<commit_message>
chore: update IPO data 2026-09-15
</commit_message>
<xml_diff>
--- a/IPO_analysis.xlsx
+++ b/IPO_analysis.xlsx
@@ -618,7 +618,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>기준일 2026-09-14 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
+          <t>기준일 2026-09-15 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
         </is>
       </c>
     </row>
@@ -11298,7 +11298,11 @@
           <t>09-10~09-11</t>
         </is>
       </c>
-      <c r="K49" s="6" t="inlineStr"/>
+      <c r="K49" s="6" t="inlineStr">
+        <is>
+          <t>4,885.53</t>
+        </is>
+      </c>
       <c r="L49" s="6" t="inlineStr"/>
       <c r="M49" s="6" t="inlineStr"/>
       <c r="N49" s="6" t="inlineStr">
@@ -11319,7 +11323,7 @@
       </c>
       <c r="R49" s="6" t="inlineStr">
         <is>
-          <t>발행조건확정</t>
+          <t>청약완료·상장대기</t>
         </is>
       </c>
     </row>
@@ -11370,7 +11374,11 @@
           <t>09-10~09-11</t>
         </is>
       </c>
-      <c r="K50" s="6" t="inlineStr"/>
+      <c r="K50" s="6" t="inlineStr">
+        <is>
+          <t>6,777.78</t>
+        </is>
+      </c>
       <c r="L50" s="6" t="inlineStr"/>
       <c r="M50" s="6" t="inlineStr"/>
       <c r="N50" s="18" t="inlineStr">
@@ -11391,146 +11399,150 @@
       </c>
       <c r="R50" s="6" t="inlineStr">
         <is>
-          <t>발행조건확정</t>
+          <t>청약완료·상장대기</t>
         </is>
       </c>
     </row>
     <row r="51" ht="30" customHeight="1">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>와이즈플래닛컴퍼니</t>
+          <t>한국제17호스팩</t>
         </is>
       </c>
       <c r="B51" s="6" t="inlineStr">
         <is>
-          <t>09-04~09-10</t>
-        </is>
-      </c>
-      <c r="C51" s="6" t="inlineStr">
-        <is>
-          <t>10,000~12,000</t>
+          <t>09-07~09-08</t>
+        </is>
+      </c>
+      <c r="C51" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="D51" s="7" t="inlineStr">
         <is>
-          <t>1,600,000</t>
+          <t>7,000,000</t>
         </is>
       </c>
       <c r="E51" s="7" t="inlineStr">
         <is>
-          <t>19,200,000,000</t>
-        </is>
-      </c>
-      <c r="F51" s="6" t="inlineStr">
-        <is>
-          <t>20.04배 (PER)</t>
+          <t>14,000,000,000</t>
+        </is>
+      </c>
+      <c r="F51" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
-          <t>12,000</t>
+          <t>2,000</t>
         </is>
       </c>
       <c r="H51" s="6" t="n">
-        <v>1248.47</v>
+        <v>1270.51</v>
       </c>
       <c r="I51" s="6" t="n">
-        <v>2323</v>
+        <v>2040</v>
       </c>
       <c r="J51" s="6" t="inlineStr">
         <is>
-          <t>09-14~09-15</t>
-        </is>
-      </c>
-      <c r="K51" s="6" t="inlineStr"/>
+          <t>09-10~09-11</t>
+        </is>
+      </c>
+      <c r="K51" s="6" t="inlineStr">
+        <is>
+          <t>8,291.55</t>
+        </is>
+      </c>
       <c r="L51" s="6" t="inlineStr"/>
       <c r="M51" s="6" t="inlineStr"/>
-      <c r="N51" s="6" t="inlineStr">
-        <is>
-          <t>대신증권</t>
+      <c r="N51" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="O51" s="6" t="inlineStr"/>
-      <c r="P51" s="7" t="inlineStr">
-        <is>
-          <t>494,400,000</t>
+      <c r="P51" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="Q51" s="6" t="inlineStr">
         <is>
-          <t>3.0%</t>
+          <t>50%</t>
         </is>
       </c>
       <c r="R51" s="6" t="inlineStr">
         <is>
-          <t>발행조건확정</t>
+          <t>청약완료·상장대기</t>
         </is>
       </c>
     </row>
     <row r="52" ht="30" customHeight="1">
       <c r="A52" s="6" t="inlineStr">
         <is>
-          <t>한국제17호스팩</t>
+          <t>와이즈플래닛컴퍼니</t>
         </is>
       </c>
       <c r="B52" s="6" t="inlineStr">
         <is>
-          <t>09-07~09-08</t>
-        </is>
-      </c>
-      <c r="C52" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>09-04~09-10</t>
+        </is>
+      </c>
+      <c r="C52" s="6" t="inlineStr">
+        <is>
+          <t>10,000~12,000</t>
         </is>
       </c>
       <c r="D52" s="7" t="inlineStr">
         <is>
-          <t>7,000,000</t>
+          <t>1,600,000</t>
         </is>
       </c>
       <c r="E52" s="7" t="inlineStr">
         <is>
-          <t>14,000,000,000</t>
-        </is>
-      </c>
-      <c r="F52" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>19,200,000,000</t>
+        </is>
+      </c>
+      <c r="F52" s="6" t="inlineStr">
+        <is>
+          <t>20.04배 (PER)</t>
         </is>
       </c>
       <c r="G52" s="6" t="inlineStr">
         <is>
-          <t>2,000</t>
+          <t>12,000</t>
         </is>
       </c>
       <c r="H52" s="6" t="n">
-        <v>1270.51</v>
+        <v>1248.47</v>
       </c>
       <c r="I52" s="6" t="n">
-        <v>2040</v>
+        <v>2323</v>
       </c>
       <c r="J52" s="6" t="inlineStr">
         <is>
-          <t>09-10~09-11</t>
+          <t>09-14~09-15</t>
         </is>
       </c>
       <c r="K52" s="6" t="inlineStr"/>
       <c r="L52" s="6" t="inlineStr"/>
       <c r="M52" s="6" t="inlineStr"/>
-      <c r="N52" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="N52" s="6" t="inlineStr">
+        <is>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="O52" s="6" t="inlineStr"/>
-      <c r="P52" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="P52" s="7" t="inlineStr">
+        <is>
+          <t>494,400,000</t>
         </is>
       </c>
       <c r="Q52" s="6" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>3.0%</t>
         </is>
       </c>
       <c r="R52" s="6" t="inlineStr">
@@ -11618,40 +11630,48 @@
     <row r="54" ht="30" customHeight="1">
       <c r="A54" s="6" t="inlineStr">
         <is>
-          <t>브릴스</t>
+          <t>글로벌테크놀로지</t>
         </is>
       </c>
       <c r="B54" s="6" t="inlineStr">
         <is>
-          <t>08-31~09-04</t>
+          <t>09-07~09-11</t>
         </is>
       </c>
       <c r="C54" s="6" t="inlineStr">
         <is>
-          <t>16,500~19,500</t>
+          <t>13,000~15,000</t>
         </is>
       </c>
       <c r="D54" s="7" t="inlineStr">
         <is>
-          <t>1,200,000</t>
+          <t>4,000,000</t>
         </is>
       </c>
       <c r="E54" s="7" t="inlineStr">
         <is>
-          <t>19,800,000,000</t>
+          <t>40,000,000,000</t>
         </is>
       </c>
       <c r="F54" s="6" t="inlineStr">
         <is>
-          <t>13.44 (PSR)</t>
-        </is>
-      </c>
-      <c r="G54" s="6" t="inlineStr"/>
-      <c r="H54" s="6" t="inlineStr"/>
-      <c r="I54" s="6" t="inlineStr"/>
+          <t>19.22배 (PER)</t>
+        </is>
+      </c>
+      <c r="G54" s="6" t="inlineStr">
+        <is>
+          <t>10,000</t>
+        </is>
+      </c>
+      <c r="H54" s="6" t="n">
+        <v>123.19</v>
+      </c>
+      <c r="I54" s="6" t="n">
+        <v>961</v>
+      </c>
       <c r="J54" s="6" t="inlineStr">
         <is>
-          <t>09-08~09-09</t>
+          <t>09-16~09-17</t>
         </is>
       </c>
       <c r="K54" s="6" t="inlineStr"/>
@@ -11659,60 +11679,68 @@
       <c r="M54" s="6" t="inlineStr"/>
       <c r="N54" s="6" t="inlineStr">
         <is>
-          <t>아이비케이투자증권</t>
+          <t>한국투자증권</t>
         </is>
       </c>
       <c r="O54" s="6" t="inlineStr"/>
       <c r="P54" s="7" t="inlineStr">
         <is>
-          <t>713,790,000</t>
-        </is>
-      </c>
-      <c r="Q54" s="6" t="inlineStr">
-        <is>
-          <t>3.5%</t>
+          <t>2,119,999,960</t>
+        </is>
+      </c>
+      <c r="Q54" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="R54" s="6" t="inlineStr">
         <is>
-          <t>정정</t>
+          <t>발행조건확정</t>
         </is>
       </c>
     </row>
     <row r="55" ht="30" customHeight="1">
       <c r="A55" s="6" t="inlineStr">
         <is>
-          <t>글로벌테크놀로지</t>
+          <t>덕산넵코어스</t>
         </is>
       </c>
       <c r="B55" s="6" t="inlineStr">
         <is>
-          <t>09-07~09-11</t>
+          <t>09-08~09-14</t>
         </is>
       </c>
       <c r="C55" s="6" t="inlineStr">
         <is>
-          <t>13,000~15,000</t>
+          <t>12,400~14,600</t>
         </is>
       </c>
       <c r="D55" s="7" t="inlineStr">
         <is>
-          <t>4,000,000</t>
+          <t>3,000,000</t>
         </is>
       </c>
       <c r="E55" s="7" t="inlineStr">
         <is>
-          <t>52,000,000,000</t>
+          <t>43,800,000,000</t>
         </is>
       </c>
       <c r="F55" s="6" t="inlineStr">
         <is>
-          <t>19.22배 (PER)</t>
-        </is>
-      </c>
-      <c r="G55" s="6" t="inlineStr"/>
-      <c r="H55" s="6" t="inlineStr"/>
-      <c r="I55" s="6" t="inlineStr"/>
+          <t>32.57배 (PER)</t>
+        </is>
+      </c>
+      <c r="G55" s="6" t="inlineStr">
+        <is>
+          <t>14,600</t>
+        </is>
+      </c>
+      <c r="H55" s="6" t="n">
+        <v>868.64</v>
+      </c>
+      <c r="I55" s="6" t="n">
+        <v>2269</v>
+      </c>
       <c r="J55" s="6" t="inlineStr">
         <is>
           <t>09-16~09-17</t>
@@ -11723,55 +11751,55 @@
       <c r="M55" s="6" t="inlineStr"/>
       <c r="N55" s="6" t="inlineStr">
         <is>
-          <t>한국투자증권</t>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="O55" s="6" t="inlineStr"/>
       <c r="P55" s="7" t="inlineStr">
         <is>
-          <t>2,119,999,960</t>
-        </is>
-      </c>
-      <c r="Q55" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>1,413,399,926</t>
+        </is>
+      </c>
+      <c r="Q55" s="6" t="inlineStr">
+        <is>
+          <t>3.7%</t>
         </is>
       </c>
       <c r="R55" s="6" t="inlineStr">
         <is>
-          <t>정정</t>
+          <t>발행조건확정</t>
         </is>
       </c>
     </row>
     <row r="56" ht="30" customHeight="1">
       <c r="A56" s="6" t="inlineStr">
         <is>
-          <t>덕산넵코어스</t>
+          <t>브릴스</t>
         </is>
       </c>
       <c r="B56" s="6" t="inlineStr">
         <is>
-          <t>09-08~09-14</t>
+          <t>08-31~09-04</t>
         </is>
       </c>
       <c r="C56" s="6" t="inlineStr">
         <is>
-          <t>12,400~14,600</t>
+          <t>16,500~19,500</t>
         </is>
       </c>
       <c r="D56" s="7" t="inlineStr">
         <is>
-          <t>3,000,000</t>
+          <t>1,200,000</t>
         </is>
       </c>
       <c r="E56" s="7" t="inlineStr">
         <is>
-          <t>37,200,000,000</t>
+          <t>19,800,000,000</t>
         </is>
       </c>
       <c r="F56" s="6" t="inlineStr">
         <is>
-          <t>32.57배 (PER)</t>
+          <t>13.44 (PSR)</t>
         </is>
       </c>
       <c r="G56" s="6" t="inlineStr"/>
@@ -11779,7 +11807,7 @@
       <c r="I56" s="6" t="inlineStr"/>
       <c r="J56" s="6" t="inlineStr">
         <is>
-          <t>09-16~09-17</t>
+          <t>09-08~09-09</t>
         </is>
       </c>
       <c r="K56" s="6" t="inlineStr"/>
@@ -11787,18 +11815,18 @@
       <c r="M56" s="6" t="inlineStr"/>
       <c r="N56" s="6" t="inlineStr">
         <is>
-          <t>대신증권</t>
+          <t>아이비케이투자증권</t>
         </is>
       </c>
       <c r="O56" s="6" t="inlineStr"/>
       <c r="P56" s="7" t="inlineStr">
         <is>
-          <t>1,413,399,926</t>
+          <t>713,790,000</t>
         </is>
       </c>
       <c r="Q56" s="6" t="inlineStr">
         <is>
-          <t>3.7%</t>
+          <t>3.5%</t>
         </is>
       </c>
       <c r="R56" s="6" t="inlineStr">
@@ -12390,32 +12418,32 @@
     <row r="66" ht="30" customHeight="1">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>크리에이츠</t>
+          <t>다비오</t>
         </is>
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
-          <t>10-12~10-16</t>
+          <t>10-07~10-14</t>
         </is>
       </c>
       <c r="C66" s="6" t="inlineStr">
         <is>
-          <t>15,000~18,000</t>
+          <t>12,300~16,600</t>
         </is>
       </c>
       <c r="D66" s="7" t="inlineStr">
         <is>
-          <t>1,400,000</t>
+          <t>1,000,000</t>
         </is>
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
-          <t>21,000,000,000</t>
+          <t>12,300,000,000</t>
         </is>
       </c>
       <c r="F66" s="6" t="inlineStr">
         <is>
-          <t>19.15배 (PER)</t>
+          <t>26.70배 (PER)</t>
         </is>
       </c>
       <c r="G66" s="6" t="inlineStr"/>
@@ -12423,7 +12451,7 @@
       <c r="I66" s="6" t="inlineStr"/>
       <c r="J66" s="6" t="inlineStr">
         <is>
-          <t>10-20~10-21</t>
+          <t>10-19~10-20</t>
         </is>
       </c>
       <c r="K66" s="6" t="inlineStr"/>
@@ -12431,18 +12459,18 @@
       <c r="M66" s="6" t="inlineStr"/>
       <c r="N66" s="6" t="inlineStr">
         <is>
-          <t>삼성증권</t>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="O66" s="6" t="inlineStr"/>
       <c r="P66" s="7" t="inlineStr">
         <is>
-          <t>865,200,000</t>
+          <t>570,105,000</t>
         </is>
       </c>
       <c r="Q66" s="6" t="inlineStr">
         <is>
-          <t>4.0%</t>
+          <t>4.5%</t>
         </is>
       </c>
       <c r="R66" s="6" t="inlineStr">
@@ -12454,59 +12482,59 @@
     <row r="67" ht="30" customHeight="1">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>바로팜</t>
-        </is>
-      </c>
-      <c r="B67" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>크리에이츠</t>
+        </is>
+      </c>
+      <c r="B67" s="6" t="inlineStr">
+        <is>
+          <t>10-12~10-16</t>
         </is>
       </c>
       <c r="C67" s="6" t="inlineStr">
         <is>
-          <t>16,400~20,200</t>
+          <t>15,000~18,000</t>
         </is>
       </c>
       <c r="D67" s="7" t="inlineStr">
         <is>
-          <t>1,780,000</t>
+          <t>1,400,000</t>
         </is>
       </c>
       <c r="E67" s="7" t="inlineStr">
         <is>
-          <t>29,192,000,000</t>
+          <t>21,000,000,000</t>
         </is>
       </c>
       <c r="F67" s="6" t="inlineStr">
         <is>
-          <t>24.95배 (PER)</t>
+          <t>19.15배 (PER)</t>
         </is>
       </c>
       <c r="G67" s="6" t="inlineStr"/>
       <c r="H67" s="6" t="inlineStr"/>
       <c r="I67" s="6" t="inlineStr"/>
-      <c r="J67" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="J67" s="6" t="inlineStr">
+        <is>
+          <t>10-20~10-21</t>
         </is>
       </c>
       <c r="K67" s="6" t="inlineStr"/>
       <c r="L67" s="6" t="inlineStr"/>
       <c r="M67" s="6" t="inlineStr"/>
-      <c r="N67" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="N67" s="6" t="inlineStr">
+        <is>
+          <t>삼성증권</t>
         </is>
       </c>
       <c r="O67" s="6" t="inlineStr"/>
-      <c r="P67" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="Q67" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="P67" s="7" t="inlineStr">
+        <is>
+          <t>865,200,000</t>
+        </is>
+      </c>
+      <c r="Q67" s="6" t="inlineStr">
+        <is>
+          <t>4.0%</t>
         </is>
       </c>
       <c r="R67" s="6" t="inlineStr">
@@ -12518,7 +12546,7 @@
     <row r="68" ht="30" customHeight="1">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>디티에스</t>
+          <t>바로팜</t>
         </is>
       </c>
       <c r="B68" s="18" t="inlineStr">
@@ -12526,24 +12554,24 @@
           <t>수집예정</t>
         </is>
       </c>
-      <c r="C68" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="D68" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="E68" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="F68" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="C68" s="6" t="inlineStr">
+        <is>
+          <t>16,400~20,200</t>
+        </is>
+      </c>
+      <c r="D68" s="7" t="inlineStr">
+        <is>
+          <t>1,780,000</t>
+        </is>
+      </c>
+      <c r="E68" s="7" t="inlineStr">
+        <is>
+          <t>29,192,000,000</t>
+        </is>
+      </c>
+      <c r="F68" s="6" t="inlineStr">
+        <is>
+          <t>24.95배 (PER)</t>
         </is>
       </c>
       <c r="G68" s="6" t="inlineStr"/>
@@ -12575,14 +12603,14 @@
       </c>
       <c r="R68" s="6" t="inlineStr">
         <is>
-          <t>신고서 대기</t>
+          <t>최초</t>
         </is>
       </c>
     </row>
     <row r="69" ht="30" customHeight="1">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>한화플러스제6호스팩</t>
+          <t>디티에스</t>
         </is>
       </c>
       <c r="B69" s="18" t="inlineStr">
@@ -12646,7 +12674,7 @@
     <row r="70" ht="30" customHeight="1">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>다비오</t>
+          <t>한화플러스제6호스팩</t>
         </is>
       </c>
       <c r="B70" s="18" t="inlineStr">
@@ -13628,7 +13656,7 @@
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>한국투자증권</t>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="B22" s="6" t="n">
@@ -13636,22 +13664,22 @@
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>122,800,000,000</t>
+          <t>122,050,000,000</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>대신증권</t>
+          <t>한국투자증권</t>
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>103,150,000,000</t>
+          <t>110,800,000,000</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update IPO data 2026-09-16
</commit_message>
<xml_diff>
--- a/IPO_analysis.xlsx
+++ b/IPO_analysis.xlsx
@@ -618,7 +618,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>기준일 2026-09-15 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
+          <t>기준일 2026-09-16 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
         </is>
       </c>
     </row>
@@ -11482,48 +11482,48 @@
     <row r="52" ht="30" customHeight="1">
       <c r="A52" s="6" t="inlineStr">
         <is>
-          <t>와이즈플래닛컴퍼니</t>
+          <t>브릴스</t>
         </is>
       </c>
       <c r="B52" s="6" t="inlineStr">
         <is>
-          <t>09-04~09-10</t>
+          <t>08-31~09-04</t>
         </is>
       </c>
       <c r="C52" s="6" t="inlineStr">
         <is>
-          <t>10,000~12,000</t>
+          <t>16,500~19,500</t>
         </is>
       </c>
       <c r="D52" s="7" t="inlineStr">
         <is>
-          <t>1,600,000</t>
+          <t>1,200,000</t>
         </is>
       </c>
       <c r="E52" s="7" t="inlineStr">
         <is>
-          <t>19,200,000,000</t>
+          <t>23,400,000,000</t>
         </is>
       </c>
       <c r="F52" s="6" t="inlineStr">
         <is>
-          <t>20.04배 (PER)</t>
+          <t>13.44 (PSR)</t>
         </is>
       </c>
       <c r="G52" s="6" t="inlineStr">
         <is>
-          <t>12,000</t>
+          <t>19,500</t>
         </is>
       </c>
       <c r="H52" s="6" t="n">
-        <v>1248.47</v>
+        <v>1187.74</v>
       </c>
       <c r="I52" s="6" t="n">
-        <v>2323</v>
+        <v>2181</v>
       </c>
       <c r="J52" s="6" t="inlineStr">
         <is>
-          <t>09-14~09-15</t>
+          <t>09-08~09-09</t>
         </is>
       </c>
       <c r="K52" s="6" t="inlineStr"/>
@@ -11531,18 +11531,18 @@
       <c r="M52" s="6" t="inlineStr"/>
       <c r="N52" s="6" t="inlineStr">
         <is>
-          <t>대신증권</t>
+          <t>아이비케이투자증권</t>
         </is>
       </c>
       <c r="O52" s="6" t="inlineStr"/>
       <c r="P52" s="7" t="inlineStr">
         <is>
-          <t>494,400,000</t>
+          <t>713,790,000</t>
         </is>
       </c>
       <c r="Q52" s="6" t="inlineStr">
         <is>
-          <t>3.0%</t>
+          <t>3.5%</t>
         </is>
       </c>
       <c r="R52" s="6" t="inlineStr">
@@ -11554,17 +11554,17 @@
     <row r="53" ht="30" customHeight="1">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t>빅웨이브로보틱스</t>
+          <t>와이즈플래닛컴퍼니</t>
         </is>
       </c>
       <c r="B53" s="6" t="inlineStr">
         <is>
-          <t>09-07~09-11</t>
+          <t>09-04~09-10</t>
         </is>
       </c>
       <c r="C53" s="6" t="inlineStr">
         <is>
-          <t>15,000~18,000</t>
+          <t>10,000~12,000</t>
         </is>
       </c>
       <c r="D53" s="7" t="inlineStr">
@@ -11574,28 +11574,28 @@
       </c>
       <c r="E53" s="7" t="inlineStr">
         <is>
-          <t>28,800,000,000</t>
+          <t>19,200,000,000</t>
         </is>
       </c>
       <c r="F53" s="6" t="inlineStr">
         <is>
-          <t>11.15 (PSR)</t>
+          <t>20.04배 (PER)</t>
         </is>
       </c>
       <c r="G53" s="6" t="inlineStr">
         <is>
-          <t>18,000</t>
+          <t>12,000</t>
         </is>
       </c>
       <c r="H53" s="6" t="n">
-        <v>1109.37</v>
+        <v>1248.47</v>
       </c>
       <c r="I53" s="6" t="n">
-        <v>2255</v>
+        <v>2323</v>
       </c>
       <c r="J53" s="6" t="inlineStr">
         <is>
-          <t>09-15~09-16</t>
+          <t>09-14~09-15</t>
         </is>
       </c>
       <c r="K53" s="6" t="inlineStr"/>
@@ -11603,17 +11603,13 @@
       <c r="M53" s="6" t="inlineStr"/>
       <c r="N53" s="6" t="inlineStr">
         <is>
-          <t>유진투자증권</t>
-        </is>
-      </c>
-      <c r="O53" s="6" t="inlineStr">
-        <is>
-          <t>미래</t>
-        </is>
-      </c>
+          <t>대신증권</t>
+        </is>
+      </c>
+      <c r="O53" s="6" t="inlineStr"/>
       <c r="P53" s="7" t="inlineStr">
         <is>
-          <t>378,216,000</t>
+          <t>494,400,000</t>
         </is>
       </c>
       <c r="Q53" s="6" t="inlineStr">
@@ -11630,7 +11626,7 @@
     <row r="54" ht="30" customHeight="1">
       <c r="A54" s="6" t="inlineStr">
         <is>
-          <t>글로벌테크놀로지</t>
+          <t>빅웨이브로보틱스</t>
         </is>
       </c>
       <c r="B54" s="6" t="inlineStr">
@@ -11640,38 +11636,38 @@
       </c>
       <c r="C54" s="6" t="inlineStr">
         <is>
-          <t>13,000~15,000</t>
+          <t>15,000~18,000</t>
         </is>
       </c>
       <c r="D54" s="7" t="inlineStr">
         <is>
-          <t>4,000,000</t>
+          <t>1,600,000</t>
         </is>
       </c>
       <c r="E54" s="7" t="inlineStr">
         <is>
-          <t>40,000,000,000</t>
+          <t>28,800,000,000</t>
         </is>
       </c>
       <c r="F54" s="6" t="inlineStr">
         <is>
-          <t>19.22배 (PER)</t>
+          <t>11.15 (PSR)</t>
         </is>
       </c>
       <c r="G54" s="6" t="inlineStr">
         <is>
-          <t>10,000</t>
+          <t>18,000</t>
         </is>
       </c>
       <c r="H54" s="6" t="n">
-        <v>123.19</v>
+        <v>1109.37</v>
       </c>
       <c r="I54" s="6" t="n">
-        <v>961</v>
+        <v>2255</v>
       </c>
       <c r="J54" s="6" t="inlineStr">
         <is>
-          <t>09-16~09-17</t>
+          <t>09-15~09-16</t>
         </is>
       </c>
       <c r="K54" s="6" t="inlineStr"/>
@@ -11679,18 +11675,22 @@
       <c r="M54" s="6" t="inlineStr"/>
       <c r="N54" s="6" t="inlineStr">
         <is>
-          <t>한국투자증권</t>
-        </is>
-      </c>
-      <c r="O54" s="6" t="inlineStr"/>
+          <t>유진투자증권</t>
+        </is>
+      </c>
+      <c r="O54" s="6" t="inlineStr">
+        <is>
+          <t>미래</t>
+        </is>
+      </c>
       <c r="P54" s="7" t="inlineStr">
         <is>
-          <t>2,119,999,960</t>
-        </is>
-      </c>
-      <c r="Q54" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>378,216,000</t>
+        </is>
+      </c>
+      <c r="Q54" s="6" t="inlineStr">
+        <is>
+          <t>3.0%</t>
         </is>
       </c>
       <c r="R54" s="6" t="inlineStr">
@@ -11702,44 +11702,44 @@
     <row r="55" ht="30" customHeight="1">
       <c r="A55" s="6" t="inlineStr">
         <is>
-          <t>덕산넵코어스</t>
+          <t>글로벌테크놀로지</t>
         </is>
       </c>
       <c r="B55" s="6" t="inlineStr">
         <is>
-          <t>09-08~09-14</t>
+          <t>09-07~09-11</t>
         </is>
       </c>
       <c r="C55" s="6" t="inlineStr">
         <is>
-          <t>12,400~14,600</t>
+          <t>13,000~15,000</t>
         </is>
       </c>
       <c r="D55" s="7" t="inlineStr">
         <is>
-          <t>3,000,000</t>
+          <t>4,000,000</t>
         </is>
       </c>
       <c r="E55" s="7" t="inlineStr">
         <is>
-          <t>43,800,000,000</t>
+          <t>40,000,000,000</t>
         </is>
       </c>
       <c r="F55" s="6" t="inlineStr">
         <is>
-          <t>32.57배 (PER)</t>
+          <t>19.22배 (PER)</t>
         </is>
       </c>
       <c r="G55" s="6" t="inlineStr">
         <is>
-          <t>14,600</t>
+          <t>10,000</t>
         </is>
       </c>
       <c r="H55" s="6" t="n">
-        <v>868.64</v>
+        <v>123.19</v>
       </c>
       <c r="I55" s="6" t="n">
-        <v>2269</v>
+        <v>961</v>
       </c>
       <c r="J55" s="6" t="inlineStr">
         <is>
@@ -11751,18 +11751,18 @@
       <c r="M55" s="6" t="inlineStr"/>
       <c r="N55" s="6" t="inlineStr">
         <is>
-          <t>대신증권</t>
+          <t>한국투자증권</t>
         </is>
       </c>
       <c r="O55" s="6" t="inlineStr"/>
       <c r="P55" s="7" t="inlineStr">
         <is>
-          <t>1,413,399,926</t>
-        </is>
-      </c>
-      <c r="Q55" s="6" t="inlineStr">
-        <is>
-          <t>3.7%</t>
+          <t>2,119,999,960</t>
+        </is>
+      </c>
+      <c r="Q55" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="R55" s="6" t="inlineStr">
@@ -11774,40 +11774,48 @@
     <row r="56" ht="30" customHeight="1">
       <c r="A56" s="6" t="inlineStr">
         <is>
-          <t>브릴스</t>
+          <t>덕산넵코어스</t>
         </is>
       </c>
       <c r="B56" s="6" t="inlineStr">
         <is>
-          <t>08-31~09-04</t>
+          <t>09-08~09-14</t>
         </is>
       </c>
       <c r="C56" s="6" t="inlineStr">
         <is>
-          <t>16,500~19,500</t>
+          <t>12,400~14,600</t>
         </is>
       </c>
       <c r="D56" s="7" t="inlineStr">
         <is>
-          <t>1,200,000</t>
+          <t>3,000,000</t>
         </is>
       </c>
       <c r="E56" s="7" t="inlineStr">
         <is>
-          <t>19,800,000,000</t>
+          <t>43,800,000,000</t>
         </is>
       </c>
       <c r="F56" s="6" t="inlineStr">
         <is>
-          <t>13.44 (PSR)</t>
-        </is>
-      </c>
-      <c r="G56" s="6" t="inlineStr"/>
-      <c r="H56" s="6" t="inlineStr"/>
-      <c r="I56" s="6" t="inlineStr"/>
+          <t>32.57배 (PER)</t>
+        </is>
+      </c>
+      <c r="G56" s="6" t="inlineStr">
+        <is>
+          <t>14,600</t>
+        </is>
+      </c>
+      <c r="H56" s="6" t="n">
+        <v>868.64</v>
+      </c>
+      <c r="I56" s="6" t="n">
+        <v>2269</v>
+      </c>
       <c r="J56" s="6" t="inlineStr">
         <is>
-          <t>09-08~09-09</t>
+          <t>09-16~09-17</t>
         </is>
       </c>
       <c r="K56" s="6" t="inlineStr"/>
@@ -11815,23 +11823,23 @@
       <c r="M56" s="6" t="inlineStr"/>
       <c r="N56" s="6" t="inlineStr">
         <is>
-          <t>아이비케이투자증권</t>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="O56" s="6" t="inlineStr"/>
       <c r="P56" s="7" t="inlineStr">
         <is>
-          <t>713,790,000</t>
+          <t>1,413,399,926</t>
         </is>
       </c>
       <c r="Q56" s="6" t="inlineStr">
         <is>
-          <t>3.5%</t>
+          <t>3.7%</t>
         </is>
       </c>
       <c r="R56" s="6" t="inlineStr">
         <is>
-          <t>정정</t>
+          <t>발행조건확정</t>
         </is>
       </c>
     </row>
@@ -12546,59 +12554,59 @@
     <row r="68" ht="30" customHeight="1">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>바로팜</t>
-        </is>
-      </c>
-      <c r="B68" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>인텔리빅스</t>
+        </is>
+      </c>
+      <c r="B68" s="6" t="inlineStr">
+        <is>
+          <t>10-12~10-16</t>
         </is>
       </c>
       <c r="C68" s="6" t="inlineStr">
         <is>
-          <t>16,400~20,200</t>
+          <t>7,600~9,000</t>
         </is>
       </c>
       <c r="D68" s="7" t="inlineStr">
         <is>
-          <t>1,780,000</t>
+          <t>2,500,000</t>
         </is>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
-          <t>29,192,000,000</t>
+          <t>19,000,000,000</t>
         </is>
       </c>
       <c r="F68" s="6" t="inlineStr">
         <is>
-          <t>24.95배 (PER)</t>
+          <t>22.02배 (PER)</t>
         </is>
       </c>
       <c r="G68" s="6" t="inlineStr"/>
       <c r="H68" s="6" t="inlineStr"/>
       <c r="I68" s="6" t="inlineStr"/>
-      <c r="J68" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="J68" s="6" t="inlineStr">
+        <is>
+          <t>10-21~10-22</t>
         </is>
       </c>
       <c r="K68" s="6" t="inlineStr"/>
       <c r="L68" s="6" t="inlineStr"/>
       <c r="M68" s="6" t="inlineStr"/>
-      <c r="N68" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="N68" s="6" t="inlineStr">
+        <is>
+          <t>미래에셋증권</t>
         </is>
       </c>
       <c r="O68" s="6" t="inlineStr"/>
-      <c r="P68" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="Q68" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="P68" s="7" t="inlineStr">
+        <is>
+          <t>782,800,000</t>
+        </is>
+      </c>
+      <c r="Q68" s="6" t="inlineStr">
+        <is>
+          <t>4.0%</t>
         </is>
       </c>
       <c r="R68" s="6" t="inlineStr">
@@ -12610,7 +12618,7 @@
     <row r="69" ht="30" customHeight="1">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>디티에스</t>
+          <t>바로팜</t>
         </is>
       </c>
       <c r="B69" s="18" t="inlineStr">
@@ -12618,24 +12626,24 @@
           <t>수집예정</t>
         </is>
       </c>
-      <c r="C69" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="D69" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="E69" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="F69" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="C69" s="6" t="inlineStr">
+        <is>
+          <t>16,400~20,200</t>
+        </is>
+      </c>
+      <c r="D69" s="7" t="inlineStr">
+        <is>
+          <t>1,780,000</t>
+        </is>
+      </c>
+      <c r="E69" s="7" t="inlineStr">
+        <is>
+          <t>29,192,000,000</t>
+        </is>
+      </c>
+      <c r="F69" s="6" t="inlineStr">
+        <is>
+          <t>24.95배 (PER)</t>
         </is>
       </c>
       <c r="G69" s="6" t="inlineStr"/>
@@ -12667,14 +12675,14 @@
       </c>
       <c r="R69" s="6" t="inlineStr">
         <is>
-          <t>신고서 대기</t>
+          <t>최초</t>
         </is>
       </c>
     </row>
     <row r="70" ht="30" customHeight="1">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>한화플러스제6호스팩</t>
+          <t>디티에스</t>
         </is>
       </c>
       <c r="B70" s="18" t="inlineStr">
@@ -12738,7 +12746,7 @@
     <row r="71" ht="30" customHeight="1">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>하나에어로다이내믹스</t>
+          <t>한화플러스제6호스팩</t>
         </is>
       </c>
       <c r="B71" s="18" t="inlineStr">
@@ -12802,7 +12810,7 @@
     <row r="72" ht="30" customHeight="1">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>에이엔에이치스트럭쳐</t>
+          <t>하나에어로다이내믹스</t>
         </is>
       </c>
       <c r="B72" s="18" t="inlineStr">
@@ -12866,7 +12874,7 @@
     <row r="73" ht="30" customHeight="1">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>인텔리빅스</t>
+          <t>에이엔에이치스트럭쳐</t>
         </is>
       </c>
       <c r="B73" s="18" t="inlineStr">
@@ -13671,30 +13679,30 @@
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>한국투자증권</t>
+          <t>미래에셋증권</t>
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>110,800,000,000</t>
+          <t>115,560,000,000</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>미래에셋증권</t>
+          <t>한국투자증권</t>
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>96,560,000,000</t>
+          <t>110,800,000,000</t>
         </is>
       </c>
     </row>
@@ -13709,7 +13717,7 @@
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>72,600,000,000</t>
+          <t>76,200,000,000</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update IPO data 2026-09-28
</commit_message>
<xml_diff>
--- a/IPO_analysis.xlsx
+++ b/IPO_analysis.xlsx
@@ -618,14 +618,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>기준일 2026-09-27 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
+          <t>기준일 2026-09-28 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>■ 심사 신청(진행중)  (47건)</t>
+          <t>■ 심사 신청(진행중)  (44건)</t>
         </is>
       </c>
       <c r="B4" s="4" t="n"/>
@@ -1910,7 +1910,7 @@
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>솔리스</t>
+          <t>이노보테라퓨틱스</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
@@ -1920,7 +1920,7 @@
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
-          <t>스팩 소멸합병</t>
+          <t>신규상장</t>
         </is>
       </c>
       <c r="E28" s="6" t="inlineStr">
@@ -1928,17 +1928,29 @@
           <t>FY25</t>
         </is>
       </c>
-      <c r="F28" s="7" t="inlineStr"/>
-      <c r="G28" s="7" t="inlineStr"/>
-      <c r="H28" s="7" t="inlineStr"/>
+      <c r="F28" s="7" t="inlineStr">
+        <is>
+          <t>209</t>
+        </is>
+      </c>
+      <c r="G28" s="7" t="inlineStr">
+        <is>
+          <t>-5,429</t>
+        </is>
+      </c>
+      <c r="H28" s="7" t="inlineStr">
+        <is>
+          <t>-53,200</t>
+        </is>
+      </c>
       <c r="I28" s="6" t="inlineStr">
         <is>
-          <t>금융 지원 서비스업</t>
+          <t>의약품 제조업</t>
         </is>
       </c>
       <c r="J28" s="6" t="inlineStr">
         <is>
-          <t>한화</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="K28" s="6" t="inlineStr">
@@ -1950,17 +1962,17 @@
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>이노보테라퓨틱스</t>
+          <t>에스에프씨</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>코스닥</t>
+          <t>유가</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr">
@@ -1975,27 +1987,27 @@
       </c>
       <c r="F29" s="7" t="inlineStr">
         <is>
-          <t>209</t>
+          <t>160,792</t>
         </is>
       </c>
       <c r="G29" s="7" t="inlineStr">
         <is>
-          <t>-5,429</t>
+          <t>25,509</t>
         </is>
       </c>
       <c r="H29" s="7" t="inlineStr">
         <is>
-          <t>-53,200</t>
+          <t>243,562</t>
         </is>
       </c>
       <c r="I29" s="6" t="inlineStr">
         <is>
-          <t>의약품 제조업</t>
+          <t>기타 화학제품 제조업</t>
         </is>
       </c>
       <c r="J29" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>미래, 한국</t>
         </is>
       </c>
       <c r="K29" s="6" t="inlineStr">
@@ -2007,17 +2019,17 @@
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>에스에프씨</t>
+          <t>아델</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>유가</t>
+          <t>코스닥</t>
         </is>
       </c>
       <c r="D30" s="6" t="inlineStr">
@@ -2032,27 +2044,27 @@
       </c>
       <c r="F30" s="7" t="inlineStr">
         <is>
-          <t>160,792</t>
+          <t>62,057</t>
         </is>
       </c>
       <c r="G30" s="7" t="inlineStr">
         <is>
-          <t>25,509</t>
+          <t>-64,210</t>
         </is>
       </c>
       <c r="H30" s="7" t="inlineStr">
         <is>
-          <t>243,562</t>
+          <t>-80,776</t>
         </is>
       </c>
       <c r="I30" s="6" t="inlineStr">
         <is>
-          <t>기타 화학제품 제조업</t>
+          <t>그외 기타 전문, 과학 및 기술 서비스업</t>
         </is>
       </c>
       <c r="J30" s="6" t="inlineStr">
         <is>
-          <t>미래, 한국</t>
+          <t>삼성, 미래</t>
         </is>
       </c>
       <c r="K30" s="6" t="inlineStr">
@@ -2064,12 +2076,12 @@
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>아델</t>
+          <t>에버온</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
@@ -2089,27 +2101,27 @@
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>62,057</t>
+          <t>65,225</t>
         </is>
       </c>
       <c r="G31" s="7" t="inlineStr">
         <is>
-          <t>-64,210</t>
+          <t>-3,606</t>
         </is>
       </c>
       <c r="H31" s="7" t="inlineStr">
         <is>
-          <t>-80,776</t>
+          <t>54,955</t>
         </is>
       </c>
       <c r="I31" s="6" t="inlineStr">
         <is>
-          <t>그외 기타 전문, 과학 및 기술 서비스업</t>
+          <t>전기업</t>
         </is>
       </c>
       <c r="J31" s="6" t="inlineStr">
         <is>
-          <t>삼성, 미래</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K31" s="6" t="inlineStr">
@@ -2121,12 +2133,12 @@
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>에버온</t>
+          <t>엔키화이트햇</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr">
@@ -2146,27 +2158,27 @@
       </c>
       <c r="F32" s="7" t="inlineStr">
         <is>
-          <t>65,225</t>
+          <t>14,176</t>
         </is>
       </c>
       <c r="G32" s="7" t="inlineStr">
         <is>
-          <t>-3,606</t>
+          <t>-3,211</t>
         </is>
       </c>
       <c r="H32" s="7" t="inlineStr">
         <is>
-          <t>54,955</t>
+          <t>8,338</t>
         </is>
       </c>
       <c r="I32" s="6" t="inlineStr">
         <is>
-          <t>전기업</t>
+          <t>소프트웨어 개발 및 공급업</t>
         </is>
       </c>
       <c r="J32" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>신영</t>
         </is>
       </c>
       <c r="K32" s="6" t="inlineStr">
@@ -2178,12 +2190,12 @@
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>엔키화이트햇</t>
+          <t>씨아이에스케미칼</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
@@ -2203,27 +2215,27 @@
       </c>
       <c r="F33" s="7" t="inlineStr">
         <is>
-          <t>14,176</t>
+          <t>15,985</t>
         </is>
       </c>
       <c r="G33" s="7" t="inlineStr">
         <is>
-          <t>-3,211</t>
+          <t>-11,440</t>
         </is>
       </c>
       <c r="H33" s="7" t="inlineStr">
         <is>
-          <t>8,338</t>
+          <t>23,706</t>
         </is>
       </c>
       <c r="I33" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어 개발 및 공급업</t>
+          <t>기초 화학물질 제조업</t>
         </is>
       </c>
       <c r="J33" s="6" t="inlineStr">
         <is>
-          <t>신영</t>
+          <t>KB</t>
         </is>
       </c>
       <c r="K33" s="6" t="inlineStr">
@@ -2235,12 +2247,12 @@
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>씨아이에스케미칼</t>
+          <t>엠디에스코리아</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
@@ -2260,27 +2272,27 @@
       </c>
       <c r="F34" s="7" t="inlineStr">
         <is>
-          <t>15,985</t>
+          <t>97,972</t>
         </is>
       </c>
       <c r="G34" s="7" t="inlineStr">
         <is>
-          <t>-11,440</t>
+          <t>6,512</t>
         </is>
       </c>
       <c r="H34" s="7" t="inlineStr">
         <is>
-          <t>23,706</t>
+          <t>53,818</t>
         </is>
       </c>
       <c r="I34" s="6" t="inlineStr">
         <is>
-          <t>기초 화학물질 제조업</t>
+          <t>기타 식품 제조업</t>
         </is>
       </c>
       <c r="J34" s="6" t="inlineStr">
         <is>
-          <t>KB</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K34" s="6" t="inlineStr">
@@ -2292,12 +2304,12 @@
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>엠디에스코리아</t>
+          <t>동승</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
@@ -2317,27 +2329,27 @@
       </c>
       <c r="F35" s="7" t="inlineStr">
         <is>
-          <t>97,972</t>
+          <t>78,625</t>
         </is>
       </c>
       <c r="G35" s="7" t="inlineStr">
         <is>
-          <t>6,512</t>
+          <t>14,525</t>
         </is>
       </c>
       <c r="H35" s="7" t="inlineStr">
         <is>
-          <t>53,818</t>
+          <t>5,438</t>
         </is>
       </c>
       <c r="I35" s="6" t="inlineStr">
         <is>
-          <t>기타 식품 제조업</t>
+          <t>부동산 임대 및 공급업</t>
         </is>
       </c>
       <c r="J35" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K35" s="6" t="inlineStr">
@@ -2354,7 +2366,7 @@
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>동승</t>
+          <t>에프엠더블유</t>
         </is>
       </c>
       <c r="C36" s="6" t="inlineStr">
@@ -2364,7 +2376,7 @@
       </c>
       <c r="D36" s="6" t="inlineStr">
         <is>
-          <t>신규상장</t>
+          <t>스팩 소멸합병</t>
         </is>
       </c>
       <c r="E36" s="6" t="inlineStr">
@@ -2374,27 +2386,27 @@
       </c>
       <c r="F36" s="7" t="inlineStr">
         <is>
-          <t>78,625</t>
+          <t>30,282</t>
         </is>
       </c>
       <c r="G36" s="7" t="inlineStr">
         <is>
-          <t>14,525</t>
+          <t>4,762</t>
         </is>
       </c>
       <c r="H36" s="7" t="inlineStr">
         <is>
-          <t>5,438</t>
+          <t>32</t>
         </is>
       </c>
       <c r="I36" s="6" t="inlineStr">
         <is>
-          <t>부동산 임대 및 공급업</t>
+          <t>기타 식품 제조업</t>
         </is>
       </c>
       <c r="J36" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>유진</t>
         </is>
       </c>
       <c r="K36" s="6" t="inlineStr">
@@ -2406,22 +2418,22 @@
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>셀트릭스</t>
+          <t>소노인터내셔널</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>코스닥</t>
+          <t>유가</t>
         </is>
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
-          <t>스팩 소멸합병</t>
+          <t>신규상장</t>
         </is>
       </c>
       <c r="E37" s="6" t="inlineStr">
@@ -2431,27 +2443,27 @@
       </c>
       <c r="F37" s="7" t="inlineStr">
         <is>
-          <t>16,976</t>
+          <t>2,093,051</t>
         </is>
       </c>
       <c r="G37" s="7" t="inlineStr">
         <is>
-          <t>4,545</t>
+          <t>-148,064</t>
         </is>
       </c>
       <c r="H37" s="7" t="inlineStr">
         <is>
-          <t>2,213</t>
+          <t>852,372</t>
         </is>
       </c>
       <c r="I37" s="6" t="inlineStr">
         <is>
-          <t>의료용품 및 기타 의약 관련제품 제조업</t>
+          <t>일반 및 생활 숙박시설 운영업</t>
         </is>
       </c>
       <c r="J37" s="6" t="inlineStr">
         <is>
-          <t>IBK</t>
+          <t>대신, 미래</t>
         </is>
       </c>
       <c r="K37" s="6" t="inlineStr">
@@ -2463,12 +2475,12 @@
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>에프엠더블유</t>
+          <t>싸이몬</t>
         </is>
       </c>
       <c r="C38" s="6" t="inlineStr">
@@ -2478,7 +2490,7 @@
       </c>
       <c r="D38" s="6" t="inlineStr">
         <is>
-          <t>스팩 소멸합병</t>
+          <t>신규상장</t>
         </is>
       </c>
       <c r="E38" s="6" t="inlineStr">
@@ -2488,27 +2500,27 @@
       </c>
       <c r="F38" s="7" t="inlineStr">
         <is>
-          <t>30,282</t>
+          <t>48,695</t>
         </is>
       </c>
       <c r="G38" s="7" t="inlineStr">
         <is>
-          <t>4,762</t>
+          <t>15,714</t>
         </is>
       </c>
       <c r="H38" s="7" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>61,761</t>
         </is>
       </c>
       <c r="I38" s="6" t="inlineStr">
         <is>
-          <t>기타 식품 제조업</t>
+          <t>측정, 시험, 항해, 제어 및 기타 정밀기기 제조업</t>
         </is>
       </c>
       <c r="J38" s="6" t="inlineStr">
         <is>
-          <t>유진</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K38" s="6" t="inlineStr">
@@ -2520,17 +2532,17 @@
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>소노인터내셔널</t>
+          <t>바이다</t>
         </is>
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>유가</t>
+          <t>코스닥</t>
         </is>
       </c>
       <c r="D39" s="6" t="inlineStr">
@@ -2545,27 +2557,27 @@
       </c>
       <c r="F39" s="7" t="inlineStr">
         <is>
-          <t>2,093,051</t>
+          <t>14,432</t>
         </is>
       </c>
       <c r="G39" s="7" t="inlineStr">
         <is>
-          <t>-148,064</t>
+          <t>-3,951</t>
         </is>
       </c>
       <c r="H39" s="7" t="inlineStr">
         <is>
-          <t>852,372</t>
+          <t>15,108</t>
         </is>
       </c>
       <c r="I39" s="6" t="inlineStr">
         <is>
-          <t>일반 및 생활 숙박시설 운영업</t>
+          <t>전자부품 제조업</t>
         </is>
       </c>
       <c r="J39" s="6" t="inlineStr">
         <is>
-          <t>대신, 미래</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K39" s="6" t="inlineStr">
@@ -2577,12 +2589,12 @@
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>싸이몬</t>
+          <t>아이알큐더스</t>
         </is>
       </c>
       <c r="C40" s="6" t="inlineStr">
@@ -2602,27 +2614,27 @@
       </c>
       <c r="F40" s="7" t="inlineStr">
         <is>
-          <t>48,695</t>
+          <t>10,231</t>
         </is>
       </c>
       <c r="G40" s="7" t="inlineStr">
         <is>
-          <t>15,714</t>
+          <t>-986</t>
         </is>
       </c>
       <c r="H40" s="7" t="inlineStr">
         <is>
-          <t>61,761</t>
+          <t>1,800</t>
         </is>
       </c>
       <c r="I40" s="6" t="inlineStr">
         <is>
-          <t>측정, 시험, 항해, 제어 및 기타 정밀기기 제조업</t>
+          <t>소프트웨어 개발 및 공급업</t>
         </is>
       </c>
       <c r="J40" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>DB</t>
         </is>
       </c>
       <c r="K40" s="6" t="inlineStr">
@@ -2634,12 +2646,12 @@
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>바이다</t>
+          <t>씨엔티테크</t>
         </is>
       </c>
       <c r="C41" s="6" t="inlineStr">
@@ -2659,27 +2671,27 @@
       </c>
       <c r="F41" s="7" t="inlineStr">
         <is>
-          <t>14,432</t>
+          <t>27,015</t>
         </is>
       </c>
       <c r="G41" s="7" t="inlineStr">
         <is>
-          <t>-3,951</t>
+          <t>3,987</t>
         </is>
       </c>
       <c r="H41" s="7" t="inlineStr">
         <is>
-          <t>15,108</t>
+          <t>2,613</t>
         </is>
       </c>
       <c r="I41" s="6" t="inlineStr">
         <is>
-          <t>전자부품 제조업</t>
+          <t>소프트웨어 개발 및 공급업</t>
         </is>
       </c>
       <c r="J41" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>한화, 하나</t>
         </is>
       </c>
       <c r="K41" s="6" t="inlineStr">
@@ -2691,12 +2703,12 @@
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B42" s="6" t="inlineStr">
         <is>
-          <t>럭스코</t>
+          <t>제이앤티지</t>
         </is>
       </c>
       <c r="C42" s="6" t="inlineStr">
@@ -2706,7 +2718,7 @@
       </c>
       <c r="D42" s="6" t="inlineStr">
         <is>
-          <t>스팩 소멸합병</t>
+          <t>신규상장</t>
         </is>
       </c>
       <c r="E42" s="6" t="inlineStr">
@@ -2716,27 +2728,27 @@
       </c>
       <c r="F42" s="7" t="inlineStr">
         <is>
-          <t>67,976</t>
+          <t>72,378</t>
         </is>
       </c>
       <c r="G42" s="7" t="inlineStr">
         <is>
-          <t>6,893</t>
+          <t>9,904</t>
         </is>
       </c>
       <c r="H42" s="7" t="inlineStr">
         <is>
-          <t>1,000</t>
+          <t>6,743</t>
         </is>
       </c>
       <c r="I42" s="6" t="inlineStr">
         <is>
-          <t>전동기, 발전기 및 전기 변환 · 공급 · 제어 장치 제조업</t>
+          <t>전자부품 제조업</t>
         </is>
       </c>
       <c r="J42" s="6" t="inlineStr">
         <is>
-          <t>IBK</t>
+          <t>대신, NH</t>
         </is>
       </c>
       <c r="K42" s="6" t="inlineStr">
@@ -2748,12 +2760,12 @@
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B43" s="6" t="inlineStr">
         <is>
-          <t>아이알큐더스</t>
+          <t>인터엑스</t>
         </is>
       </c>
       <c r="C43" s="6" t="inlineStr">
@@ -2773,17 +2785,17 @@
       </c>
       <c r="F43" s="7" t="inlineStr">
         <is>
-          <t>10,231</t>
+          <t>8,645</t>
         </is>
       </c>
       <c r="G43" s="7" t="inlineStr">
         <is>
-          <t>-986</t>
+          <t>-20,272</t>
         </is>
       </c>
       <c r="H43" s="7" t="inlineStr">
         <is>
-          <t>1,800</t>
+          <t>4,530</t>
         </is>
       </c>
       <c r="I43" s="6" t="inlineStr">
@@ -2793,7 +2805,7 @@
       </c>
       <c r="J43" s="6" t="inlineStr">
         <is>
-          <t>DB</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="K43" s="6" t="inlineStr">
@@ -2805,12 +2817,12 @@
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B44" s="6" t="inlineStr">
         <is>
-          <t>씨엔티테크</t>
+          <t>삼홍아크튜리온</t>
         </is>
       </c>
       <c r="C44" s="6" t="inlineStr">
@@ -2830,27 +2842,27 @@
       </c>
       <c r="F44" s="7" t="inlineStr">
         <is>
-          <t>27,015</t>
+          <t>26,162</t>
         </is>
       </c>
       <c r="G44" s="7" t="inlineStr">
         <is>
-          <t>3,987</t>
+          <t>-10,314</t>
         </is>
       </c>
       <c r="H44" s="7" t="inlineStr">
         <is>
-          <t>2,613</t>
+          <t>6,369</t>
         </is>
       </c>
       <c r="I44" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어 개발 및 공급업</t>
+          <t>구조용 금속제품, 탱크 및 증기발생기 제조업</t>
         </is>
       </c>
       <c r="J44" s="6" t="inlineStr">
         <is>
-          <t>한화, 하나</t>
+          <t>삼성, 미래</t>
         </is>
       </c>
       <c r="K44" s="6" t="inlineStr">
@@ -2862,12 +2874,12 @@
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B45" s="6" t="inlineStr">
         <is>
-          <t>제이앤티지</t>
+          <t>넥스트에어로스페이스</t>
         </is>
       </c>
       <c r="C45" s="6" t="inlineStr">
@@ -2887,27 +2899,27 @@
       </c>
       <c r="F45" s="7" t="inlineStr">
         <is>
-          <t>72,378</t>
+          <t>12,084</t>
         </is>
       </c>
       <c r="G45" s="7" t="inlineStr">
         <is>
-          <t>9,904</t>
+          <t>-17,270</t>
         </is>
       </c>
       <c r="H45" s="7" t="inlineStr">
         <is>
-          <t>6,743</t>
+          <t>6,158</t>
         </is>
       </c>
       <c r="I45" s="6" t="inlineStr">
         <is>
-          <t>전자부품 제조업</t>
+          <t>유인 항공기, 항공우주선 및 보조장치 제조업</t>
         </is>
       </c>
       <c r="J45" s="6" t="inlineStr">
         <is>
-          <t>대신, NH</t>
+          <t>삼성</t>
         </is>
       </c>
       <c r="K45" s="6" t="inlineStr">
@@ -2919,12 +2931,12 @@
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B46" s="6" t="inlineStr">
         <is>
-          <t>인터엑스</t>
+          <t>비앤비코리아</t>
         </is>
       </c>
       <c r="C46" s="6" t="inlineStr">
@@ -2944,27 +2956,27 @@
       </c>
       <c r="F46" s="7" t="inlineStr">
         <is>
-          <t>8,645</t>
+          <t>141,169</t>
         </is>
       </c>
       <c r="G46" s="7" t="inlineStr">
         <is>
-          <t>-20,272</t>
+          <t>21,406</t>
         </is>
       </c>
       <c r="H46" s="7" t="inlineStr">
         <is>
-          <t>4,530</t>
+          <t>43,932</t>
         </is>
       </c>
       <c r="I46" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어 개발 및 공급업</t>
+          <t>기타 화학제품 제조업</t>
         </is>
       </c>
       <c r="J46" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K46" s="6" t="inlineStr">
@@ -2976,12 +2988,12 @@
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B47" s="6" t="inlineStr">
         <is>
-          <t>삼홍아크튜리온</t>
+          <t>오토핸즈</t>
         </is>
       </c>
       <c r="C47" s="6" t="inlineStr">
@@ -2991,7 +3003,7 @@
       </c>
       <c r="D47" s="6" t="inlineStr">
         <is>
-          <t>신규상장</t>
+          <t>스팩 소멸합병</t>
         </is>
       </c>
       <c r="E47" s="6" t="inlineStr">
@@ -3001,27 +3013,27 @@
       </c>
       <c r="F47" s="7" t="inlineStr">
         <is>
-          <t>26,162</t>
+          <t>238,564</t>
         </is>
       </c>
       <c r="G47" s="7" t="inlineStr">
         <is>
-          <t>-10,314</t>
+          <t>6,047</t>
         </is>
       </c>
       <c r="H47" s="7" t="inlineStr">
         <is>
-          <t>6,369</t>
+          <t>6,129</t>
         </is>
       </c>
       <c r="I47" s="6" t="inlineStr">
         <is>
-          <t>구조용 금속제품, 탱크 및 증기발생기 제조업</t>
+          <t>자동차 판매업</t>
         </is>
       </c>
       <c r="J47" s="6" t="inlineStr">
         <is>
-          <t>삼성, 미래</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K47" s="6" t="inlineStr">
@@ -3033,12 +3045,12 @@
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B48" s="6" t="inlineStr">
         <is>
-          <t>넥스트에어로스페이스</t>
+          <t>아이벡스메디칼시스템즈</t>
         </is>
       </c>
       <c r="C48" s="6" t="inlineStr">
@@ -3058,27 +3070,27 @@
       </c>
       <c r="F48" s="7" t="inlineStr">
         <is>
-          <t>12,084</t>
+          <t>15,282</t>
         </is>
       </c>
       <c r="G48" s="7" t="inlineStr">
         <is>
-          <t>-17,270</t>
+          <t>-7,227</t>
         </is>
       </c>
       <c r="H48" s="7" t="inlineStr">
         <is>
-          <t>6,158</t>
+          <t>744</t>
         </is>
       </c>
       <c r="I48" s="6" t="inlineStr">
         <is>
-          <t>유인 항공기, 항공우주선 및 보조장치 제조업</t>
+          <t>의료용 기기 제조업</t>
         </is>
       </c>
       <c r="J48" s="6" t="inlineStr">
         <is>
-          <t>삼성</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K48" s="6" t="inlineStr">
@@ -3090,12 +3102,12 @@
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="B49" s="6" t="inlineStr">
         <is>
-          <t>비앤비코리아</t>
+          <t>피지티</t>
         </is>
       </c>
       <c r="C49" s="6" t="inlineStr">
@@ -3115,17 +3127,17 @@
       </c>
       <c r="F49" s="7" t="inlineStr">
         <is>
-          <t>141,169</t>
+          <t>40,141</t>
         </is>
       </c>
       <c r="G49" s="7" t="inlineStr">
         <is>
-          <t>21,406</t>
+          <t>-69,722</t>
         </is>
       </c>
       <c r="H49" s="7" t="inlineStr">
         <is>
-          <t>43,932</t>
+          <t>6,029</t>
         </is>
       </c>
       <c r="I49" s="6" t="inlineStr">
@@ -3135,7 +3147,7 @@
       </c>
       <c r="J49" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="K49" s="6" t="inlineStr">
@@ -3144,248 +3156,236 @@
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="6" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
-        </is>
-      </c>
-      <c r="B50" s="6" t="inlineStr">
-        <is>
-          <t>오토핸즈</t>
-        </is>
-      </c>
-      <c r="C50" s="6" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t>■ 심사 승인  (70건)</t>
+        </is>
+      </c>
+      <c r="B51" s="4" t="n"/>
+      <c r="C51" s="4" t="n"/>
+      <c r="D51" s="4" t="n"/>
+      <c r="E51" s="4" t="n"/>
+      <c r="F51" s="4" t="n"/>
+      <c r="G51" s="4" t="n"/>
+      <c r="H51" s="4" t="n"/>
+      <c r="I51" s="4" t="n"/>
+      <c r="J51" s="4" t="n"/>
+      <c r="K51" s="4" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>일자</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t>회사명</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>시장</t>
+        </is>
+      </c>
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>상장유형</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>기준연도</t>
+        </is>
+      </c>
+      <c r="F52" s="5" t="inlineStr">
+        <is>
+          <t>매출액</t>
+        </is>
+      </c>
+      <c r="G52" s="5" t="inlineStr">
+        <is>
+          <t>순이익</t>
+        </is>
+      </c>
+      <c r="H52" s="5" t="inlineStr">
+        <is>
+          <t>자기자본</t>
+        </is>
+      </c>
+      <c r="I52" s="5" t="inlineStr">
+        <is>
+          <t>업종</t>
+        </is>
+      </c>
+      <c r="J52" s="5" t="inlineStr">
+        <is>
+          <t>대표주관사</t>
+        </is>
+      </c>
+      <c r="K52" s="5" t="inlineStr">
+        <is>
+          <t>현황</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B53" s="6" t="inlineStr">
+        <is>
+          <t>셀트릭스</t>
+        </is>
+      </c>
+      <c r="C53" s="6" t="inlineStr">
         <is>
           <t>코스닥</t>
         </is>
       </c>
-      <c r="D50" s="6" t="inlineStr">
+      <c r="D53" s="6" t="inlineStr">
         <is>
           <t>스팩 소멸합병</t>
         </is>
       </c>
-      <c r="E50" s="6" t="inlineStr">
+      <c r="E53" s="6" t="inlineStr">
         <is>
           <t>FY25</t>
         </is>
       </c>
-      <c r="F50" s="7" t="inlineStr">
-        <is>
-          <t>238,564</t>
-        </is>
-      </c>
-      <c r="G50" s="7" t="inlineStr">
-        <is>
-          <t>6,047</t>
-        </is>
-      </c>
-      <c r="H50" s="7" t="inlineStr">
-        <is>
-          <t>6,129</t>
-        </is>
-      </c>
-      <c r="I50" s="6" t="inlineStr">
-        <is>
-          <t>자동차 판매업</t>
-        </is>
-      </c>
-      <c r="J50" s="6" t="inlineStr">
-        <is>
-          <t>미래</t>
-        </is>
-      </c>
-      <c r="K50" s="6" t="inlineStr">
-        <is>
-          <t>예심 진행중</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="6" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-      <c r="B51" s="6" t="inlineStr">
-        <is>
-          <t>아이벡스메디칼시스템즈</t>
-        </is>
-      </c>
-      <c r="C51" s="6" t="inlineStr">
+      <c r="F53" s="7" t="inlineStr">
+        <is>
+          <t>16,976</t>
+        </is>
+      </c>
+      <c r="G53" s="7" t="inlineStr">
+        <is>
+          <t>4,545</t>
+        </is>
+      </c>
+      <c r="H53" s="7" t="inlineStr">
+        <is>
+          <t>2,213</t>
+        </is>
+      </c>
+      <c r="I53" s="6" t="inlineStr">
+        <is>
+          <t>의료용품 및 기타 의약 관련제품 제조업</t>
+        </is>
+      </c>
+      <c r="J53" s="6" t="inlineStr">
+        <is>
+          <t>IBK</t>
+        </is>
+      </c>
+      <c r="K53" s="6" t="inlineStr">
+        <is>
+          <t>상장전</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B54" s="6" t="inlineStr">
+        <is>
+          <t>럭스코</t>
+        </is>
+      </c>
+      <c r="C54" s="6" t="inlineStr">
         <is>
           <t>코스닥</t>
         </is>
       </c>
-      <c r="D51" s="6" t="inlineStr">
-        <is>
-          <t>신규상장</t>
-        </is>
-      </c>
-      <c r="E51" s="6" t="inlineStr">
+      <c r="D54" s="6" t="inlineStr">
+        <is>
+          <t>스팩 소멸합병</t>
+        </is>
+      </c>
+      <c r="E54" s="6" t="inlineStr">
         <is>
           <t>FY25</t>
         </is>
       </c>
-      <c r="F51" s="7" t="inlineStr">
-        <is>
-          <t>15,282</t>
-        </is>
-      </c>
-      <c r="G51" s="7" t="inlineStr">
-        <is>
-          <t>-7,227</t>
-        </is>
-      </c>
-      <c r="H51" s="7" t="inlineStr">
-        <is>
-          <t>744</t>
-        </is>
-      </c>
-      <c r="I51" s="6" t="inlineStr">
-        <is>
-          <t>의료용 기기 제조업</t>
-        </is>
-      </c>
-      <c r="J51" s="6" t="inlineStr">
-        <is>
-          <t>NH</t>
-        </is>
-      </c>
-      <c r="K51" s="6" t="inlineStr">
-        <is>
-          <t>예심 진행중</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="6" t="inlineStr">
-        <is>
-          <t>2026-02-27</t>
-        </is>
-      </c>
-      <c r="B52" s="6" t="inlineStr">
-        <is>
-          <t>피지티</t>
-        </is>
-      </c>
-      <c r="C52" s="6" t="inlineStr">
+      <c r="F54" s="7" t="inlineStr">
+        <is>
+          <t>67,976</t>
+        </is>
+      </c>
+      <c r="G54" s="7" t="inlineStr">
+        <is>
+          <t>6,893</t>
+        </is>
+      </c>
+      <c r="H54" s="7" t="inlineStr">
+        <is>
+          <t>1,000</t>
+        </is>
+      </c>
+      <c r="I54" s="6" t="inlineStr">
+        <is>
+          <t>전동기, 발전기 및 전기 변환 · 공급 · 제어 장치 제조업</t>
+        </is>
+      </c>
+      <c r="J54" s="6" t="inlineStr">
+        <is>
+          <t>IBK</t>
+        </is>
+      </c>
+      <c r="K54" s="6" t="inlineStr">
+        <is>
+          <t>상장전</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B55" s="6" t="inlineStr">
+        <is>
+          <t>솔리스</t>
+        </is>
+      </c>
+      <c r="C55" s="6" t="inlineStr">
         <is>
           <t>코스닥</t>
         </is>
       </c>
-      <c r="D52" s="6" t="inlineStr">
-        <is>
-          <t>신규상장</t>
-        </is>
-      </c>
-      <c r="E52" s="6" t="inlineStr">
+      <c r="D55" s="6" t="inlineStr">
+        <is>
+          <t>스팩 소멸합병</t>
+        </is>
+      </c>
+      <c r="E55" s="6" t="inlineStr">
         <is>
           <t>FY25</t>
         </is>
       </c>
-      <c r="F52" s="7" t="inlineStr">
-        <is>
-          <t>40,141</t>
-        </is>
-      </c>
-      <c r="G52" s="7" t="inlineStr">
-        <is>
-          <t>-69,722</t>
-        </is>
-      </c>
-      <c r="H52" s="7" t="inlineStr">
-        <is>
-          <t>6,029</t>
-        </is>
-      </c>
-      <c r="I52" s="6" t="inlineStr">
-        <is>
-          <t>기타 화학제품 제조업</t>
-        </is>
-      </c>
-      <c r="J52" s="6" t="inlineStr">
-        <is>
-          <t>한국</t>
-        </is>
-      </c>
-      <c r="K52" s="6" t="inlineStr">
-        <is>
-          <t>예심 진행중</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="3" t="inlineStr">
-        <is>
-          <t>■ 심사 승인  (67건)</t>
-        </is>
-      </c>
-      <c r="B54" s="4" t="n"/>
-      <c r="C54" s="4" t="n"/>
-      <c r="D54" s="4" t="n"/>
-      <c r="E54" s="4" t="n"/>
-      <c r="F54" s="4" t="n"/>
-      <c r="G54" s="4" t="n"/>
-      <c r="H54" s="4" t="n"/>
-      <c r="I54" s="4" t="n"/>
-      <c r="J54" s="4" t="n"/>
-      <c r="K54" s="4" t="n"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="5" t="inlineStr">
-        <is>
-          <t>일자</t>
-        </is>
-      </c>
-      <c r="B55" s="5" t="inlineStr">
-        <is>
-          <t>회사명</t>
-        </is>
-      </c>
-      <c r="C55" s="5" t="inlineStr">
-        <is>
-          <t>시장</t>
-        </is>
-      </c>
-      <c r="D55" s="5" t="inlineStr">
-        <is>
-          <t>상장유형</t>
-        </is>
-      </c>
-      <c r="E55" s="5" t="inlineStr">
-        <is>
-          <t>기준연도</t>
-        </is>
-      </c>
-      <c r="F55" s="5" t="inlineStr">
-        <is>
-          <t>매출액</t>
-        </is>
-      </c>
-      <c r="G55" s="5" t="inlineStr">
-        <is>
-          <t>순이익</t>
-        </is>
-      </c>
-      <c r="H55" s="5" t="inlineStr">
-        <is>
-          <t>자기자본</t>
-        </is>
-      </c>
-      <c r="I55" s="5" t="inlineStr">
-        <is>
-          <t>업종</t>
-        </is>
-      </c>
-      <c r="J55" s="5" t="inlineStr">
-        <is>
-          <t>대표주관사</t>
-        </is>
-      </c>
-      <c r="K55" s="5" t="inlineStr">
-        <is>
-          <t>현황</t>
+      <c r="F55" s="7" t="inlineStr"/>
+      <c r="G55" s="7" t="inlineStr"/>
+      <c r="H55" s="7" t="inlineStr"/>
+      <c r="I55" s="6" t="inlineStr">
+        <is>
+          <t>금융 지원 서비스업</t>
+        </is>
+      </c>
+      <c r="J55" s="6" t="inlineStr">
+        <is>
+          <t>한화</t>
+        </is>
+      </c>
+      <c r="K55" s="6" t="inlineStr">
+        <is>
+          <t>상장전</t>
         </is>
       </c>
     </row>
@@ -5083,7 +5083,7 @@
       </c>
       <c r="K85" s="6" t="inlineStr">
         <is>
-          <t>상장전</t>
+          <t>상장승인(상장예정)</t>
         </is>
       </c>
     </row>
@@ -8179,7 +8179,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R88"/>
+  <dimension ref="A1:R91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -11937,7 +11937,7 @@
     <row r="52" ht="22" customHeight="1">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>■ 공모 진행 (예심 승인법인)  (32건)</t>
+          <t>■ 공모 진행 (예심 승인법인)  (35건)</t>
         </is>
       </c>
       <c r="B52" s="4" t="n"/>
@@ -12345,7 +12345,7 @@
     <row r="58" ht="30" customHeight="1">
       <c r="A58" s="6" t="inlineStr">
         <is>
-          <t>멜콘</t>
+          <t>진코스텍</t>
         </is>
       </c>
       <c r="B58" s="6" t="inlineStr">
@@ -12355,30 +12355,38 @@
       </c>
       <c r="C58" s="6" t="inlineStr">
         <is>
-          <t>10,700~12,300</t>
+          <t>19,500~23,500</t>
         </is>
       </c>
       <c r="D58" s="7" t="inlineStr">
         <is>
-          <t>2,500,000</t>
+          <t>852,000</t>
         </is>
       </c>
       <c r="E58" s="7" t="inlineStr">
         <is>
-          <t>26,750,000,000</t>
+          <t>16,614,000,000</t>
         </is>
       </c>
       <c r="F58" s="6" t="inlineStr">
         <is>
-          <t>26.18배 (PER)</t>
-        </is>
-      </c>
-      <c r="G58" s="6" t="inlineStr"/>
-      <c r="H58" s="6" t="inlineStr"/>
-      <c r="I58" s="6" t="inlineStr"/>
+          <t>17.61배 (PER)</t>
+        </is>
+      </c>
+      <c r="G58" s="6" t="inlineStr">
+        <is>
+          <t>19,500</t>
+        </is>
+      </c>
+      <c r="H58" s="6" t="n">
+        <v>1097.62</v>
+      </c>
+      <c r="I58" s="6" t="n">
+        <v>2006</v>
+      </c>
       <c r="J58" s="6" t="inlineStr">
         <is>
-          <t>10-01~10-02</t>
+          <t>10-02~10-06</t>
         </is>
       </c>
       <c r="K58" s="6" t="inlineStr"/>
@@ -12386,30 +12394,30 @@
       <c r="M58" s="6" t="inlineStr"/>
       <c r="N58" s="6" t="inlineStr">
         <is>
-          <t>대신증권</t>
+          <t>하나증권</t>
         </is>
       </c>
       <c r="O58" s="6" t="inlineStr"/>
       <c r="P58" s="7" t="inlineStr">
         <is>
-          <t>826,575,000</t>
+          <t>697,788,000</t>
         </is>
       </c>
       <c r="Q58" s="6" t="inlineStr">
         <is>
-          <t>3.0%</t>
+          <t>4.0%</t>
         </is>
       </c>
       <c r="R58" s="6" t="inlineStr">
         <is>
-          <t>정정</t>
+          <t>발행조건확정</t>
         </is>
       </c>
     </row>
     <row r="59" ht="30" customHeight="1">
       <c r="A59" s="6" t="inlineStr">
         <is>
-          <t>진코스텍</t>
+          <t>멜콘</t>
         </is>
       </c>
       <c r="B59" s="6" t="inlineStr">
@@ -12419,22 +12427,22 @@
       </c>
       <c r="C59" s="6" t="inlineStr">
         <is>
-          <t>19,500~23,500</t>
+          <t>10,700~12,300</t>
         </is>
       </c>
       <c r="D59" s="7" t="inlineStr">
         <is>
-          <t>852,000</t>
+          <t>2,500,000</t>
         </is>
       </c>
       <c r="E59" s="7" t="inlineStr">
         <is>
-          <t>16,614,000,000</t>
+          <t>26,750,000,000</t>
         </is>
       </c>
       <c r="F59" s="6" t="inlineStr">
         <is>
-          <t>17.61배 (PER)</t>
+          <t>26.18배 (PER)</t>
         </is>
       </c>
       <c r="G59" s="6" t="inlineStr"/>
@@ -12442,7 +12450,7 @@
       <c r="I59" s="6" t="inlineStr"/>
       <c r="J59" s="6" t="inlineStr">
         <is>
-          <t>10-02~10-06</t>
+          <t>10-01~10-02</t>
         </is>
       </c>
       <c r="K59" s="6" t="inlineStr"/>
@@ -12450,18 +12458,18 @@
       <c r="M59" s="6" t="inlineStr"/>
       <c r="N59" s="6" t="inlineStr">
         <is>
-          <t>하나증권</t>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="O59" s="6" t="inlineStr"/>
       <c r="P59" s="7" t="inlineStr">
         <is>
-          <t>697,788,000</t>
+          <t>826,575,000</t>
         </is>
       </c>
       <c r="Q59" s="6" t="inlineStr">
         <is>
-          <t>4.0%</t>
+          <t>3.0%</t>
         </is>
       </c>
       <c r="R59" s="6" t="inlineStr">
@@ -13373,32 +13381,32 @@
     <row r="74" ht="30" customHeight="1">
       <c r="A74" s="6" t="inlineStr">
         <is>
-          <t>하나에어로다이내믹스</t>
+          <t>넥스아이</t>
         </is>
       </c>
       <c r="B74" s="6" t="inlineStr">
         <is>
-          <t>11-02~11-06</t>
+          <t>10-22~10-28</t>
         </is>
       </c>
       <c r="C74" s="6" t="inlineStr">
         <is>
-          <t>4,700~5,700</t>
+          <t>10,500~13,000</t>
         </is>
       </c>
       <c r="D74" s="7" t="inlineStr">
         <is>
-          <t>4,400,000</t>
+          <t>5,000,000</t>
         </is>
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
-          <t>20,680,000,000</t>
+          <t>52,500,000,000</t>
         </is>
       </c>
       <c r="F74" s="6" t="inlineStr">
         <is>
-          <t>17.89배 (EV/EBITDA)</t>
+          <t>19.15배 (PER)</t>
         </is>
       </c>
       <c r="G74" s="6" t="inlineStr"/>
@@ -13406,7 +13414,7 @@
       <c r="I74" s="6" t="inlineStr"/>
       <c r="J74" s="6" t="inlineStr">
         <is>
-          <t>11-10~11-11</t>
+          <t>11-03~11-04</t>
         </is>
       </c>
       <c r="K74" s="6" t="inlineStr"/>
@@ -13414,18 +13422,18 @@
       <c r="M74" s="6" t="inlineStr"/>
       <c r="N74" s="6" t="inlineStr">
         <is>
-          <t>아이비케이투자증권</t>
+          <t>한국투자증권</t>
         </is>
       </c>
       <c r="O74" s="6" t="inlineStr"/>
       <c r="P74" s="7" t="inlineStr">
         <is>
-          <t>850,000,000</t>
-        </is>
-      </c>
-      <c r="Q74" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>2,407,500,000</t>
+        </is>
+      </c>
+      <c r="Q74" s="6" t="inlineStr">
+        <is>
+          <t>4.5%</t>
         </is>
       </c>
       <c r="R74" s="6" t="inlineStr">
@@ -13437,54 +13445,54 @@
     <row r="75" ht="30" customHeight="1">
       <c r="A75" s="6" t="inlineStr">
         <is>
-          <t>바로팜</t>
-        </is>
-      </c>
-      <c r="B75" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>하나에어로다이내믹스</t>
+        </is>
+      </c>
+      <c r="B75" s="6" t="inlineStr">
+        <is>
+          <t>11-02~11-06</t>
         </is>
       </c>
       <c r="C75" s="6" t="inlineStr">
         <is>
-          <t>16,400~20,200</t>
+          <t>4,700~5,700</t>
         </is>
       </c>
       <c r="D75" s="7" t="inlineStr">
         <is>
-          <t>1,780,000</t>
+          <t>4,400,000</t>
         </is>
       </c>
       <c r="E75" s="7" t="inlineStr">
         <is>
-          <t>29,192,000,000</t>
+          <t>20,680,000,000</t>
         </is>
       </c>
       <c r="F75" s="6" t="inlineStr">
         <is>
-          <t>24.95배 (PER)</t>
+          <t>17.89배 (EV/EBITDA)</t>
         </is>
       </c>
       <c r="G75" s="6" t="inlineStr"/>
       <c r="H75" s="6" t="inlineStr"/>
       <c r="I75" s="6" t="inlineStr"/>
-      <c r="J75" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="J75" s="6" t="inlineStr">
+        <is>
+          <t>11-10~11-11</t>
         </is>
       </c>
       <c r="K75" s="6" t="inlineStr"/>
       <c r="L75" s="6" t="inlineStr"/>
       <c r="M75" s="6" t="inlineStr"/>
-      <c r="N75" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="N75" s="6" t="inlineStr">
+        <is>
+          <t>아이비케이투자증권</t>
         </is>
       </c>
       <c r="O75" s="6" t="inlineStr"/>
-      <c r="P75" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="P75" s="7" t="inlineStr">
+        <is>
+          <t>850,000,000</t>
         </is>
       </c>
       <c r="Q75" s="18" t="inlineStr">
@@ -13501,7 +13509,7 @@
     <row r="76" ht="30" customHeight="1">
       <c r="A76" s="6" t="inlineStr">
         <is>
-          <t>디티에스</t>
+          <t>바로팜</t>
         </is>
       </c>
       <c r="B76" s="18" t="inlineStr">
@@ -13509,24 +13517,24 @@
           <t>수집예정</t>
         </is>
       </c>
-      <c r="C76" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="D76" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="E76" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="F76" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="C76" s="6" t="inlineStr">
+        <is>
+          <t>16,400~20,200</t>
+        </is>
+      </c>
+      <c r="D76" s="7" t="inlineStr">
+        <is>
+          <t>1,780,000</t>
+        </is>
+      </c>
+      <c r="E76" s="7" t="inlineStr">
+        <is>
+          <t>29,192,000,000</t>
+        </is>
+      </c>
+      <c r="F76" s="6" t="inlineStr">
+        <is>
+          <t>24.95배 (PER)</t>
         </is>
       </c>
       <c r="G76" s="6" t="inlineStr"/>
@@ -13558,14 +13566,14 @@
       </c>
       <c r="R76" s="6" t="inlineStr">
         <is>
-          <t>신고서 대기</t>
+          <t>최초</t>
         </is>
       </c>
     </row>
     <row r="77" ht="30" customHeight="1">
       <c r="A77" s="6" t="inlineStr">
         <is>
-          <t>에이엔에이치스트럭쳐</t>
+          <t>디티에스</t>
         </is>
       </c>
       <c r="B77" s="18" t="inlineStr">
@@ -13629,7 +13637,7 @@
     <row r="78" ht="30" customHeight="1">
       <c r="A78" s="6" t="inlineStr">
         <is>
-          <t>이에스티</t>
+          <t>에이엔에이치스트럭쳐</t>
         </is>
       </c>
       <c r="B78" s="18" t="inlineStr">
@@ -13693,7 +13701,7 @@
     <row r="79" ht="30" customHeight="1">
       <c r="A79" s="6" t="inlineStr">
         <is>
-          <t>영광와이케이엠씨</t>
+          <t>이에스티</t>
         </is>
       </c>
       <c r="B79" s="18" t="inlineStr">
@@ -13757,7 +13765,7 @@
     <row r="80" ht="30" customHeight="1">
       <c r="A80" s="6" t="inlineStr">
         <is>
-          <t>동원파츠</t>
+          <t>영광와이케이엠씨</t>
         </is>
       </c>
       <c r="B80" s="18" t="inlineStr">
@@ -13821,7 +13829,7 @@
     <row r="81" ht="30" customHeight="1">
       <c r="A81" s="6" t="inlineStr">
         <is>
-          <t>케이엠에프</t>
+          <t>동원파츠</t>
         </is>
       </c>
       <c r="B81" s="18" t="inlineStr">
@@ -13885,7 +13893,7 @@
     <row r="82" ht="30" customHeight="1">
       <c r="A82" s="6" t="inlineStr">
         <is>
-          <t>넥스아이</t>
+          <t>케이엠에프</t>
         </is>
       </c>
       <c r="B82" s="18" t="inlineStr">
@@ -14074,22 +14082,214 @@
         </is>
       </c>
     </row>
-    <row r="86">
-      <c r="A86" s="20" t="inlineStr">
+    <row r="85" ht="30" customHeight="1">
+      <c r="A85" s="6" t="inlineStr">
+        <is>
+          <t>셀트릭스</t>
+        </is>
+      </c>
+      <c r="B85" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="C85" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="D85" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="E85" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="F85" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="G85" s="6" t="inlineStr"/>
+      <c r="H85" s="6" t="inlineStr"/>
+      <c r="I85" s="6" t="inlineStr"/>
+      <c r="J85" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="K85" s="6" t="inlineStr"/>
+      <c r="L85" s="6" t="inlineStr"/>
+      <c r="M85" s="6" t="inlineStr"/>
+      <c r="N85" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="O85" s="6" t="inlineStr"/>
+      <c r="P85" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="Q85" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="R85" s="6" t="inlineStr">
+        <is>
+          <t>신고서 대기</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="30" customHeight="1">
+      <c r="A86" s="6" t="inlineStr">
+        <is>
+          <t>럭스코</t>
+        </is>
+      </c>
+      <c r="B86" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="C86" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="D86" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="E86" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="F86" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="G86" s="6" t="inlineStr"/>
+      <c r="H86" s="6" t="inlineStr"/>
+      <c r="I86" s="6" t="inlineStr"/>
+      <c r="J86" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="K86" s="6" t="inlineStr"/>
+      <c r="L86" s="6" t="inlineStr"/>
+      <c r="M86" s="6" t="inlineStr"/>
+      <c r="N86" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="O86" s="6" t="inlineStr"/>
+      <c r="P86" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="Q86" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="R86" s="6" t="inlineStr">
+        <is>
+          <t>신고서 대기</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="30" customHeight="1">
+      <c r="A87" s="6" t="inlineStr">
+        <is>
+          <t>솔리스</t>
+        </is>
+      </c>
+      <c r="B87" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="C87" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="D87" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="E87" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="F87" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="G87" s="6" t="inlineStr"/>
+      <c r="H87" s="6" t="inlineStr"/>
+      <c r="I87" s="6" t="inlineStr"/>
+      <c r="J87" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="K87" s="6" t="inlineStr"/>
+      <c r="L87" s="6" t="inlineStr"/>
+      <c r="M87" s="6" t="inlineStr"/>
+      <c r="N87" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="O87" s="6" t="inlineStr"/>
+      <c r="P87" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="Q87" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="R87" s="6" t="inlineStr">
+        <is>
+          <t>신고서 대기</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="20" t="inlineStr">
         <is>
           <t>※ 상장 완료 = KIND 신규상장 페이지 기준(스팩합병 포함) · 스팩 공모상장은 밴드·밸류에이션 등 해당없음(공모가 2,000원 고정).</t>
         </is>
       </c>
     </row>
-    <row r="87">
-      <c r="A87" s="20" t="inlineStr">
+    <row r="90">
+      <c r="A90" s="20" t="inlineStr">
         <is>
           <t>※ 기재정정 신고서 내 정정 전·후 병존 → 자동수집은 "정정 후" 값만 취함.</t>
         </is>
       </c>
     </row>
-    <row r="88">
-      <c r="A88" s="20" t="inlineStr">
+    <row r="91">
+      <c r="A91" s="20" t="inlineStr">
         <is>
           <t>※ 청약경쟁률=일반투자자 청약수량÷최종배정수량 · "MM-DD~"는 종료일 자동수집 예정.</t>
         </is>
@@ -14369,7 +14569,7 @@
         <v>11</v>
       </c>
       <c r="C14" s="6" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D14" s="6" t="n">
         <v>0</v>
@@ -14468,30 +14668,30 @@
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>미래에셋증권㈜</t>
+          <t>한국투자증권</t>
         </is>
       </c>
       <c r="B21" s="6" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>156,428,800,000</t>
+          <t>194,940,000,000</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>한국투자증권</t>
+          <t>미래에셋증권㈜</t>
         </is>
       </c>
       <c r="B22" s="6" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>142,440,000,000</t>
+          <t>156,428,800,000</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update IPO data 2026-10-06
</commit_message>
<xml_diff>
--- a/IPO_analysis.xlsx
+++ b/IPO_analysis.xlsx
@@ -618,14 +618,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>기준일 2026-10-05 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
+          <t>기준일 2026-10-06 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>■ 심사 신청(진행중)  (47건)</t>
+          <t>■ 심사 신청(진행중)  (46건)</t>
         </is>
       </c>
       <c r="B4" s="4" t="n"/>
@@ -1746,17 +1746,17 @@
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>우리투자제1호스팩</t>
+          <t>에스텍시스템</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>코스닥</t>
+          <t>유가</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
@@ -1769,17 +1769,29 @@
           <t>FY25</t>
         </is>
       </c>
-      <c r="F25" s="7" t="inlineStr"/>
-      <c r="G25" s="7" t="inlineStr"/>
-      <c r="H25" s="7" t="inlineStr"/>
+      <c r="F25" s="7" t="inlineStr">
+        <is>
+          <t>975,224</t>
+        </is>
+      </c>
+      <c r="G25" s="7" t="inlineStr">
+        <is>
+          <t>24,647</t>
+        </is>
+      </c>
+      <c r="H25" s="7" t="inlineStr">
+        <is>
+          <t>237,182</t>
+        </is>
+      </c>
       <c r="I25" s="6" t="inlineStr">
         <is>
-          <t>기타 금융업</t>
+          <t>경비, 경호 및 탐정업</t>
         </is>
       </c>
       <c r="J25" s="6" t="inlineStr">
         <is>
-          <t>주식회사 우리투자증권</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K25" s="6" t="inlineStr">
@@ -1791,17 +1803,17 @@
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>에스텍시스템</t>
+          <t>범한메카텍</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>유가</t>
+          <t>코스닥</t>
         </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
@@ -1816,27 +1828,27 @@
       </c>
       <c r="F26" s="7" t="inlineStr">
         <is>
-          <t>975,224</t>
+          <t>339,209</t>
         </is>
       </c>
       <c r="G26" s="7" t="inlineStr">
         <is>
-          <t>24,647</t>
+          <t>-18,141</t>
         </is>
       </c>
       <c r="H26" s="7" t="inlineStr">
         <is>
-          <t>237,182</t>
+          <t>265,955</t>
         </is>
       </c>
       <c r="I26" s="6" t="inlineStr">
         <is>
-          <t>경비, 경호 및 탐정업</t>
+          <t>구조용 금속제품, 탱크 및 증기발생기 제조업</t>
         </is>
       </c>
       <c r="J26" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>유진, NH</t>
         </is>
       </c>
       <c r="K26" s="6" t="inlineStr">
@@ -1853,7 +1865,7 @@
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>범한메카텍</t>
+          <t>케이티이</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
@@ -1873,27 +1885,27 @@
       </c>
       <c r="F27" s="7" t="inlineStr">
         <is>
-          <t>339,209</t>
+          <t>173,901</t>
         </is>
       </c>
       <c r="G27" s="7" t="inlineStr">
         <is>
-          <t>-18,141</t>
+          <t>14,243</t>
         </is>
       </c>
       <c r="H27" s="7" t="inlineStr">
         <is>
-          <t>265,955</t>
+          <t>94,928</t>
         </is>
       </c>
       <c r="I27" s="6" t="inlineStr">
         <is>
-          <t>구조용 금속제품, 탱크 및 증기발생기 제조업</t>
+          <t>전동기, 발전기 및 전기 변환 · 공급 · 제어 장치 제조업</t>
         </is>
       </c>
       <c r="J27" s="6" t="inlineStr">
         <is>
-          <t>유진, NH</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K27" s="6" t="inlineStr">
@@ -1905,12 +1917,12 @@
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>케이티이</t>
+          <t>데스틴파워</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
@@ -1930,17 +1942,17 @@
       </c>
       <c r="F28" s="7" t="inlineStr">
         <is>
-          <t>173,901</t>
+          <t>29,851</t>
         </is>
       </c>
       <c r="G28" s="7" t="inlineStr">
         <is>
-          <t>14,243</t>
+          <t>5,852</t>
         </is>
       </c>
       <c r="H28" s="7" t="inlineStr">
         <is>
-          <t>94,928</t>
+          <t>-30,114</t>
         </is>
       </c>
       <c r="I28" s="6" t="inlineStr">
@@ -1950,7 +1962,7 @@
       </c>
       <c r="J28" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="K28" s="6" t="inlineStr">
@@ -1967,7 +1979,7 @@
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>데스틴파워</t>
+          <t>유림테크</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
@@ -1987,27 +1999,27 @@
       </c>
       <c r="F29" s="7" t="inlineStr">
         <is>
-          <t>29,851</t>
+          <t>102,586</t>
         </is>
       </c>
       <c r="G29" s="7" t="inlineStr">
         <is>
-          <t>5,852</t>
+          <t>-18,278</t>
         </is>
       </c>
       <c r="H29" s="7" t="inlineStr">
         <is>
-          <t>-30,114</t>
+          <t>-4,832</t>
         </is>
       </c>
       <c r="I29" s="6" t="inlineStr">
         <is>
-          <t>전동기, 발전기 및 전기 변환 · 공급 · 제어 장치 제조업</t>
+          <t>자동차 신품 부품 제조업</t>
         </is>
       </c>
       <c r="J29" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>대신</t>
         </is>
       </c>
       <c r="K29" s="6" t="inlineStr">
@@ -2019,12 +2031,12 @@
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>유림테크</t>
+          <t>이노보테라퓨틱스</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
@@ -2044,27 +2056,27 @@
       </c>
       <c r="F30" s="7" t="inlineStr">
         <is>
-          <t>102,586</t>
+          <t>209</t>
         </is>
       </c>
       <c r="G30" s="7" t="inlineStr">
         <is>
-          <t>-18,278</t>
+          <t>-5,429</t>
         </is>
       </c>
       <c r="H30" s="7" t="inlineStr">
         <is>
-          <t>-4,832</t>
+          <t>-53,200</t>
         </is>
       </c>
       <c r="I30" s="6" t="inlineStr">
         <is>
-          <t>자동차 신품 부품 제조업</t>
+          <t>의약품 제조업</t>
         </is>
       </c>
       <c r="J30" s="6" t="inlineStr">
         <is>
-          <t>대신</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="K30" s="6" t="inlineStr">
@@ -2076,17 +2088,17 @@
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>이노보테라퓨틱스</t>
+          <t>에스에프씨</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>코스닥</t>
+          <t>유가</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr">
@@ -2101,27 +2113,27 @@
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>209</t>
+          <t>160,792</t>
         </is>
       </c>
       <c r="G31" s="7" t="inlineStr">
         <is>
-          <t>-5,429</t>
+          <t>25,509</t>
         </is>
       </c>
       <c r="H31" s="7" t="inlineStr">
         <is>
-          <t>-53,200</t>
+          <t>243,562</t>
         </is>
       </c>
       <c r="I31" s="6" t="inlineStr">
         <is>
-          <t>의약품 제조업</t>
+          <t>기타 화학제품 제조업</t>
         </is>
       </c>
       <c r="J31" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>미래, 한국</t>
         </is>
       </c>
       <c r="K31" s="6" t="inlineStr">
@@ -2133,17 +2145,17 @@
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>에스에프씨</t>
+          <t>아델</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>유가</t>
+          <t>코스닥</t>
         </is>
       </c>
       <c r="D32" s="6" t="inlineStr">
@@ -2158,27 +2170,27 @@
       </c>
       <c r="F32" s="7" t="inlineStr">
         <is>
-          <t>160,792</t>
+          <t>62,057</t>
         </is>
       </c>
       <c r="G32" s="7" t="inlineStr">
         <is>
-          <t>25,509</t>
+          <t>-64,210</t>
         </is>
       </c>
       <c r="H32" s="7" t="inlineStr">
         <is>
-          <t>243,562</t>
+          <t>-80,776</t>
         </is>
       </c>
       <c r="I32" s="6" t="inlineStr">
         <is>
-          <t>기타 화학제품 제조업</t>
+          <t>그외 기타 전문, 과학 및 기술 서비스업</t>
         </is>
       </c>
       <c r="J32" s="6" t="inlineStr">
         <is>
-          <t>미래, 한국</t>
+          <t>삼성, 미래</t>
         </is>
       </c>
       <c r="K32" s="6" t="inlineStr">
@@ -2190,12 +2202,12 @@
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>아델</t>
+          <t>에버온</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
@@ -2215,27 +2227,27 @@
       </c>
       <c r="F33" s="7" t="inlineStr">
         <is>
-          <t>62,057</t>
+          <t>65,225</t>
         </is>
       </c>
       <c r="G33" s="7" t="inlineStr">
         <is>
-          <t>-64,210</t>
+          <t>-3,606</t>
         </is>
       </c>
       <c r="H33" s="7" t="inlineStr">
         <is>
-          <t>-80,776</t>
+          <t>54,955</t>
         </is>
       </c>
       <c r="I33" s="6" t="inlineStr">
         <is>
-          <t>그외 기타 전문, 과학 및 기술 서비스업</t>
+          <t>전기업</t>
         </is>
       </c>
       <c r="J33" s="6" t="inlineStr">
         <is>
-          <t>삼성, 미래</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K33" s="6" t="inlineStr">
@@ -2247,12 +2259,12 @@
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>에버온</t>
+          <t>엔키화이트햇</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
@@ -2272,27 +2284,27 @@
       </c>
       <c r="F34" s="7" t="inlineStr">
         <is>
-          <t>65,225</t>
+          <t>14,176</t>
         </is>
       </c>
       <c r="G34" s="7" t="inlineStr">
         <is>
-          <t>-3,606</t>
+          <t>-3,211</t>
         </is>
       </c>
       <c r="H34" s="7" t="inlineStr">
         <is>
-          <t>54,955</t>
+          <t>8,338</t>
         </is>
       </c>
       <c r="I34" s="6" t="inlineStr">
         <is>
-          <t>전기업</t>
+          <t>소프트웨어 개발 및 공급업</t>
         </is>
       </c>
       <c r="J34" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>신영</t>
         </is>
       </c>
       <c r="K34" s="6" t="inlineStr">
@@ -2304,12 +2316,12 @@
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>엔키화이트햇</t>
+          <t>씨아이에스케미칼</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
@@ -2329,27 +2341,27 @@
       </c>
       <c r="F35" s="7" t="inlineStr">
         <is>
-          <t>14,176</t>
+          <t>15,985</t>
         </is>
       </c>
       <c r="G35" s="7" t="inlineStr">
         <is>
-          <t>-3,211</t>
+          <t>-11,440</t>
         </is>
       </c>
       <c r="H35" s="7" t="inlineStr">
         <is>
-          <t>8,338</t>
+          <t>23,706</t>
         </is>
       </c>
       <c r="I35" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어 개발 및 공급업</t>
+          <t>기초 화학물질 제조업</t>
         </is>
       </c>
       <c r="J35" s="6" t="inlineStr">
         <is>
-          <t>신영</t>
+          <t>KB</t>
         </is>
       </c>
       <c r="K35" s="6" t="inlineStr">
@@ -2361,12 +2373,12 @@
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>씨아이에스케미칼</t>
+          <t>엠디에스코리아</t>
         </is>
       </c>
       <c r="C36" s="6" t="inlineStr">
@@ -2386,27 +2398,27 @@
       </c>
       <c r="F36" s="7" t="inlineStr">
         <is>
-          <t>15,985</t>
+          <t>97,972</t>
         </is>
       </c>
       <c r="G36" s="7" t="inlineStr">
         <is>
-          <t>-11,440</t>
+          <t>6,512</t>
         </is>
       </c>
       <c r="H36" s="7" t="inlineStr">
         <is>
-          <t>23,706</t>
+          <t>53,818</t>
         </is>
       </c>
       <c r="I36" s="6" t="inlineStr">
         <is>
-          <t>기초 화학물질 제조업</t>
+          <t>기타 식품 제조업</t>
         </is>
       </c>
       <c r="J36" s="6" t="inlineStr">
         <is>
-          <t>KB</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K36" s="6" t="inlineStr">
@@ -2418,12 +2430,12 @@
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>엠디에스코리아</t>
+          <t>동승</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
@@ -2443,27 +2455,27 @@
       </c>
       <c r="F37" s="7" t="inlineStr">
         <is>
-          <t>97,972</t>
+          <t>78,625</t>
         </is>
       </c>
       <c r="G37" s="7" t="inlineStr">
         <is>
-          <t>6,512</t>
+          <t>14,525</t>
         </is>
       </c>
       <c r="H37" s="7" t="inlineStr">
         <is>
-          <t>53,818</t>
+          <t>5,438</t>
         </is>
       </c>
       <c r="I37" s="6" t="inlineStr">
         <is>
-          <t>기타 식품 제조업</t>
+          <t>부동산 임대 및 공급업</t>
         </is>
       </c>
       <c r="J37" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K37" s="6" t="inlineStr">
@@ -2480,7 +2492,7 @@
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>동승</t>
+          <t>에프엠더블유</t>
         </is>
       </c>
       <c r="C38" s="6" t="inlineStr">
@@ -2490,7 +2502,7 @@
       </c>
       <c r="D38" s="6" t="inlineStr">
         <is>
-          <t>신규상장</t>
+          <t>스팩 소멸합병</t>
         </is>
       </c>
       <c r="E38" s="6" t="inlineStr">
@@ -2500,27 +2512,27 @@
       </c>
       <c r="F38" s="7" t="inlineStr">
         <is>
-          <t>78,625</t>
+          <t>30,282</t>
         </is>
       </c>
       <c r="G38" s="7" t="inlineStr">
         <is>
-          <t>14,525</t>
+          <t>4,762</t>
         </is>
       </c>
       <c r="H38" s="7" t="inlineStr">
         <is>
-          <t>5,438</t>
+          <t>32</t>
         </is>
       </c>
       <c r="I38" s="6" t="inlineStr">
         <is>
-          <t>부동산 임대 및 공급업</t>
+          <t>기타 식품 제조업</t>
         </is>
       </c>
       <c r="J38" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>유진</t>
         </is>
       </c>
       <c r="K38" s="6" t="inlineStr">
@@ -2532,22 +2544,22 @@
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>에프엠더블유</t>
+          <t>소노인터내셔널</t>
         </is>
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>코스닥</t>
+          <t>유가</t>
         </is>
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
-          <t>스팩 소멸합병</t>
+          <t>신규상장</t>
         </is>
       </c>
       <c r="E39" s="6" t="inlineStr">
@@ -2557,27 +2569,27 @@
       </c>
       <c r="F39" s="7" t="inlineStr">
         <is>
-          <t>30,282</t>
+          <t>2,093,051</t>
         </is>
       </c>
       <c r="G39" s="7" t="inlineStr">
         <is>
-          <t>4,762</t>
+          <t>-148,064</t>
         </is>
       </c>
       <c r="H39" s="7" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>852,372</t>
         </is>
       </c>
       <c r="I39" s="6" t="inlineStr">
         <is>
-          <t>기타 식품 제조업</t>
+          <t>일반 및 생활 숙박시설 운영업</t>
         </is>
       </c>
       <c r="J39" s="6" t="inlineStr">
         <is>
-          <t>유진</t>
+          <t>대신, 미래</t>
         </is>
       </c>
       <c r="K39" s="6" t="inlineStr">
@@ -2589,17 +2601,17 @@
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>소노인터내셔널</t>
+          <t>싸이몬</t>
         </is>
       </c>
       <c r="C40" s="6" t="inlineStr">
         <is>
-          <t>유가</t>
+          <t>코스닥</t>
         </is>
       </c>
       <c r="D40" s="6" t="inlineStr">
@@ -2614,27 +2626,27 @@
       </c>
       <c r="F40" s="7" t="inlineStr">
         <is>
-          <t>2,093,051</t>
+          <t>48,695</t>
         </is>
       </c>
       <c r="G40" s="7" t="inlineStr">
         <is>
-          <t>-148,064</t>
+          <t>15,714</t>
         </is>
       </c>
       <c r="H40" s="7" t="inlineStr">
         <is>
-          <t>852,372</t>
+          <t>61,761</t>
         </is>
       </c>
       <c r="I40" s="6" t="inlineStr">
         <is>
-          <t>일반 및 생활 숙박시설 운영업</t>
+          <t>측정, 시험, 항해, 제어 및 기타 정밀기기 제조업</t>
         </is>
       </c>
       <c r="J40" s="6" t="inlineStr">
         <is>
-          <t>대신, 미래</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K40" s="6" t="inlineStr">
@@ -2646,12 +2658,12 @@
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>싸이몬</t>
+          <t>바이다</t>
         </is>
       </c>
       <c r="C41" s="6" t="inlineStr">
@@ -2671,27 +2683,27 @@
       </c>
       <c r="F41" s="7" t="inlineStr">
         <is>
-          <t>48,695</t>
+          <t>14,432</t>
         </is>
       </c>
       <c r="G41" s="7" t="inlineStr">
         <is>
-          <t>15,714</t>
+          <t>-3,951</t>
         </is>
       </c>
       <c r="H41" s="7" t="inlineStr">
         <is>
-          <t>61,761</t>
+          <t>15,108</t>
         </is>
       </c>
       <c r="I41" s="6" t="inlineStr">
         <is>
-          <t>측정, 시험, 항해, 제어 및 기타 정밀기기 제조업</t>
+          <t>전자부품 제조업</t>
         </is>
       </c>
       <c r="J41" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K41" s="6" t="inlineStr">
@@ -2703,12 +2715,12 @@
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B42" s="6" t="inlineStr">
         <is>
-          <t>바이다</t>
+          <t>아이알큐더스</t>
         </is>
       </c>
       <c r="C42" s="6" t="inlineStr">
@@ -2728,27 +2740,27 @@
       </c>
       <c r="F42" s="7" t="inlineStr">
         <is>
-          <t>14,432</t>
+          <t>10,231</t>
         </is>
       </c>
       <c r="G42" s="7" t="inlineStr">
         <is>
-          <t>-3,951</t>
+          <t>-986</t>
         </is>
       </c>
       <c r="H42" s="7" t="inlineStr">
         <is>
-          <t>15,108</t>
+          <t>1,800</t>
         </is>
       </c>
       <c r="I42" s="6" t="inlineStr">
         <is>
-          <t>전자부품 제조업</t>
+          <t>소프트웨어 개발 및 공급업</t>
         </is>
       </c>
       <c r="J42" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>DB</t>
         </is>
       </c>
       <c r="K42" s="6" t="inlineStr">
@@ -2760,12 +2772,12 @@
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B43" s="6" t="inlineStr">
         <is>
-          <t>아이알큐더스</t>
+          <t>씨엔티테크</t>
         </is>
       </c>
       <c r="C43" s="6" t="inlineStr">
@@ -2785,17 +2797,17 @@
       </c>
       <c r="F43" s="7" t="inlineStr">
         <is>
-          <t>10,231</t>
+          <t>27,015</t>
         </is>
       </c>
       <c r="G43" s="7" t="inlineStr">
         <is>
-          <t>-986</t>
+          <t>3,987</t>
         </is>
       </c>
       <c r="H43" s="7" t="inlineStr">
         <is>
-          <t>1,800</t>
+          <t>2,613</t>
         </is>
       </c>
       <c r="I43" s="6" t="inlineStr">
@@ -2805,7 +2817,7 @@
       </c>
       <c r="J43" s="6" t="inlineStr">
         <is>
-          <t>DB</t>
+          <t>한화, 하나</t>
         </is>
       </c>
       <c r="K43" s="6" t="inlineStr">
@@ -2822,7 +2834,7 @@
       </c>
       <c r="B44" s="6" t="inlineStr">
         <is>
-          <t>씨엔티테크</t>
+          <t>제이앤티지</t>
         </is>
       </c>
       <c r="C44" s="6" t="inlineStr">
@@ -2842,27 +2854,27 @@
       </c>
       <c r="F44" s="7" t="inlineStr">
         <is>
-          <t>27,015</t>
+          <t>72,378</t>
         </is>
       </c>
       <c r="G44" s="7" t="inlineStr">
         <is>
-          <t>3,987</t>
+          <t>9,904</t>
         </is>
       </c>
       <c r="H44" s="7" t="inlineStr">
         <is>
-          <t>2,613</t>
+          <t>6,743</t>
         </is>
       </c>
       <c r="I44" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어 개발 및 공급업</t>
+          <t>전자부품 제조업</t>
         </is>
       </c>
       <c r="J44" s="6" t="inlineStr">
         <is>
-          <t>한화, 하나</t>
+          <t>대신, NH</t>
         </is>
       </c>
       <c r="K44" s="6" t="inlineStr">
@@ -2874,12 +2886,12 @@
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B45" s="6" t="inlineStr">
         <is>
-          <t>제이앤티지</t>
+          <t>인터엑스</t>
         </is>
       </c>
       <c r="C45" s="6" t="inlineStr">
@@ -2899,27 +2911,27 @@
       </c>
       <c r="F45" s="7" t="inlineStr">
         <is>
-          <t>72,378</t>
+          <t>8,645</t>
         </is>
       </c>
       <c r="G45" s="7" t="inlineStr">
         <is>
-          <t>9,904</t>
+          <t>-20,272</t>
         </is>
       </c>
       <c r="H45" s="7" t="inlineStr">
         <is>
-          <t>6,743</t>
+          <t>4,530</t>
         </is>
       </c>
       <c r="I45" s="6" t="inlineStr">
         <is>
-          <t>전자부품 제조업</t>
+          <t>소프트웨어 개발 및 공급업</t>
         </is>
       </c>
       <c r="J45" s="6" t="inlineStr">
         <is>
-          <t>대신, NH</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="K45" s="6" t="inlineStr">
@@ -2931,12 +2943,12 @@
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B46" s="6" t="inlineStr">
         <is>
-          <t>인터엑스</t>
+          <t>삼홍아크튜리온</t>
         </is>
       </c>
       <c r="C46" s="6" t="inlineStr">
@@ -2956,27 +2968,27 @@
       </c>
       <c r="F46" s="7" t="inlineStr">
         <is>
-          <t>8,645</t>
+          <t>26,162</t>
         </is>
       </c>
       <c r="G46" s="7" t="inlineStr">
         <is>
-          <t>-20,272</t>
+          <t>-10,314</t>
         </is>
       </c>
       <c r="H46" s="7" t="inlineStr">
         <is>
-          <t>4,530</t>
+          <t>6,369</t>
         </is>
       </c>
       <c r="I46" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어 개발 및 공급업</t>
+          <t>구조용 금속제품, 탱크 및 증기발생기 제조업</t>
         </is>
       </c>
       <c r="J46" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>삼성, 미래</t>
         </is>
       </c>
       <c r="K46" s="6" t="inlineStr">
@@ -2988,12 +3000,12 @@
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B47" s="6" t="inlineStr">
         <is>
-          <t>삼홍아크튜리온</t>
+          <t>넥스트에어로스페이스</t>
         </is>
       </c>
       <c r="C47" s="6" t="inlineStr">
@@ -3013,27 +3025,27 @@
       </c>
       <c r="F47" s="7" t="inlineStr">
         <is>
-          <t>26,162</t>
+          <t>12,084</t>
         </is>
       </c>
       <c r="G47" s="7" t="inlineStr">
         <is>
-          <t>-10,314</t>
+          <t>-17,270</t>
         </is>
       </c>
       <c r="H47" s="7" t="inlineStr">
         <is>
-          <t>6,369</t>
+          <t>6,158</t>
         </is>
       </c>
       <c r="I47" s="6" t="inlineStr">
         <is>
-          <t>구조용 금속제품, 탱크 및 증기발생기 제조업</t>
+          <t>유인 항공기, 항공우주선 및 보조장치 제조업</t>
         </is>
       </c>
       <c r="J47" s="6" t="inlineStr">
         <is>
-          <t>삼성, 미래</t>
+          <t>삼성</t>
         </is>
       </c>
       <c r="K47" s="6" t="inlineStr">
@@ -3050,7 +3062,7 @@
       </c>
       <c r="B48" s="6" t="inlineStr">
         <is>
-          <t>넥스트에어로스페이스</t>
+          <t>비앤비코리아</t>
         </is>
       </c>
       <c r="C48" s="6" t="inlineStr">
@@ -3070,27 +3082,27 @@
       </c>
       <c r="F48" s="7" t="inlineStr">
         <is>
-          <t>12,084</t>
+          <t>141,169</t>
         </is>
       </c>
       <c r="G48" s="7" t="inlineStr">
         <is>
-          <t>-17,270</t>
+          <t>21,406</t>
         </is>
       </c>
       <c r="H48" s="7" t="inlineStr">
         <is>
-          <t>6,158</t>
+          <t>43,932</t>
         </is>
       </c>
       <c r="I48" s="6" t="inlineStr">
         <is>
-          <t>유인 항공기, 항공우주선 및 보조장치 제조업</t>
+          <t>기타 화학제품 제조업</t>
         </is>
       </c>
       <c r="J48" s="6" t="inlineStr">
         <is>
-          <t>삼성</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K48" s="6" t="inlineStr">
@@ -3102,12 +3114,12 @@
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B49" s="6" t="inlineStr">
         <is>
-          <t>비앤비코리아</t>
+          <t>오토핸즈</t>
         </is>
       </c>
       <c r="C49" s="6" t="inlineStr">
@@ -3117,7 +3129,7 @@
       </c>
       <c r="D49" s="6" t="inlineStr">
         <is>
-          <t>신규상장</t>
+          <t>스팩 소멸합병</t>
         </is>
       </c>
       <c r="E49" s="6" t="inlineStr">
@@ -3127,22 +3139,22 @@
       </c>
       <c r="F49" s="7" t="inlineStr">
         <is>
-          <t>141,169</t>
+          <t>238,564</t>
         </is>
       </c>
       <c r="G49" s="7" t="inlineStr">
         <is>
-          <t>21,406</t>
+          <t>6,047</t>
         </is>
       </c>
       <c r="H49" s="7" t="inlineStr">
         <is>
-          <t>43,932</t>
+          <t>6,129</t>
         </is>
       </c>
       <c r="I49" s="6" t="inlineStr">
         <is>
-          <t>기타 화학제품 제조업</t>
+          <t>자동차 판매업</t>
         </is>
       </c>
       <c r="J49" s="6" t="inlineStr">
@@ -3159,12 +3171,12 @@
     <row r="50">
       <c r="A50" s="6" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B50" s="6" t="inlineStr">
         <is>
-          <t>오토핸즈</t>
+          <t>아이벡스메디칼시스템즈</t>
         </is>
       </c>
       <c r="C50" s="6" t="inlineStr">
@@ -3174,7 +3186,7 @@
       </c>
       <c r="D50" s="6" t="inlineStr">
         <is>
-          <t>스팩 소멸합병</t>
+          <t>신규상장</t>
         </is>
       </c>
       <c r="E50" s="6" t="inlineStr">
@@ -3184,27 +3196,27 @@
       </c>
       <c r="F50" s="7" t="inlineStr">
         <is>
-          <t>238,564</t>
+          <t>15,282</t>
         </is>
       </c>
       <c r="G50" s="7" t="inlineStr">
         <is>
-          <t>6,047</t>
+          <t>-7,227</t>
         </is>
       </c>
       <c r="H50" s="7" t="inlineStr">
         <is>
-          <t>6,129</t>
+          <t>744</t>
         </is>
       </c>
       <c r="I50" s="6" t="inlineStr">
         <is>
-          <t>자동차 판매업</t>
+          <t>의료용 기기 제조업</t>
         </is>
       </c>
       <c r="J50" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K50" s="6" t="inlineStr">
@@ -3216,12 +3228,12 @@
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="B51" s="6" t="inlineStr">
         <is>
-          <t>아이벡스메디칼시스템즈</t>
+          <t>피지티</t>
         </is>
       </c>
       <c r="C51" s="6" t="inlineStr">
@@ -3241,27 +3253,27 @@
       </c>
       <c r="F51" s="7" t="inlineStr">
         <is>
-          <t>15,282</t>
+          <t>40,141</t>
         </is>
       </c>
       <c r="G51" s="7" t="inlineStr">
         <is>
-          <t>-7,227</t>
+          <t>-69,722</t>
         </is>
       </c>
       <c r="H51" s="7" t="inlineStr">
         <is>
-          <t>744</t>
+          <t>6,029</t>
         </is>
       </c>
       <c r="I51" s="6" t="inlineStr">
         <is>
-          <t>의료용 기기 제조업</t>
+          <t>기타 화학제품 제조업</t>
         </is>
       </c>
       <c r="J51" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="K51" s="6" t="inlineStr">
@@ -3270,134 +3282,122 @@
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="6" t="inlineStr">
-        <is>
-          <t>2026-02-27</t>
-        </is>
-      </c>
-      <c r="B52" s="6" t="inlineStr">
-        <is>
-          <t>피지티</t>
-        </is>
-      </c>
-      <c r="C52" s="6" t="inlineStr">
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>■ 심사 승인  (71건)</t>
+        </is>
+      </c>
+      <c r="B53" s="4" t="n"/>
+      <c r="C53" s="4" t="n"/>
+      <c r="D53" s="4" t="n"/>
+      <c r="E53" s="4" t="n"/>
+      <c r="F53" s="4" t="n"/>
+      <c r="G53" s="4" t="n"/>
+      <c r="H53" s="4" t="n"/>
+      <c r="I53" s="4" t="n"/>
+      <c r="J53" s="4" t="n"/>
+      <c r="K53" s="4" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>일자</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="inlineStr">
+        <is>
+          <t>회사명</t>
+        </is>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>시장</t>
+        </is>
+      </c>
+      <c r="D54" s="5" t="inlineStr">
+        <is>
+          <t>상장유형</t>
+        </is>
+      </c>
+      <c r="E54" s="5" t="inlineStr">
+        <is>
+          <t>기준연도</t>
+        </is>
+      </c>
+      <c r="F54" s="5" t="inlineStr">
+        <is>
+          <t>매출액</t>
+        </is>
+      </c>
+      <c r="G54" s="5" t="inlineStr">
+        <is>
+          <t>순이익</t>
+        </is>
+      </c>
+      <c r="H54" s="5" t="inlineStr">
+        <is>
+          <t>자기자본</t>
+        </is>
+      </c>
+      <c r="I54" s="5" t="inlineStr">
+        <is>
+          <t>업종</t>
+        </is>
+      </c>
+      <c r="J54" s="5" t="inlineStr">
+        <is>
+          <t>대표주관사</t>
+        </is>
+      </c>
+      <c r="K54" s="5" t="inlineStr">
+        <is>
+          <t>현황</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B55" s="6" t="inlineStr">
+        <is>
+          <t>우리투자제1호스팩</t>
+        </is>
+      </c>
+      <c r="C55" s="6" t="inlineStr">
         <is>
           <t>코스닥</t>
         </is>
       </c>
-      <c r="D52" s="6" t="inlineStr">
+      <c r="D55" s="6" t="inlineStr">
         <is>
           <t>신규상장</t>
         </is>
       </c>
-      <c r="E52" s="6" t="inlineStr">
+      <c r="E55" s="6" t="inlineStr">
         <is>
           <t>FY25</t>
         </is>
       </c>
-      <c r="F52" s="7" t="inlineStr">
-        <is>
-          <t>40,141</t>
-        </is>
-      </c>
-      <c r="G52" s="7" t="inlineStr">
-        <is>
-          <t>-69,722</t>
-        </is>
-      </c>
-      <c r="H52" s="7" t="inlineStr">
-        <is>
-          <t>6,029</t>
-        </is>
-      </c>
-      <c r="I52" s="6" t="inlineStr">
-        <is>
-          <t>기타 화학제품 제조업</t>
-        </is>
-      </c>
-      <c r="J52" s="6" t="inlineStr">
-        <is>
-          <t>한국</t>
-        </is>
-      </c>
-      <c r="K52" s="6" t="inlineStr">
-        <is>
-          <t>예심 진행중</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="3" t="inlineStr">
-        <is>
-          <t>■ 심사 승인  (70건)</t>
-        </is>
-      </c>
-      <c r="B54" s="4" t="n"/>
-      <c r="C54" s="4" t="n"/>
-      <c r="D54" s="4" t="n"/>
-      <c r="E54" s="4" t="n"/>
-      <c r="F54" s="4" t="n"/>
-      <c r="G54" s="4" t="n"/>
-      <c r="H54" s="4" t="n"/>
-      <c r="I54" s="4" t="n"/>
-      <c r="J54" s="4" t="n"/>
-      <c r="K54" s="4" t="n"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="5" t="inlineStr">
-        <is>
-          <t>일자</t>
-        </is>
-      </c>
-      <c r="B55" s="5" t="inlineStr">
-        <is>
-          <t>회사명</t>
-        </is>
-      </c>
-      <c r="C55" s="5" t="inlineStr">
-        <is>
-          <t>시장</t>
-        </is>
-      </c>
-      <c r="D55" s="5" t="inlineStr">
-        <is>
-          <t>상장유형</t>
-        </is>
-      </c>
-      <c r="E55" s="5" t="inlineStr">
-        <is>
-          <t>기준연도</t>
-        </is>
-      </c>
-      <c r="F55" s="5" t="inlineStr">
-        <is>
-          <t>매출액</t>
-        </is>
-      </c>
-      <c r="G55" s="5" t="inlineStr">
-        <is>
-          <t>순이익</t>
-        </is>
-      </c>
-      <c r="H55" s="5" t="inlineStr">
-        <is>
-          <t>자기자본</t>
-        </is>
-      </c>
-      <c r="I55" s="5" t="inlineStr">
-        <is>
-          <t>업종</t>
-        </is>
-      </c>
-      <c r="J55" s="5" t="inlineStr">
-        <is>
-          <t>대표주관사</t>
-        </is>
-      </c>
-      <c r="K55" s="5" t="inlineStr">
-        <is>
-          <t>현황</t>
+      <c r="F55" s="7" t="inlineStr"/>
+      <c r="G55" s="7" t="inlineStr"/>
+      <c r="H55" s="7" t="inlineStr"/>
+      <c r="I55" s="6" t="inlineStr">
+        <is>
+          <t>기타 금융업</t>
+        </is>
+      </c>
+      <c r="J55" s="6" t="inlineStr">
+        <is>
+          <t>주식회사 우리투자증권</t>
+        </is>
+      </c>
+      <c r="K55" s="6" t="inlineStr">
+        <is>
+          <t>상장전</t>
         </is>
       </c>
     </row>
@@ -8350,7 +8350,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R91"/>
+  <dimension ref="A1:R92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -12432,7 +12432,7 @@
     <row r="56" ht="22" customHeight="1">
       <c r="A56" s="3" t="inlineStr">
         <is>
-          <t>■ 공모 진행 (예심 승인법인)  (31건)</t>
+          <t>■ 공모 진행 (예심 승인법인)  (32건)</t>
         </is>
       </c>
       <c r="B56" s="4" t="n"/>
@@ -12696,7 +12696,7 @@
       </c>
       <c r="E60" s="7" t="inlineStr">
         <is>
-          <t>156,428,800,000</t>
+          <t>201,091,000,000</t>
         </is>
       </c>
       <c r="F60" s="6" t="inlineStr">
@@ -12704,9 +12704,17 @@
           <t>27.13배 (EV/EBITDA)</t>
         </is>
       </c>
-      <c r="G60" s="6" t="inlineStr"/>
-      <c r="H60" s="6" t="inlineStr"/>
-      <c r="I60" s="6" t="inlineStr"/>
+      <c r="G60" s="6" t="inlineStr">
+        <is>
+          <t>90,500</t>
+        </is>
+      </c>
+      <c r="H60" s="6" t="n">
+        <v>388.84</v>
+      </c>
+      <c r="I60" s="6" t="n">
+        <v>2367</v>
+      </c>
       <c r="J60" s="6" t="inlineStr">
         <is>
           <t>10-07~10-08</t>
@@ -12737,7 +12745,7 @@
       </c>
       <c r="R60" s="6" t="inlineStr">
         <is>
-          <t>정정</t>
+          <t>발행조건확정</t>
         </is>
       </c>
     </row>
@@ -12936,32 +12944,32 @@
     <row r="64" ht="30" customHeight="1">
       <c r="A64" s="6" t="inlineStr">
         <is>
-          <t>에스케이증권제14호기업인수목적</t>
+          <t>다비오</t>
         </is>
       </c>
       <c r="B64" s="6" t="inlineStr">
         <is>
-          <t>10-12~10-13</t>
-        </is>
-      </c>
-      <c r="C64" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>10-07~10-14</t>
+        </is>
+      </c>
+      <c r="C64" s="6" t="inlineStr">
+        <is>
+          <t>12,300~16,600</t>
         </is>
       </c>
       <c r="D64" s="7" t="inlineStr">
         <is>
-          <t>6,500,000</t>
+          <t>1,000,000</t>
         </is>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
-          <t>13,000,000,000</t>
-        </is>
-      </c>
-      <c r="F64" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>12,300,000,000</t>
+        </is>
+      </c>
+      <c r="F64" s="6" t="inlineStr">
+        <is>
+          <t>26.70배 (PER)</t>
         </is>
       </c>
       <c r="G64" s="6" t="inlineStr"/>
@@ -12969,26 +12977,26 @@
       <c r="I64" s="6" t="inlineStr"/>
       <c r="J64" s="6" t="inlineStr">
         <is>
-          <t>10-15~10-16</t>
+          <t>10-19~10-20</t>
         </is>
       </c>
       <c r="K64" s="6" t="inlineStr"/>
       <c r="L64" s="6" t="inlineStr"/>
       <c r="M64" s="6" t="inlineStr"/>
-      <c r="N64" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="N64" s="6" t="inlineStr">
+        <is>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="O64" s="6" t="inlineStr"/>
-      <c r="P64" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="P64" s="7" t="inlineStr">
+        <is>
+          <t>570,105,000</t>
         </is>
       </c>
       <c r="Q64" s="6" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>4.5%</t>
         </is>
       </c>
       <c r="R64" s="6" t="inlineStr">
@@ -13000,32 +13008,32 @@
     <row r="65" ht="30" customHeight="1">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>크리에이츠</t>
+          <t>에스케이증권제14호기업인수목적</t>
         </is>
       </c>
       <c r="B65" s="6" t="inlineStr">
         <is>
-          <t>10-12~10-16</t>
-        </is>
-      </c>
-      <c r="C65" s="6" t="inlineStr">
-        <is>
-          <t>15,000~18,000</t>
+          <t>10-12~10-13</t>
+        </is>
+      </c>
+      <c r="C65" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="D65" s="7" t="inlineStr">
         <is>
-          <t>1,400,000</t>
+          <t>6,500,000</t>
         </is>
       </c>
       <c r="E65" s="7" t="inlineStr">
         <is>
-          <t>21,000,000,000</t>
-        </is>
-      </c>
-      <c r="F65" s="6" t="inlineStr">
-        <is>
-          <t>19.15배 (PER)</t>
+          <t>13,000,000,000</t>
+        </is>
+      </c>
+      <c r="F65" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="G65" s="6" t="inlineStr"/>
@@ -13033,26 +13041,26 @@
       <c r="I65" s="6" t="inlineStr"/>
       <c r="J65" s="6" t="inlineStr">
         <is>
-          <t>10-20~10-21</t>
+          <t>10-15~10-16</t>
         </is>
       </c>
       <c r="K65" s="6" t="inlineStr"/>
       <c r="L65" s="6" t="inlineStr"/>
       <c r="M65" s="6" t="inlineStr"/>
-      <c r="N65" s="6" t="inlineStr">
-        <is>
-          <t>삼성증권</t>
+      <c r="N65" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="O65" s="6" t="inlineStr"/>
-      <c r="P65" s="7" t="inlineStr">
-        <is>
-          <t>865,200,000</t>
+      <c r="P65" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="Q65" s="6" t="inlineStr">
         <is>
-          <t>4.0%</t>
+          <t>50%</t>
         </is>
       </c>
       <c r="R65" s="6" t="inlineStr">
@@ -13064,32 +13072,32 @@
     <row r="66" ht="30" customHeight="1">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>래블업</t>
+          <t>크리에이츠</t>
         </is>
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
-          <t>10-13~10-19</t>
+          <t>10-12~10-16</t>
         </is>
       </c>
       <c r="C66" s="6" t="inlineStr">
         <is>
-          <t>19,000~22,000</t>
+          <t>15,000~18,000</t>
         </is>
       </c>
       <c r="D66" s="7" t="inlineStr">
         <is>
-          <t>2,180,000</t>
+          <t>1,400,000</t>
         </is>
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
-          <t>41,420,000,000</t>
+          <t>21,000,000,000</t>
         </is>
       </c>
       <c r="F66" s="6" t="inlineStr">
         <is>
-          <t>33.6배 (PER)</t>
+          <t>19.15배 (PER)</t>
         </is>
       </c>
       <c r="G66" s="6" t="inlineStr"/>
@@ -13097,7 +13105,7 @@
       <c r="I66" s="6" t="inlineStr"/>
       <c r="J66" s="6" t="inlineStr">
         <is>
-          <t>10-22~10-23</t>
+          <t>10-20~10-21</t>
         </is>
       </c>
       <c r="K66" s="6" t="inlineStr"/>
@@ -13105,18 +13113,18 @@
       <c r="M66" s="6" t="inlineStr"/>
       <c r="N66" s="6" t="inlineStr">
         <is>
-          <t>NH투자증권</t>
+          <t>삼성증권</t>
         </is>
       </c>
       <c r="O66" s="6" t="inlineStr"/>
       <c r="P66" s="7" t="inlineStr">
         <is>
-          <t>1,908,899,000</t>
+          <t>865,200,000</t>
         </is>
       </c>
       <c r="Q66" s="6" t="inlineStr">
         <is>
-          <t>4.5%</t>
+          <t>4.0%</t>
         </is>
       </c>
       <c r="R66" s="6" t="inlineStr">
@@ -13128,32 +13136,32 @@
     <row r="67" ht="30" customHeight="1">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>엠비디</t>
+          <t>래블업</t>
         </is>
       </c>
       <c r="B67" s="6" t="inlineStr">
         <is>
-          <t>10-16~10-22</t>
+          <t>10-13~10-19</t>
         </is>
       </c>
       <c r="C67" s="6" t="inlineStr">
         <is>
-          <t>9,600~11,700</t>
+          <t>19,000~22,000</t>
         </is>
       </c>
       <c r="D67" s="7" t="inlineStr">
         <is>
-          <t>2,000,000</t>
+          <t>2,180,000</t>
         </is>
       </c>
       <c r="E67" s="7" t="inlineStr">
         <is>
-          <t>19,200,000,000</t>
+          <t>41,420,000,000</t>
         </is>
       </c>
       <c r="F67" s="6" t="inlineStr">
         <is>
-          <t>26.87배 (PER)</t>
+          <t>33.6배 (PER)</t>
         </is>
       </c>
       <c r="G67" s="6" t="inlineStr"/>
@@ -13161,7 +13169,7 @@
       <c r="I67" s="6" t="inlineStr"/>
       <c r="J67" s="6" t="inlineStr">
         <is>
-          <t>10-28~10-29</t>
+          <t>10-22~10-23</t>
         </is>
       </c>
       <c r="K67" s="6" t="inlineStr"/>
@@ -13169,18 +13177,18 @@
       <c r="M67" s="6" t="inlineStr"/>
       <c r="N67" s="6" t="inlineStr">
         <is>
-          <t>하나증권</t>
+          <t>NH투자증권</t>
         </is>
       </c>
       <c r="O67" s="6" t="inlineStr"/>
       <c r="P67" s="7" t="inlineStr">
         <is>
-          <t>988,800,000</t>
+          <t>1,908,899,000</t>
         </is>
       </c>
       <c r="Q67" s="6" t="inlineStr">
         <is>
-          <t>5.0%</t>
+          <t>4.5%</t>
         </is>
       </c>
       <c r="R67" s="6" t="inlineStr">
@@ -13192,40 +13200,40 @@
     <row r="68" ht="30" customHeight="1">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>바로팜</t>
-        </is>
-      </c>
-      <c r="B68" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="C68" s="6" t="inlineStr">
-        <is>
-          <t>16,400~20,200</t>
+          <t>한화플러스제6호스팩</t>
+        </is>
+      </c>
+      <c r="B68" s="6" t="inlineStr">
+        <is>
+          <t>10-14~10-15</t>
+        </is>
+      </c>
+      <c r="C68" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="D68" s="7" t="inlineStr">
         <is>
-          <t>1,780,000</t>
+          <t>6,000,000</t>
         </is>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
-          <t>29,192,000,000</t>
-        </is>
-      </c>
-      <c r="F68" s="6" t="inlineStr">
-        <is>
-          <t>24.95배 (PER)</t>
+          <t>12,000,000,000</t>
+        </is>
+      </c>
+      <c r="F68" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="G68" s="6" t="inlineStr"/>
       <c r="H68" s="6" t="inlineStr"/>
       <c r="I68" s="6" t="inlineStr"/>
-      <c r="J68" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="J68" s="6" t="inlineStr">
+        <is>
+          <t>10-20~10-21</t>
         </is>
       </c>
       <c r="K68" s="6" t="inlineStr"/>
@@ -13242,9 +13250,9 @@
           <t>수집예정</t>
         </is>
       </c>
-      <c r="Q68" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="Q68" s="6" t="inlineStr">
+        <is>
+          <t>3.50%</t>
         </is>
       </c>
       <c r="R68" s="6" t="inlineStr">
@@ -13256,59 +13264,59 @@
     <row r="69" ht="30" customHeight="1">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>셀트릭스</t>
-        </is>
-      </c>
-      <c r="B69" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="C69" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="D69" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="E69" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="F69" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>엠비디</t>
+        </is>
+      </c>
+      <c r="B69" s="6" t="inlineStr">
+        <is>
+          <t>10-16~10-22</t>
+        </is>
+      </c>
+      <c r="C69" s="6" t="inlineStr">
+        <is>
+          <t>9,600~11,700</t>
+        </is>
+      </c>
+      <c r="D69" s="7" t="inlineStr">
+        <is>
+          <t>2,000,000</t>
+        </is>
+      </c>
+      <c r="E69" s="7" t="inlineStr">
+        <is>
+          <t>19,200,000,000</t>
+        </is>
+      </c>
+      <c r="F69" s="6" t="inlineStr">
+        <is>
+          <t>26.87배 (PER)</t>
         </is>
       </c>
       <c r="G69" s="6" t="inlineStr"/>
       <c r="H69" s="6" t="inlineStr"/>
       <c r="I69" s="6" t="inlineStr"/>
-      <c r="J69" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="J69" s="6" t="inlineStr">
+        <is>
+          <t>10-28~10-29</t>
         </is>
       </c>
       <c r="K69" s="6" t="inlineStr"/>
       <c r="L69" s="6" t="inlineStr"/>
       <c r="M69" s="6" t="inlineStr"/>
-      <c r="N69" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="N69" s="6" t="inlineStr">
+        <is>
+          <t>하나증권</t>
         </is>
       </c>
       <c r="O69" s="6" t="inlineStr"/>
-      <c r="P69" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="Q69" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="P69" s="7" t="inlineStr">
+        <is>
+          <t>988,800,000</t>
+        </is>
+      </c>
+      <c r="Q69" s="6" t="inlineStr">
+        <is>
+          <t>5.0%</t>
         </is>
       </c>
       <c r="R69" s="6" t="inlineStr">
@@ -13320,160 +13328,160 @@
     <row r="70" ht="30" customHeight="1">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>다비오</t>
-        </is>
-      </c>
-      <c r="B70" s="6" t="inlineStr">
-        <is>
-          <t>10-07~10-14</t>
+          <t>바로팜</t>
+        </is>
+      </c>
+      <c r="B70" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr">
         <is>
-          <t>12,300~16,600</t>
+          <t>16,400~20,200</t>
         </is>
       </c>
       <c r="D70" s="7" t="inlineStr">
         <is>
-          <t>1,000,000</t>
+          <t>1,780,000</t>
         </is>
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
-          <t>12,300,000,000</t>
+          <t>29,192,000,000</t>
         </is>
       </c>
       <c r="F70" s="6" t="inlineStr">
         <is>
-          <t>26.70배 (PER)</t>
+          <t>24.95배 (PER)</t>
         </is>
       </c>
       <c r="G70" s="6" t="inlineStr"/>
       <c r="H70" s="6" t="inlineStr"/>
       <c r="I70" s="6" t="inlineStr"/>
-      <c r="J70" s="6" t="inlineStr">
-        <is>
-          <t>10-19~10-20</t>
+      <c r="J70" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="K70" s="6" t="inlineStr"/>
       <c r="L70" s="6" t="inlineStr"/>
       <c r="M70" s="6" t="inlineStr"/>
-      <c r="N70" s="6" t="inlineStr">
-        <is>
-          <t>대신증권</t>
+      <c r="N70" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="O70" s="6" t="inlineStr"/>
-      <c r="P70" s="7" t="inlineStr">
-        <is>
-          <t>570,105,000</t>
-        </is>
-      </c>
-      <c r="Q70" s="6" t="inlineStr">
-        <is>
-          <t>4.5%</t>
+      <c r="P70" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="Q70" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="R70" s="6" t="inlineStr">
         <is>
-          <t>최초</t>
+          <t>정정</t>
         </is>
       </c>
     </row>
     <row r="71" ht="30" customHeight="1">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>인텔리빅스</t>
-        </is>
-      </c>
-      <c r="B71" s="6" t="inlineStr">
-        <is>
-          <t>10-12~10-16</t>
-        </is>
-      </c>
-      <c r="C71" s="6" t="inlineStr">
-        <is>
-          <t>7,600~9,000</t>
-        </is>
-      </c>
-      <c r="D71" s="7" t="inlineStr">
-        <is>
-          <t>2,500,000</t>
-        </is>
-      </c>
-      <c r="E71" s="7" t="inlineStr">
-        <is>
-          <t>19,000,000,000</t>
-        </is>
-      </c>
-      <c r="F71" s="6" t="inlineStr">
-        <is>
-          <t>22.02배 (PER)</t>
+          <t>셀트릭스</t>
+        </is>
+      </c>
+      <c r="B71" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="C71" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="D71" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="E71" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="F71" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="G71" s="6" t="inlineStr"/>
       <c r="H71" s="6" t="inlineStr"/>
       <c r="I71" s="6" t="inlineStr"/>
-      <c r="J71" s="6" t="inlineStr">
-        <is>
-          <t>10-21~10-22</t>
+      <c r="J71" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="K71" s="6" t="inlineStr"/>
       <c r="L71" s="6" t="inlineStr"/>
       <c r="M71" s="6" t="inlineStr"/>
-      <c r="N71" s="6" t="inlineStr">
-        <is>
-          <t>미래에셋증권</t>
+      <c r="N71" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="O71" s="6" t="inlineStr"/>
-      <c r="P71" s="7" t="inlineStr">
-        <is>
-          <t>782,800,000</t>
-        </is>
-      </c>
-      <c r="Q71" s="6" t="inlineStr">
-        <is>
-          <t>4.0%</t>
+      <c r="P71" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="Q71" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="R71" s="6" t="inlineStr">
         <is>
-          <t>최초</t>
+          <t>정정</t>
         </is>
       </c>
     </row>
     <row r="72" ht="30" customHeight="1">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>영광</t>
+          <t>인텔리빅스</t>
         </is>
       </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>10-13~10-19</t>
+          <t>10-12~10-16</t>
         </is>
       </c>
       <c r="C72" s="6" t="inlineStr">
         <is>
-          <t>14,000~17,000</t>
+          <t>7,600~9,000</t>
         </is>
       </c>
       <c r="D72" s="7" t="inlineStr">
         <is>
-          <t>2,260,000</t>
+          <t>2,500,000</t>
         </is>
       </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
-          <t>31,640,000,000</t>
+          <t>19,000,000,000</t>
         </is>
       </c>
       <c r="F72" s="6" t="inlineStr">
         <is>
-          <t>11.98배 (EV/EBITDA)</t>
+          <t>22.02배 (PER)</t>
         </is>
       </c>
       <c r="G72" s="6" t="inlineStr"/>
@@ -13481,7 +13489,7 @@
       <c r="I72" s="6" t="inlineStr"/>
       <c r="J72" s="6" t="inlineStr">
         <is>
-          <t>10-22~10-23</t>
+          <t>10-21~10-22</t>
         </is>
       </c>
       <c r="K72" s="6" t="inlineStr"/>
@@ -13489,18 +13497,18 @@
       <c r="M72" s="6" t="inlineStr"/>
       <c r="N72" s="6" t="inlineStr">
         <is>
-          <t>한국투자증권</t>
+          <t>미래에셋증권</t>
         </is>
       </c>
       <c r="O72" s="6" t="inlineStr"/>
       <c r="P72" s="7" t="inlineStr">
         <is>
-          <t>977,676,000</t>
-        </is>
-      </c>
-      <c r="Q72" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>782,800,000</t>
+        </is>
+      </c>
+      <c r="Q72" s="6" t="inlineStr">
+        <is>
+          <t>4.0%</t>
         </is>
       </c>
       <c r="R72" s="6" t="inlineStr">
@@ -13512,32 +13520,32 @@
     <row r="73" ht="30" customHeight="1">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>한화플러스제6호스팩</t>
+          <t>영광</t>
         </is>
       </c>
       <c r="B73" s="6" t="inlineStr">
         <is>
-          <t>10-14~10-15</t>
-        </is>
-      </c>
-      <c r="C73" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>10-13~10-19</t>
+        </is>
+      </c>
+      <c r="C73" s="6" t="inlineStr">
+        <is>
+          <t>14,000~17,000</t>
         </is>
       </c>
       <c r="D73" s="7" t="inlineStr">
         <is>
-          <t>6,000,000</t>
+          <t>2,260,000</t>
         </is>
       </c>
       <c r="E73" s="7" t="inlineStr">
         <is>
-          <t>12,000,000,000</t>
-        </is>
-      </c>
-      <c r="F73" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>31,640,000,000</t>
+        </is>
+      </c>
+      <c r="F73" s="6" t="inlineStr">
+        <is>
+          <t>11.98배 (EV/EBITDA)</t>
         </is>
       </c>
       <c r="G73" s="6" t="inlineStr"/>
@@ -13545,26 +13553,26 @@
       <c r="I73" s="6" t="inlineStr"/>
       <c r="J73" s="6" t="inlineStr">
         <is>
-          <t>10-20~10-21</t>
+          <t>10-22~10-23</t>
         </is>
       </c>
       <c r="K73" s="6" t="inlineStr"/>
       <c r="L73" s="6" t="inlineStr"/>
       <c r="M73" s="6" t="inlineStr"/>
-      <c r="N73" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="N73" s="6" t="inlineStr">
+        <is>
+          <t>한국투자증권</t>
         </is>
       </c>
       <c r="O73" s="6" t="inlineStr"/>
-      <c r="P73" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="Q73" s="6" t="inlineStr">
-        <is>
-          <t>3.50%</t>
+      <c r="P73" s="7" t="inlineStr">
+        <is>
+          <t>977,676,000</t>
+        </is>
+      </c>
+      <c r="Q73" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="R73" s="6" t="inlineStr">
@@ -14024,7 +14032,7 @@
     <row r="81" ht="30" customHeight="1">
       <c r="A81" s="6" t="inlineStr">
         <is>
-          <t>솔리스</t>
+          <t>럭스코</t>
         </is>
       </c>
       <c r="B81" s="18" t="inlineStr">
@@ -14088,7 +14096,7 @@
     <row r="82" ht="30" customHeight="1">
       <c r="A82" s="6" t="inlineStr">
         <is>
-          <t>디티에스</t>
+          <t>솔리스</t>
         </is>
       </c>
       <c r="B82" s="18" t="inlineStr">
@@ -14145,14 +14153,14 @@
       </c>
       <c r="R82" s="6" t="inlineStr">
         <is>
-          <t>신고서 대기</t>
+          <t>최초</t>
         </is>
       </c>
     </row>
     <row r="83" ht="30" customHeight="1">
       <c r="A83" s="6" t="inlineStr">
         <is>
-          <t>에이엔에이치스트럭쳐</t>
+          <t>디티에스</t>
         </is>
       </c>
       <c r="B83" s="18" t="inlineStr">
@@ -14216,7 +14224,7 @@
     <row r="84" ht="30" customHeight="1">
       <c r="A84" s="6" t="inlineStr">
         <is>
-          <t>이에스티</t>
+          <t>에이엔에이치스트럭쳐</t>
         </is>
       </c>
       <c r="B84" s="18" t="inlineStr">
@@ -14280,7 +14288,7 @@
     <row r="85" ht="30" customHeight="1">
       <c r="A85" s="6" t="inlineStr">
         <is>
-          <t>영광와이케이엠씨</t>
+          <t>이에스티</t>
         </is>
       </c>
       <c r="B85" s="18" t="inlineStr">
@@ -14344,7 +14352,7 @@
     <row r="86" ht="30" customHeight="1">
       <c r="A86" s="6" t="inlineStr">
         <is>
-          <t>제논</t>
+          <t>영광와이케이엠씨</t>
         </is>
       </c>
       <c r="B86" s="18" t="inlineStr">
@@ -14408,7 +14416,7 @@
     <row r="87" ht="30" customHeight="1">
       <c r="A87" s="6" t="inlineStr">
         <is>
-          <t>럭스코</t>
+          <t>제논</t>
         </is>
       </c>
       <c r="B87" s="18" t="inlineStr">
@@ -14469,22 +14477,86 @@
         </is>
       </c>
     </row>
-    <row r="89">
-      <c r="A89" s="20" t="inlineStr">
-        <is>
-          <t>※ 상장 완료 = KIND 신규상장 페이지 기준(스팩합병 포함) · 스팩 공모상장은 밴드·밸류에이션 등 해당없음(공모가 2,000원 고정).</t>
+    <row r="88" ht="30" customHeight="1">
+      <c r="A88" s="6" t="inlineStr">
+        <is>
+          <t>우리투자제1호스팩</t>
+        </is>
+      </c>
+      <c r="B88" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="C88" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="D88" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="E88" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="F88" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="G88" s="6" t="inlineStr"/>
+      <c r="H88" s="6" t="inlineStr"/>
+      <c r="I88" s="6" t="inlineStr"/>
+      <c r="J88" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="K88" s="6" t="inlineStr"/>
+      <c r="L88" s="6" t="inlineStr"/>
+      <c r="M88" s="6" t="inlineStr"/>
+      <c r="N88" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="O88" s="6" t="inlineStr"/>
+      <c r="P88" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="Q88" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="R88" s="6" t="inlineStr">
+        <is>
+          <t>신고서 대기</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="20" t="inlineStr">
         <is>
-          <t>※ 기재정정 신고서 내 정정 전·후 병존 → 자동수집은 "정정 후" 값만 취함.</t>
+          <t>※ 상장 완료 = KIND 신규상장 페이지 기준(스팩합병 포함) · 스팩 공모상장은 밴드·밸류에이션 등 해당없음(공모가 2,000원 고정).</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="20" t="inlineStr">
+        <is>
+          <t>※ 기재정정 신고서 내 정정 전·후 병존 → 자동수집은 "정정 후" 값만 취함.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="20" t="inlineStr">
         <is>
           <t>※ 청약경쟁률=일반투자자 청약수량÷최종배정수량 · "MM-DD~"는 종료일 자동수집 예정.</t>
         </is>
@@ -14787,7 +14859,7 @@
         <v>1</v>
       </c>
       <c r="C15" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D15" s="6" t="n">
         <v>0</v>
@@ -14909,7 +14981,7 @@
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>156,428,800,000</t>
+          <t>201,091,000,000</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update IPO data 2026-10-07
</commit_message>
<xml_diff>
--- a/IPO_analysis.xlsx
+++ b/IPO_analysis.xlsx
@@ -592,7 +592,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K146"/>
+  <dimension ref="A1:K147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -618,14 +618,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>기준일 2026-10-06 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
+          <t>기준일 2026-10-07 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>■ 심사 신청(진행중)  (46건)</t>
+          <t>■ 심사 신청(진행중)  (44건)</t>
         </is>
       </c>
       <c r="B4" s="4" t="n"/>
@@ -699,12 +699,12 @@
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>뱅크샐러드</t>
+          <t>베르티스</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
@@ -724,27 +724,27 @@
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>25,994</t>
+          <t>5,119</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
-          <t>-59,792</t>
+          <t>-12,903</t>
         </is>
       </c>
       <c r="H6" s="7" t="inlineStr">
         <is>
-          <t>28,335</t>
+          <t>-16,364</t>
         </is>
       </c>
       <c r="I6" s="6" t="inlineStr">
         <is>
-          <t>금융 지원 서비스업</t>
+          <t>의료용품 및 기타 의약 관련제품 제조업</t>
         </is>
       </c>
       <c r="J6" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>대신</t>
         </is>
       </c>
       <c r="K6" s="6" t="inlineStr">
@@ -756,12 +756,12 @@
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>키노톤</t>
+          <t>뱅크샐러드</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -781,27 +781,27 @@
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>46,943</t>
+          <t>25,994</t>
         </is>
       </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
-          <t>4,222</t>
+          <t>-59,792</t>
         </is>
       </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
-          <t>19,112</t>
+          <t>28,335</t>
         </is>
       </c>
       <c r="I7" s="6" t="inlineStr">
         <is>
-          <t>건축기술, 엔지니어링 및 관련 기술 서비스업</t>
+          <t>금융 지원 서비스업</t>
         </is>
       </c>
       <c r="J7" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K7" s="6" t="inlineStr">
@@ -818,7 +818,7 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>티에스모스트</t>
+          <t>키노톤</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
@@ -838,27 +838,27 @@
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>156,198</t>
+          <t>46,943</t>
         </is>
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
-          <t>5,666</t>
+          <t>4,222</t>
         </is>
       </c>
       <c r="H8" s="7" t="inlineStr">
         <is>
-          <t>25,181</t>
+          <t>19,112</t>
         </is>
       </c>
       <c r="I8" s="6" t="inlineStr">
         <is>
-          <t>자동차 신품 부품 제조업</t>
+          <t>건축기술, 엔지니어링 및 관련 기술 서비스업</t>
         </is>
       </c>
       <c r="J8" s="6" t="inlineStr">
         <is>
-          <t>신한</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="K8" s="6" t="inlineStr">
@@ -870,12 +870,12 @@
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>셀렉트스타</t>
+          <t>티에스모스트</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
@@ -895,27 +895,27 @@
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>11,616</t>
+          <t>156,198</t>
         </is>
       </c>
       <c r="G9" s="7" t="inlineStr">
         <is>
-          <t>-9,883</t>
+          <t>5,666</t>
         </is>
       </c>
       <c r="H9" s="7" t="inlineStr">
         <is>
-          <t>-34,511</t>
+          <t>25,181</t>
         </is>
       </c>
       <c r="I9" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어 개발 및 공급업</t>
+          <t>자동차 신품 부품 제조업</t>
         </is>
       </c>
       <c r="J9" s="6" t="inlineStr">
         <is>
-          <t>대신</t>
+          <t>신한</t>
         </is>
       </c>
       <c r="K9" s="6" t="inlineStr">
@@ -927,12 +927,12 @@
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>서북</t>
+          <t>셀렉트스타</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -952,27 +952,27 @@
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>60,439</t>
+          <t>11,616</t>
         </is>
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
-          <t>-8,764</t>
+          <t>-9,883</t>
         </is>
       </c>
       <c r="H10" s="7" t="inlineStr">
         <is>
-          <t>4,485</t>
+          <t>-34,511</t>
         </is>
       </c>
       <c r="I10" s="6" t="inlineStr">
         <is>
-          <t>사진장비 및 광학기기 제조업</t>
+          <t>소프트웨어 개발 및 공급업</t>
         </is>
       </c>
       <c r="J10" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>대신</t>
         </is>
       </c>
       <c r="K10" s="6" t="inlineStr">
@@ -989,7 +989,7 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>에이스엔지니어링</t>
+          <t>서북</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -1009,27 +1009,27 @@
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>307,911</t>
+          <t>60,439</t>
         </is>
       </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
-          <t>-101,468</t>
+          <t>-8,764</t>
         </is>
       </c>
       <c r="H11" s="7" t="inlineStr">
         <is>
-          <t>83,159</t>
+          <t>4,485</t>
         </is>
       </c>
       <c r="I11" s="6" t="inlineStr">
         <is>
-          <t>전동기, 발전기 및 전기 변환 · 공급 · 제어 장치 제조업</t>
+          <t>사진장비 및 광학기기 제조업</t>
         </is>
       </c>
       <c r="J11" s="6" t="inlineStr">
         <is>
-          <t>대신, 미래, 키움</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K11" s="6" t="inlineStr">
@@ -1046,7 +1046,7 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>플렉스시스템</t>
+          <t>에이스엔지니어링</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
@@ -1066,27 +1066,27 @@
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>10,894</t>
+          <t>307,911</t>
         </is>
       </c>
       <c r="G12" s="7" t="inlineStr">
         <is>
-          <t>-2,342</t>
+          <t>-101,468</t>
         </is>
       </c>
       <c r="H12" s="7" t="inlineStr">
         <is>
-          <t>3,014</t>
+          <t>83,159</t>
         </is>
       </c>
       <c r="I12" s="6" t="inlineStr">
         <is>
-          <t>측정, 시험, 항해, 제어 및 기타 정밀기기 제조업; 광학기기 제외</t>
+          <t>전동기, 발전기 및 전기 변환 · 공급 · 제어 장치 제조업</t>
         </is>
       </c>
       <c r="J12" s="6" t="inlineStr">
         <is>
-          <t>대신</t>
+          <t>대신, 미래, 키움</t>
         </is>
       </c>
       <c r="K12" s="6" t="inlineStr">
@@ -1098,12 +1098,12 @@
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>엠아이티</t>
+          <t>플렉스시스템</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
@@ -1123,27 +1123,27 @@
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>14,921</t>
+          <t>10,894</t>
         </is>
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
-          <t>1,181</t>
+          <t>-2,342</t>
         </is>
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
-          <t>28,026</t>
+          <t>3,014</t>
         </is>
       </c>
       <c r="I13" s="6" t="inlineStr">
         <is>
-          <t>특수 목적용 기계 제조업</t>
+          <t>측정, 시험, 항해, 제어 및 기타 정밀기기 제조업; 광학기기 제외</t>
         </is>
       </c>
       <c r="J13" s="6" t="inlineStr">
         <is>
-          <t>삼성</t>
+          <t>대신</t>
         </is>
       </c>
       <c r="K13" s="6" t="inlineStr">
@@ -1160,7 +1160,7 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>큐로드</t>
+          <t>엠아이티</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
@@ -1170,7 +1170,7 @@
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>스팩 소멸합병</t>
+          <t>신규상장</t>
         </is>
       </c>
       <c r="E14" s="6" t="inlineStr">
@@ -1178,17 +1178,29 @@
           <t>FY25</t>
         </is>
       </c>
-      <c r="F14" s="7" t="inlineStr"/>
-      <c r="G14" s="7" t="inlineStr"/>
-      <c r="H14" s="7" t="inlineStr"/>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>14,921</t>
+        </is>
+      </c>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>1,181</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>28,026</t>
+        </is>
+      </c>
       <c r="I14" s="6" t="inlineStr">
         <is>
-          <t>금융 지원 서비스업</t>
+          <t>특수 목적용 기계 제조업</t>
         </is>
       </c>
       <c r="J14" s="6" t="inlineStr">
         <is>
-          <t>교보</t>
+          <t>삼성</t>
         </is>
       </c>
       <c r="K14" s="6" t="inlineStr">
@@ -1200,12 +1212,12 @@
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>노바셀테크놀로지</t>
+          <t>큐로드</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
@@ -1215,7 +1227,7 @@
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>신규상장</t>
+          <t>스팩 소멸합병</t>
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr">
@@ -1223,29 +1235,17 @@
           <t>FY25</t>
         </is>
       </c>
-      <c r="F15" s="7" t="inlineStr">
-        <is>
-          <t>377</t>
-        </is>
-      </c>
-      <c r="G15" s="7" t="inlineStr">
-        <is>
-          <t>-4,606</t>
-        </is>
-      </c>
-      <c r="H15" s="7" t="inlineStr">
-        <is>
-          <t>-15,458</t>
-        </is>
-      </c>
+      <c r="F15" s="7" t="inlineStr"/>
+      <c r="G15" s="7" t="inlineStr"/>
+      <c r="H15" s="7" t="inlineStr"/>
       <c r="I15" s="6" t="inlineStr">
         <is>
-          <t>자연과학 및 공학 연구개발업</t>
+          <t>금융 지원 서비스업</t>
         </is>
       </c>
       <c r="J15" s="6" t="inlineStr">
         <is>
-          <t>키움</t>
+          <t>교보</t>
         </is>
       </c>
       <c r="K15" s="6" t="inlineStr">
@@ -1257,12 +1257,12 @@
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>(주)태석광학</t>
+          <t>노바셀테크놀로지</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
@@ -1282,27 +1282,27 @@
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
-          <t>79,804</t>
+          <t>377</t>
         </is>
       </c>
       <c r="G16" s="7" t="inlineStr">
         <is>
-          <t>4,721</t>
+          <t>-4,606</t>
         </is>
       </c>
       <c r="H16" s="7" t="inlineStr">
         <is>
-          <t>7,228</t>
+          <t>-15,458</t>
         </is>
       </c>
       <c r="I16" s="6" t="inlineStr">
         <is>
-          <t>생활용품 도매업</t>
+          <t>자연과학 및 공학 연구개발업</t>
         </is>
       </c>
       <c r="J16" s="6" t="inlineStr">
         <is>
-          <t>신한, 대신</t>
+          <t>키움</t>
         </is>
       </c>
       <c r="K16" s="6" t="inlineStr">
@@ -1314,12 +1314,12 @@
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>엑티브온</t>
+          <t>(주)태석광학</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
@@ -1329,7 +1329,7 @@
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>스팩 소멸합병</t>
+          <t>신규상장</t>
         </is>
       </c>
       <c r="E17" s="6" t="inlineStr">
@@ -1337,17 +1337,29 @@
           <t>FY25</t>
         </is>
       </c>
-      <c r="F17" s="7" t="inlineStr"/>
-      <c r="G17" s="7" t="inlineStr"/>
-      <c r="H17" s="7" t="inlineStr"/>
+      <c r="F17" s="7" t="inlineStr">
+        <is>
+          <t>79,804</t>
+        </is>
+      </c>
+      <c r="G17" s="7" t="inlineStr">
+        <is>
+          <t>4,721</t>
+        </is>
+      </c>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>7,228</t>
+        </is>
+      </c>
       <c r="I17" s="6" t="inlineStr">
         <is>
-          <t>금융 지원 서비스업</t>
+          <t>생활용품 도매업</t>
         </is>
       </c>
       <c r="J17" s="6" t="inlineStr">
         <is>
-          <t>키움</t>
+          <t>신한, 대신</t>
         </is>
       </c>
       <c r="K17" s="6" t="inlineStr">
@@ -1359,12 +1371,12 @@
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>씨앤엠</t>
+          <t>엑티브온</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
@@ -1374,7 +1386,7 @@
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
-          <t>신규상장</t>
+          <t>스팩 소멸합병</t>
         </is>
       </c>
       <c r="E18" s="6" t="inlineStr">
@@ -1382,29 +1394,17 @@
           <t>FY25</t>
         </is>
       </c>
-      <c r="F18" s="7" t="inlineStr">
-        <is>
-          <t>238,489</t>
-        </is>
-      </c>
-      <c r="G18" s="7" t="inlineStr">
-        <is>
-          <t>19,869</t>
-        </is>
-      </c>
-      <c r="H18" s="7" t="inlineStr">
-        <is>
-          <t>112,262</t>
-        </is>
-      </c>
+      <c r="F18" s="7" t="inlineStr"/>
+      <c r="G18" s="7" t="inlineStr"/>
+      <c r="H18" s="7" t="inlineStr"/>
       <c r="I18" s="6" t="inlineStr">
         <is>
-          <t>전동기, 발전기 및 전기 변환 · 공급 · 제어 장치 제조업</t>
+          <t>금융 지원 서비스업</t>
         </is>
       </c>
       <c r="J18" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>키움</t>
         </is>
       </c>
       <c r="K18" s="6" t="inlineStr">
@@ -1416,17 +1416,17 @@
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>무신사</t>
+          <t>씨앤엠</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>유가</t>
+          <t>코스닥</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
@@ -1441,27 +1441,27 @@
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>1,352,930</t>
+          <t>238,489</t>
         </is>
       </c>
       <c r="G19" s="7" t="inlineStr">
         <is>
-          <t>-10,571</t>
+          <t>19,869</t>
         </is>
       </c>
       <c r="H19" s="7" t="inlineStr">
         <is>
-          <t>243,731</t>
+          <t>112,262</t>
         </is>
       </c>
       <c r="I19" s="6" t="inlineStr">
         <is>
-          <t>섬유, 의복, 신발 및 가죽제품 소매업</t>
+          <t>전동기, 발전기 및 전기 변환 · 공급 · 제어 장치 제조업</t>
         </is>
       </c>
       <c r="J19" s="6" t="inlineStr">
         <is>
-          <t>한국, 씨티그룹글로벌마켓증권(주), KB, 제이피모간증권회사 서울지점</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="K19" s="6" t="inlineStr">
@@ -1473,17 +1473,17 @@
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>마더스제약</t>
+          <t>무신사</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>코스닥</t>
+          <t>유가</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
@@ -1498,27 +1498,27 @@
       </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
-          <t>228,830</t>
+          <t>1,352,930</t>
         </is>
       </c>
       <c r="G20" s="7" t="inlineStr">
         <is>
-          <t>11,204</t>
+          <t>-10,571</t>
         </is>
       </c>
       <c r="H20" s="7" t="inlineStr">
         <is>
-          <t>57,394</t>
+          <t>243,731</t>
         </is>
       </c>
       <c r="I20" s="6" t="inlineStr">
         <is>
-          <t>의약품 제조업</t>
+          <t>섬유, 의복, 신발 및 가죽제품 소매업</t>
         </is>
       </c>
       <c r="J20" s="6" t="inlineStr">
         <is>
-          <t>NH, KB</t>
+          <t>한국, 씨티그룹글로벌마켓증권(주), KB, 제이피모간증권회사 서울지점</t>
         </is>
       </c>
       <c r="K20" s="6" t="inlineStr">
@@ -2259,12 +2259,12 @@
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>엔키화이트햇</t>
+          <t>씨아이에스케미칼</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
@@ -2284,27 +2284,27 @@
       </c>
       <c r="F34" s="7" t="inlineStr">
         <is>
-          <t>14,176</t>
+          <t>15,985</t>
         </is>
       </c>
       <c r="G34" s="7" t="inlineStr">
         <is>
-          <t>-3,211</t>
+          <t>-11,440</t>
         </is>
       </c>
       <c r="H34" s="7" t="inlineStr">
         <is>
-          <t>8,338</t>
+          <t>23,706</t>
         </is>
       </c>
       <c r="I34" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어 개발 및 공급업</t>
+          <t>기초 화학물질 제조업</t>
         </is>
       </c>
       <c r="J34" s="6" t="inlineStr">
         <is>
-          <t>신영</t>
+          <t>KB</t>
         </is>
       </c>
       <c r="K34" s="6" t="inlineStr">
@@ -2316,12 +2316,12 @@
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>씨아이에스케미칼</t>
+          <t>엠디에스코리아</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
@@ -2341,27 +2341,27 @@
       </c>
       <c r="F35" s="7" t="inlineStr">
         <is>
-          <t>15,985</t>
+          <t>97,972</t>
         </is>
       </c>
       <c r="G35" s="7" t="inlineStr">
         <is>
-          <t>-11,440</t>
+          <t>6,512</t>
         </is>
       </c>
       <c r="H35" s="7" t="inlineStr">
         <is>
-          <t>23,706</t>
+          <t>53,818</t>
         </is>
       </c>
       <c r="I35" s="6" t="inlineStr">
         <is>
-          <t>기초 화학물질 제조업</t>
+          <t>기타 식품 제조업</t>
         </is>
       </c>
       <c r="J35" s="6" t="inlineStr">
         <is>
-          <t>KB</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K35" s="6" t="inlineStr">
@@ -2373,12 +2373,12 @@
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>엠디에스코리아</t>
+          <t>동승</t>
         </is>
       </c>
       <c r="C36" s="6" t="inlineStr">
@@ -2398,27 +2398,27 @@
       </c>
       <c r="F36" s="7" t="inlineStr">
         <is>
-          <t>97,972</t>
+          <t>78,625</t>
         </is>
       </c>
       <c r="G36" s="7" t="inlineStr">
         <is>
-          <t>6,512</t>
+          <t>14,525</t>
         </is>
       </c>
       <c r="H36" s="7" t="inlineStr">
         <is>
-          <t>53,818</t>
+          <t>5,438</t>
         </is>
       </c>
       <c r="I36" s="6" t="inlineStr">
         <is>
-          <t>기타 식품 제조업</t>
+          <t>부동산 임대 및 공급업</t>
         </is>
       </c>
       <c r="J36" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K36" s="6" t="inlineStr">
@@ -2435,7 +2435,7 @@
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>동승</t>
+          <t>에프엠더블유</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
@@ -2445,7 +2445,7 @@
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
-          <t>신규상장</t>
+          <t>스팩 소멸합병</t>
         </is>
       </c>
       <c r="E37" s="6" t="inlineStr">
@@ -2455,27 +2455,27 @@
       </c>
       <c r="F37" s="7" t="inlineStr">
         <is>
-          <t>78,625</t>
+          <t>30,282</t>
         </is>
       </c>
       <c r="G37" s="7" t="inlineStr">
         <is>
-          <t>14,525</t>
+          <t>4,762</t>
         </is>
       </c>
       <c r="H37" s="7" t="inlineStr">
         <is>
-          <t>5,438</t>
+          <t>32</t>
         </is>
       </c>
       <c r="I37" s="6" t="inlineStr">
         <is>
-          <t>부동산 임대 및 공급업</t>
+          <t>기타 식품 제조업</t>
         </is>
       </c>
       <c r="J37" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>유진</t>
         </is>
       </c>
       <c r="K37" s="6" t="inlineStr">
@@ -2487,22 +2487,22 @@
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>에프엠더블유</t>
+          <t>소노인터내셔널</t>
         </is>
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
-          <t>코스닥</t>
+          <t>유가</t>
         </is>
       </c>
       <c r="D38" s="6" t="inlineStr">
         <is>
-          <t>스팩 소멸합병</t>
+          <t>신규상장</t>
         </is>
       </c>
       <c r="E38" s="6" t="inlineStr">
@@ -2512,27 +2512,27 @@
       </c>
       <c r="F38" s="7" t="inlineStr">
         <is>
-          <t>30,282</t>
+          <t>2,093,051</t>
         </is>
       </c>
       <c r="G38" s="7" t="inlineStr">
         <is>
-          <t>4,762</t>
+          <t>-148,064</t>
         </is>
       </c>
       <c r="H38" s="7" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>852,372</t>
         </is>
       </c>
       <c r="I38" s="6" t="inlineStr">
         <is>
-          <t>기타 식품 제조업</t>
+          <t>일반 및 생활 숙박시설 운영업</t>
         </is>
       </c>
       <c r="J38" s="6" t="inlineStr">
         <is>
-          <t>유진</t>
+          <t>대신, 미래</t>
         </is>
       </c>
       <c r="K38" s="6" t="inlineStr">
@@ -2544,17 +2544,17 @@
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>소노인터내셔널</t>
+          <t>싸이몬</t>
         </is>
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>유가</t>
+          <t>코스닥</t>
         </is>
       </c>
       <c r="D39" s="6" t="inlineStr">
@@ -2569,27 +2569,27 @@
       </c>
       <c r="F39" s="7" t="inlineStr">
         <is>
-          <t>2,093,051</t>
+          <t>48,695</t>
         </is>
       </c>
       <c r="G39" s="7" t="inlineStr">
         <is>
-          <t>-148,064</t>
+          <t>15,714</t>
         </is>
       </c>
       <c r="H39" s="7" t="inlineStr">
         <is>
-          <t>852,372</t>
+          <t>61,761</t>
         </is>
       </c>
       <c r="I39" s="6" t="inlineStr">
         <is>
-          <t>일반 및 생활 숙박시설 운영업</t>
+          <t>측정, 시험, 항해, 제어 및 기타 정밀기기 제조업</t>
         </is>
       </c>
       <c r="J39" s="6" t="inlineStr">
         <is>
-          <t>대신, 미래</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K39" s="6" t="inlineStr">
@@ -2601,12 +2601,12 @@
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>싸이몬</t>
+          <t>바이다</t>
         </is>
       </c>
       <c r="C40" s="6" t="inlineStr">
@@ -2626,27 +2626,27 @@
       </c>
       <c r="F40" s="7" t="inlineStr">
         <is>
-          <t>48,695</t>
+          <t>14,432</t>
         </is>
       </c>
       <c r="G40" s="7" t="inlineStr">
         <is>
-          <t>15,714</t>
+          <t>-3,951</t>
         </is>
       </c>
       <c r="H40" s="7" t="inlineStr">
         <is>
-          <t>61,761</t>
+          <t>15,108</t>
         </is>
       </c>
       <c r="I40" s="6" t="inlineStr">
         <is>
-          <t>측정, 시험, 항해, 제어 및 기타 정밀기기 제조업</t>
+          <t>전자부품 제조업</t>
         </is>
       </c>
       <c r="J40" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K40" s="6" t="inlineStr">
@@ -2658,12 +2658,12 @@
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>바이다</t>
+          <t>아이알큐더스</t>
         </is>
       </c>
       <c r="C41" s="6" t="inlineStr">
@@ -2683,27 +2683,27 @@
       </c>
       <c r="F41" s="7" t="inlineStr">
         <is>
-          <t>14,432</t>
+          <t>10,231</t>
         </is>
       </c>
       <c r="G41" s="7" t="inlineStr">
         <is>
-          <t>-3,951</t>
+          <t>-986</t>
         </is>
       </c>
       <c r="H41" s="7" t="inlineStr">
         <is>
-          <t>15,108</t>
+          <t>1,800</t>
         </is>
       </c>
       <c r="I41" s="6" t="inlineStr">
         <is>
-          <t>전자부품 제조업</t>
+          <t>소프트웨어 개발 및 공급업</t>
         </is>
       </c>
       <c r="J41" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>DB</t>
         </is>
       </c>
       <c r="K41" s="6" t="inlineStr">
@@ -2715,12 +2715,12 @@
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B42" s="6" t="inlineStr">
         <is>
-          <t>아이알큐더스</t>
+          <t>씨엔티테크</t>
         </is>
       </c>
       <c r="C42" s="6" t="inlineStr">
@@ -2740,17 +2740,17 @@
       </c>
       <c r="F42" s="7" t="inlineStr">
         <is>
-          <t>10,231</t>
+          <t>27,015</t>
         </is>
       </c>
       <c r="G42" s="7" t="inlineStr">
         <is>
-          <t>-986</t>
+          <t>3,987</t>
         </is>
       </c>
       <c r="H42" s="7" t="inlineStr">
         <is>
-          <t>1,800</t>
+          <t>2,613</t>
         </is>
       </c>
       <c r="I42" s="6" t="inlineStr">
@@ -2760,7 +2760,7 @@
       </c>
       <c r="J42" s="6" t="inlineStr">
         <is>
-          <t>DB</t>
+          <t>한화, 하나</t>
         </is>
       </c>
       <c r="K42" s="6" t="inlineStr">
@@ -2777,7 +2777,7 @@
       </c>
       <c r="B43" s="6" t="inlineStr">
         <is>
-          <t>씨엔티테크</t>
+          <t>제이앤티지</t>
         </is>
       </c>
       <c r="C43" s="6" t="inlineStr">
@@ -2797,27 +2797,27 @@
       </c>
       <c r="F43" s="7" t="inlineStr">
         <is>
-          <t>27,015</t>
+          <t>72,378</t>
         </is>
       </c>
       <c r="G43" s="7" t="inlineStr">
         <is>
-          <t>3,987</t>
+          <t>9,904</t>
         </is>
       </c>
       <c r="H43" s="7" t="inlineStr">
         <is>
-          <t>2,613</t>
+          <t>6,743</t>
         </is>
       </c>
       <c r="I43" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어 개발 및 공급업</t>
+          <t>전자부품 제조업</t>
         </is>
       </c>
       <c r="J43" s="6" t="inlineStr">
         <is>
-          <t>한화, 하나</t>
+          <t>대신, NH</t>
         </is>
       </c>
       <c r="K43" s="6" t="inlineStr">
@@ -2829,12 +2829,12 @@
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B44" s="6" t="inlineStr">
         <is>
-          <t>제이앤티지</t>
+          <t>인터엑스</t>
         </is>
       </c>
       <c r="C44" s="6" t="inlineStr">
@@ -2854,27 +2854,27 @@
       </c>
       <c r="F44" s="7" t="inlineStr">
         <is>
-          <t>72,378</t>
+          <t>8,645</t>
         </is>
       </c>
       <c r="G44" s="7" t="inlineStr">
         <is>
-          <t>9,904</t>
+          <t>-20,272</t>
         </is>
       </c>
       <c r="H44" s="7" t="inlineStr">
         <is>
-          <t>6,743</t>
+          <t>4,530</t>
         </is>
       </c>
       <c r="I44" s="6" t="inlineStr">
         <is>
-          <t>전자부품 제조업</t>
+          <t>소프트웨어 개발 및 공급업</t>
         </is>
       </c>
       <c r="J44" s="6" t="inlineStr">
         <is>
-          <t>대신, NH</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="K44" s="6" t="inlineStr">
@@ -2886,12 +2886,12 @@
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B45" s="6" t="inlineStr">
         <is>
-          <t>인터엑스</t>
+          <t>삼홍아크튜리온</t>
         </is>
       </c>
       <c r="C45" s="6" t="inlineStr">
@@ -2911,27 +2911,27 @@
       </c>
       <c r="F45" s="7" t="inlineStr">
         <is>
-          <t>8,645</t>
+          <t>26,162</t>
         </is>
       </c>
       <c r="G45" s="7" t="inlineStr">
         <is>
-          <t>-20,272</t>
+          <t>-10,314</t>
         </is>
       </c>
       <c r="H45" s="7" t="inlineStr">
         <is>
-          <t>4,530</t>
+          <t>6,369</t>
         </is>
       </c>
       <c r="I45" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어 개발 및 공급업</t>
+          <t>구조용 금속제품, 탱크 및 증기발생기 제조업</t>
         </is>
       </c>
       <c r="J45" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>삼성, 미래</t>
         </is>
       </c>
       <c r="K45" s="6" t="inlineStr">
@@ -2943,12 +2943,12 @@
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B46" s="6" t="inlineStr">
         <is>
-          <t>삼홍아크튜리온</t>
+          <t>비앤비코리아</t>
         </is>
       </c>
       <c r="C46" s="6" t="inlineStr">
@@ -2968,27 +2968,27 @@
       </c>
       <c r="F46" s="7" t="inlineStr">
         <is>
-          <t>26,162</t>
+          <t>141,169</t>
         </is>
       </c>
       <c r="G46" s="7" t="inlineStr">
         <is>
-          <t>-10,314</t>
+          <t>21,406</t>
         </is>
       </c>
       <c r="H46" s="7" t="inlineStr">
         <is>
-          <t>6,369</t>
+          <t>43,932</t>
         </is>
       </c>
       <c r="I46" s="6" t="inlineStr">
         <is>
-          <t>구조용 금속제품, 탱크 및 증기발생기 제조업</t>
+          <t>기타 화학제품 제조업</t>
         </is>
       </c>
       <c r="J46" s="6" t="inlineStr">
         <is>
-          <t>삼성, 미래</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K46" s="6" t="inlineStr">
@@ -3000,12 +3000,12 @@
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B47" s="6" t="inlineStr">
         <is>
-          <t>넥스트에어로스페이스</t>
+          <t>오토핸즈</t>
         </is>
       </c>
       <c r="C47" s="6" t="inlineStr">
@@ -3015,7 +3015,7 @@
       </c>
       <c r="D47" s="6" t="inlineStr">
         <is>
-          <t>신규상장</t>
+          <t>스팩 소멸합병</t>
         </is>
       </c>
       <c r="E47" s="6" t="inlineStr">
@@ -3025,27 +3025,27 @@
       </c>
       <c r="F47" s="7" t="inlineStr">
         <is>
-          <t>12,084</t>
+          <t>238,564</t>
         </is>
       </c>
       <c r="G47" s="7" t="inlineStr">
         <is>
-          <t>-17,270</t>
+          <t>6,047</t>
         </is>
       </c>
       <c r="H47" s="7" t="inlineStr">
         <is>
-          <t>6,158</t>
+          <t>6,129</t>
         </is>
       </c>
       <c r="I47" s="6" t="inlineStr">
         <is>
-          <t>유인 항공기, 항공우주선 및 보조장치 제조업</t>
+          <t>자동차 판매업</t>
         </is>
       </c>
       <c r="J47" s="6" t="inlineStr">
         <is>
-          <t>삼성</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K47" s="6" t="inlineStr">
@@ -3057,12 +3057,12 @@
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B48" s="6" t="inlineStr">
         <is>
-          <t>비앤비코리아</t>
+          <t>아이벡스메디칼시스템즈</t>
         </is>
       </c>
       <c r="C48" s="6" t="inlineStr">
@@ -3082,27 +3082,27 @@
       </c>
       <c r="F48" s="7" t="inlineStr">
         <is>
-          <t>141,169</t>
+          <t>15,282</t>
         </is>
       </c>
       <c r="G48" s="7" t="inlineStr">
         <is>
-          <t>21,406</t>
+          <t>-7,227</t>
         </is>
       </c>
       <c r="H48" s="7" t="inlineStr">
         <is>
-          <t>43,932</t>
+          <t>744</t>
         </is>
       </c>
       <c r="I48" s="6" t="inlineStr">
         <is>
-          <t>기타 화학제품 제조업</t>
+          <t>의료용 기기 제조업</t>
         </is>
       </c>
       <c r="J48" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K48" s="6" t="inlineStr">
@@ -3114,12 +3114,12 @@
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="B49" s="6" t="inlineStr">
         <is>
-          <t>오토핸즈</t>
+          <t>피지티</t>
         </is>
       </c>
       <c r="C49" s="6" t="inlineStr">
@@ -3129,7 +3129,7 @@
       </c>
       <c r="D49" s="6" t="inlineStr">
         <is>
-          <t>스팩 소멸합병</t>
+          <t>신규상장</t>
         </is>
       </c>
       <c r="E49" s="6" t="inlineStr">
@@ -3139,27 +3139,27 @@
       </c>
       <c r="F49" s="7" t="inlineStr">
         <is>
-          <t>238,564</t>
+          <t>40,141</t>
         </is>
       </c>
       <c r="G49" s="7" t="inlineStr">
         <is>
-          <t>6,047</t>
+          <t>-69,722</t>
         </is>
       </c>
       <c r="H49" s="7" t="inlineStr">
         <is>
-          <t>6,129</t>
+          <t>6,029</t>
         </is>
       </c>
       <c r="I49" s="6" t="inlineStr">
         <is>
-          <t>자동차 판매업</t>
+          <t>기타 화학제품 제조업</t>
         </is>
       </c>
       <c r="J49" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="K49" s="6" t="inlineStr">
@@ -3168,191 +3168,191 @@
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="6" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-      <c r="B50" s="6" t="inlineStr">
-        <is>
-          <t>아이벡스메디칼시스템즈</t>
-        </is>
-      </c>
-      <c r="C50" s="6" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t>■ 심사 승인  (73건)</t>
+        </is>
+      </c>
+      <c r="B51" s="4" t="n"/>
+      <c r="C51" s="4" t="n"/>
+      <c r="D51" s="4" t="n"/>
+      <c r="E51" s="4" t="n"/>
+      <c r="F51" s="4" t="n"/>
+      <c r="G51" s="4" t="n"/>
+      <c r="H51" s="4" t="n"/>
+      <c r="I51" s="4" t="n"/>
+      <c r="J51" s="4" t="n"/>
+      <c r="K51" s="4" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>일자</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t>회사명</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>시장</t>
+        </is>
+      </c>
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>상장유형</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>기준연도</t>
+        </is>
+      </c>
+      <c r="F52" s="5" t="inlineStr">
+        <is>
+          <t>매출액</t>
+        </is>
+      </c>
+      <c r="G52" s="5" t="inlineStr">
+        <is>
+          <t>순이익</t>
+        </is>
+      </c>
+      <c r="H52" s="5" t="inlineStr">
+        <is>
+          <t>자기자본</t>
+        </is>
+      </c>
+      <c r="I52" s="5" t="inlineStr">
+        <is>
+          <t>업종</t>
+        </is>
+      </c>
+      <c r="J52" s="5" t="inlineStr">
+        <is>
+          <t>대표주관사</t>
+        </is>
+      </c>
+      <c r="K52" s="5" t="inlineStr">
+        <is>
+          <t>현황</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B53" s="6" t="inlineStr">
+        <is>
+          <t>엔키화이트햇</t>
+        </is>
+      </c>
+      <c r="C53" s="6" t="inlineStr">
         <is>
           <t>코스닥</t>
         </is>
       </c>
-      <c r="D50" s="6" t="inlineStr">
+      <c r="D53" s="6" t="inlineStr">
         <is>
           <t>신규상장</t>
         </is>
       </c>
-      <c r="E50" s="6" t="inlineStr">
+      <c r="E53" s="6" t="inlineStr">
         <is>
           <t>FY25</t>
         </is>
       </c>
-      <c r="F50" s="7" t="inlineStr">
-        <is>
-          <t>15,282</t>
-        </is>
-      </c>
-      <c r="G50" s="7" t="inlineStr">
-        <is>
-          <t>-7,227</t>
-        </is>
-      </c>
-      <c r="H50" s="7" t="inlineStr">
-        <is>
-          <t>744</t>
-        </is>
-      </c>
-      <c r="I50" s="6" t="inlineStr">
-        <is>
-          <t>의료용 기기 제조업</t>
-        </is>
-      </c>
-      <c r="J50" s="6" t="inlineStr">
-        <is>
-          <t>NH</t>
-        </is>
-      </c>
-      <c r="K50" s="6" t="inlineStr">
-        <is>
-          <t>예심 진행중</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="6" t="inlineStr">
-        <is>
-          <t>2026-02-27</t>
-        </is>
-      </c>
-      <c r="B51" s="6" t="inlineStr">
-        <is>
-          <t>피지티</t>
-        </is>
-      </c>
-      <c r="C51" s="6" t="inlineStr">
+      <c r="F53" s="7" t="inlineStr">
+        <is>
+          <t>14,176</t>
+        </is>
+      </c>
+      <c r="G53" s="7" t="inlineStr">
+        <is>
+          <t>-3,211</t>
+        </is>
+      </c>
+      <c r="H53" s="7" t="inlineStr">
+        <is>
+          <t>8,338</t>
+        </is>
+      </c>
+      <c r="I53" s="6" t="inlineStr">
+        <is>
+          <t>소프트웨어 개발 및 공급업</t>
+        </is>
+      </c>
+      <c r="J53" s="6" t="inlineStr">
+        <is>
+          <t>신영</t>
+        </is>
+      </c>
+      <c r="K53" s="6" t="inlineStr">
+        <is>
+          <t>상장전</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B54" s="6" t="inlineStr">
+        <is>
+          <t>마더스제약</t>
+        </is>
+      </c>
+      <c r="C54" s="6" t="inlineStr">
         <is>
           <t>코스닥</t>
         </is>
       </c>
-      <c r="D51" s="6" t="inlineStr">
+      <c r="D54" s="6" t="inlineStr">
         <is>
           <t>신규상장</t>
         </is>
       </c>
-      <c r="E51" s="6" t="inlineStr">
+      <c r="E54" s="6" t="inlineStr">
         <is>
           <t>FY25</t>
         </is>
       </c>
-      <c r="F51" s="7" t="inlineStr">
-        <is>
-          <t>40,141</t>
-        </is>
-      </c>
-      <c r="G51" s="7" t="inlineStr">
-        <is>
-          <t>-69,722</t>
-        </is>
-      </c>
-      <c r="H51" s="7" t="inlineStr">
-        <is>
-          <t>6,029</t>
-        </is>
-      </c>
-      <c r="I51" s="6" t="inlineStr">
-        <is>
-          <t>기타 화학제품 제조업</t>
-        </is>
-      </c>
-      <c r="J51" s="6" t="inlineStr">
-        <is>
-          <t>한국</t>
-        </is>
-      </c>
-      <c r="K51" s="6" t="inlineStr">
-        <is>
-          <t>예심 진행중</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="3" t="inlineStr">
-        <is>
-          <t>■ 심사 승인  (71건)</t>
-        </is>
-      </c>
-      <c r="B53" s="4" t="n"/>
-      <c r="C53" s="4" t="n"/>
-      <c r="D53" s="4" t="n"/>
-      <c r="E53" s="4" t="n"/>
-      <c r="F53" s="4" t="n"/>
-      <c r="G53" s="4" t="n"/>
-      <c r="H53" s="4" t="n"/>
-      <c r="I53" s="4" t="n"/>
-      <c r="J53" s="4" t="n"/>
-      <c r="K53" s="4" t="n"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="5" t="inlineStr">
-        <is>
-          <t>일자</t>
-        </is>
-      </c>
-      <c r="B54" s="5" t="inlineStr">
-        <is>
-          <t>회사명</t>
-        </is>
-      </c>
-      <c r="C54" s="5" t="inlineStr">
-        <is>
-          <t>시장</t>
-        </is>
-      </c>
-      <c r="D54" s="5" t="inlineStr">
-        <is>
-          <t>상장유형</t>
-        </is>
-      </c>
-      <c r="E54" s="5" t="inlineStr">
-        <is>
-          <t>기준연도</t>
-        </is>
-      </c>
-      <c r="F54" s="5" t="inlineStr">
-        <is>
-          <t>매출액</t>
-        </is>
-      </c>
-      <c r="G54" s="5" t="inlineStr">
-        <is>
-          <t>순이익</t>
-        </is>
-      </c>
-      <c r="H54" s="5" t="inlineStr">
-        <is>
-          <t>자기자본</t>
-        </is>
-      </c>
-      <c r="I54" s="5" t="inlineStr">
-        <is>
-          <t>업종</t>
-        </is>
-      </c>
-      <c r="J54" s="5" t="inlineStr">
-        <is>
-          <t>대표주관사</t>
-        </is>
-      </c>
-      <c r="K54" s="5" t="inlineStr">
-        <is>
-          <t>현황</t>
+      <c r="F54" s="7" t="inlineStr">
+        <is>
+          <t>228,830</t>
+        </is>
+      </c>
+      <c r="G54" s="7" t="inlineStr">
+        <is>
+          <t>11,204</t>
+        </is>
+      </c>
+      <c r="H54" s="7" t="inlineStr">
+        <is>
+          <t>57,394</t>
+        </is>
+      </c>
+      <c r="I54" s="6" t="inlineStr">
+        <is>
+          <t>의약품 제조업</t>
+        </is>
+      </c>
+      <c r="J54" s="6" t="inlineStr">
+        <is>
+          <t>NH, KB</t>
+        </is>
+      </c>
+      <c r="K54" s="6" t="inlineStr">
+        <is>
+          <t>상장전</t>
         </is>
       </c>
     </row>
@@ -7242,7 +7242,7 @@
     <row r="127">
       <c r="A127" s="3" t="inlineStr">
         <is>
-          <t>■ 철회·미승인  (18건)</t>
+          <t>■ 철회·미승인  (19건)</t>
         </is>
       </c>
       <c r="B127" s="4" t="n"/>
@@ -7316,12 +7316,12 @@
     <row r="129">
       <c r="A129" s="6" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="B129" s="6" t="inlineStr">
         <is>
-          <t>텔레픽스</t>
+          <t>넥스트에어로스페이스</t>
         </is>
       </c>
       <c r="C129" s="6" t="inlineStr">
@@ -7341,27 +7341,27 @@
       </c>
       <c r="F129" s="7" t="inlineStr">
         <is>
-          <t>4,896</t>
+          <t>12,084</t>
         </is>
       </c>
       <c r="G129" s="7" t="inlineStr">
         <is>
-          <t>-16,214</t>
+          <t>-17,270</t>
         </is>
       </c>
       <c r="H129" s="7" t="inlineStr">
         <is>
-          <t>9,146</t>
+          <t>6,158</t>
         </is>
       </c>
       <c r="I129" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어 개발 및 공급업</t>
+          <t>유인 항공기, 항공우주선 및 보조장치 제조업</t>
         </is>
       </c>
       <c r="J129" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>삼성</t>
         </is>
       </c>
       <c r="K129" s="6" t="inlineStr">
@@ -7373,12 +7373,12 @@
     <row r="130">
       <c r="A130" s="6" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B130" s="6" t="inlineStr">
         <is>
-          <t>씨엠디엘</t>
+          <t>텔레픽스</t>
         </is>
       </c>
       <c r="C130" s="6" t="inlineStr">
@@ -7388,37 +7388,37 @@
       </c>
       <c r="D130" s="6" t="inlineStr">
         <is>
-          <t>스팩 소멸합병</t>
+          <t>신규상장</t>
         </is>
       </c>
       <c r="E130" s="6" t="inlineStr">
         <is>
-          <t>FY24</t>
+          <t>FY25</t>
         </is>
       </c>
       <c r="F130" s="7" t="inlineStr">
         <is>
-          <t>39,991</t>
+          <t>4,896</t>
         </is>
       </c>
       <c r="G130" s="7" t="inlineStr">
         <is>
-          <t>3,541</t>
+          <t>-16,214</t>
         </is>
       </c>
       <c r="H130" s="7" t="inlineStr">
         <is>
-          <t>503</t>
+          <t>9,146</t>
         </is>
       </c>
       <c r="I130" s="6" t="inlineStr">
         <is>
-          <t>기타 기초 유기 화학물질 제조업</t>
+          <t>소프트웨어 개발 및 공급업</t>
         </is>
       </c>
       <c r="J130" s="6" t="inlineStr">
         <is>
-          <t>교보</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K130" s="6" t="inlineStr">
@@ -7430,12 +7430,12 @@
     <row r="131">
       <c r="A131" s="6" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B131" s="6" t="inlineStr">
         <is>
-          <t>모비어스</t>
+          <t>씨엠디엘</t>
         </is>
       </c>
       <c r="C131" s="6" t="inlineStr">
@@ -7445,37 +7445,37 @@
       </c>
       <c r="D131" s="6" t="inlineStr">
         <is>
-          <t>신규상장</t>
+          <t>스팩 소멸합병</t>
         </is>
       </c>
       <c r="E131" s="6" t="inlineStr">
         <is>
-          <t>FY25</t>
+          <t>FY24</t>
         </is>
       </c>
       <c r="F131" s="7" t="inlineStr">
         <is>
-          <t>31,989</t>
+          <t>39,991</t>
         </is>
       </c>
       <c r="G131" s="7" t="inlineStr">
         <is>
-          <t>-45,307</t>
+          <t>3,541</t>
         </is>
       </c>
       <c r="H131" s="7" t="inlineStr">
         <is>
-          <t>-96,707</t>
+          <t>503</t>
         </is>
       </c>
       <c r="I131" s="6" t="inlineStr">
         <is>
-          <t>컴퓨터 프로그래밍, 시스템 통합 및 관리업</t>
+          <t>기타 기초 유기 화학물질 제조업</t>
         </is>
       </c>
       <c r="J131" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>교보</t>
         </is>
       </c>
       <c r="K131" s="6" t="inlineStr">
@@ -7487,12 +7487,12 @@
     <row r="132">
       <c r="A132" s="6" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B132" s="6" t="inlineStr">
         <is>
-          <t>넥스트젠바이오</t>
+          <t>모비어스</t>
         </is>
       </c>
       <c r="C132" s="6" t="inlineStr">
@@ -7507,32 +7507,32 @@
       </c>
       <c r="E132" s="6" t="inlineStr">
         <is>
-          <t>FY24</t>
+          <t>FY25</t>
         </is>
       </c>
       <c r="F132" s="7" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>31,989</t>
         </is>
       </c>
       <c r="G132" s="7" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>-45,307</t>
         </is>
       </c>
       <c r="H132" s="7" t="inlineStr">
         <is>
-          <t>4,792</t>
+          <t>-96,707</t>
         </is>
       </c>
       <c r="I132" s="6" t="inlineStr">
         <is>
-          <t>자연과학 및 공학 연구개발업</t>
+          <t>컴퓨터 프로그래밍, 시스템 통합 및 관리업</t>
         </is>
       </c>
       <c r="J132" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K132" s="6" t="inlineStr">
@@ -7544,12 +7544,12 @@
     <row r="133">
       <c r="A133" s="6" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B133" s="6" t="inlineStr">
         <is>
-          <t>파워큐브세미</t>
+          <t>넥스트젠바이오</t>
         </is>
       </c>
       <c r="C133" s="6" t="inlineStr">
@@ -7564,32 +7564,32 @@
       </c>
       <c r="E133" s="6" t="inlineStr">
         <is>
-          <t>FY25</t>
+          <t>FY24</t>
         </is>
       </c>
       <c r="F133" s="7" t="inlineStr">
         <is>
-          <t>10,341</t>
+          <t>100</t>
         </is>
       </c>
       <c r="G133" s="7" t="inlineStr">
         <is>
-          <t>-10,837</t>
+          <t>69</t>
         </is>
       </c>
       <c r="H133" s="7" t="inlineStr">
         <is>
-          <t>841</t>
+          <t>4,792</t>
         </is>
       </c>
       <c r="I133" s="6" t="inlineStr">
         <is>
-          <t>반도체 제조업</t>
+          <t>자연과학 및 공학 연구개발업</t>
         </is>
       </c>
       <c r="J133" s="6" t="inlineStr">
         <is>
-          <t>하나, BNK</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="K133" s="6" t="inlineStr">
@@ -7601,12 +7601,12 @@
     <row r="134">
       <c r="A134" s="6" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B134" s="6" t="inlineStr">
         <is>
-          <t>제이피이노베이션</t>
+          <t>파워큐브세미</t>
         </is>
       </c>
       <c r="C134" s="6" t="inlineStr">
@@ -7626,27 +7626,27 @@
       </c>
       <c r="F134" s="7" t="inlineStr">
         <is>
-          <t>56,324</t>
+          <t>10,341</t>
         </is>
       </c>
       <c r="G134" s="7" t="inlineStr">
         <is>
-          <t>5,588</t>
+          <t>-10,837</t>
         </is>
       </c>
       <c r="H134" s="7" t="inlineStr">
         <is>
-          <t>3,684</t>
+          <t>841</t>
         </is>
       </c>
       <c r="I134" s="6" t="inlineStr">
         <is>
-          <t>특수 목적용 기계 제조업</t>
+          <t>반도체 제조업</t>
         </is>
       </c>
       <c r="J134" s="6" t="inlineStr">
         <is>
-          <t>삼성</t>
+          <t>하나, BNK</t>
         </is>
       </c>
       <c r="K134" s="6" t="inlineStr">
@@ -7658,12 +7658,12 @@
     <row r="135">
       <c r="A135" s="6" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B135" s="6" t="inlineStr">
         <is>
-          <t>케이솔루션</t>
+          <t>제이피이노베이션</t>
         </is>
       </c>
       <c r="C135" s="6" t="inlineStr">
@@ -7673,7 +7673,7 @@
       </c>
       <c r="D135" s="6" t="inlineStr">
         <is>
-          <t>스팩 존속합병</t>
+          <t>신규상장</t>
         </is>
       </c>
       <c r="E135" s="6" t="inlineStr">
@@ -7683,27 +7683,27 @@
       </c>
       <c r="F135" s="7" t="inlineStr">
         <is>
-          <t>34,565</t>
+          <t>56,324</t>
         </is>
       </c>
       <c r="G135" s="7" t="inlineStr">
         <is>
-          <t>1,158</t>
+          <t>5,588</t>
         </is>
       </c>
       <c r="H135" s="7" t="inlineStr">
         <is>
-          <t>653</t>
+          <t>3,684</t>
         </is>
       </c>
       <c r="I135" s="6" t="inlineStr">
         <is>
-          <t>차체 및 특장차 제조업</t>
+          <t>특수 목적용 기계 제조업</t>
         </is>
       </c>
       <c r="J135" s="6" t="inlineStr">
         <is>
-          <t>DB</t>
+          <t>삼성</t>
         </is>
       </c>
       <c r="K135" s="6" t="inlineStr">
@@ -7715,12 +7715,12 @@
     <row r="136">
       <c r="A136" s="6" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B136" s="6" t="inlineStr">
         <is>
-          <t>디토닉</t>
+          <t>케이솔루션</t>
         </is>
       </c>
       <c r="C136" s="6" t="inlineStr">
@@ -7730,37 +7730,37 @@
       </c>
       <c r="D136" s="6" t="inlineStr">
         <is>
-          <t>신규상장</t>
+          <t>스팩 존속합병</t>
         </is>
       </c>
       <c r="E136" s="6" t="inlineStr">
         <is>
-          <t>FY24</t>
+          <t>FY25</t>
         </is>
       </c>
       <c r="F136" s="7" t="inlineStr">
         <is>
-          <t>31,293</t>
+          <t>34,565</t>
         </is>
       </c>
       <c r="G136" s="7" t="inlineStr">
         <is>
-          <t>-1,633</t>
+          <t>1,158</t>
         </is>
       </c>
       <c r="H136" s="7" t="inlineStr">
         <is>
-          <t>-21,926</t>
+          <t>653</t>
         </is>
       </c>
       <c r="I136" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어 개발 및 공급업</t>
+          <t>차체 및 특장차 제조업</t>
         </is>
       </c>
       <c r="J136" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>DB</t>
         </is>
       </c>
       <c r="K136" s="6" t="inlineStr">
@@ -7772,12 +7772,12 @@
     <row r="137">
       <c r="A137" s="6" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="B137" s="6" t="inlineStr">
         <is>
-          <t>에스케이팩</t>
+          <t>디토닉</t>
         </is>
       </c>
       <c r="C137" s="6" t="inlineStr">
@@ -7787,7 +7787,7 @@
       </c>
       <c r="D137" s="6" t="inlineStr">
         <is>
-          <t>스팩 소멸합병</t>
+          <t>신규상장</t>
         </is>
       </c>
       <c r="E137" s="6" t="inlineStr">
@@ -7797,27 +7797,27 @@
       </c>
       <c r="F137" s="7" t="inlineStr">
         <is>
-          <t>27,310</t>
+          <t>31,293</t>
         </is>
       </c>
       <c r="G137" s="7" t="inlineStr">
         <is>
-          <t>2,257</t>
+          <t>-1,633</t>
         </is>
       </c>
       <c r="H137" s="7" t="inlineStr">
         <is>
-          <t>3,207</t>
+          <t>-21,926</t>
         </is>
       </c>
       <c r="I137" s="6" t="inlineStr">
         <is>
-          <t>용기 세척, 포장 및 충전기 제조업</t>
+          <t>소프트웨어 개발 및 공급업</t>
         </is>
       </c>
       <c r="J137" s="6" t="inlineStr">
         <is>
-          <t>교보</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K137" s="6" t="inlineStr">
@@ -7829,12 +7829,12 @@
     <row r="138">
       <c r="A138" s="6" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="B138" s="6" t="inlineStr">
         <is>
-          <t>메타넷엑스</t>
+          <t>에스케이팩</t>
         </is>
       </c>
       <c r="C138" s="6" t="inlineStr">
@@ -7844,7 +7844,7 @@
       </c>
       <c r="D138" s="6" t="inlineStr">
         <is>
-          <t>신규상장</t>
+          <t>스팩 소멸합병</t>
         </is>
       </c>
       <c r="E138" s="6" t="inlineStr">
@@ -7854,27 +7854,27 @@
       </c>
       <c r="F138" s="7" t="inlineStr">
         <is>
-          <t>244,130</t>
+          <t>27,310</t>
         </is>
       </c>
       <c r="G138" s="7" t="inlineStr">
         <is>
-          <t>13,455</t>
+          <t>2,257</t>
         </is>
       </c>
       <c r="H138" s="7" t="inlineStr">
         <is>
-          <t>9,995</t>
+          <t>3,207</t>
         </is>
       </c>
       <c r="I138" s="6" t="inlineStr">
         <is>
-          <t>컴퓨터 프로그래밍, 시스템 통합 및 관리업</t>
+          <t>용기 세척, 포장 및 충전기 제조업</t>
         </is>
       </c>
       <c r="J138" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>교보</t>
         </is>
       </c>
       <c r="K138" s="6" t="inlineStr">
@@ -7886,12 +7886,12 @@
     <row r="139">
       <c r="A139" s="6" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="B139" s="6" t="inlineStr">
         <is>
-          <t>무아스</t>
+          <t>메타넷엑스</t>
         </is>
       </c>
       <c r="C139" s="6" t="inlineStr">
@@ -7901,7 +7901,7 @@
       </c>
       <c r="D139" s="6" t="inlineStr">
         <is>
-          <t>스팩 소멸합병</t>
+          <t>신규상장</t>
         </is>
       </c>
       <c r="E139" s="6" t="inlineStr">
@@ -7911,27 +7911,27 @@
       </c>
       <c r="F139" s="7" t="inlineStr">
         <is>
-          <t>41,813</t>
+          <t>244,130</t>
         </is>
       </c>
       <c r="G139" s="7" t="inlineStr">
         <is>
-          <t>3,903</t>
+          <t>13,455</t>
         </is>
       </c>
       <c r="H139" s="7" t="inlineStr">
         <is>
-          <t>532</t>
+          <t>9,995</t>
         </is>
       </c>
       <c r="I139" s="6" t="inlineStr">
         <is>
-          <t>가정용 전기기기 제조업</t>
+          <t>컴퓨터 프로그래밍, 시스템 통합 및 관리업</t>
         </is>
       </c>
       <c r="J139" s="6" t="inlineStr">
         <is>
-          <t>신한</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K139" s="6" t="inlineStr">
@@ -7948,7 +7948,7 @@
       </c>
       <c r="B140" s="6" t="inlineStr">
         <is>
-          <t>유빅스테라퓨틱스</t>
+          <t>무아스</t>
         </is>
       </c>
       <c r="C140" s="6" t="inlineStr">
@@ -7958,7 +7958,7 @@
       </c>
       <c r="D140" s="6" t="inlineStr">
         <is>
-          <t>신규상장</t>
+          <t>스팩 소멸합병</t>
         </is>
       </c>
       <c r="E140" s="6" t="inlineStr">
@@ -7968,27 +7968,27 @@
       </c>
       <c r="F140" s="7" t="inlineStr">
         <is>
-          <t>1,071</t>
+          <t>41,813</t>
         </is>
       </c>
       <c r="G140" s="7" t="inlineStr">
         <is>
-          <t>-15,145</t>
+          <t>3,903</t>
         </is>
       </c>
       <c r="H140" s="7" t="inlineStr">
         <is>
-          <t>5,489</t>
+          <t>532</t>
         </is>
       </c>
       <c r="I140" s="6" t="inlineStr">
         <is>
-          <t>자연과학 및 공학 연구개발업</t>
+          <t>가정용 전기기기 제조업</t>
         </is>
       </c>
       <c r="J140" s="6" t="inlineStr">
         <is>
-          <t>대신</t>
+          <t>신한</t>
         </is>
       </c>
       <c r="K140" s="6" t="inlineStr">
@@ -8000,12 +8000,12 @@
     <row r="141">
       <c r="A141" s="6" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B141" s="6" t="inlineStr">
         <is>
-          <t>코드잇</t>
+          <t>유빅스테라퓨틱스</t>
         </is>
       </c>
       <c r="C141" s="6" t="inlineStr">
@@ -8025,27 +8025,27 @@
       </c>
       <c r="F141" s="7" t="inlineStr">
         <is>
-          <t>30,747</t>
+          <t>1,071</t>
         </is>
       </c>
       <c r="G141" s="7" t="inlineStr">
         <is>
-          <t>6,652</t>
+          <t>-15,145</t>
         </is>
       </c>
       <c r="H141" s="7" t="inlineStr">
         <is>
-          <t>2,403</t>
+          <t>5,489</t>
         </is>
       </c>
       <c r="I141" s="6" t="inlineStr">
         <is>
-          <t>교육지원 서비스업</t>
+          <t>자연과학 및 공학 연구개발업</t>
         </is>
       </c>
       <c r="J141" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>대신</t>
         </is>
       </c>
       <c r="K141" s="6" t="inlineStr">
@@ -8057,12 +8057,12 @@
     <row r="142">
       <c r="A142" s="6" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="B142" s="6" t="inlineStr">
         <is>
-          <t>한컴인스페이스</t>
+          <t>코드잇</t>
         </is>
       </c>
       <c r="C142" s="6" t="inlineStr">
@@ -8082,44 +8082,44 @@
       </c>
       <c r="F142" s="7" t="inlineStr">
         <is>
-          <t>23,492</t>
+          <t>30,747</t>
         </is>
       </c>
       <c r="G142" s="7" t="inlineStr">
         <is>
-          <t>-3,104</t>
+          <t>6,652</t>
         </is>
       </c>
       <c r="H142" s="7" t="inlineStr">
         <is>
-          <t>5,815</t>
+          <t>2,403</t>
         </is>
       </c>
       <c r="I142" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어 개발 및 공급업</t>
+          <t>교육지원 서비스업</t>
         </is>
       </c>
       <c r="J142" s="6" t="inlineStr">
         <is>
-          <t>대신</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K142" s="6" t="inlineStr">
         <is>
-          <t>심사 미승인</t>
+          <t>심사 철회</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="6" t="inlineStr">
         <is>
-          <t>2026-01-28</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B143" s="6" t="inlineStr">
         <is>
-          <t>크몽</t>
+          <t>한컴인스페이스</t>
         </is>
       </c>
       <c r="C143" s="6" t="inlineStr">
@@ -8139,44 +8139,44 @@
       </c>
       <c r="F143" s="7" t="inlineStr">
         <is>
-          <t>48,572</t>
+          <t>23,492</t>
         </is>
       </c>
       <c r="G143" s="7" t="inlineStr">
         <is>
-          <t>3,988</t>
+          <t>-3,104</t>
         </is>
       </c>
       <c r="H143" s="7" t="inlineStr">
         <is>
-          <t>4,930</t>
+          <t>5,815</t>
         </is>
       </c>
       <c r="I143" s="6" t="inlineStr">
         <is>
-          <t>기타 정보 서비스업</t>
+          <t>소프트웨어 개발 및 공급업</t>
         </is>
       </c>
       <c r="J143" s="6" t="inlineStr">
         <is>
-          <t>삼성</t>
+          <t>대신</t>
         </is>
       </c>
       <c r="K143" s="6" t="inlineStr">
         <is>
-          <t>심사 철회</t>
+          <t>심사 미승인</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="6" t="inlineStr">
         <is>
-          <t>2026-01-27</t>
+          <t>2026-01-28</t>
         </is>
       </c>
       <c r="B144" s="6" t="inlineStr">
         <is>
-          <t>한화플러스제6호스팩</t>
+          <t>크몽</t>
         </is>
       </c>
       <c r="C144" s="6" t="inlineStr">
@@ -8196,27 +8196,27 @@
       </c>
       <c r="F144" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>48,572</t>
         </is>
       </c>
       <c r="G144" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>3,988</t>
         </is>
       </c>
       <c r="H144" s="7" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>4,930</t>
         </is>
       </c>
       <c r="I144" s="6" t="inlineStr">
         <is>
-          <t>기타 금융업</t>
+          <t>기타 정보 서비스업</t>
         </is>
       </c>
       <c r="J144" s="6" t="inlineStr">
         <is>
-          <t>한화</t>
+          <t>삼성</t>
         </is>
       </c>
       <c r="K144" s="6" t="inlineStr">
@@ -8228,17 +8228,17 @@
     <row r="145">
       <c r="A145" s="6" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-27</t>
         </is>
       </c>
       <c r="B145" s="6" t="inlineStr">
         <is>
-          <t>에식스솔루션즈</t>
+          <t>한화플러스제6호스팩</t>
         </is>
       </c>
       <c r="C145" s="6" t="inlineStr">
         <is>
-          <t>유가</t>
+          <t>코스닥</t>
         </is>
       </c>
       <c r="D145" s="6" t="inlineStr">
@@ -8253,27 +8253,27 @@
       </c>
       <c r="F145" s="7" t="inlineStr">
         <is>
-          <t>2,461</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G145" s="7" t="inlineStr">
         <is>
-          <t>46</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H145" s="7" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>41</t>
         </is>
       </c>
       <c r="I145" s="6" t="inlineStr">
         <is>
-          <t>절연선 및 케이블 제조업</t>
+          <t>기타 금융업</t>
         </is>
       </c>
       <c r="J145" s="6" t="inlineStr">
         <is>
-          <t>한국, 미래</t>
+          <t>한화</t>
         </is>
       </c>
       <c r="K145" s="6" t="inlineStr">
@@ -8285,55 +8285,112 @@
     <row r="146">
       <c r="A146" s="6" t="inlineStr">
         <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="B146" s="6" t="inlineStr">
+        <is>
+          <t>에식스솔루션즈</t>
+        </is>
+      </c>
+      <c r="C146" s="6" t="inlineStr">
+        <is>
+          <t>유가</t>
+        </is>
+      </c>
+      <c r="D146" s="6" t="inlineStr">
+        <is>
+          <t>신규상장</t>
+        </is>
+      </c>
+      <c r="E146" s="6" t="inlineStr">
+        <is>
+          <t>FY24</t>
+        </is>
+      </c>
+      <c r="F146" s="7" t="inlineStr">
+        <is>
+          <t>2,461</t>
+        </is>
+      </c>
+      <c r="G146" s="7" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
+      <c r="H146" s="7" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I146" s="6" t="inlineStr">
+        <is>
+          <t>절연선 및 케이블 제조업</t>
+        </is>
+      </c>
+      <c r="J146" s="6" t="inlineStr">
+        <is>
+          <t>한국, 미래</t>
+        </is>
+      </c>
+      <c r="K146" s="6" t="inlineStr">
+        <is>
+          <t>심사 철회</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="6" t="inlineStr">
+        <is>
           <t>2026-01-23</t>
         </is>
       </c>
-      <c r="B146" s="6" t="inlineStr">
+      <c r="B147" s="6" t="inlineStr">
         <is>
           <t>에코크레이션</t>
         </is>
       </c>
-      <c r="C146" s="6" t="inlineStr">
+      <c r="C147" s="6" t="inlineStr">
         <is>
           <t>코스닥</t>
         </is>
       </c>
-      <c r="D146" s="6" t="inlineStr">
+      <c r="D147" s="6" t="inlineStr">
         <is>
           <t>신규상장</t>
         </is>
       </c>
-      <c r="E146" s="6" t="inlineStr">
+      <c r="E147" s="6" t="inlineStr">
         <is>
           <t>FY24</t>
         </is>
       </c>
-      <c r="F146" s="7" t="inlineStr">
+      <c r="F147" s="7" t="inlineStr">
         <is>
           <t>18,544</t>
         </is>
       </c>
-      <c r="G146" s="7" t="inlineStr">
+      <c r="G147" s="7" t="inlineStr">
         <is>
           <t>-15,634</t>
         </is>
       </c>
-      <c r="H146" s="7" t="inlineStr">
+      <c r="H147" s="7" t="inlineStr">
         <is>
           <t>4,550</t>
         </is>
       </c>
-      <c r="I146" s="6" t="inlineStr">
+      <c r="I147" s="6" t="inlineStr">
         <is>
           <t>일반 목적용 기계 제조업</t>
         </is>
       </c>
-      <c r="J146" s="6" t="inlineStr">
+      <c r="J147" s="6" t="inlineStr">
         <is>
           <t>키움</t>
         </is>
       </c>
-      <c r="K146" s="6" t="inlineStr">
+      <c r="K147" s="6" t="inlineStr">
         <is>
           <t>심사 철회</t>
         </is>
@@ -8350,7 +8407,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R92"/>
+  <dimension ref="A1:R94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -12432,7 +12489,7 @@
     <row r="56" ht="22" customHeight="1">
       <c r="A56" s="3" t="inlineStr">
         <is>
-          <t>■ 공모 진행 (예심 승인법인)  (32건)</t>
+          <t>■ 공모 진행 (예심 승인법인)  (34건)</t>
         </is>
       </c>
       <c r="B56" s="4" t="n"/>
@@ -12576,7 +12633,11 @@
           <t>10-01~10-02</t>
         </is>
       </c>
-      <c r="K58" s="6" t="inlineStr"/>
+      <c r="K58" s="6" t="inlineStr">
+        <is>
+          <t>4,284.98</t>
+        </is>
+      </c>
       <c r="L58" s="6" t="inlineStr"/>
       <c r="M58" s="6" t="inlineStr"/>
       <c r="N58" s="6" t="inlineStr">
@@ -12597,7 +12658,7 @@
       </c>
       <c r="R58" s="6" t="inlineStr">
         <is>
-          <t>발행조건확정</t>
+          <t>청약완료·상장대기</t>
         </is>
       </c>
     </row>
@@ -12772,7 +12833,7 @@
       </c>
       <c r="E61" s="7" t="inlineStr">
         <is>
-          <t>27,200,000,000</t>
+          <t>31,200,000,000</t>
         </is>
       </c>
       <c r="F61" s="6" t="inlineStr">
@@ -12780,9 +12841,17 @@
           <t>30.89배 (PER)</t>
         </is>
       </c>
-      <c r="G61" s="6" t="inlineStr"/>
-      <c r="H61" s="6" t="inlineStr"/>
-      <c r="I61" s="6" t="inlineStr"/>
+      <c r="G61" s="6" t="inlineStr">
+        <is>
+          <t>7,800</t>
+        </is>
+      </c>
+      <c r="H61" s="6" t="n">
+        <v>1096.56</v>
+      </c>
+      <c r="I61" s="6" t="n">
+        <v>2269</v>
+      </c>
       <c r="J61" s="6" t="inlineStr">
         <is>
           <t>10-12~10-13</t>
@@ -12809,7 +12878,7 @@
       </c>
       <c r="R61" s="6" t="inlineStr">
         <is>
-          <t>정정</t>
+          <t>발행조건확정</t>
         </is>
       </c>
     </row>
@@ -13456,96 +13525,96 @@
     <row r="72" ht="30" customHeight="1">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>인텔리빅스</t>
-        </is>
-      </c>
-      <c r="B72" s="6" t="inlineStr">
-        <is>
-          <t>10-12~10-16</t>
-        </is>
-      </c>
-      <c r="C72" s="6" t="inlineStr">
-        <is>
-          <t>7,600~9,000</t>
-        </is>
-      </c>
-      <c r="D72" s="7" t="inlineStr">
-        <is>
-          <t>2,500,000</t>
-        </is>
-      </c>
-      <c r="E72" s="7" t="inlineStr">
-        <is>
-          <t>19,000,000,000</t>
-        </is>
-      </c>
-      <c r="F72" s="6" t="inlineStr">
-        <is>
-          <t>22.02배 (PER)</t>
+          <t>솔리스</t>
+        </is>
+      </c>
+      <c r="B72" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="C72" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="D72" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="E72" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="F72" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="G72" s="6" t="inlineStr"/>
       <c r="H72" s="6" t="inlineStr"/>
       <c r="I72" s="6" t="inlineStr"/>
-      <c r="J72" s="6" t="inlineStr">
-        <is>
-          <t>10-21~10-22</t>
+      <c r="J72" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="K72" s="6" t="inlineStr"/>
       <c r="L72" s="6" t="inlineStr"/>
       <c r="M72" s="6" t="inlineStr"/>
-      <c r="N72" s="6" t="inlineStr">
-        <is>
-          <t>미래에셋증권</t>
+      <c r="N72" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="O72" s="6" t="inlineStr"/>
-      <c r="P72" s="7" t="inlineStr">
-        <is>
-          <t>782,800,000</t>
-        </is>
-      </c>
-      <c r="Q72" s="6" t="inlineStr">
-        <is>
-          <t>4.0%</t>
+      <c r="P72" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="Q72" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="R72" s="6" t="inlineStr">
         <is>
-          <t>최초</t>
+          <t>정정</t>
         </is>
       </c>
     </row>
     <row r="73" ht="30" customHeight="1">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>영광</t>
+          <t>인텔리빅스</t>
         </is>
       </c>
       <c r="B73" s="6" t="inlineStr">
         <is>
-          <t>10-13~10-19</t>
+          <t>10-12~10-16</t>
         </is>
       </c>
       <c r="C73" s="6" t="inlineStr">
         <is>
-          <t>14,000~17,000</t>
+          <t>7,600~9,000</t>
         </is>
       </c>
       <c r="D73" s="7" t="inlineStr">
         <is>
-          <t>2,260,000</t>
+          <t>2,500,000</t>
         </is>
       </c>
       <c r="E73" s="7" t="inlineStr">
         <is>
-          <t>31,640,000,000</t>
+          <t>19,000,000,000</t>
         </is>
       </c>
       <c r="F73" s="6" t="inlineStr">
         <is>
-          <t>11.98배 (EV/EBITDA)</t>
+          <t>22.02배 (PER)</t>
         </is>
       </c>
       <c r="G73" s="6" t="inlineStr"/>
@@ -13553,7 +13622,7 @@
       <c r="I73" s="6" t="inlineStr"/>
       <c r="J73" s="6" t="inlineStr">
         <is>
-          <t>10-22~10-23</t>
+          <t>10-21~10-22</t>
         </is>
       </c>
       <c r="K73" s="6" t="inlineStr"/>
@@ -13561,18 +13630,18 @@
       <c r="M73" s="6" t="inlineStr"/>
       <c r="N73" s="6" t="inlineStr">
         <is>
-          <t>한국투자증권</t>
+          <t>미래에셋증권</t>
         </is>
       </c>
       <c r="O73" s="6" t="inlineStr"/>
       <c r="P73" s="7" t="inlineStr">
         <is>
-          <t>977,676,000</t>
-        </is>
-      </c>
-      <c r="Q73" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>782,800,000</t>
+        </is>
+      </c>
+      <c r="Q73" s="6" t="inlineStr">
+        <is>
+          <t>4.0%</t>
         </is>
       </c>
       <c r="R73" s="6" t="inlineStr">
@@ -13584,32 +13653,32 @@
     <row r="74" ht="30" customHeight="1">
       <c r="A74" s="6" t="inlineStr">
         <is>
-          <t>에이엘로봇</t>
+          <t>영광</t>
         </is>
       </c>
       <c r="B74" s="6" t="inlineStr">
         <is>
-          <t>10-15~10-21</t>
+          <t>10-13~10-19</t>
         </is>
       </c>
       <c r="C74" s="6" t="inlineStr">
         <is>
-          <t>15,700~17,600</t>
+          <t>14,000~17,000</t>
         </is>
       </c>
       <c r="D74" s="7" t="inlineStr">
         <is>
-          <t>2,400,000</t>
+          <t>2,260,000</t>
         </is>
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
-          <t>37,680,000,000</t>
+          <t>31,640,000,000</t>
         </is>
       </c>
       <c r="F74" s="6" t="inlineStr">
         <is>
-          <t>37.17배 (PER)</t>
+          <t>11.98배 (EV/EBITDA)</t>
         </is>
       </c>
       <c r="G74" s="6" t="inlineStr"/>
@@ -13617,7 +13686,7 @@
       <c r="I74" s="6" t="inlineStr"/>
       <c r="J74" s="6" t="inlineStr">
         <is>
-          <t>10-26~10-27</t>
+          <t>10-22~10-23</t>
         </is>
       </c>
       <c r="K74" s="6" t="inlineStr"/>
@@ -13625,18 +13694,18 @@
       <c r="M74" s="6" t="inlineStr"/>
       <c r="N74" s="6" t="inlineStr">
         <is>
-          <t>대신증권</t>
+          <t>한국투자증권</t>
         </is>
       </c>
       <c r="O74" s="6" t="inlineStr"/>
       <c r="P74" s="7" t="inlineStr">
         <is>
-          <t>1,160,399,874</t>
-        </is>
-      </c>
-      <c r="Q74" s="6" t="inlineStr">
-        <is>
-          <t>3.0%</t>
+          <t>977,676,000</t>
+        </is>
+      </c>
+      <c r="Q74" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="R74" s="6" t="inlineStr">
@@ -13648,32 +13717,32 @@
     <row r="75" ht="30" customHeight="1">
       <c r="A75" s="6" t="inlineStr">
         <is>
-          <t>아이엠스팩1호</t>
+          <t>에이엘로봇</t>
         </is>
       </c>
       <c r="B75" s="6" t="inlineStr">
         <is>
-          <t>10-19~10-20</t>
-        </is>
-      </c>
-      <c r="C75" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>10-15~10-21</t>
+        </is>
+      </c>
+      <c r="C75" s="6" t="inlineStr">
+        <is>
+          <t>15,700~17,600</t>
         </is>
       </c>
       <c r="D75" s="7" t="inlineStr">
         <is>
-          <t>5,000,000</t>
+          <t>2,400,000</t>
         </is>
       </c>
       <c r="E75" s="7" t="inlineStr">
         <is>
-          <t>10,000,000,000</t>
-        </is>
-      </c>
-      <c r="F75" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>37,680,000,000</t>
+        </is>
+      </c>
+      <c r="F75" s="6" t="inlineStr">
+        <is>
+          <t>37.17배 (PER)</t>
         </is>
       </c>
       <c r="G75" s="6" t="inlineStr"/>
@@ -13687,20 +13756,20 @@
       <c r="K75" s="6" t="inlineStr"/>
       <c r="L75" s="6" t="inlineStr"/>
       <c r="M75" s="6" t="inlineStr"/>
-      <c r="N75" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="N75" s="6" t="inlineStr">
+        <is>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="O75" s="6" t="inlineStr"/>
-      <c r="P75" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="P75" s="7" t="inlineStr">
+        <is>
+          <t>1,160,399,874</t>
         </is>
       </c>
       <c r="Q75" s="6" t="inlineStr">
         <is>
-          <t>3.00%</t>
+          <t>3.0%</t>
         </is>
       </c>
       <c r="R75" s="6" t="inlineStr">
@@ -13712,32 +13781,32 @@
     <row r="76" ht="30" customHeight="1">
       <c r="A76" s="6" t="inlineStr">
         <is>
-          <t>옵토닉스</t>
+          <t>아이엠스팩1호</t>
         </is>
       </c>
       <c r="B76" s="6" t="inlineStr">
         <is>
-          <t>10-21~10-27</t>
-        </is>
-      </c>
-      <c r="C76" s="6" t="inlineStr">
-        <is>
-          <t>10,000~12,000</t>
+          <t>10-19~10-20</t>
+        </is>
+      </c>
+      <c r="C76" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="D76" s="7" t="inlineStr">
         <is>
-          <t>2,200,000</t>
+          <t>5,000,000</t>
         </is>
       </c>
       <c r="E76" s="7" t="inlineStr">
         <is>
-          <t>22,000,000,000</t>
-        </is>
-      </c>
-      <c r="F76" s="6" t="inlineStr">
-        <is>
-          <t>25.27배 (EV/EBITDA)</t>
+          <t>10,000,000,000</t>
+        </is>
+      </c>
+      <c r="F76" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="G76" s="6" t="inlineStr"/>
@@ -13745,26 +13814,26 @@
       <c r="I76" s="6" t="inlineStr"/>
       <c r="J76" s="6" t="inlineStr">
         <is>
-          <t>11-05~11-06</t>
+          <t>10-26~10-27</t>
         </is>
       </c>
       <c r="K76" s="6" t="inlineStr"/>
       <c r="L76" s="6" t="inlineStr"/>
       <c r="M76" s="6" t="inlineStr"/>
-      <c r="N76" s="6" t="inlineStr">
-        <is>
-          <t>한국투자증권</t>
+      <c r="N76" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="O76" s="6" t="inlineStr"/>
-      <c r="P76" s="7" t="inlineStr">
-        <is>
-          <t>1,133,000,000</t>
+      <c r="P76" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="Q76" s="6" t="inlineStr">
         <is>
-          <t>5.0%</t>
+          <t>3.00%</t>
         </is>
       </c>
       <c r="R76" s="6" t="inlineStr">
@@ -13776,32 +13845,32 @@
     <row r="77" ht="30" customHeight="1">
       <c r="A77" s="6" t="inlineStr">
         <is>
-          <t>동원파츠</t>
+          <t>옵토닉스</t>
         </is>
       </c>
       <c r="B77" s="6" t="inlineStr">
         <is>
-          <t>10-22~10-28</t>
+          <t>10-21~10-27</t>
         </is>
       </c>
       <c r="C77" s="6" t="inlineStr">
         <is>
-          <t>23,000~26,500</t>
+          <t>10,000~12,000</t>
         </is>
       </c>
       <c r="D77" s="7" t="inlineStr">
         <is>
-          <t>2,030,000</t>
+          <t>2,200,000</t>
         </is>
       </c>
       <c r="E77" s="7" t="inlineStr">
         <is>
-          <t>46,690,000,000</t>
+          <t>22,000,000,000</t>
         </is>
       </c>
       <c r="F77" s="6" t="inlineStr">
         <is>
-          <t>22.91배 (PER)</t>
+          <t>25.27배 (EV/EBITDA)</t>
         </is>
       </c>
       <c r="G77" s="6" t="inlineStr"/>
@@ -13809,7 +13878,7 @@
       <c r="I77" s="6" t="inlineStr"/>
       <c r="J77" s="6" t="inlineStr">
         <is>
-          <t>11-02~11-03</t>
+          <t>11-05~11-06</t>
         </is>
       </c>
       <c r="K77" s="6" t="inlineStr"/>
@@ -13817,18 +13886,18 @@
       <c r="M77" s="6" t="inlineStr"/>
       <c r="N77" s="6" t="inlineStr">
         <is>
-          <t>삼성증권</t>
+          <t>한국투자증권</t>
         </is>
       </c>
       <c r="O77" s="6" t="inlineStr"/>
       <c r="P77" s="7" t="inlineStr">
         <is>
-          <t>1,430,699,820</t>
+          <t>1,133,000,000</t>
         </is>
       </c>
       <c r="Q77" s="6" t="inlineStr">
         <is>
-          <t>3.0%</t>
+          <t>5.0%</t>
         </is>
       </c>
       <c r="R77" s="6" t="inlineStr">
@@ -13840,7 +13909,7 @@
     <row r="78" ht="30" customHeight="1">
       <c r="A78" s="6" t="inlineStr">
         <is>
-          <t>넥스아이</t>
+          <t>동원파츠</t>
         </is>
       </c>
       <c r="B78" s="6" t="inlineStr">
@@ -13850,22 +13919,22 @@
       </c>
       <c r="C78" s="6" t="inlineStr">
         <is>
-          <t>10,500~13,000</t>
+          <t>23,000~26,500</t>
         </is>
       </c>
       <c r="D78" s="7" t="inlineStr">
         <is>
-          <t>5,000,000</t>
+          <t>2,030,000</t>
         </is>
       </c>
       <c r="E78" s="7" t="inlineStr">
         <is>
-          <t>52,500,000,000</t>
+          <t>46,690,000,000</t>
         </is>
       </c>
       <c r="F78" s="6" t="inlineStr">
         <is>
-          <t>19.15배 (PER)</t>
+          <t>22.91배 (PER)</t>
         </is>
       </c>
       <c r="G78" s="6" t="inlineStr"/>
@@ -13873,7 +13942,7 @@
       <c r="I78" s="6" t="inlineStr"/>
       <c r="J78" s="6" t="inlineStr">
         <is>
-          <t>11-03~11-04</t>
+          <t>11-02~11-03</t>
         </is>
       </c>
       <c r="K78" s="6" t="inlineStr"/>
@@ -13881,18 +13950,18 @@
       <c r="M78" s="6" t="inlineStr"/>
       <c r="N78" s="6" t="inlineStr">
         <is>
-          <t>한국투자증권</t>
+          <t>삼성증권</t>
         </is>
       </c>
       <c r="O78" s="6" t="inlineStr"/>
       <c r="P78" s="7" t="inlineStr">
         <is>
-          <t>2,407,500,000</t>
+          <t>1,430,699,820</t>
         </is>
       </c>
       <c r="Q78" s="6" t="inlineStr">
         <is>
-          <t>4.5%</t>
+          <t>3.0%</t>
         </is>
       </c>
       <c r="R78" s="6" t="inlineStr">
@@ -13904,32 +13973,32 @@
     <row r="79" ht="30" customHeight="1">
       <c r="A79" s="6" t="inlineStr">
         <is>
-          <t>하나에어로다이내믹스</t>
+          <t>넥스아이</t>
         </is>
       </c>
       <c r="B79" s="6" t="inlineStr">
         <is>
-          <t>11-02~11-06</t>
+          <t>10-22~10-28</t>
         </is>
       </c>
       <c r="C79" s="6" t="inlineStr">
         <is>
-          <t>4,700~5,700</t>
+          <t>10,500~13,000</t>
         </is>
       </c>
       <c r="D79" s="7" t="inlineStr">
         <is>
-          <t>4,400,000</t>
+          <t>5,000,000</t>
         </is>
       </c>
       <c r="E79" s="7" t="inlineStr">
         <is>
-          <t>20,680,000,000</t>
+          <t>52,500,000,000</t>
         </is>
       </c>
       <c r="F79" s="6" t="inlineStr">
         <is>
-          <t>17.89배 (EV/EBITDA)</t>
+          <t>19.15배 (PER)</t>
         </is>
       </c>
       <c r="G79" s="6" t="inlineStr"/>
@@ -13937,7 +14006,7 @@
       <c r="I79" s="6" t="inlineStr"/>
       <c r="J79" s="6" t="inlineStr">
         <is>
-          <t>11-10~11-11</t>
+          <t>11-03~11-04</t>
         </is>
       </c>
       <c r="K79" s="6" t="inlineStr"/>
@@ -13945,18 +14014,18 @@
       <c r="M79" s="6" t="inlineStr"/>
       <c r="N79" s="6" t="inlineStr">
         <is>
-          <t>아이비케이투자증권</t>
+          <t>한국투자증권</t>
         </is>
       </c>
       <c r="O79" s="6" t="inlineStr"/>
       <c r="P79" s="7" t="inlineStr">
         <is>
-          <t>850,000,000</t>
-        </is>
-      </c>
-      <c r="Q79" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>2,407,500,000</t>
+        </is>
+      </c>
+      <c r="Q79" s="6" t="inlineStr">
+        <is>
+          <t>4.5%</t>
         </is>
       </c>
       <c r="R79" s="6" t="inlineStr">
@@ -13968,32 +14037,32 @@
     <row r="80" ht="30" customHeight="1">
       <c r="A80" s="6" t="inlineStr">
         <is>
-          <t>케이엠에프</t>
+          <t>제논</t>
         </is>
       </c>
       <c r="B80" s="6" t="inlineStr">
         <is>
-          <t>11-16~11-20</t>
+          <t>10-26~10-30</t>
         </is>
       </c>
       <c r="C80" s="6" t="inlineStr">
         <is>
-          <t>15,000~17,800</t>
+          <t>9,700~12,200</t>
         </is>
       </c>
       <c r="D80" s="7" t="inlineStr">
         <is>
-          <t>2,000,000</t>
+          <t>2,200,000</t>
         </is>
       </c>
       <c r="E80" s="7" t="inlineStr">
         <is>
-          <t>30,000,000,000</t>
+          <t>21,340,000,000</t>
         </is>
       </c>
       <c r="F80" s="6" t="inlineStr">
         <is>
-          <t>18.53배 (PER)</t>
+          <t>36.49배 (PER)</t>
         </is>
       </c>
       <c r="G80" s="6" t="inlineStr"/>
@@ -14001,7 +14070,7 @@
       <c r="I80" s="6" t="inlineStr"/>
       <c r="J80" s="6" t="inlineStr">
         <is>
-          <t>11-24~11-25</t>
+          <t>11-04~11-05</t>
         </is>
       </c>
       <c r="K80" s="6" t="inlineStr"/>
@@ -14009,18 +14078,18 @@
       <c r="M80" s="6" t="inlineStr"/>
       <c r="N80" s="6" t="inlineStr">
         <is>
-          <t>아이비케이투자증권</t>
+          <t>삼성증권</t>
         </is>
       </c>
       <c r="O80" s="6" t="inlineStr"/>
       <c r="P80" s="7" t="inlineStr">
         <is>
-          <t>927,000,000</t>
+          <t>835,247,600</t>
         </is>
       </c>
       <c r="Q80" s="6" t="inlineStr">
         <is>
-          <t>3.0%</t>
+          <t>3.80%</t>
         </is>
       </c>
       <c r="R80" s="6" t="inlineStr">
@@ -14032,54 +14101,54 @@
     <row r="81" ht="30" customHeight="1">
       <c r="A81" s="6" t="inlineStr">
         <is>
-          <t>럭스코</t>
-        </is>
-      </c>
-      <c r="B81" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="C81" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="D81" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="E81" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="F81" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>하나에어로다이내믹스</t>
+        </is>
+      </c>
+      <c r="B81" s="6" t="inlineStr">
+        <is>
+          <t>11-02~11-06</t>
+        </is>
+      </c>
+      <c r="C81" s="6" t="inlineStr">
+        <is>
+          <t>4,700~5,700</t>
+        </is>
+      </c>
+      <c r="D81" s="7" t="inlineStr">
+        <is>
+          <t>4,400,000</t>
+        </is>
+      </c>
+      <c r="E81" s="7" t="inlineStr">
+        <is>
+          <t>20,680,000,000</t>
+        </is>
+      </c>
+      <c r="F81" s="6" t="inlineStr">
+        <is>
+          <t>17.89배 (EV/EBITDA)</t>
         </is>
       </c>
       <c r="G81" s="6" t="inlineStr"/>
       <c r="H81" s="6" t="inlineStr"/>
       <c r="I81" s="6" t="inlineStr"/>
-      <c r="J81" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="J81" s="6" t="inlineStr">
+        <is>
+          <t>11-10~11-11</t>
         </is>
       </c>
       <c r="K81" s="6" t="inlineStr"/>
       <c r="L81" s="6" t="inlineStr"/>
       <c r="M81" s="6" t="inlineStr"/>
-      <c r="N81" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="N81" s="6" t="inlineStr">
+        <is>
+          <t>아이비케이투자증권</t>
         </is>
       </c>
       <c r="O81" s="6" t="inlineStr"/>
-      <c r="P81" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="P81" s="7" t="inlineStr">
+        <is>
+          <t>850,000,000</t>
         </is>
       </c>
       <c r="Q81" s="18" t="inlineStr">
@@ -14096,59 +14165,59 @@
     <row r="82" ht="30" customHeight="1">
       <c r="A82" s="6" t="inlineStr">
         <is>
-          <t>솔리스</t>
-        </is>
-      </c>
-      <c r="B82" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="C82" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="D82" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="E82" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="F82" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>케이엠에프</t>
+        </is>
+      </c>
+      <c r="B82" s="6" t="inlineStr">
+        <is>
+          <t>11-16~11-20</t>
+        </is>
+      </c>
+      <c r="C82" s="6" t="inlineStr">
+        <is>
+          <t>15,000~17,800</t>
+        </is>
+      </c>
+      <c r="D82" s="7" t="inlineStr">
+        <is>
+          <t>2,000,000</t>
+        </is>
+      </c>
+      <c r="E82" s="7" t="inlineStr">
+        <is>
+          <t>30,000,000,000</t>
+        </is>
+      </c>
+      <c r="F82" s="6" t="inlineStr">
+        <is>
+          <t>18.53배 (PER)</t>
         </is>
       </c>
       <c r="G82" s="6" t="inlineStr"/>
       <c r="H82" s="6" t="inlineStr"/>
       <c r="I82" s="6" t="inlineStr"/>
-      <c r="J82" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="J82" s="6" t="inlineStr">
+        <is>
+          <t>11-24~11-25</t>
         </is>
       </c>
       <c r="K82" s="6" t="inlineStr"/>
       <c r="L82" s="6" t="inlineStr"/>
       <c r="M82" s="6" t="inlineStr"/>
-      <c r="N82" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="N82" s="6" t="inlineStr">
+        <is>
+          <t>아이비케이투자증권</t>
         </is>
       </c>
       <c r="O82" s="6" t="inlineStr"/>
-      <c r="P82" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="Q82" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="P82" s="7" t="inlineStr">
+        <is>
+          <t>927,000,000</t>
+        </is>
+      </c>
+      <c r="Q82" s="6" t="inlineStr">
+        <is>
+          <t>3.0%</t>
         </is>
       </c>
       <c r="R82" s="6" t="inlineStr">
@@ -14160,7 +14229,7 @@
     <row r="83" ht="30" customHeight="1">
       <c r="A83" s="6" t="inlineStr">
         <is>
-          <t>디티에스</t>
+          <t>럭스코</t>
         </is>
       </c>
       <c r="B83" s="18" t="inlineStr">
@@ -14217,14 +14286,14 @@
       </c>
       <c r="R83" s="6" t="inlineStr">
         <is>
-          <t>신고서 대기</t>
+          <t>최초</t>
         </is>
       </c>
     </row>
     <row r="84" ht="30" customHeight="1">
       <c r="A84" s="6" t="inlineStr">
         <is>
-          <t>에이엔에이치스트럭쳐</t>
+          <t>디티에스</t>
         </is>
       </c>
       <c r="B84" s="18" t="inlineStr">
@@ -14288,7 +14357,7 @@
     <row r="85" ht="30" customHeight="1">
       <c r="A85" s="6" t="inlineStr">
         <is>
-          <t>이에스티</t>
+          <t>에이엔에이치스트럭쳐</t>
         </is>
       </c>
       <c r="B85" s="18" t="inlineStr">
@@ -14352,7 +14421,7 @@
     <row r="86" ht="30" customHeight="1">
       <c r="A86" s="6" t="inlineStr">
         <is>
-          <t>영광와이케이엠씨</t>
+          <t>이에스티</t>
         </is>
       </c>
       <c r="B86" s="18" t="inlineStr">
@@ -14416,7 +14485,7 @@
     <row r="87" ht="30" customHeight="1">
       <c r="A87" s="6" t="inlineStr">
         <is>
-          <t>제논</t>
+          <t>영광와이케이엠씨</t>
         </is>
       </c>
       <c r="B87" s="18" t="inlineStr">
@@ -14541,22 +14610,150 @@
         </is>
       </c>
     </row>
-    <row r="90">
-      <c r="A90" s="20" t="inlineStr">
-        <is>
-          <t>※ 상장 완료 = KIND 신규상장 페이지 기준(스팩합병 포함) · 스팩 공모상장은 밴드·밸류에이션 등 해당없음(공모가 2,000원 고정).</t>
-        </is>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" s="20" t="inlineStr">
-        <is>
-          <t>※ 기재정정 신고서 내 정정 전·후 병존 → 자동수집은 "정정 후" 값만 취함.</t>
+    <row r="89" ht="30" customHeight="1">
+      <c r="A89" s="6" t="inlineStr">
+        <is>
+          <t>엔키화이트햇</t>
+        </is>
+      </c>
+      <c r="B89" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="C89" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="D89" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="E89" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="F89" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="G89" s="6" t="inlineStr"/>
+      <c r="H89" s="6" t="inlineStr"/>
+      <c r="I89" s="6" t="inlineStr"/>
+      <c r="J89" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="K89" s="6" t="inlineStr"/>
+      <c r="L89" s="6" t="inlineStr"/>
+      <c r="M89" s="6" t="inlineStr"/>
+      <c r="N89" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="O89" s="6" t="inlineStr"/>
+      <c r="P89" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="Q89" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="R89" s="6" t="inlineStr">
+        <is>
+          <t>신고서 대기</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="30" customHeight="1">
+      <c r="A90" s="6" t="inlineStr">
+        <is>
+          <t>마더스제약</t>
+        </is>
+      </c>
+      <c r="B90" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="C90" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="D90" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="E90" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="F90" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="G90" s="6" t="inlineStr"/>
+      <c r="H90" s="6" t="inlineStr"/>
+      <c r="I90" s="6" t="inlineStr"/>
+      <c r="J90" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="K90" s="6" t="inlineStr"/>
+      <c r="L90" s="6" t="inlineStr"/>
+      <c r="M90" s="6" t="inlineStr"/>
+      <c r="N90" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="O90" s="6" t="inlineStr"/>
+      <c r="P90" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="Q90" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="R90" s="6" t="inlineStr">
+        <is>
+          <t>신고서 대기</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="20" t="inlineStr">
+        <is>
+          <t>※ 상장 완료 = KIND 신규상장 페이지 기준(스팩합병 포함) · 스팩 공모상장은 밴드·밸류에이션 등 해당없음(공모가 2,000원 고정).</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="20" t="inlineStr">
+        <is>
+          <t>※ 기재정정 신고서 내 정정 전·후 병존 → 자동수집은 "정정 후" 값만 취함.</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="20" t="inlineStr">
         <is>
           <t>※ 청약경쟁률=일반투자자 청약수량÷최종배정수량 · "MM-DD~"는 종료일 자동수집 예정.</t>
         </is>
@@ -14747,7 +14944,7 @@
         <v>4</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E10" s="6" t="n">
         <v>3</v>
@@ -14856,10 +15053,10 @@
         </is>
       </c>
       <c r="B15" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C15" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D15" s="6" t="n">
         <v>0</v>
@@ -14932,11 +15129,11 @@
         </is>
       </c>
       <c r="B20" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>262,674,000,000</t>
+          <t>284,014,000,000</t>
         </is>
       </c>
     </row>
@@ -15093,7 +15290,7 @@
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>신한투자증권</t>
+          <t>KB증권</t>
         </is>
       </c>
       <c r="B31" s="6" t="n">
@@ -15101,14 +15298,14 @@
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>30,240,000,000</t>
+          <t>31,200,000,000</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>KB증권</t>
+          <t>신한투자증권</t>
         </is>
       </c>
       <c r="B32" s="6" t="n">
@@ -15116,7 +15313,7 @@
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>27,200,000,000</t>
+          <t>30,240,000,000</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update IPO data 2026-10-08
</commit_message>
<xml_diff>
--- a/IPO_analysis.xlsx
+++ b/IPO_analysis.xlsx
@@ -592,7 +592,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K147"/>
+  <dimension ref="A1:K148"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -618,14 +618,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>기준일 2026-10-07 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
+          <t>기준일 2026-10-08 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>■ 심사 신청(진행중)  (44건)</t>
+          <t>■ 심사 신청(진행중)  (41건)</t>
         </is>
       </c>
       <c r="B4" s="4" t="n"/>
@@ -699,12 +699,12 @@
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>베르티스</t>
+          <t>세미솔루션</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
@@ -724,27 +724,27 @@
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>5,119</t>
+          <t>16,266</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
-          <t>-12,903</t>
+          <t>791</t>
         </is>
       </c>
       <c r="H6" s="7" t="inlineStr">
         <is>
-          <t>-16,364</t>
+          <t>9,629</t>
         </is>
       </c>
       <c r="I6" s="6" t="inlineStr">
         <is>
-          <t>의료용품 및 기타 의약 관련제품 제조업</t>
+          <t>반도체 제조업</t>
         </is>
       </c>
       <c r="J6" s="6" t="inlineStr">
         <is>
-          <t>대신</t>
+          <t>DB</t>
         </is>
       </c>
       <c r="K6" s="6" t="inlineStr">
@@ -756,12 +756,12 @@
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>뱅크샐러드</t>
+          <t>베르티스</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -781,27 +781,27 @@
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>25,994</t>
+          <t>5,119</t>
         </is>
       </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
-          <t>-59,792</t>
+          <t>-12,903</t>
         </is>
       </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
-          <t>28,335</t>
+          <t>-16,364</t>
         </is>
       </c>
       <c r="I7" s="6" t="inlineStr">
         <is>
-          <t>금융 지원 서비스업</t>
+          <t>의료용품 및 기타 의약 관련제품 제조업</t>
         </is>
       </c>
       <c r="J7" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>대신</t>
         </is>
       </c>
       <c r="K7" s="6" t="inlineStr">
@@ -813,12 +813,12 @@
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>키노톤</t>
+          <t>뱅크샐러드</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
@@ -838,27 +838,27 @@
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>46,943</t>
+          <t>25,994</t>
         </is>
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
-          <t>4,222</t>
+          <t>-59,792</t>
         </is>
       </c>
       <c r="H8" s="7" t="inlineStr">
         <is>
-          <t>19,112</t>
+          <t>28,335</t>
         </is>
       </c>
       <c r="I8" s="6" t="inlineStr">
         <is>
-          <t>건축기술, 엔지니어링 및 관련 기술 서비스업</t>
+          <t>금융 지원 서비스업</t>
         </is>
       </c>
       <c r="J8" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K8" s="6" t="inlineStr">
@@ -875,7 +875,7 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>티에스모스트</t>
+          <t>키노톤</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
@@ -895,27 +895,27 @@
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>156,198</t>
+          <t>46,943</t>
         </is>
       </c>
       <c r="G9" s="7" t="inlineStr">
         <is>
-          <t>5,666</t>
+          <t>4,222</t>
         </is>
       </c>
       <c r="H9" s="7" t="inlineStr">
         <is>
-          <t>25,181</t>
+          <t>19,112</t>
         </is>
       </c>
       <c r="I9" s="6" t="inlineStr">
         <is>
-          <t>자동차 신품 부품 제조업</t>
+          <t>건축기술, 엔지니어링 및 관련 기술 서비스업</t>
         </is>
       </c>
       <c r="J9" s="6" t="inlineStr">
         <is>
-          <t>신한</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="K9" s="6" t="inlineStr">
@@ -927,12 +927,12 @@
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>셀렉트스타</t>
+          <t>티에스모스트</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -952,27 +952,27 @@
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>11,616</t>
+          <t>156,198</t>
         </is>
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
-          <t>-9,883</t>
+          <t>5,666</t>
         </is>
       </c>
       <c r="H10" s="7" t="inlineStr">
         <is>
-          <t>-34,511</t>
+          <t>25,181</t>
         </is>
       </c>
       <c r="I10" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어 개발 및 공급업</t>
+          <t>자동차 신품 부품 제조업</t>
         </is>
       </c>
       <c r="J10" s="6" t="inlineStr">
         <is>
-          <t>대신</t>
+          <t>신한</t>
         </is>
       </c>
       <c r="K10" s="6" t="inlineStr">
@@ -984,12 +984,12 @@
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>서북</t>
+          <t>셀렉트스타</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -1009,27 +1009,27 @@
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>60,439</t>
+          <t>11,616</t>
         </is>
       </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
-          <t>-8,764</t>
+          <t>-9,883</t>
         </is>
       </c>
       <c r="H11" s="7" t="inlineStr">
         <is>
-          <t>4,485</t>
+          <t>-34,511</t>
         </is>
       </c>
       <c r="I11" s="6" t="inlineStr">
         <is>
-          <t>사진장비 및 광학기기 제조업</t>
+          <t>소프트웨어 개발 및 공급업</t>
         </is>
       </c>
       <c r="J11" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>대신</t>
         </is>
       </c>
       <c r="K11" s="6" t="inlineStr">
@@ -1046,7 +1046,7 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>에이스엔지니어링</t>
+          <t>서북</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
@@ -1066,27 +1066,27 @@
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>307,911</t>
+          <t>60,439</t>
         </is>
       </c>
       <c r="G12" s="7" t="inlineStr">
         <is>
-          <t>-101,468</t>
+          <t>-8,764</t>
         </is>
       </c>
       <c r="H12" s="7" t="inlineStr">
         <is>
-          <t>83,159</t>
+          <t>4,485</t>
         </is>
       </c>
       <c r="I12" s="6" t="inlineStr">
         <is>
-          <t>전동기, 발전기 및 전기 변환 · 공급 · 제어 장치 제조업</t>
+          <t>사진장비 및 광학기기 제조업</t>
         </is>
       </c>
       <c r="J12" s="6" t="inlineStr">
         <is>
-          <t>대신, 미래, 키움</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K12" s="6" t="inlineStr">
@@ -1103,7 +1103,7 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>플렉스시스템</t>
+          <t>에이스엔지니어링</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
@@ -1123,27 +1123,27 @@
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>10,894</t>
+          <t>307,911</t>
         </is>
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
-          <t>-2,342</t>
+          <t>-101,468</t>
         </is>
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
-          <t>3,014</t>
+          <t>83,159</t>
         </is>
       </c>
       <c r="I13" s="6" t="inlineStr">
         <is>
-          <t>측정, 시험, 항해, 제어 및 기타 정밀기기 제조업; 광학기기 제외</t>
+          <t>전동기, 발전기 및 전기 변환 · 공급 · 제어 장치 제조업</t>
         </is>
       </c>
       <c r="J13" s="6" t="inlineStr">
         <is>
-          <t>대신</t>
+          <t>대신, 미래, 키움</t>
         </is>
       </c>
       <c r="K13" s="6" t="inlineStr">
@@ -1155,12 +1155,12 @@
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>엠아이티</t>
+          <t>플렉스시스템</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
@@ -1180,27 +1180,27 @@
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
-          <t>14,921</t>
+          <t>10,894</t>
         </is>
       </c>
       <c r="G14" s="7" t="inlineStr">
         <is>
-          <t>1,181</t>
+          <t>-2,342</t>
         </is>
       </c>
       <c r="H14" s="7" t="inlineStr">
         <is>
-          <t>28,026</t>
+          <t>3,014</t>
         </is>
       </c>
       <c r="I14" s="6" t="inlineStr">
         <is>
-          <t>특수 목적용 기계 제조업</t>
+          <t>측정, 시험, 항해, 제어 및 기타 정밀기기 제조업; 광학기기 제외</t>
         </is>
       </c>
       <c r="J14" s="6" t="inlineStr">
         <is>
-          <t>삼성</t>
+          <t>대신</t>
         </is>
       </c>
       <c r="K14" s="6" t="inlineStr">
@@ -1217,7 +1217,7 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>큐로드</t>
+          <t>엠아이티</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
@@ -1227,7 +1227,7 @@
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>스팩 소멸합병</t>
+          <t>신규상장</t>
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr">
@@ -1235,17 +1235,29 @@
           <t>FY25</t>
         </is>
       </c>
-      <c r="F15" s="7" t="inlineStr"/>
-      <c r="G15" s="7" t="inlineStr"/>
-      <c r="H15" s="7" t="inlineStr"/>
+      <c r="F15" s="7" t="inlineStr">
+        <is>
+          <t>14,921</t>
+        </is>
+      </c>
+      <c r="G15" s="7" t="inlineStr">
+        <is>
+          <t>1,181</t>
+        </is>
+      </c>
+      <c r="H15" s="7" t="inlineStr">
+        <is>
+          <t>28,026</t>
+        </is>
+      </c>
       <c r="I15" s="6" t="inlineStr">
         <is>
-          <t>금융 지원 서비스업</t>
+          <t>특수 목적용 기계 제조업</t>
         </is>
       </c>
       <c r="J15" s="6" t="inlineStr">
         <is>
-          <t>교보</t>
+          <t>삼성</t>
         </is>
       </c>
       <c r="K15" s="6" t="inlineStr">
@@ -1257,12 +1269,12 @@
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>노바셀테크놀로지</t>
+          <t>큐로드</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
@@ -1272,7 +1284,7 @@
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t>신규상장</t>
+          <t>스팩 소멸합병</t>
         </is>
       </c>
       <c r="E16" s="6" t="inlineStr">
@@ -1280,29 +1292,17 @@
           <t>FY25</t>
         </is>
       </c>
-      <c r="F16" s="7" t="inlineStr">
-        <is>
-          <t>377</t>
-        </is>
-      </c>
-      <c r="G16" s="7" t="inlineStr">
-        <is>
-          <t>-4,606</t>
-        </is>
-      </c>
-      <c r="H16" s="7" t="inlineStr">
-        <is>
-          <t>-15,458</t>
-        </is>
-      </c>
+      <c r="F16" s="7" t="inlineStr"/>
+      <c r="G16" s="7" t="inlineStr"/>
+      <c r="H16" s="7" t="inlineStr"/>
       <c r="I16" s="6" t="inlineStr">
         <is>
-          <t>자연과학 및 공학 연구개발업</t>
+          <t>금융 지원 서비스업</t>
         </is>
       </c>
       <c r="J16" s="6" t="inlineStr">
         <is>
-          <t>키움</t>
+          <t>교보</t>
         </is>
       </c>
       <c r="K16" s="6" t="inlineStr">
@@ -1314,12 +1314,12 @@
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>(주)태석광학</t>
+          <t>노바셀테크놀로지</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
@@ -1339,27 +1339,27 @@
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
-          <t>79,804</t>
+          <t>377</t>
         </is>
       </c>
       <c r="G17" s="7" t="inlineStr">
         <is>
-          <t>4,721</t>
+          <t>-4,606</t>
         </is>
       </c>
       <c r="H17" s="7" t="inlineStr">
         <is>
-          <t>7,228</t>
+          <t>-15,458</t>
         </is>
       </c>
       <c r="I17" s="6" t="inlineStr">
         <is>
-          <t>생활용품 도매업</t>
+          <t>자연과학 및 공학 연구개발업</t>
         </is>
       </c>
       <c r="J17" s="6" t="inlineStr">
         <is>
-          <t>신한, 대신</t>
+          <t>키움</t>
         </is>
       </c>
       <c r="K17" s="6" t="inlineStr">
@@ -1371,12 +1371,12 @@
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>엑티브온</t>
+          <t>(주)태석광학</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
-          <t>스팩 소멸합병</t>
+          <t>신규상장</t>
         </is>
       </c>
       <c r="E18" s="6" t="inlineStr">
@@ -1394,17 +1394,29 @@
           <t>FY25</t>
         </is>
       </c>
-      <c r="F18" s="7" t="inlineStr"/>
-      <c r="G18" s="7" t="inlineStr"/>
-      <c r="H18" s="7" t="inlineStr"/>
+      <c r="F18" s="7" t="inlineStr">
+        <is>
+          <t>79,804</t>
+        </is>
+      </c>
+      <c r="G18" s="7" t="inlineStr">
+        <is>
+          <t>4,721</t>
+        </is>
+      </c>
+      <c r="H18" s="7" t="inlineStr">
+        <is>
+          <t>7,228</t>
+        </is>
+      </c>
       <c r="I18" s="6" t="inlineStr">
         <is>
-          <t>금융 지원 서비스업</t>
+          <t>생활용품 도매업</t>
         </is>
       </c>
       <c r="J18" s="6" t="inlineStr">
         <is>
-          <t>키움</t>
+          <t>신한, 대신</t>
         </is>
       </c>
       <c r="K18" s="6" t="inlineStr">
@@ -1416,12 +1428,12 @@
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>씨앤엠</t>
+          <t>엑티브온</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
@@ -1431,7 +1443,7 @@
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>신규상장</t>
+          <t>스팩 소멸합병</t>
         </is>
       </c>
       <c r="E19" s="6" t="inlineStr">
@@ -1439,29 +1451,17 @@
           <t>FY25</t>
         </is>
       </c>
-      <c r="F19" s="7" t="inlineStr">
-        <is>
-          <t>238,489</t>
-        </is>
-      </c>
-      <c r="G19" s="7" t="inlineStr">
-        <is>
-          <t>19,869</t>
-        </is>
-      </c>
-      <c r="H19" s="7" t="inlineStr">
-        <is>
-          <t>112,262</t>
-        </is>
-      </c>
+      <c r="F19" s="7" t="inlineStr"/>
+      <c r="G19" s="7" t="inlineStr"/>
+      <c r="H19" s="7" t="inlineStr"/>
       <c r="I19" s="6" t="inlineStr">
         <is>
-          <t>전동기, 발전기 및 전기 변환 · 공급 · 제어 장치 제조업</t>
+          <t>금융 지원 서비스업</t>
         </is>
       </c>
       <c r="J19" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>키움</t>
         </is>
       </c>
       <c r="K19" s="6" t="inlineStr">
@@ -1746,17 +1746,17 @@
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>에스텍시스템</t>
+          <t>범한메카텍</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>유가</t>
+          <t>코스닥</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
@@ -1771,27 +1771,27 @@
       </c>
       <c r="F25" s="7" t="inlineStr">
         <is>
-          <t>975,224</t>
+          <t>339,209</t>
         </is>
       </c>
       <c r="G25" s="7" t="inlineStr">
         <is>
-          <t>24,647</t>
+          <t>-18,141</t>
         </is>
       </c>
       <c r="H25" s="7" t="inlineStr">
         <is>
-          <t>237,182</t>
+          <t>265,955</t>
         </is>
       </c>
       <c r="I25" s="6" t="inlineStr">
         <is>
-          <t>경비, 경호 및 탐정업</t>
+          <t>구조용 금속제품, 탱크 및 증기발생기 제조업</t>
         </is>
       </c>
       <c r="J25" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>유진, NH</t>
         </is>
       </c>
       <c r="K25" s="6" t="inlineStr">
@@ -1803,12 +1803,12 @@
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>범한메카텍</t>
+          <t>데스틴파워</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
@@ -1828,27 +1828,27 @@
       </c>
       <c r="F26" s="7" t="inlineStr">
         <is>
-          <t>339,209</t>
+          <t>29,851</t>
         </is>
       </c>
       <c r="G26" s="7" t="inlineStr">
         <is>
-          <t>-18,141</t>
+          <t>5,852</t>
         </is>
       </c>
       <c r="H26" s="7" t="inlineStr">
         <is>
-          <t>265,955</t>
+          <t>-30,114</t>
         </is>
       </c>
       <c r="I26" s="6" t="inlineStr">
         <is>
-          <t>구조용 금속제품, 탱크 및 증기발생기 제조업</t>
+          <t>전동기, 발전기 및 전기 변환 · 공급 · 제어 장치 제조업</t>
         </is>
       </c>
       <c r="J26" s="6" t="inlineStr">
         <is>
-          <t>유진, NH</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="K26" s="6" t="inlineStr">
@@ -1860,12 +1860,12 @@
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>케이티이</t>
+          <t>유림테크</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
@@ -1885,27 +1885,27 @@
       </c>
       <c r="F27" s="7" t="inlineStr">
         <is>
-          <t>173,901</t>
+          <t>102,586</t>
         </is>
       </c>
       <c r="G27" s="7" t="inlineStr">
         <is>
-          <t>14,243</t>
+          <t>-18,278</t>
         </is>
       </c>
       <c r="H27" s="7" t="inlineStr">
         <is>
-          <t>94,928</t>
+          <t>-4,832</t>
         </is>
       </c>
       <c r="I27" s="6" t="inlineStr">
         <is>
-          <t>전동기, 발전기 및 전기 변환 · 공급 · 제어 장치 제조업</t>
+          <t>자동차 신품 부품 제조업</t>
         </is>
       </c>
       <c r="J27" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>대신</t>
         </is>
       </c>
       <c r="K27" s="6" t="inlineStr">
@@ -1917,12 +1917,12 @@
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>데스틴파워</t>
+          <t>이노보테라퓨틱스</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
@@ -1942,22 +1942,22 @@
       </c>
       <c r="F28" s="7" t="inlineStr">
         <is>
-          <t>29,851</t>
+          <t>209</t>
         </is>
       </c>
       <c r="G28" s="7" t="inlineStr">
         <is>
-          <t>5,852</t>
+          <t>-5,429</t>
         </is>
       </c>
       <c r="H28" s="7" t="inlineStr">
         <is>
-          <t>-30,114</t>
+          <t>-53,200</t>
         </is>
       </c>
       <c r="I28" s="6" t="inlineStr">
         <is>
-          <t>전동기, 발전기 및 전기 변환 · 공급 · 제어 장치 제조업</t>
+          <t>의약품 제조업</t>
         </is>
       </c>
       <c r="J28" s="6" t="inlineStr">
@@ -1974,17 +1974,17 @@
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>유림테크</t>
+          <t>에스에프씨</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>코스닥</t>
+          <t>유가</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr">
@@ -1999,27 +1999,27 @@
       </c>
       <c r="F29" s="7" t="inlineStr">
         <is>
-          <t>102,586</t>
+          <t>160,792</t>
         </is>
       </c>
       <c r="G29" s="7" t="inlineStr">
         <is>
-          <t>-18,278</t>
+          <t>25,509</t>
         </is>
       </c>
       <c r="H29" s="7" t="inlineStr">
         <is>
-          <t>-4,832</t>
+          <t>243,562</t>
         </is>
       </c>
       <c r="I29" s="6" t="inlineStr">
         <is>
-          <t>자동차 신품 부품 제조업</t>
+          <t>기타 화학제품 제조업</t>
         </is>
       </c>
       <c r="J29" s="6" t="inlineStr">
         <is>
-          <t>대신</t>
+          <t>미래, 한국</t>
         </is>
       </c>
       <c r="K29" s="6" t="inlineStr">
@@ -2031,12 +2031,12 @@
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>이노보테라퓨틱스</t>
+          <t>에버온</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
@@ -2056,27 +2056,27 @@
       </c>
       <c r="F30" s="7" t="inlineStr">
         <is>
-          <t>209</t>
+          <t>65,225</t>
         </is>
       </c>
       <c r="G30" s="7" t="inlineStr">
         <is>
-          <t>-5,429</t>
+          <t>-3,606</t>
         </is>
       </c>
       <c r="H30" s="7" t="inlineStr">
         <is>
-          <t>-53,200</t>
+          <t>54,955</t>
         </is>
       </c>
       <c r="I30" s="6" t="inlineStr">
         <is>
-          <t>의약품 제조업</t>
+          <t>전기업</t>
         </is>
       </c>
       <c r="J30" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K30" s="6" t="inlineStr">
@@ -2088,17 +2088,17 @@
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>에스에프씨</t>
+          <t>씨아이에스케미칼</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>유가</t>
+          <t>코스닥</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr">
@@ -2113,27 +2113,27 @@
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>160,792</t>
+          <t>15,985</t>
         </is>
       </c>
       <c r="G31" s="7" t="inlineStr">
         <is>
-          <t>25,509</t>
+          <t>-11,440</t>
         </is>
       </c>
       <c r="H31" s="7" t="inlineStr">
         <is>
-          <t>243,562</t>
+          <t>23,706</t>
         </is>
       </c>
       <c r="I31" s="6" t="inlineStr">
         <is>
-          <t>기타 화학제품 제조업</t>
+          <t>기초 화학물질 제조업</t>
         </is>
       </c>
       <c r="J31" s="6" t="inlineStr">
         <is>
-          <t>미래, 한국</t>
+          <t>KB</t>
         </is>
       </c>
       <c r="K31" s="6" t="inlineStr">
@@ -2145,12 +2145,12 @@
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>아델</t>
+          <t>엠디에스코리아</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr">
@@ -2170,27 +2170,27 @@
       </c>
       <c r="F32" s="7" t="inlineStr">
         <is>
-          <t>62,057</t>
+          <t>97,972</t>
         </is>
       </c>
       <c r="G32" s="7" t="inlineStr">
         <is>
-          <t>-64,210</t>
+          <t>6,512</t>
         </is>
       </c>
       <c r="H32" s="7" t="inlineStr">
         <is>
-          <t>-80,776</t>
+          <t>53,818</t>
         </is>
       </c>
       <c r="I32" s="6" t="inlineStr">
         <is>
-          <t>그외 기타 전문, 과학 및 기술 서비스업</t>
+          <t>기타 식품 제조업</t>
         </is>
       </c>
       <c r="J32" s="6" t="inlineStr">
         <is>
-          <t>삼성, 미래</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K32" s="6" t="inlineStr">
@@ -2202,12 +2202,12 @@
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>에버온</t>
+          <t>동승</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
@@ -2227,27 +2227,27 @@
       </c>
       <c r="F33" s="7" t="inlineStr">
         <is>
-          <t>65,225</t>
+          <t>78,625</t>
         </is>
       </c>
       <c r="G33" s="7" t="inlineStr">
         <is>
-          <t>-3,606</t>
+          <t>14,525</t>
         </is>
       </c>
       <c r="H33" s="7" t="inlineStr">
         <is>
-          <t>54,955</t>
+          <t>5,438</t>
         </is>
       </c>
       <c r="I33" s="6" t="inlineStr">
         <is>
-          <t>전기업</t>
+          <t>부동산 임대 및 공급업</t>
         </is>
       </c>
       <c r="J33" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K33" s="6" t="inlineStr">
@@ -2259,12 +2259,12 @@
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>씨아이에스케미칼</t>
+          <t>에프엠더블유</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
@@ -2274,7 +2274,7 @@
       </c>
       <c r="D34" s="6" t="inlineStr">
         <is>
-          <t>신규상장</t>
+          <t>스팩 소멸합병</t>
         </is>
       </c>
       <c r="E34" s="6" t="inlineStr">
@@ -2284,27 +2284,27 @@
       </c>
       <c r="F34" s="7" t="inlineStr">
         <is>
-          <t>15,985</t>
+          <t>30,282</t>
         </is>
       </c>
       <c r="G34" s="7" t="inlineStr">
         <is>
-          <t>-11,440</t>
+          <t>4,762</t>
         </is>
       </c>
       <c r="H34" s="7" t="inlineStr">
         <is>
-          <t>23,706</t>
+          <t>32</t>
         </is>
       </c>
       <c r="I34" s="6" t="inlineStr">
         <is>
-          <t>기초 화학물질 제조업</t>
+          <t>기타 식품 제조업</t>
         </is>
       </c>
       <c r="J34" s="6" t="inlineStr">
         <is>
-          <t>KB</t>
+          <t>유진</t>
         </is>
       </c>
       <c r="K34" s="6" t="inlineStr">
@@ -2316,17 +2316,17 @@
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>엠디에스코리아</t>
+          <t>소노인터내셔널</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>코스닥</t>
+          <t>유가</t>
         </is>
       </c>
       <c r="D35" s="6" t="inlineStr">
@@ -2341,27 +2341,27 @@
       </c>
       <c r="F35" s="7" t="inlineStr">
         <is>
-          <t>97,972</t>
+          <t>2,093,051</t>
         </is>
       </c>
       <c r="G35" s="7" t="inlineStr">
         <is>
-          <t>6,512</t>
+          <t>-148,064</t>
         </is>
       </c>
       <c r="H35" s="7" t="inlineStr">
         <is>
-          <t>53,818</t>
+          <t>852,372</t>
         </is>
       </c>
       <c r="I35" s="6" t="inlineStr">
         <is>
-          <t>기타 식품 제조업</t>
+          <t>일반 및 생활 숙박시설 운영업</t>
         </is>
       </c>
       <c r="J35" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>대신, 미래</t>
         </is>
       </c>
       <c r="K35" s="6" t="inlineStr">
@@ -2373,12 +2373,12 @@
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>동승</t>
+          <t>싸이몬</t>
         </is>
       </c>
       <c r="C36" s="6" t="inlineStr">
@@ -2398,27 +2398,27 @@
       </c>
       <c r="F36" s="7" t="inlineStr">
         <is>
-          <t>78,625</t>
+          <t>48,695</t>
         </is>
       </c>
       <c r="G36" s="7" t="inlineStr">
         <is>
-          <t>14,525</t>
+          <t>15,714</t>
         </is>
       </c>
       <c r="H36" s="7" t="inlineStr">
         <is>
-          <t>5,438</t>
+          <t>61,761</t>
         </is>
       </c>
       <c r="I36" s="6" t="inlineStr">
         <is>
-          <t>부동산 임대 및 공급업</t>
+          <t>측정, 시험, 항해, 제어 및 기타 정밀기기 제조업</t>
         </is>
       </c>
       <c r="J36" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K36" s="6" t="inlineStr">
@@ -2430,12 +2430,12 @@
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>에프엠더블유</t>
+          <t>바이다</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
@@ -2445,7 +2445,7 @@
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
-          <t>스팩 소멸합병</t>
+          <t>신규상장</t>
         </is>
       </c>
       <c r="E37" s="6" t="inlineStr">
@@ -2455,27 +2455,27 @@
       </c>
       <c r="F37" s="7" t="inlineStr">
         <is>
-          <t>30,282</t>
+          <t>14,432</t>
         </is>
       </c>
       <c r="G37" s="7" t="inlineStr">
         <is>
-          <t>4,762</t>
+          <t>-3,951</t>
         </is>
       </c>
       <c r="H37" s="7" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>15,108</t>
         </is>
       </c>
       <c r="I37" s="6" t="inlineStr">
         <is>
-          <t>기타 식품 제조업</t>
+          <t>전자부품 제조업</t>
         </is>
       </c>
       <c r="J37" s="6" t="inlineStr">
         <is>
-          <t>유진</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K37" s="6" t="inlineStr">
@@ -2487,17 +2487,17 @@
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>소노인터내셔널</t>
+          <t>아이알큐더스</t>
         </is>
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
-          <t>유가</t>
+          <t>코스닥</t>
         </is>
       </c>
       <c r="D38" s="6" t="inlineStr">
@@ -2512,27 +2512,27 @@
       </c>
       <c r="F38" s="7" t="inlineStr">
         <is>
-          <t>2,093,051</t>
+          <t>10,231</t>
         </is>
       </c>
       <c r="G38" s="7" t="inlineStr">
         <is>
-          <t>-148,064</t>
+          <t>-986</t>
         </is>
       </c>
       <c r="H38" s="7" t="inlineStr">
         <is>
-          <t>852,372</t>
+          <t>1,800</t>
         </is>
       </c>
       <c r="I38" s="6" t="inlineStr">
         <is>
-          <t>일반 및 생활 숙박시설 운영업</t>
+          <t>소프트웨어 개발 및 공급업</t>
         </is>
       </c>
       <c r="J38" s="6" t="inlineStr">
         <is>
-          <t>대신, 미래</t>
+          <t>DB</t>
         </is>
       </c>
       <c r="K38" s="6" t="inlineStr">
@@ -2544,12 +2544,12 @@
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>싸이몬</t>
+          <t>씨엔티테크</t>
         </is>
       </c>
       <c r="C39" s="6" t="inlineStr">
@@ -2569,27 +2569,27 @@
       </c>
       <c r="F39" s="7" t="inlineStr">
         <is>
-          <t>48,695</t>
+          <t>27,015</t>
         </is>
       </c>
       <c r="G39" s="7" t="inlineStr">
         <is>
-          <t>15,714</t>
+          <t>3,987</t>
         </is>
       </c>
       <c r="H39" s="7" t="inlineStr">
         <is>
-          <t>61,761</t>
+          <t>2,613</t>
         </is>
       </c>
       <c r="I39" s="6" t="inlineStr">
         <is>
-          <t>측정, 시험, 항해, 제어 및 기타 정밀기기 제조업</t>
+          <t>소프트웨어 개발 및 공급업</t>
         </is>
       </c>
       <c r="J39" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>한화, 하나</t>
         </is>
       </c>
       <c r="K39" s="6" t="inlineStr">
@@ -2601,12 +2601,12 @@
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>바이다</t>
+          <t>제이앤티지</t>
         </is>
       </c>
       <c r="C40" s="6" t="inlineStr">
@@ -2626,17 +2626,17 @@
       </c>
       <c r="F40" s="7" t="inlineStr">
         <is>
-          <t>14,432</t>
+          <t>72,378</t>
         </is>
       </c>
       <c r="G40" s="7" t="inlineStr">
         <is>
-          <t>-3,951</t>
+          <t>9,904</t>
         </is>
       </c>
       <c r="H40" s="7" t="inlineStr">
         <is>
-          <t>15,108</t>
+          <t>6,743</t>
         </is>
       </c>
       <c r="I40" s="6" t="inlineStr">
@@ -2646,7 +2646,7 @@
       </c>
       <c r="J40" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>대신, NH</t>
         </is>
       </c>
       <c r="K40" s="6" t="inlineStr">
@@ -2658,12 +2658,12 @@
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>아이알큐더스</t>
+          <t>인터엑스</t>
         </is>
       </c>
       <c r="C41" s="6" t="inlineStr">
@@ -2683,17 +2683,17 @@
       </c>
       <c r="F41" s="7" t="inlineStr">
         <is>
-          <t>10,231</t>
+          <t>8,645</t>
         </is>
       </c>
       <c r="G41" s="7" t="inlineStr">
         <is>
-          <t>-986</t>
+          <t>-20,272</t>
         </is>
       </c>
       <c r="H41" s="7" t="inlineStr">
         <is>
-          <t>1,800</t>
+          <t>4,530</t>
         </is>
       </c>
       <c r="I41" s="6" t="inlineStr">
@@ -2703,7 +2703,7 @@
       </c>
       <c r="J41" s="6" t="inlineStr">
         <is>
-          <t>DB</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="K41" s="6" t="inlineStr">
@@ -2715,12 +2715,12 @@
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B42" s="6" t="inlineStr">
         <is>
-          <t>씨엔티테크</t>
+          <t>삼홍아크튜리온</t>
         </is>
       </c>
       <c r="C42" s="6" t="inlineStr">
@@ -2740,27 +2740,27 @@
       </c>
       <c r="F42" s="7" t="inlineStr">
         <is>
-          <t>27,015</t>
+          <t>26,162</t>
         </is>
       </c>
       <c r="G42" s="7" t="inlineStr">
         <is>
-          <t>3,987</t>
+          <t>-10,314</t>
         </is>
       </c>
       <c r="H42" s="7" t="inlineStr">
         <is>
-          <t>2,613</t>
+          <t>6,369</t>
         </is>
       </c>
       <c r="I42" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어 개발 및 공급업</t>
+          <t>구조용 금속제품, 탱크 및 증기발생기 제조업</t>
         </is>
       </c>
       <c r="J42" s="6" t="inlineStr">
         <is>
-          <t>한화, 하나</t>
+          <t>삼성, 미래</t>
         </is>
       </c>
       <c r="K42" s="6" t="inlineStr">
@@ -2772,12 +2772,12 @@
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B43" s="6" t="inlineStr">
         <is>
-          <t>제이앤티지</t>
+          <t>비앤비코리아</t>
         </is>
       </c>
       <c r="C43" s="6" t="inlineStr">
@@ -2797,27 +2797,27 @@
       </c>
       <c r="F43" s="7" t="inlineStr">
         <is>
-          <t>72,378</t>
+          <t>141,169</t>
         </is>
       </c>
       <c r="G43" s="7" t="inlineStr">
         <is>
-          <t>9,904</t>
+          <t>21,406</t>
         </is>
       </c>
       <c r="H43" s="7" t="inlineStr">
         <is>
-          <t>6,743</t>
+          <t>43,932</t>
         </is>
       </c>
       <c r="I43" s="6" t="inlineStr">
         <is>
-          <t>전자부품 제조업</t>
+          <t>기타 화학제품 제조업</t>
         </is>
       </c>
       <c r="J43" s="6" t="inlineStr">
         <is>
-          <t>대신, NH</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K43" s="6" t="inlineStr">
@@ -2829,12 +2829,12 @@
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B44" s="6" t="inlineStr">
         <is>
-          <t>인터엑스</t>
+          <t>오토핸즈</t>
         </is>
       </c>
       <c r="C44" s="6" t="inlineStr">
@@ -2844,7 +2844,7 @@
       </c>
       <c r="D44" s="6" t="inlineStr">
         <is>
-          <t>신규상장</t>
+          <t>스팩 소멸합병</t>
         </is>
       </c>
       <c r="E44" s="6" t="inlineStr">
@@ -2854,27 +2854,27 @@
       </c>
       <c r="F44" s="7" t="inlineStr">
         <is>
-          <t>8,645</t>
+          <t>238,564</t>
         </is>
       </c>
       <c r="G44" s="7" t="inlineStr">
         <is>
-          <t>-20,272</t>
+          <t>6,047</t>
         </is>
       </c>
       <c r="H44" s="7" t="inlineStr">
         <is>
-          <t>4,530</t>
+          <t>6,129</t>
         </is>
       </c>
       <c r="I44" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어 개발 및 공급업</t>
+          <t>자동차 판매업</t>
         </is>
       </c>
       <c r="J44" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K44" s="6" t="inlineStr">
@@ -2886,12 +2886,12 @@
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B45" s="6" t="inlineStr">
         <is>
-          <t>삼홍아크튜리온</t>
+          <t>아이벡스메디칼시스템즈</t>
         </is>
       </c>
       <c r="C45" s="6" t="inlineStr">
@@ -2911,27 +2911,27 @@
       </c>
       <c r="F45" s="7" t="inlineStr">
         <is>
-          <t>26,162</t>
+          <t>15,282</t>
         </is>
       </c>
       <c r="G45" s="7" t="inlineStr">
         <is>
-          <t>-10,314</t>
+          <t>-7,227</t>
         </is>
       </c>
       <c r="H45" s="7" t="inlineStr">
         <is>
-          <t>6,369</t>
+          <t>744</t>
         </is>
       </c>
       <c r="I45" s="6" t="inlineStr">
         <is>
-          <t>구조용 금속제품, 탱크 및 증기발생기 제조업</t>
+          <t>의료용 기기 제조업</t>
         </is>
       </c>
       <c r="J45" s="6" t="inlineStr">
         <is>
-          <t>삼성, 미래</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K45" s="6" t="inlineStr">
@@ -2943,12 +2943,12 @@
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="B46" s="6" t="inlineStr">
         <is>
-          <t>비앤비코리아</t>
+          <t>피지티</t>
         </is>
       </c>
       <c r="C46" s="6" t="inlineStr">
@@ -2968,17 +2968,17 @@
       </c>
       <c r="F46" s="7" t="inlineStr">
         <is>
-          <t>141,169</t>
+          <t>40,141</t>
         </is>
       </c>
       <c r="G46" s="7" t="inlineStr">
         <is>
-          <t>21,406</t>
+          <t>-69,722</t>
         </is>
       </c>
       <c r="H46" s="7" t="inlineStr">
         <is>
-          <t>43,932</t>
+          <t>6,029</t>
         </is>
       </c>
       <c r="I46" s="6" t="inlineStr">
@@ -2988,7 +2988,7 @@
       </c>
       <c r="J46" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="K46" s="6" t="inlineStr">
@@ -2997,248 +2997,248 @@
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="6" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
-        </is>
-      </c>
-      <c r="B47" s="6" t="inlineStr">
-        <is>
-          <t>오토핸즈</t>
-        </is>
-      </c>
-      <c r="C47" s="6" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>■ 심사 승인  (76건)</t>
+        </is>
+      </c>
+      <c r="B48" s="4" t="n"/>
+      <c r="C48" s="4" t="n"/>
+      <c r="D48" s="4" t="n"/>
+      <c r="E48" s="4" t="n"/>
+      <c r="F48" s="4" t="n"/>
+      <c r="G48" s="4" t="n"/>
+      <c r="H48" s="4" t="n"/>
+      <c r="I48" s="4" t="n"/>
+      <c r="J48" s="4" t="n"/>
+      <c r="K48" s="4" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>일자</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>회사명</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>시장</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t>상장유형</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>기준연도</t>
+        </is>
+      </c>
+      <c r="F49" s="5" t="inlineStr">
+        <is>
+          <t>매출액</t>
+        </is>
+      </c>
+      <c r="G49" s="5" t="inlineStr">
+        <is>
+          <t>순이익</t>
+        </is>
+      </c>
+      <c r="H49" s="5" t="inlineStr">
+        <is>
+          <t>자기자본</t>
+        </is>
+      </c>
+      <c r="I49" s="5" t="inlineStr">
+        <is>
+          <t>업종</t>
+        </is>
+      </c>
+      <c r="J49" s="5" t="inlineStr">
+        <is>
+          <t>대표주관사</t>
+        </is>
+      </c>
+      <c r="K49" s="5" t="inlineStr">
+        <is>
+          <t>현황</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B50" s="6" t="inlineStr">
+        <is>
+          <t>아델</t>
+        </is>
+      </c>
+      <c r="C50" s="6" t="inlineStr">
         <is>
           <t>코스닥</t>
         </is>
       </c>
-      <c r="D47" s="6" t="inlineStr">
-        <is>
-          <t>스팩 소멸합병</t>
-        </is>
-      </c>
-      <c r="E47" s="6" t="inlineStr">
+      <c r="D50" s="6" t="inlineStr">
+        <is>
+          <t>신규상장</t>
+        </is>
+      </c>
+      <c r="E50" s="6" t="inlineStr">
         <is>
           <t>FY25</t>
         </is>
       </c>
-      <c r="F47" s="7" t="inlineStr">
-        <is>
-          <t>238,564</t>
-        </is>
-      </c>
-      <c r="G47" s="7" t="inlineStr">
-        <is>
-          <t>6,047</t>
-        </is>
-      </c>
-      <c r="H47" s="7" t="inlineStr">
-        <is>
-          <t>6,129</t>
-        </is>
-      </c>
-      <c r="I47" s="6" t="inlineStr">
-        <is>
-          <t>자동차 판매업</t>
-        </is>
-      </c>
-      <c r="J47" s="6" t="inlineStr">
-        <is>
-          <t>미래</t>
-        </is>
-      </c>
-      <c r="K47" s="6" t="inlineStr">
-        <is>
-          <t>예심 진행중</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="6" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-      <c r="B48" s="6" t="inlineStr">
-        <is>
-          <t>아이벡스메디칼시스템즈</t>
-        </is>
-      </c>
-      <c r="C48" s="6" t="inlineStr">
+      <c r="F50" s="7" t="inlineStr">
+        <is>
+          <t>62,057</t>
+        </is>
+      </c>
+      <c r="G50" s="7" t="inlineStr">
+        <is>
+          <t>-64,210</t>
+        </is>
+      </c>
+      <c r="H50" s="7" t="inlineStr">
+        <is>
+          <t>-80,776</t>
+        </is>
+      </c>
+      <c r="I50" s="6" t="inlineStr">
+        <is>
+          <t>그외 기타 전문, 과학 및 기술 서비스업</t>
+        </is>
+      </c>
+      <c r="J50" s="6" t="inlineStr">
+        <is>
+          <t>삼성, 미래</t>
+        </is>
+      </c>
+      <c r="K50" s="6" t="inlineStr">
+        <is>
+          <t>상장전</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B51" s="6" t="inlineStr">
+        <is>
+          <t>케이티이</t>
+        </is>
+      </c>
+      <c r="C51" s="6" t="inlineStr">
         <is>
           <t>코스닥</t>
         </is>
       </c>
-      <c r="D48" s="6" t="inlineStr">
+      <c r="D51" s="6" t="inlineStr">
         <is>
           <t>신규상장</t>
         </is>
       </c>
-      <c r="E48" s="6" t="inlineStr">
+      <c r="E51" s="6" t="inlineStr">
         <is>
           <t>FY25</t>
         </is>
       </c>
-      <c r="F48" s="7" t="inlineStr">
-        <is>
-          <t>15,282</t>
-        </is>
-      </c>
-      <c r="G48" s="7" t="inlineStr">
-        <is>
-          <t>-7,227</t>
-        </is>
-      </c>
-      <c r="H48" s="7" t="inlineStr">
-        <is>
-          <t>744</t>
-        </is>
-      </c>
-      <c r="I48" s="6" t="inlineStr">
-        <is>
-          <t>의료용 기기 제조업</t>
-        </is>
-      </c>
-      <c r="J48" s="6" t="inlineStr">
+      <c r="F51" s="7" t="inlineStr">
+        <is>
+          <t>173,901</t>
+        </is>
+      </c>
+      <c r="G51" s="7" t="inlineStr">
+        <is>
+          <t>14,243</t>
+        </is>
+      </c>
+      <c r="H51" s="7" t="inlineStr">
+        <is>
+          <t>94,928</t>
+        </is>
+      </c>
+      <c r="I51" s="6" t="inlineStr">
+        <is>
+          <t>전동기, 발전기 및 전기 변환 · 공급 · 제어 장치 제조업</t>
+        </is>
+      </c>
+      <c r="J51" s="6" t="inlineStr">
         <is>
           <t>NH</t>
         </is>
       </c>
-      <c r="K48" s="6" t="inlineStr">
-        <is>
-          <t>예심 진행중</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="6" t="inlineStr">
-        <is>
-          <t>2026-02-27</t>
-        </is>
-      </c>
-      <c r="B49" s="6" t="inlineStr">
-        <is>
-          <t>피지티</t>
-        </is>
-      </c>
-      <c r="C49" s="6" t="inlineStr">
+      <c r="K51" s="6" t="inlineStr">
+        <is>
+          <t>상장전</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B52" s="6" t="inlineStr">
+        <is>
+          <t>씨앤엠</t>
+        </is>
+      </c>
+      <c r="C52" s="6" t="inlineStr">
         <is>
           <t>코스닥</t>
         </is>
       </c>
-      <c r="D49" s="6" t="inlineStr">
+      <c r="D52" s="6" t="inlineStr">
         <is>
           <t>신규상장</t>
         </is>
       </c>
-      <c r="E49" s="6" t="inlineStr">
+      <c r="E52" s="6" t="inlineStr">
         <is>
           <t>FY25</t>
         </is>
       </c>
-      <c r="F49" s="7" t="inlineStr">
-        <is>
-          <t>40,141</t>
-        </is>
-      </c>
-      <c r="G49" s="7" t="inlineStr">
-        <is>
-          <t>-69,722</t>
-        </is>
-      </c>
-      <c r="H49" s="7" t="inlineStr">
-        <is>
-          <t>6,029</t>
-        </is>
-      </c>
-      <c r="I49" s="6" t="inlineStr">
-        <is>
-          <t>기타 화학제품 제조업</t>
-        </is>
-      </c>
-      <c r="J49" s="6" t="inlineStr">
+      <c r="F52" s="7" t="inlineStr">
+        <is>
+          <t>238,489</t>
+        </is>
+      </c>
+      <c r="G52" s="7" t="inlineStr">
+        <is>
+          <t>19,869</t>
+        </is>
+      </c>
+      <c r="H52" s="7" t="inlineStr">
+        <is>
+          <t>112,262</t>
+        </is>
+      </c>
+      <c r="I52" s="6" t="inlineStr">
+        <is>
+          <t>전동기, 발전기 및 전기 변환 · 공급 · 제어 장치 제조업</t>
+        </is>
+      </c>
+      <c r="J52" s="6" t="inlineStr">
         <is>
           <t>한국</t>
         </is>
       </c>
-      <c r="K49" s="6" t="inlineStr">
-        <is>
-          <t>예심 진행중</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="3" t="inlineStr">
-        <is>
-          <t>■ 심사 승인  (73건)</t>
-        </is>
-      </c>
-      <c r="B51" s="4" t="n"/>
-      <c r="C51" s="4" t="n"/>
-      <c r="D51" s="4" t="n"/>
-      <c r="E51" s="4" t="n"/>
-      <c r="F51" s="4" t="n"/>
-      <c r="G51" s="4" t="n"/>
-      <c r="H51" s="4" t="n"/>
-      <c r="I51" s="4" t="n"/>
-      <c r="J51" s="4" t="n"/>
-      <c r="K51" s="4" t="n"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="5" t="inlineStr">
-        <is>
-          <t>일자</t>
-        </is>
-      </c>
-      <c r="B52" s="5" t="inlineStr">
-        <is>
-          <t>회사명</t>
-        </is>
-      </c>
-      <c r="C52" s="5" t="inlineStr">
-        <is>
-          <t>시장</t>
-        </is>
-      </c>
-      <c r="D52" s="5" t="inlineStr">
-        <is>
-          <t>상장유형</t>
-        </is>
-      </c>
-      <c r="E52" s="5" t="inlineStr">
-        <is>
-          <t>기준연도</t>
-        </is>
-      </c>
-      <c r="F52" s="5" t="inlineStr">
-        <is>
-          <t>매출액</t>
-        </is>
-      </c>
-      <c r="G52" s="5" t="inlineStr">
-        <is>
-          <t>순이익</t>
-        </is>
-      </c>
-      <c r="H52" s="5" t="inlineStr">
-        <is>
-          <t>자기자본</t>
-        </is>
-      </c>
-      <c r="I52" s="5" t="inlineStr">
-        <is>
-          <t>업종</t>
-        </is>
-      </c>
-      <c r="J52" s="5" t="inlineStr">
-        <is>
-          <t>대표주관사</t>
-        </is>
-      </c>
-      <c r="K52" s="5" t="inlineStr">
-        <is>
-          <t>현황</t>
+      <c r="K52" s="6" t="inlineStr">
+        <is>
+          <t>상장전</t>
         </is>
       </c>
     </row>
@@ -7242,7 +7242,7 @@
     <row r="127">
       <c r="A127" s="3" t="inlineStr">
         <is>
-          <t>■ 철회·미승인  (19건)</t>
+          <t>■ 철회·미승인  (20건)</t>
         </is>
       </c>
       <c r="B127" s="4" t="n"/>
@@ -7316,17 +7316,17 @@
     <row r="129">
       <c r="A129" s="6" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B129" s="6" t="inlineStr">
         <is>
-          <t>넥스트에어로스페이스</t>
+          <t>에스텍시스템</t>
         </is>
       </c>
       <c r="C129" s="6" t="inlineStr">
         <is>
-          <t>코스닥</t>
+          <t>유가</t>
         </is>
       </c>
       <c r="D129" s="6" t="inlineStr">
@@ -7341,27 +7341,27 @@
       </c>
       <c r="F129" s="7" t="inlineStr">
         <is>
-          <t>12,084</t>
+          <t>975,224</t>
         </is>
       </c>
       <c r="G129" s="7" t="inlineStr">
         <is>
-          <t>-17,270</t>
+          <t>24,647</t>
         </is>
       </c>
       <c r="H129" s="7" t="inlineStr">
         <is>
-          <t>6,158</t>
+          <t>237,182</t>
         </is>
       </c>
       <c r="I129" s="6" t="inlineStr">
         <is>
-          <t>유인 항공기, 항공우주선 및 보조장치 제조업</t>
+          <t>경비, 경호 및 탐정업</t>
         </is>
       </c>
       <c r="J129" s="6" t="inlineStr">
         <is>
-          <t>삼성</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K129" s="6" t="inlineStr">
@@ -7373,12 +7373,12 @@
     <row r="130">
       <c r="A130" s="6" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="B130" s="6" t="inlineStr">
         <is>
-          <t>텔레픽스</t>
+          <t>넥스트에어로스페이스</t>
         </is>
       </c>
       <c r="C130" s="6" t="inlineStr">
@@ -7398,27 +7398,27 @@
       </c>
       <c r="F130" s="7" t="inlineStr">
         <is>
-          <t>4,896</t>
+          <t>12,084</t>
         </is>
       </c>
       <c r="G130" s="7" t="inlineStr">
         <is>
-          <t>-16,214</t>
+          <t>-17,270</t>
         </is>
       </c>
       <c r="H130" s="7" t="inlineStr">
         <is>
-          <t>9,146</t>
+          <t>6,158</t>
         </is>
       </c>
       <c r="I130" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어 개발 및 공급업</t>
+          <t>유인 항공기, 항공우주선 및 보조장치 제조업</t>
         </is>
       </c>
       <c r="J130" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>삼성</t>
         </is>
       </c>
       <c r="K130" s="6" t="inlineStr">
@@ -7430,12 +7430,12 @@
     <row r="131">
       <c r="A131" s="6" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B131" s="6" t="inlineStr">
         <is>
-          <t>씨엠디엘</t>
+          <t>텔레픽스</t>
         </is>
       </c>
       <c r="C131" s="6" t="inlineStr">
@@ -7445,37 +7445,37 @@
       </c>
       <c r="D131" s="6" t="inlineStr">
         <is>
-          <t>스팩 소멸합병</t>
+          <t>신규상장</t>
         </is>
       </c>
       <c r="E131" s="6" t="inlineStr">
         <is>
-          <t>FY24</t>
+          <t>FY25</t>
         </is>
       </c>
       <c r="F131" s="7" t="inlineStr">
         <is>
-          <t>39,991</t>
+          <t>4,896</t>
         </is>
       </c>
       <c r="G131" s="7" t="inlineStr">
         <is>
-          <t>3,541</t>
+          <t>-16,214</t>
         </is>
       </c>
       <c r="H131" s="7" t="inlineStr">
         <is>
-          <t>503</t>
+          <t>9,146</t>
         </is>
       </c>
       <c r="I131" s="6" t="inlineStr">
         <is>
-          <t>기타 기초 유기 화학물질 제조업</t>
+          <t>소프트웨어 개발 및 공급업</t>
         </is>
       </c>
       <c r="J131" s="6" t="inlineStr">
         <is>
-          <t>교보</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K131" s="6" t="inlineStr">
@@ -7487,12 +7487,12 @@
     <row r="132">
       <c r="A132" s="6" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B132" s="6" t="inlineStr">
         <is>
-          <t>모비어스</t>
+          <t>씨엠디엘</t>
         </is>
       </c>
       <c r="C132" s="6" t="inlineStr">
@@ -7502,37 +7502,37 @@
       </c>
       <c r="D132" s="6" t="inlineStr">
         <is>
-          <t>신규상장</t>
+          <t>스팩 소멸합병</t>
         </is>
       </c>
       <c r="E132" s="6" t="inlineStr">
         <is>
-          <t>FY25</t>
+          <t>FY24</t>
         </is>
       </c>
       <c r="F132" s="7" t="inlineStr">
         <is>
-          <t>31,989</t>
+          <t>39,991</t>
         </is>
       </c>
       <c r="G132" s="7" t="inlineStr">
         <is>
-          <t>-45,307</t>
+          <t>3,541</t>
         </is>
       </c>
       <c r="H132" s="7" t="inlineStr">
         <is>
-          <t>-96,707</t>
+          <t>503</t>
         </is>
       </c>
       <c r="I132" s="6" t="inlineStr">
         <is>
-          <t>컴퓨터 프로그래밍, 시스템 통합 및 관리업</t>
+          <t>기타 기초 유기 화학물질 제조업</t>
         </is>
       </c>
       <c r="J132" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>교보</t>
         </is>
       </c>
       <c r="K132" s="6" t="inlineStr">
@@ -7544,12 +7544,12 @@
     <row r="133">
       <c r="A133" s="6" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B133" s="6" t="inlineStr">
         <is>
-          <t>넥스트젠바이오</t>
+          <t>모비어스</t>
         </is>
       </c>
       <c r="C133" s="6" t="inlineStr">
@@ -7564,32 +7564,32 @@
       </c>
       <c r="E133" s="6" t="inlineStr">
         <is>
-          <t>FY24</t>
+          <t>FY25</t>
         </is>
       </c>
       <c r="F133" s="7" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>31,989</t>
         </is>
       </c>
       <c r="G133" s="7" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>-45,307</t>
         </is>
       </c>
       <c r="H133" s="7" t="inlineStr">
         <is>
-          <t>4,792</t>
+          <t>-96,707</t>
         </is>
       </c>
       <c r="I133" s="6" t="inlineStr">
         <is>
-          <t>자연과학 및 공학 연구개발업</t>
+          <t>컴퓨터 프로그래밍, 시스템 통합 및 관리업</t>
         </is>
       </c>
       <c r="J133" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K133" s="6" t="inlineStr">
@@ -7601,12 +7601,12 @@
     <row r="134">
       <c r="A134" s="6" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B134" s="6" t="inlineStr">
         <is>
-          <t>파워큐브세미</t>
+          <t>넥스트젠바이오</t>
         </is>
       </c>
       <c r="C134" s="6" t="inlineStr">
@@ -7621,32 +7621,32 @@
       </c>
       <c r="E134" s="6" t="inlineStr">
         <is>
-          <t>FY25</t>
+          <t>FY24</t>
         </is>
       </c>
       <c r="F134" s="7" t="inlineStr">
         <is>
-          <t>10,341</t>
+          <t>100</t>
         </is>
       </c>
       <c r="G134" s="7" t="inlineStr">
         <is>
-          <t>-10,837</t>
+          <t>69</t>
         </is>
       </c>
       <c r="H134" s="7" t="inlineStr">
         <is>
-          <t>841</t>
+          <t>4,792</t>
         </is>
       </c>
       <c r="I134" s="6" t="inlineStr">
         <is>
-          <t>반도체 제조업</t>
+          <t>자연과학 및 공학 연구개발업</t>
         </is>
       </c>
       <c r="J134" s="6" t="inlineStr">
         <is>
-          <t>하나, BNK</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="K134" s="6" t="inlineStr">
@@ -7658,12 +7658,12 @@
     <row r="135">
       <c r="A135" s="6" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B135" s="6" t="inlineStr">
         <is>
-          <t>제이피이노베이션</t>
+          <t>파워큐브세미</t>
         </is>
       </c>
       <c r="C135" s="6" t="inlineStr">
@@ -7683,27 +7683,27 @@
       </c>
       <c r="F135" s="7" t="inlineStr">
         <is>
-          <t>56,324</t>
+          <t>10,341</t>
         </is>
       </c>
       <c r="G135" s="7" t="inlineStr">
         <is>
-          <t>5,588</t>
+          <t>-10,837</t>
         </is>
       </c>
       <c r="H135" s="7" t="inlineStr">
         <is>
-          <t>3,684</t>
+          <t>841</t>
         </is>
       </c>
       <c r="I135" s="6" t="inlineStr">
         <is>
-          <t>특수 목적용 기계 제조업</t>
+          <t>반도체 제조업</t>
         </is>
       </c>
       <c r="J135" s="6" t="inlineStr">
         <is>
-          <t>삼성</t>
+          <t>하나, BNK</t>
         </is>
       </c>
       <c r="K135" s="6" t="inlineStr">
@@ -7715,12 +7715,12 @@
     <row r="136">
       <c r="A136" s="6" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B136" s="6" t="inlineStr">
         <is>
-          <t>케이솔루션</t>
+          <t>제이피이노베이션</t>
         </is>
       </c>
       <c r="C136" s="6" t="inlineStr">
@@ -7730,7 +7730,7 @@
       </c>
       <c r="D136" s="6" t="inlineStr">
         <is>
-          <t>스팩 존속합병</t>
+          <t>신규상장</t>
         </is>
       </c>
       <c r="E136" s="6" t="inlineStr">
@@ -7740,27 +7740,27 @@
       </c>
       <c r="F136" s="7" t="inlineStr">
         <is>
-          <t>34,565</t>
+          <t>56,324</t>
         </is>
       </c>
       <c r="G136" s="7" t="inlineStr">
         <is>
-          <t>1,158</t>
+          <t>5,588</t>
         </is>
       </c>
       <c r="H136" s="7" t="inlineStr">
         <is>
-          <t>653</t>
+          <t>3,684</t>
         </is>
       </c>
       <c r="I136" s="6" t="inlineStr">
         <is>
-          <t>차체 및 특장차 제조업</t>
+          <t>특수 목적용 기계 제조업</t>
         </is>
       </c>
       <c r="J136" s="6" t="inlineStr">
         <is>
-          <t>DB</t>
+          <t>삼성</t>
         </is>
       </c>
       <c r="K136" s="6" t="inlineStr">
@@ -7772,12 +7772,12 @@
     <row r="137">
       <c r="A137" s="6" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B137" s="6" t="inlineStr">
         <is>
-          <t>디토닉</t>
+          <t>케이솔루션</t>
         </is>
       </c>
       <c r="C137" s="6" t="inlineStr">
@@ -7787,37 +7787,37 @@
       </c>
       <c r="D137" s="6" t="inlineStr">
         <is>
-          <t>신규상장</t>
+          <t>스팩 존속합병</t>
         </is>
       </c>
       <c r="E137" s="6" t="inlineStr">
         <is>
-          <t>FY24</t>
+          <t>FY25</t>
         </is>
       </c>
       <c r="F137" s="7" t="inlineStr">
         <is>
-          <t>31,293</t>
+          <t>34,565</t>
         </is>
       </c>
       <c r="G137" s="7" t="inlineStr">
         <is>
-          <t>-1,633</t>
+          <t>1,158</t>
         </is>
       </c>
       <c r="H137" s="7" t="inlineStr">
         <is>
-          <t>-21,926</t>
+          <t>653</t>
         </is>
       </c>
       <c r="I137" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어 개발 및 공급업</t>
+          <t>차체 및 특장차 제조업</t>
         </is>
       </c>
       <c r="J137" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>DB</t>
         </is>
       </c>
       <c r="K137" s="6" t="inlineStr">
@@ -7829,12 +7829,12 @@
     <row r="138">
       <c r="A138" s="6" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="B138" s="6" t="inlineStr">
         <is>
-          <t>에스케이팩</t>
+          <t>디토닉</t>
         </is>
       </c>
       <c r="C138" s="6" t="inlineStr">
@@ -7844,7 +7844,7 @@
       </c>
       <c r="D138" s="6" t="inlineStr">
         <is>
-          <t>스팩 소멸합병</t>
+          <t>신규상장</t>
         </is>
       </c>
       <c r="E138" s="6" t="inlineStr">
@@ -7854,27 +7854,27 @@
       </c>
       <c r="F138" s="7" t="inlineStr">
         <is>
-          <t>27,310</t>
+          <t>31,293</t>
         </is>
       </c>
       <c r="G138" s="7" t="inlineStr">
         <is>
-          <t>2,257</t>
+          <t>-1,633</t>
         </is>
       </c>
       <c r="H138" s="7" t="inlineStr">
         <is>
-          <t>3,207</t>
+          <t>-21,926</t>
         </is>
       </c>
       <c r="I138" s="6" t="inlineStr">
         <is>
-          <t>용기 세척, 포장 및 충전기 제조업</t>
+          <t>소프트웨어 개발 및 공급업</t>
         </is>
       </c>
       <c r="J138" s="6" t="inlineStr">
         <is>
-          <t>교보</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K138" s="6" t="inlineStr">
@@ -7886,12 +7886,12 @@
     <row r="139">
       <c r="A139" s="6" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="B139" s="6" t="inlineStr">
         <is>
-          <t>메타넷엑스</t>
+          <t>에스케이팩</t>
         </is>
       </c>
       <c r="C139" s="6" t="inlineStr">
@@ -7901,7 +7901,7 @@
       </c>
       <c r="D139" s="6" t="inlineStr">
         <is>
-          <t>신규상장</t>
+          <t>스팩 소멸합병</t>
         </is>
       </c>
       <c r="E139" s="6" t="inlineStr">
@@ -7911,27 +7911,27 @@
       </c>
       <c r="F139" s="7" t="inlineStr">
         <is>
-          <t>244,130</t>
+          <t>27,310</t>
         </is>
       </c>
       <c r="G139" s="7" t="inlineStr">
         <is>
-          <t>13,455</t>
+          <t>2,257</t>
         </is>
       </c>
       <c r="H139" s="7" t="inlineStr">
         <is>
-          <t>9,995</t>
+          <t>3,207</t>
         </is>
       </c>
       <c r="I139" s="6" t="inlineStr">
         <is>
-          <t>컴퓨터 프로그래밍, 시스템 통합 및 관리업</t>
+          <t>용기 세척, 포장 및 충전기 제조업</t>
         </is>
       </c>
       <c r="J139" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>교보</t>
         </is>
       </c>
       <c r="K139" s="6" t="inlineStr">
@@ -7943,12 +7943,12 @@
     <row r="140">
       <c r="A140" s="6" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="B140" s="6" t="inlineStr">
         <is>
-          <t>무아스</t>
+          <t>메타넷엑스</t>
         </is>
       </c>
       <c r="C140" s="6" t="inlineStr">
@@ -7958,7 +7958,7 @@
       </c>
       <c r="D140" s="6" t="inlineStr">
         <is>
-          <t>스팩 소멸합병</t>
+          <t>신규상장</t>
         </is>
       </c>
       <c r="E140" s="6" t="inlineStr">
@@ -7968,27 +7968,27 @@
       </c>
       <c r="F140" s="7" t="inlineStr">
         <is>
-          <t>41,813</t>
+          <t>244,130</t>
         </is>
       </c>
       <c r="G140" s="7" t="inlineStr">
         <is>
-          <t>3,903</t>
+          <t>13,455</t>
         </is>
       </c>
       <c r="H140" s="7" t="inlineStr">
         <is>
-          <t>532</t>
+          <t>9,995</t>
         </is>
       </c>
       <c r="I140" s="6" t="inlineStr">
         <is>
-          <t>가정용 전기기기 제조업</t>
+          <t>컴퓨터 프로그래밍, 시스템 통합 및 관리업</t>
         </is>
       </c>
       <c r="J140" s="6" t="inlineStr">
         <is>
-          <t>신한</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K140" s="6" t="inlineStr">
@@ -8005,7 +8005,7 @@
       </c>
       <c r="B141" s="6" t="inlineStr">
         <is>
-          <t>유빅스테라퓨틱스</t>
+          <t>무아스</t>
         </is>
       </c>
       <c r="C141" s="6" t="inlineStr">
@@ -8015,7 +8015,7 @@
       </c>
       <c r="D141" s="6" t="inlineStr">
         <is>
-          <t>신규상장</t>
+          <t>스팩 소멸합병</t>
         </is>
       </c>
       <c r="E141" s="6" t="inlineStr">
@@ -8025,27 +8025,27 @@
       </c>
       <c r="F141" s="7" t="inlineStr">
         <is>
-          <t>1,071</t>
+          <t>41,813</t>
         </is>
       </c>
       <c r="G141" s="7" t="inlineStr">
         <is>
-          <t>-15,145</t>
+          <t>3,903</t>
         </is>
       </c>
       <c r="H141" s="7" t="inlineStr">
         <is>
-          <t>5,489</t>
+          <t>532</t>
         </is>
       </c>
       <c r="I141" s="6" t="inlineStr">
         <is>
-          <t>자연과학 및 공학 연구개발업</t>
+          <t>가정용 전기기기 제조업</t>
         </is>
       </c>
       <c r="J141" s="6" t="inlineStr">
         <is>
-          <t>대신</t>
+          <t>신한</t>
         </is>
       </c>
       <c r="K141" s="6" t="inlineStr">
@@ -8057,12 +8057,12 @@
     <row r="142">
       <c r="A142" s="6" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B142" s="6" t="inlineStr">
         <is>
-          <t>코드잇</t>
+          <t>유빅스테라퓨틱스</t>
         </is>
       </c>
       <c r="C142" s="6" t="inlineStr">
@@ -8082,27 +8082,27 @@
       </c>
       <c r="F142" s="7" t="inlineStr">
         <is>
-          <t>30,747</t>
+          <t>1,071</t>
         </is>
       </c>
       <c r="G142" s="7" t="inlineStr">
         <is>
-          <t>6,652</t>
+          <t>-15,145</t>
         </is>
       </c>
       <c r="H142" s="7" t="inlineStr">
         <is>
-          <t>2,403</t>
+          <t>5,489</t>
         </is>
       </c>
       <c r="I142" s="6" t="inlineStr">
         <is>
-          <t>교육지원 서비스업</t>
+          <t>자연과학 및 공학 연구개발업</t>
         </is>
       </c>
       <c r="J142" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>대신</t>
         </is>
       </c>
       <c r="K142" s="6" t="inlineStr">
@@ -8114,12 +8114,12 @@
     <row r="143">
       <c r="A143" s="6" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="B143" s="6" t="inlineStr">
         <is>
-          <t>한컴인스페이스</t>
+          <t>코드잇</t>
         </is>
       </c>
       <c r="C143" s="6" t="inlineStr">
@@ -8139,44 +8139,44 @@
       </c>
       <c r="F143" s="7" t="inlineStr">
         <is>
-          <t>23,492</t>
+          <t>30,747</t>
         </is>
       </c>
       <c r="G143" s="7" t="inlineStr">
         <is>
-          <t>-3,104</t>
+          <t>6,652</t>
         </is>
       </c>
       <c r="H143" s="7" t="inlineStr">
         <is>
-          <t>5,815</t>
+          <t>2,403</t>
         </is>
       </c>
       <c r="I143" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어 개발 및 공급업</t>
+          <t>교육지원 서비스업</t>
         </is>
       </c>
       <c r="J143" s="6" t="inlineStr">
         <is>
-          <t>대신</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K143" s="6" t="inlineStr">
         <is>
-          <t>심사 미승인</t>
+          <t>심사 철회</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="6" t="inlineStr">
         <is>
-          <t>2026-01-28</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B144" s="6" t="inlineStr">
         <is>
-          <t>크몽</t>
+          <t>한컴인스페이스</t>
         </is>
       </c>
       <c r="C144" s="6" t="inlineStr">
@@ -8196,44 +8196,44 @@
       </c>
       <c r="F144" s="7" t="inlineStr">
         <is>
-          <t>48,572</t>
+          <t>23,492</t>
         </is>
       </c>
       <c r="G144" s="7" t="inlineStr">
         <is>
-          <t>3,988</t>
+          <t>-3,104</t>
         </is>
       </c>
       <c r="H144" s="7" t="inlineStr">
         <is>
-          <t>4,930</t>
+          <t>5,815</t>
         </is>
       </c>
       <c r="I144" s="6" t="inlineStr">
         <is>
-          <t>기타 정보 서비스업</t>
+          <t>소프트웨어 개발 및 공급업</t>
         </is>
       </c>
       <c r="J144" s="6" t="inlineStr">
         <is>
-          <t>삼성</t>
+          <t>대신</t>
         </is>
       </c>
       <c r="K144" s="6" t="inlineStr">
         <is>
-          <t>심사 철회</t>
+          <t>심사 미승인</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="6" t="inlineStr">
         <is>
-          <t>2026-01-27</t>
+          <t>2026-01-28</t>
         </is>
       </c>
       <c r="B145" s="6" t="inlineStr">
         <is>
-          <t>한화플러스제6호스팩</t>
+          <t>크몽</t>
         </is>
       </c>
       <c r="C145" s="6" t="inlineStr">
@@ -8253,27 +8253,27 @@
       </c>
       <c r="F145" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>48,572</t>
         </is>
       </c>
       <c r="G145" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>3,988</t>
         </is>
       </c>
       <c r="H145" s="7" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>4,930</t>
         </is>
       </c>
       <c r="I145" s="6" t="inlineStr">
         <is>
-          <t>기타 금융업</t>
+          <t>기타 정보 서비스업</t>
         </is>
       </c>
       <c r="J145" s="6" t="inlineStr">
         <is>
-          <t>한화</t>
+          <t>삼성</t>
         </is>
       </c>
       <c r="K145" s="6" t="inlineStr">
@@ -8285,17 +8285,17 @@
     <row r="146">
       <c r="A146" s="6" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-27</t>
         </is>
       </c>
       <c r="B146" s="6" t="inlineStr">
         <is>
-          <t>에식스솔루션즈</t>
+          <t>한화플러스제6호스팩</t>
         </is>
       </c>
       <c r="C146" s="6" t="inlineStr">
         <is>
-          <t>유가</t>
+          <t>코스닥</t>
         </is>
       </c>
       <c r="D146" s="6" t="inlineStr">
@@ -8310,27 +8310,27 @@
       </c>
       <c r="F146" s="7" t="inlineStr">
         <is>
-          <t>2,461</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G146" s="7" t="inlineStr">
         <is>
-          <t>46</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H146" s="7" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>41</t>
         </is>
       </c>
       <c r="I146" s="6" t="inlineStr">
         <is>
-          <t>절연선 및 케이블 제조업</t>
+          <t>기타 금융업</t>
         </is>
       </c>
       <c r="J146" s="6" t="inlineStr">
         <is>
-          <t>한국, 미래</t>
+          <t>한화</t>
         </is>
       </c>
       <c r="K146" s="6" t="inlineStr">
@@ -8342,55 +8342,112 @@
     <row r="147">
       <c r="A147" s="6" t="inlineStr">
         <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="B147" s="6" t="inlineStr">
+        <is>
+          <t>에식스솔루션즈</t>
+        </is>
+      </c>
+      <c r="C147" s="6" t="inlineStr">
+        <is>
+          <t>유가</t>
+        </is>
+      </c>
+      <c r="D147" s="6" t="inlineStr">
+        <is>
+          <t>신규상장</t>
+        </is>
+      </c>
+      <c r="E147" s="6" t="inlineStr">
+        <is>
+          <t>FY24</t>
+        </is>
+      </c>
+      <c r="F147" s="7" t="inlineStr">
+        <is>
+          <t>2,461</t>
+        </is>
+      </c>
+      <c r="G147" s="7" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
+      <c r="H147" s="7" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I147" s="6" t="inlineStr">
+        <is>
+          <t>절연선 및 케이블 제조업</t>
+        </is>
+      </c>
+      <c r="J147" s="6" t="inlineStr">
+        <is>
+          <t>한국, 미래</t>
+        </is>
+      </c>
+      <c r="K147" s="6" t="inlineStr">
+        <is>
+          <t>심사 철회</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="6" t="inlineStr">
+        <is>
           <t>2026-01-23</t>
         </is>
       </c>
-      <c r="B147" s="6" t="inlineStr">
+      <c r="B148" s="6" t="inlineStr">
         <is>
           <t>에코크레이션</t>
         </is>
       </c>
-      <c r="C147" s="6" t="inlineStr">
+      <c r="C148" s="6" t="inlineStr">
         <is>
           <t>코스닥</t>
         </is>
       </c>
-      <c r="D147" s="6" t="inlineStr">
+      <c r="D148" s="6" t="inlineStr">
         <is>
           <t>신규상장</t>
         </is>
       </c>
-      <c r="E147" s="6" t="inlineStr">
+      <c r="E148" s="6" t="inlineStr">
         <is>
           <t>FY24</t>
         </is>
       </c>
-      <c r="F147" s="7" t="inlineStr">
+      <c r="F148" s="7" t="inlineStr">
         <is>
           <t>18,544</t>
         </is>
       </c>
-      <c r="G147" s="7" t="inlineStr">
+      <c r="G148" s="7" t="inlineStr">
         <is>
           <t>-15,634</t>
         </is>
       </c>
-      <c r="H147" s="7" t="inlineStr">
+      <c r="H148" s="7" t="inlineStr">
         <is>
           <t>4,550</t>
         </is>
       </c>
-      <c r="I147" s="6" t="inlineStr">
+      <c r="I148" s="6" t="inlineStr">
         <is>
           <t>일반 목적용 기계 제조업</t>
         </is>
       </c>
-      <c r="J147" s="6" t="inlineStr">
+      <c r="J148" s="6" t="inlineStr">
         <is>
           <t>키움</t>
         </is>
       </c>
-      <c r="K147" s="6" t="inlineStr">
+      <c r="K148" s="6" t="inlineStr">
         <is>
           <t>심사 철회</t>
         </is>
@@ -8407,7 +8464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R94"/>
+  <dimension ref="A1:R97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -12489,7 +12546,7 @@
     <row r="56" ht="22" customHeight="1">
       <c r="A56" s="3" t="inlineStr">
         <is>
-          <t>■ 공모 진행 (예심 승인법인)  (34건)</t>
+          <t>■ 공모 진행 (예심 승인법인)  (37건)</t>
         </is>
       </c>
       <c r="B56" s="4" t="n"/>
@@ -12730,7 +12787,7 @@
       </c>
       <c r="R59" s="6" t="inlineStr">
         <is>
-          <t>발행조건확정</t>
+          <t>청약완료·상장대기</t>
         </is>
       </c>
     </row>
@@ -13205,32 +13262,32 @@
     <row r="67" ht="30" customHeight="1">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>래블업</t>
+          <t>인텔리빅스</t>
         </is>
       </c>
       <c r="B67" s="6" t="inlineStr">
         <is>
-          <t>10-13~10-19</t>
+          <t>10-12~10-16</t>
         </is>
       </c>
       <c r="C67" s="6" t="inlineStr">
         <is>
-          <t>19,000~22,000</t>
+          <t>7,600~9,000</t>
         </is>
       </c>
       <c r="D67" s="7" t="inlineStr">
         <is>
-          <t>2,180,000</t>
+          <t>2,500,000</t>
         </is>
       </c>
       <c r="E67" s="7" t="inlineStr">
         <is>
-          <t>41,420,000,000</t>
+          <t>19,000,000,000</t>
         </is>
       </c>
       <c r="F67" s="6" t="inlineStr">
         <is>
-          <t>33.6배 (PER)</t>
+          <t>22.02배 (PER)</t>
         </is>
       </c>
       <c r="G67" s="6" t="inlineStr"/>
@@ -13238,7 +13295,7 @@
       <c r="I67" s="6" t="inlineStr"/>
       <c r="J67" s="6" t="inlineStr">
         <is>
-          <t>10-22~10-23</t>
+          <t>10-21~10-22</t>
         </is>
       </c>
       <c r="K67" s="6" t="inlineStr"/>
@@ -13246,18 +13303,18 @@
       <c r="M67" s="6" t="inlineStr"/>
       <c r="N67" s="6" t="inlineStr">
         <is>
-          <t>NH투자증권</t>
+          <t>미래에셋증권</t>
         </is>
       </c>
       <c r="O67" s="6" t="inlineStr"/>
       <c r="P67" s="7" t="inlineStr">
         <is>
-          <t>1,908,899,000</t>
+          <t>782,800,000</t>
         </is>
       </c>
       <c r="Q67" s="6" t="inlineStr">
         <is>
-          <t>4.5%</t>
+          <t>4.0%</t>
         </is>
       </c>
       <c r="R67" s="6" t="inlineStr">
@@ -13269,32 +13326,32 @@
     <row r="68" ht="30" customHeight="1">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>한화플러스제6호스팩</t>
+          <t>래블업</t>
         </is>
       </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t>10-14~10-15</t>
-        </is>
-      </c>
-      <c r="C68" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>10-13~10-19</t>
+        </is>
+      </c>
+      <c r="C68" s="6" t="inlineStr">
+        <is>
+          <t>19,000~22,000</t>
         </is>
       </c>
       <c r="D68" s="7" t="inlineStr">
         <is>
-          <t>6,000,000</t>
+          <t>2,180,000</t>
         </is>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
-          <t>12,000,000,000</t>
-        </is>
-      </c>
-      <c r="F68" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>41,420,000,000</t>
+        </is>
+      </c>
+      <c r="F68" s="6" t="inlineStr">
+        <is>
+          <t>33.6배 (PER)</t>
         </is>
       </c>
       <c r="G68" s="6" t="inlineStr"/>
@@ -13302,26 +13359,26 @@
       <c r="I68" s="6" t="inlineStr"/>
       <c r="J68" s="6" t="inlineStr">
         <is>
-          <t>10-20~10-21</t>
+          <t>10-22~10-23</t>
         </is>
       </c>
       <c r="K68" s="6" t="inlineStr"/>
       <c r="L68" s="6" t="inlineStr"/>
       <c r="M68" s="6" t="inlineStr"/>
-      <c r="N68" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="N68" s="6" t="inlineStr">
+        <is>
+          <t>NH투자증권</t>
         </is>
       </c>
       <c r="O68" s="6" t="inlineStr"/>
-      <c r="P68" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="P68" s="7" t="inlineStr">
+        <is>
+          <t>1,908,899,000</t>
         </is>
       </c>
       <c r="Q68" s="6" t="inlineStr">
         <is>
-          <t>3.50%</t>
+          <t>4.5%</t>
         </is>
       </c>
       <c r="R68" s="6" t="inlineStr">
@@ -13333,32 +13390,32 @@
     <row r="69" ht="30" customHeight="1">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>엠비디</t>
+          <t>한화플러스제6호스팩</t>
         </is>
       </c>
       <c r="B69" s="6" t="inlineStr">
         <is>
-          <t>10-16~10-22</t>
-        </is>
-      </c>
-      <c r="C69" s="6" t="inlineStr">
-        <is>
-          <t>9,600~11,700</t>
+          <t>10-14~10-15</t>
+        </is>
+      </c>
+      <c r="C69" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="D69" s="7" t="inlineStr">
         <is>
-          <t>2,000,000</t>
+          <t>6,000,000</t>
         </is>
       </c>
       <c r="E69" s="7" t="inlineStr">
         <is>
-          <t>19,200,000,000</t>
-        </is>
-      </c>
-      <c r="F69" s="6" t="inlineStr">
-        <is>
-          <t>26.87배 (PER)</t>
+          <t>12,000,000,000</t>
+        </is>
+      </c>
+      <c r="F69" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="G69" s="6" t="inlineStr"/>
@@ -13366,26 +13423,26 @@
       <c r="I69" s="6" t="inlineStr"/>
       <c r="J69" s="6" t="inlineStr">
         <is>
-          <t>10-28~10-29</t>
+          <t>10-20~10-21</t>
         </is>
       </c>
       <c r="K69" s="6" t="inlineStr"/>
       <c r="L69" s="6" t="inlineStr"/>
       <c r="M69" s="6" t="inlineStr"/>
-      <c r="N69" s="6" t="inlineStr">
-        <is>
-          <t>하나증권</t>
+      <c r="N69" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="O69" s="6" t="inlineStr"/>
-      <c r="P69" s="7" t="inlineStr">
-        <is>
-          <t>988,800,000</t>
+      <c r="P69" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="Q69" s="6" t="inlineStr">
         <is>
-          <t>5.0%</t>
+          <t>3.50%</t>
         </is>
       </c>
       <c r="R69" s="6" t="inlineStr">
@@ -13397,59 +13454,59 @@
     <row r="70" ht="30" customHeight="1">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>바로팜</t>
-        </is>
-      </c>
-      <c r="B70" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>엠비디</t>
+        </is>
+      </c>
+      <c r="B70" s="6" t="inlineStr">
+        <is>
+          <t>10-16~10-22</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr">
         <is>
-          <t>16,400~20,200</t>
+          <t>9,600~11,700</t>
         </is>
       </c>
       <c r="D70" s="7" t="inlineStr">
         <is>
-          <t>1,780,000</t>
+          <t>2,000,000</t>
         </is>
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
-          <t>29,192,000,000</t>
+          <t>19,200,000,000</t>
         </is>
       </c>
       <c r="F70" s="6" t="inlineStr">
         <is>
-          <t>24.95배 (PER)</t>
+          <t>26.87배 (PER)</t>
         </is>
       </c>
       <c r="G70" s="6" t="inlineStr"/>
       <c r="H70" s="6" t="inlineStr"/>
       <c r="I70" s="6" t="inlineStr"/>
-      <c r="J70" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="J70" s="6" t="inlineStr">
+        <is>
+          <t>10-28~10-29</t>
         </is>
       </c>
       <c r="K70" s="6" t="inlineStr"/>
       <c r="L70" s="6" t="inlineStr"/>
       <c r="M70" s="6" t="inlineStr"/>
-      <c r="N70" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="N70" s="6" t="inlineStr">
+        <is>
+          <t>하나증권</t>
         </is>
       </c>
       <c r="O70" s="6" t="inlineStr"/>
-      <c r="P70" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="Q70" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="P70" s="7" t="inlineStr">
+        <is>
+          <t>988,800,000</t>
+        </is>
+      </c>
+      <c r="Q70" s="6" t="inlineStr">
+        <is>
+          <t>5.0%</t>
         </is>
       </c>
       <c r="R70" s="6" t="inlineStr">
@@ -13461,7 +13518,7 @@
     <row r="71" ht="30" customHeight="1">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>셀트릭스</t>
+          <t>바로팜</t>
         </is>
       </c>
       <c r="B71" s="18" t="inlineStr">
@@ -13469,24 +13526,24 @@
           <t>수집예정</t>
         </is>
       </c>
-      <c r="C71" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="D71" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="E71" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="F71" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="C71" s="6" t="inlineStr">
+        <is>
+          <t>16,400~20,200</t>
+        </is>
+      </c>
+      <c r="D71" s="7" t="inlineStr">
+        <is>
+          <t>1,780,000</t>
+        </is>
+      </c>
+      <c r="E71" s="7" t="inlineStr">
+        <is>
+          <t>29,192,000,000</t>
+        </is>
+      </c>
+      <c r="F71" s="6" t="inlineStr">
+        <is>
+          <t>24.95배 (PER)</t>
         </is>
       </c>
       <c r="G71" s="6" t="inlineStr"/>
@@ -13525,7 +13582,7 @@
     <row r="72" ht="30" customHeight="1">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>솔리스</t>
+          <t>셀트릭스</t>
         </is>
       </c>
       <c r="B72" s="18" t="inlineStr">
@@ -13589,64 +13646,64 @@
     <row r="73" ht="30" customHeight="1">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>인텔리빅스</t>
-        </is>
-      </c>
-      <c r="B73" s="6" t="inlineStr">
-        <is>
-          <t>10-12~10-16</t>
-        </is>
-      </c>
-      <c r="C73" s="6" t="inlineStr">
-        <is>
-          <t>7,600~9,000</t>
-        </is>
-      </c>
-      <c r="D73" s="7" t="inlineStr">
-        <is>
-          <t>2,500,000</t>
-        </is>
-      </c>
-      <c r="E73" s="7" t="inlineStr">
-        <is>
-          <t>19,000,000,000</t>
-        </is>
-      </c>
-      <c r="F73" s="6" t="inlineStr">
-        <is>
-          <t>22.02배 (PER)</t>
+          <t>솔리스</t>
+        </is>
+      </c>
+      <c r="B73" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="C73" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="D73" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="E73" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="F73" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="G73" s="6" t="inlineStr"/>
       <c r="H73" s="6" t="inlineStr"/>
       <c r="I73" s="6" t="inlineStr"/>
-      <c r="J73" s="6" t="inlineStr">
-        <is>
-          <t>10-21~10-22</t>
+      <c r="J73" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="K73" s="6" t="inlineStr"/>
       <c r="L73" s="6" t="inlineStr"/>
       <c r="M73" s="6" t="inlineStr"/>
-      <c r="N73" s="6" t="inlineStr">
-        <is>
-          <t>미래에셋증권</t>
+      <c r="N73" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="O73" s="6" t="inlineStr"/>
-      <c r="P73" s="7" t="inlineStr">
-        <is>
-          <t>782,800,000</t>
-        </is>
-      </c>
-      <c r="Q73" s="6" t="inlineStr">
-        <is>
-          <t>4.0%</t>
+      <c r="P73" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="Q73" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="R73" s="6" t="inlineStr">
         <is>
-          <t>최초</t>
+          <t>정정</t>
         </is>
       </c>
     </row>
@@ -14229,7 +14286,7 @@
     <row r="83" ht="30" customHeight="1">
       <c r="A83" s="6" t="inlineStr">
         <is>
-          <t>럭스코</t>
+          <t>영광와이케이엠씨</t>
         </is>
       </c>
       <c r="B83" s="18" t="inlineStr">
@@ -14293,7 +14350,7 @@
     <row r="84" ht="30" customHeight="1">
       <c r="A84" s="6" t="inlineStr">
         <is>
-          <t>디티에스</t>
+          <t>럭스코</t>
         </is>
       </c>
       <c r="B84" s="18" t="inlineStr">
@@ -14350,14 +14407,14 @@
       </c>
       <c r="R84" s="6" t="inlineStr">
         <is>
-          <t>신고서 대기</t>
+          <t>최초</t>
         </is>
       </c>
     </row>
     <row r="85" ht="30" customHeight="1">
       <c r="A85" s="6" t="inlineStr">
         <is>
-          <t>에이엔에이치스트럭쳐</t>
+          <t>엔키화이트햇</t>
         </is>
       </c>
       <c r="B85" s="18" t="inlineStr">
@@ -14414,14 +14471,14 @@
       </c>
       <c r="R85" s="6" t="inlineStr">
         <is>
-          <t>신고서 대기</t>
+          <t>최초</t>
         </is>
       </c>
     </row>
     <row r="86" ht="30" customHeight="1">
       <c r="A86" s="6" t="inlineStr">
         <is>
-          <t>이에스티</t>
+          <t>아델</t>
         </is>
       </c>
       <c r="B86" s="18" t="inlineStr">
@@ -14478,14 +14535,14 @@
       </c>
       <c r="R86" s="6" t="inlineStr">
         <is>
-          <t>신고서 대기</t>
+          <t>corp_code 미확보(수동확인)</t>
         </is>
       </c>
     </row>
     <row r="87" ht="30" customHeight="1">
       <c r="A87" s="6" t="inlineStr">
         <is>
-          <t>영광와이케이엠씨</t>
+          <t>케이티이</t>
         </is>
       </c>
       <c r="B87" s="18" t="inlineStr">
@@ -14542,14 +14599,14 @@
       </c>
       <c r="R87" s="6" t="inlineStr">
         <is>
-          <t>신고서 대기</t>
+          <t>corp_code 미확보(수동확인)</t>
         </is>
       </c>
     </row>
     <row r="88" ht="30" customHeight="1">
       <c r="A88" s="6" t="inlineStr">
         <is>
-          <t>우리투자제1호스팩</t>
+          <t>씨앤엠</t>
         </is>
       </c>
       <c r="B88" s="18" t="inlineStr">
@@ -14606,14 +14663,14 @@
       </c>
       <c r="R88" s="6" t="inlineStr">
         <is>
-          <t>신고서 대기</t>
+          <t>corp_code 미확보(수동확인)</t>
         </is>
       </c>
     </row>
     <row r="89" ht="30" customHeight="1">
       <c r="A89" s="6" t="inlineStr">
         <is>
-          <t>엔키화이트햇</t>
+          <t>디티에스</t>
         </is>
       </c>
       <c r="B89" s="18" t="inlineStr">
@@ -14677,7 +14734,7 @@
     <row r="90" ht="30" customHeight="1">
       <c r="A90" s="6" t="inlineStr">
         <is>
-          <t>마더스제약</t>
+          <t>에이엔에이치스트럭쳐</t>
         </is>
       </c>
       <c r="B90" s="18" t="inlineStr">
@@ -14738,22 +14795,214 @@
         </is>
       </c>
     </row>
-    <row r="92">
-      <c r="A92" s="20" t="inlineStr">
+    <row r="91" ht="30" customHeight="1">
+      <c r="A91" s="6" t="inlineStr">
+        <is>
+          <t>이에스티</t>
+        </is>
+      </c>
+      <c r="B91" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="C91" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="D91" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="E91" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="F91" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="G91" s="6" t="inlineStr"/>
+      <c r="H91" s="6" t="inlineStr"/>
+      <c r="I91" s="6" t="inlineStr"/>
+      <c r="J91" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="K91" s="6" t="inlineStr"/>
+      <c r="L91" s="6" t="inlineStr"/>
+      <c r="M91" s="6" t="inlineStr"/>
+      <c r="N91" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="O91" s="6" t="inlineStr"/>
+      <c r="P91" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="Q91" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="R91" s="6" t="inlineStr">
+        <is>
+          <t>신고서 대기</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="30" customHeight="1">
+      <c r="A92" s="6" t="inlineStr">
+        <is>
+          <t>우리투자제1호스팩</t>
+        </is>
+      </c>
+      <c r="B92" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="C92" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="D92" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="E92" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="F92" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="G92" s="6" t="inlineStr"/>
+      <c r="H92" s="6" t="inlineStr"/>
+      <c r="I92" s="6" t="inlineStr"/>
+      <c r="J92" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="K92" s="6" t="inlineStr"/>
+      <c r="L92" s="6" t="inlineStr"/>
+      <c r="M92" s="6" t="inlineStr"/>
+      <c r="N92" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="O92" s="6" t="inlineStr"/>
+      <c r="P92" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="Q92" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="R92" s="6" t="inlineStr">
+        <is>
+          <t>신고서 대기</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="30" customHeight="1">
+      <c r="A93" s="6" t="inlineStr">
+        <is>
+          <t>마더스제약</t>
+        </is>
+      </c>
+      <c r="B93" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="C93" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="D93" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="E93" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="F93" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="G93" s="6" t="inlineStr"/>
+      <c r="H93" s="6" t="inlineStr"/>
+      <c r="I93" s="6" t="inlineStr"/>
+      <c r="J93" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="K93" s="6" t="inlineStr"/>
+      <c r="L93" s="6" t="inlineStr"/>
+      <c r="M93" s="6" t="inlineStr"/>
+      <c r="N93" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="O93" s="6" t="inlineStr"/>
+      <c r="P93" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="Q93" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="R93" s="6" t="inlineStr">
+        <is>
+          <t>신고서 대기</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="20" t="inlineStr">
         <is>
           <t>※ 상장 완료 = KIND 신규상장 페이지 기준(스팩합병 포함) · 스팩 공모상장은 밴드·밸류에이션 등 해당없음(공모가 2,000원 고정).</t>
         </is>
       </c>
     </row>
-    <row r="93">
-      <c r="A93" s="20" t="inlineStr">
+    <row r="96">
+      <c r="A96" s="20" t="inlineStr">
         <is>
           <t>※ 기재정정 신고서 내 정정 전·후 병존 → 자동수집은 "정정 후" 값만 취함.</t>
         </is>
       </c>
     </row>
-    <row r="94">
-      <c r="A94" s="20" t="inlineStr">
+    <row r="97">
+      <c r="A97" s="20" t="inlineStr">
         <is>
           <t>※ 청약경쟁률=일반투자자 청약수량÷최종배정수량 · "MM-DD~"는 종료일 자동수집 예정.</t>
         </is>
@@ -15053,13 +15302,13 @@
         </is>
       </c>
       <c r="B15" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C15" s="6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D15" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E15" s="6" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
chore: update IPO data 2026-10-11
</commit_message>
<xml_diff>
--- a/IPO_analysis.xlsx
+++ b/IPO_analysis.xlsx
@@ -618,7 +618,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>기준일 2026-10-10 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
+          <t>기준일 2026-10-11 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
         </is>
       </c>
     </row>
@@ -13070,32 +13070,32 @@
     <row r="64" ht="30" customHeight="1">
       <c r="A64" s="6" t="inlineStr">
         <is>
-          <t>다비오</t>
+          <t>에스케이증권제14호기업인수목적</t>
         </is>
       </c>
       <c r="B64" s="6" t="inlineStr">
         <is>
-          <t>10-07~10-14</t>
-        </is>
-      </c>
-      <c r="C64" s="6" t="inlineStr">
-        <is>
-          <t>12,300~16,600</t>
+          <t>10-12~10-13</t>
+        </is>
+      </c>
+      <c r="C64" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="D64" s="7" t="inlineStr">
         <is>
-          <t>1,000,000</t>
+          <t>6,500,000</t>
         </is>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
-          <t>12,300,000,000</t>
-        </is>
-      </c>
-      <c r="F64" s="6" t="inlineStr">
-        <is>
-          <t>26.70배 (PER)</t>
+          <t>13,000,000,000</t>
+        </is>
+      </c>
+      <c r="F64" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="G64" s="6" t="inlineStr"/>
@@ -13103,26 +13103,26 @@
       <c r="I64" s="6" t="inlineStr"/>
       <c r="J64" s="6" t="inlineStr">
         <is>
-          <t>10-19~10-20</t>
+          <t>10-15~10-16</t>
         </is>
       </c>
       <c r="K64" s="6" t="inlineStr"/>
       <c r="L64" s="6" t="inlineStr"/>
       <c r="M64" s="6" t="inlineStr"/>
-      <c r="N64" s="6" t="inlineStr">
-        <is>
-          <t>대신증권</t>
+      <c r="N64" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="O64" s="6" t="inlineStr"/>
-      <c r="P64" s="7" t="inlineStr">
-        <is>
-          <t>570,105,000</t>
+      <c r="P64" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="Q64" s="6" t="inlineStr">
         <is>
-          <t>4.5%</t>
+          <t>50%</t>
         </is>
       </c>
       <c r="R64" s="6" t="inlineStr">
@@ -13134,32 +13134,32 @@
     <row r="65" ht="30" customHeight="1">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>에스케이증권제14호기업인수목적</t>
+          <t>크리에이츠</t>
         </is>
       </c>
       <c r="B65" s="6" t="inlineStr">
         <is>
-          <t>10-12~10-13</t>
-        </is>
-      </c>
-      <c r="C65" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>10-12~10-16</t>
+        </is>
+      </c>
+      <c r="C65" s="6" t="inlineStr">
+        <is>
+          <t>15,000~18,000</t>
         </is>
       </c>
       <c r="D65" s="7" t="inlineStr">
         <is>
-          <t>6,500,000</t>
+          <t>1,400,000</t>
         </is>
       </c>
       <c r="E65" s="7" t="inlineStr">
         <is>
-          <t>13,000,000,000</t>
-        </is>
-      </c>
-      <c r="F65" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>21,000,000,000</t>
+        </is>
+      </c>
+      <c r="F65" s="6" t="inlineStr">
+        <is>
+          <t>19.15배 (PER)</t>
         </is>
       </c>
       <c r="G65" s="6" t="inlineStr"/>
@@ -13167,26 +13167,26 @@
       <c r="I65" s="6" t="inlineStr"/>
       <c r="J65" s="6" t="inlineStr">
         <is>
-          <t>10-15~10-16</t>
+          <t>10-20~10-21</t>
         </is>
       </c>
       <c r="K65" s="6" t="inlineStr"/>
       <c r="L65" s="6" t="inlineStr"/>
       <c r="M65" s="6" t="inlineStr"/>
-      <c r="N65" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="N65" s="6" t="inlineStr">
+        <is>
+          <t>삼성증권</t>
         </is>
       </c>
       <c r="O65" s="6" t="inlineStr"/>
-      <c r="P65" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="P65" s="7" t="inlineStr">
+        <is>
+          <t>865,200,000</t>
         </is>
       </c>
       <c r="Q65" s="6" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>4.0%</t>
         </is>
       </c>
       <c r="R65" s="6" t="inlineStr">
@@ -13198,7 +13198,7 @@
     <row r="66" ht="30" customHeight="1">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>크리에이츠</t>
+          <t>인텔리빅스</t>
         </is>
       </c>
       <c r="B66" s="6" t="inlineStr">
@@ -13208,22 +13208,22 @@
       </c>
       <c r="C66" s="6" t="inlineStr">
         <is>
-          <t>15,000~18,000</t>
+          <t>7,600~9,000</t>
         </is>
       </c>
       <c r="D66" s="7" t="inlineStr">
         <is>
-          <t>1,400,000</t>
+          <t>2,500,000</t>
         </is>
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
-          <t>21,000,000,000</t>
+          <t>19,000,000,000</t>
         </is>
       </c>
       <c r="F66" s="6" t="inlineStr">
         <is>
-          <t>19.15배 (PER)</t>
+          <t>22.02배 (PER)</t>
         </is>
       </c>
       <c r="G66" s="6" t="inlineStr"/>
@@ -13231,7 +13231,7 @@
       <c r="I66" s="6" t="inlineStr"/>
       <c r="J66" s="6" t="inlineStr">
         <is>
-          <t>10-20~10-21</t>
+          <t>10-21~10-22</t>
         </is>
       </c>
       <c r="K66" s="6" t="inlineStr"/>
@@ -13239,13 +13239,13 @@
       <c r="M66" s="6" t="inlineStr"/>
       <c r="N66" s="6" t="inlineStr">
         <is>
-          <t>삼성증권</t>
+          <t>미래에셋증권</t>
         </is>
       </c>
       <c r="O66" s="6" t="inlineStr"/>
       <c r="P66" s="7" t="inlineStr">
         <is>
-          <t>865,200,000</t>
+          <t>782,800,000</t>
         </is>
       </c>
       <c r="Q66" s="6" t="inlineStr">
@@ -13262,32 +13262,32 @@
     <row r="67" ht="30" customHeight="1">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>인텔리빅스</t>
+          <t>래블업</t>
         </is>
       </c>
       <c r="B67" s="6" t="inlineStr">
         <is>
-          <t>10-12~10-16</t>
+          <t>10-13~10-19</t>
         </is>
       </c>
       <c r="C67" s="6" t="inlineStr">
         <is>
-          <t>7,600~9,000</t>
+          <t>19,000~22,000</t>
         </is>
       </c>
       <c r="D67" s="7" t="inlineStr">
         <is>
-          <t>2,500,000</t>
+          <t>2,180,000</t>
         </is>
       </c>
       <c r="E67" s="7" t="inlineStr">
         <is>
-          <t>19,000,000,000</t>
+          <t>41,420,000,000</t>
         </is>
       </c>
       <c r="F67" s="6" t="inlineStr">
         <is>
-          <t>22.02배 (PER)</t>
+          <t>33.6배 (PER)</t>
         </is>
       </c>
       <c r="G67" s="6" t="inlineStr"/>
@@ -13295,7 +13295,7 @@
       <c r="I67" s="6" t="inlineStr"/>
       <c r="J67" s="6" t="inlineStr">
         <is>
-          <t>10-21~10-22</t>
+          <t>10-22~10-23</t>
         </is>
       </c>
       <c r="K67" s="6" t="inlineStr"/>
@@ -13303,18 +13303,18 @@
       <c r="M67" s="6" t="inlineStr"/>
       <c r="N67" s="6" t="inlineStr">
         <is>
-          <t>미래에셋증권</t>
+          <t>NH투자증권</t>
         </is>
       </c>
       <c r="O67" s="6" t="inlineStr"/>
       <c r="P67" s="7" t="inlineStr">
         <is>
-          <t>782,800,000</t>
+          <t>1,908,899,000</t>
         </is>
       </c>
       <c r="Q67" s="6" t="inlineStr">
         <is>
-          <t>4.0%</t>
+          <t>4.5%</t>
         </is>
       </c>
       <c r="R67" s="6" t="inlineStr">
@@ -13326,7 +13326,7 @@
     <row r="68" ht="30" customHeight="1">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>래블업</t>
+          <t>영광</t>
         </is>
       </c>
       <c r="B68" s="6" t="inlineStr">
@@ -13336,22 +13336,22 @@
       </c>
       <c r="C68" s="6" t="inlineStr">
         <is>
-          <t>19,000~22,000</t>
+          <t>14,000~17,000</t>
         </is>
       </c>
       <c r="D68" s="7" t="inlineStr">
         <is>
-          <t>2,180,000</t>
+          <t>2,260,000</t>
         </is>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
-          <t>41,420,000,000</t>
+          <t>31,640,000,000</t>
         </is>
       </c>
       <c r="F68" s="6" t="inlineStr">
         <is>
-          <t>33.6배 (PER)</t>
+          <t>11.98배 (EV/EBITDA)</t>
         </is>
       </c>
       <c r="G68" s="6" t="inlineStr"/>
@@ -13367,18 +13367,18 @@
       <c r="M68" s="6" t="inlineStr"/>
       <c r="N68" s="6" t="inlineStr">
         <is>
-          <t>NH투자증권</t>
+          <t>한국투자증권</t>
         </is>
       </c>
       <c r="O68" s="6" t="inlineStr"/>
       <c r="P68" s="7" t="inlineStr">
         <is>
-          <t>1,908,899,000</t>
-        </is>
-      </c>
-      <c r="Q68" s="6" t="inlineStr">
-        <is>
-          <t>4.5%</t>
+          <t>977,676,000</t>
+        </is>
+      </c>
+      <c r="Q68" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="R68" s="6" t="inlineStr">
@@ -13390,32 +13390,32 @@
     <row r="69" ht="30" customHeight="1">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>영광</t>
+          <t>한화플러스제6호스팩</t>
         </is>
       </c>
       <c r="B69" s="6" t="inlineStr">
         <is>
-          <t>10-13~10-19</t>
-        </is>
-      </c>
-      <c r="C69" s="6" t="inlineStr">
-        <is>
-          <t>14,000~17,000</t>
+          <t>10-14~10-15</t>
+        </is>
+      </c>
+      <c r="C69" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="D69" s="7" t="inlineStr">
         <is>
-          <t>2,260,000</t>
+          <t>6,000,000</t>
         </is>
       </c>
       <c r="E69" s="7" t="inlineStr">
         <is>
-          <t>31,640,000,000</t>
-        </is>
-      </c>
-      <c r="F69" s="6" t="inlineStr">
-        <is>
-          <t>11.98배 (EV/EBITDA)</t>
+          <t>12,000,000,000</t>
+        </is>
+      </c>
+      <c r="F69" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="G69" s="6" t="inlineStr"/>
@@ -13423,26 +13423,26 @@
       <c r="I69" s="6" t="inlineStr"/>
       <c r="J69" s="6" t="inlineStr">
         <is>
-          <t>10-22~10-23</t>
+          <t>10-20~10-21</t>
         </is>
       </c>
       <c r="K69" s="6" t="inlineStr"/>
       <c r="L69" s="6" t="inlineStr"/>
       <c r="M69" s="6" t="inlineStr"/>
-      <c r="N69" s="6" t="inlineStr">
-        <is>
-          <t>한국투자증권</t>
+      <c r="N69" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="O69" s="6" t="inlineStr"/>
-      <c r="P69" s="7" t="inlineStr">
-        <is>
-          <t>977,676,000</t>
-        </is>
-      </c>
-      <c r="Q69" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="P69" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="Q69" s="6" t="inlineStr">
+        <is>
+          <t>3.50%</t>
         </is>
       </c>
       <c r="R69" s="6" t="inlineStr">
@@ -13454,32 +13454,32 @@
     <row r="70" ht="30" customHeight="1">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>한화플러스제6호스팩</t>
+          <t>엠비디</t>
         </is>
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>10-14~10-15</t>
-        </is>
-      </c>
-      <c r="C70" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>10-16~10-22</t>
+        </is>
+      </c>
+      <c r="C70" s="6" t="inlineStr">
+        <is>
+          <t>9,600~11,700</t>
         </is>
       </c>
       <c r="D70" s="7" t="inlineStr">
         <is>
-          <t>6,000,000</t>
+          <t>2,000,000</t>
         </is>
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
-          <t>12,000,000,000</t>
-        </is>
-      </c>
-      <c r="F70" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>19,200,000,000</t>
+        </is>
+      </c>
+      <c r="F70" s="6" t="inlineStr">
+        <is>
+          <t>26.87배 (PER)</t>
         </is>
       </c>
       <c r="G70" s="6" t="inlineStr"/>
@@ -13487,26 +13487,26 @@
       <c r="I70" s="6" t="inlineStr"/>
       <c r="J70" s="6" t="inlineStr">
         <is>
-          <t>10-20~10-21</t>
+          <t>10-28~10-29</t>
         </is>
       </c>
       <c r="K70" s="6" t="inlineStr"/>
       <c r="L70" s="6" t="inlineStr"/>
       <c r="M70" s="6" t="inlineStr"/>
-      <c r="N70" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="N70" s="6" t="inlineStr">
+        <is>
+          <t>하나증권</t>
         </is>
       </c>
       <c r="O70" s="6" t="inlineStr"/>
-      <c r="P70" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="P70" s="7" t="inlineStr">
+        <is>
+          <t>988,800,000</t>
         </is>
       </c>
       <c r="Q70" s="6" t="inlineStr">
         <is>
-          <t>3.50%</t>
+          <t>5.0%</t>
         </is>
       </c>
       <c r="R70" s="6" t="inlineStr">
@@ -13518,32 +13518,32 @@
     <row r="71" ht="30" customHeight="1">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>엠비디</t>
+          <t>아이엠스팩1호</t>
         </is>
       </c>
       <c r="B71" s="6" t="inlineStr">
         <is>
-          <t>10-16~10-22</t>
-        </is>
-      </c>
-      <c r="C71" s="6" t="inlineStr">
-        <is>
-          <t>9,600~11,700</t>
+          <t>10-19~10-20</t>
+        </is>
+      </c>
+      <c r="C71" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="D71" s="7" t="inlineStr">
         <is>
-          <t>2,000,000</t>
+          <t>5,000,000</t>
         </is>
       </c>
       <c r="E71" s="7" t="inlineStr">
         <is>
-          <t>19,200,000,000</t>
-        </is>
-      </c>
-      <c r="F71" s="6" t="inlineStr">
-        <is>
-          <t>26.87배 (PER)</t>
+          <t>10,000,000,000</t>
+        </is>
+      </c>
+      <c r="F71" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="G71" s="6" t="inlineStr"/>
@@ -13551,26 +13551,26 @@
       <c r="I71" s="6" t="inlineStr"/>
       <c r="J71" s="6" t="inlineStr">
         <is>
-          <t>10-28~10-29</t>
+          <t>10-26~10-27</t>
         </is>
       </c>
       <c r="K71" s="6" t="inlineStr"/>
       <c r="L71" s="6" t="inlineStr"/>
       <c r="M71" s="6" t="inlineStr"/>
-      <c r="N71" s="6" t="inlineStr">
-        <is>
-          <t>하나증권</t>
+      <c r="N71" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="O71" s="6" t="inlineStr"/>
-      <c r="P71" s="7" t="inlineStr">
-        <is>
-          <t>988,800,000</t>
+      <c r="P71" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="Q71" s="6" t="inlineStr">
         <is>
-          <t>5.0%</t>
+          <t>3.00%</t>
         </is>
       </c>
       <c r="R71" s="6" t="inlineStr">
@@ -13582,32 +13582,32 @@
     <row r="72" ht="30" customHeight="1">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>아이엠스팩1호</t>
+          <t>다비오</t>
         </is>
       </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>10-19~10-20</t>
-        </is>
-      </c>
-      <c r="C72" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>11-02~11-06</t>
+        </is>
+      </c>
+      <c r="C72" s="6" t="inlineStr">
+        <is>
+          <t>12,300~16,600</t>
         </is>
       </c>
       <c r="D72" s="7" t="inlineStr">
         <is>
-          <t>5,000,000</t>
+          <t>1,000,000</t>
         </is>
       </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
-          <t>10,000,000,000</t>
-        </is>
-      </c>
-      <c r="F72" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>12,300,000,000</t>
+        </is>
+      </c>
+      <c r="F72" s="6" t="inlineStr">
+        <is>
+          <t>26.70배 (PER)</t>
         </is>
       </c>
       <c r="G72" s="6" t="inlineStr"/>
@@ -13615,26 +13615,26 @@
       <c r="I72" s="6" t="inlineStr"/>
       <c r="J72" s="6" t="inlineStr">
         <is>
-          <t>10-26~10-27</t>
+          <t>11-10~11-11</t>
         </is>
       </c>
       <c r="K72" s="6" t="inlineStr"/>
       <c r="L72" s="6" t="inlineStr"/>
       <c r="M72" s="6" t="inlineStr"/>
-      <c r="N72" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="N72" s="6" t="inlineStr">
+        <is>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="O72" s="6" t="inlineStr"/>
-      <c r="P72" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="P72" s="7" t="inlineStr">
+        <is>
+          <t>570,105,000</t>
         </is>
       </c>
       <c r="Q72" s="6" t="inlineStr">
         <is>
-          <t>3.00%</t>
+          <t>4.5%</t>
         </is>
       </c>
       <c r="R72" s="6" t="inlineStr">
@@ -14158,32 +14158,32 @@
     <row r="81" ht="30" customHeight="1">
       <c r="A81" s="6" t="inlineStr">
         <is>
-          <t>하나에어로다이내믹스</t>
+          <t>영광와이케이엠씨</t>
         </is>
       </c>
       <c r="B81" s="6" t="inlineStr">
         <is>
-          <t>11-02~11-06</t>
+          <t>10-27~11-02</t>
         </is>
       </c>
       <c r="C81" s="6" t="inlineStr">
         <is>
-          <t>4,700~5,700</t>
+          <t>9,400~11,000</t>
         </is>
       </c>
       <c r="D81" s="7" t="inlineStr">
         <is>
-          <t>4,400,000</t>
+          <t>2,300,000</t>
         </is>
       </c>
       <c r="E81" s="7" t="inlineStr">
         <is>
-          <t>20,680,000,000</t>
+          <t>21,620,000,000</t>
         </is>
       </c>
       <c r="F81" s="6" t="inlineStr">
         <is>
-          <t>17.89배 (EV/EBITDA)</t>
+          <t>22.91배 (PER)</t>
         </is>
       </c>
       <c r="G81" s="6" t="inlineStr"/>
@@ -14191,7 +14191,7 @@
       <c r="I81" s="6" t="inlineStr"/>
       <c r="J81" s="6" t="inlineStr">
         <is>
-          <t>11-10~11-11</t>
+          <t>11-04~11-05</t>
         </is>
       </c>
       <c r="K81" s="6" t="inlineStr"/>
@@ -14199,18 +14199,18 @@
       <c r="M81" s="6" t="inlineStr"/>
       <c r="N81" s="6" t="inlineStr">
         <is>
-          <t>아이비케이투자증권</t>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="O81" s="6" t="inlineStr"/>
       <c r="P81" s="7" t="inlineStr">
         <is>
-          <t>850,000,000</t>
-        </is>
-      </c>
-      <c r="Q81" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>1,002,087,000</t>
+        </is>
+      </c>
+      <c r="Q81" s="6" t="inlineStr">
+        <is>
+          <t>0%</t>
         </is>
       </c>
       <c r="R81" s="6" t="inlineStr">
@@ -14222,32 +14222,32 @@
     <row r="82" ht="30" customHeight="1">
       <c r="A82" s="6" t="inlineStr">
         <is>
-          <t>케이엠에프</t>
+          <t>하나에어로다이내믹스</t>
         </is>
       </c>
       <c r="B82" s="6" t="inlineStr">
         <is>
-          <t>11-16~11-20</t>
+          <t>11-02~11-06</t>
         </is>
       </c>
       <c r="C82" s="6" t="inlineStr">
         <is>
-          <t>15,000~17,800</t>
+          <t>4,700~5,700</t>
         </is>
       </c>
       <c r="D82" s="7" t="inlineStr">
         <is>
-          <t>2,000,000</t>
+          <t>4,400,000</t>
         </is>
       </c>
       <c r="E82" s="7" t="inlineStr">
         <is>
-          <t>30,000,000,000</t>
+          <t>20,680,000,000</t>
         </is>
       </c>
       <c r="F82" s="6" t="inlineStr">
         <is>
-          <t>18.53배 (PER)</t>
+          <t>17.89배 (EV/EBITDA)</t>
         </is>
       </c>
       <c r="G82" s="6" t="inlineStr"/>
@@ -14255,7 +14255,7 @@
       <c r="I82" s="6" t="inlineStr"/>
       <c r="J82" s="6" t="inlineStr">
         <is>
-          <t>11-24~11-25</t>
+          <t>11-10~11-11</t>
         </is>
       </c>
       <c r="K82" s="6" t="inlineStr"/>
@@ -14269,12 +14269,12 @@
       <c r="O82" s="6" t="inlineStr"/>
       <c r="P82" s="7" t="inlineStr">
         <is>
-          <t>927,000,000</t>
-        </is>
-      </c>
-      <c r="Q82" s="6" t="inlineStr">
-        <is>
-          <t>3.0%</t>
+          <t>850,000,000</t>
+        </is>
+      </c>
+      <c r="Q82" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="R82" s="6" t="inlineStr">
@@ -14286,59 +14286,59 @@
     <row r="83" ht="30" customHeight="1">
       <c r="A83" s="6" t="inlineStr">
         <is>
-          <t>영광와이케이엠씨</t>
-        </is>
-      </c>
-      <c r="B83" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="C83" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="D83" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="E83" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="F83" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>엔키화이트햇</t>
+        </is>
+      </c>
+      <c r="B83" s="6" t="inlineStr">
+        <is>
+          <t>11-03~11-09</t>
+        </is>
+      </c>
+      <c r="C83" s="6" t="inlineStr">
+        <is>
+          <t>13,000~16,500</t>
+        </is>
+      </c>
+      <c r="D83" s="7" t="inlineStr">
+        <is>
+          <t>1,700,000</t>
+        </is>
+      </c>
+      <c r="E83" s="7" t="inlineStr">
+        <is>
+          <t>22,100,000,000</t>
+        </is>
+      </c>
+      <c r="F83" s="6" t="inlineStr">
+        <is>
+          <t>24.86배 (PER)</t>
         </is>
       </c>
       <c r="G83" s="6" t="inlineStr"/>
       <c r="H83" s="6" t="inlineStr"/>
       <c r="I83" s="6" t="inlineStr"/>
-      <c r="J83" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="J83" s="6" t="inlineStr">
+        <is>
+          <t>11-12~11-13</t>
         </is>
       </c>
       <c r="K83" s="6" t="inlineStr"/>
       <c r="L83" s="6" t="inlineStr"/>
       <c r="M83" s="6" t="inlineStr"/>
-      <c r="N83" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="N83" s="6" t="inlineStr">
+        <is>
+          <t>신영증권</t>
         </is>
       </c>
       <c r="O83" s="6" t="inlineStr"/>
-      <c r="P83" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="Q83" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="P83" s="7" t="inlineStr">
+        <is>
+          <t>1,138,150,000</t>
+        </is>
+      </c>
+      <c r="Q83" s="6" t="inlineStr">
+        <is>
+          <t>5.0%</t>
         </is>
       </c>
       <c r="R83" s="6" t="inlineStr">
@@ -14350,59 +14350,59 @@
     <row r="84" ht="30" customHeight="1">
       <c r="A84" s="6" t="inlineStr">
         <is>
-          <t>럭스코</t>
-        </is>
-      </c>
-      <c r="B84" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="C84" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="D84" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="E84" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="F84" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>케이엠에프</t>
+        </is>
+      </c>
+      <c r="B84" s="6" t="inlineStr">
+        <is>
+          <t>11-16~11-20</t>
+        </is>
+      </c>
+      <c r="C84" s="6" t="inlineStr">
+        <is>
+          <t>15,000~17,800</t>
+        </is>
+      </c>
+      <c r="D84" s="7" t="inlineStr">
+        <is>
+          <t>2,000,000</t>
+        </is>
+      </c>
+      <c r="E84" s="7" t="inlineStr">
+        <is>
+          <t>30,000,000,000</t>
+        </is>
+      </c>
+      <c r="F84" s="6" t="inlineStr">
+        <is>
+          <t>18.53배 (PER)</t>
         </is>
       </c>
       <c r="G84" s="6" t="inlineStr"/>
       <c r="H84" s="6" t="inlineStr"/>
       <c r="I84" s="6" t="inlineStr"/>
-      <c r="J84" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="J84" s="6" t="inlineStr">
+        <is>
+          <t>11-24~11-25</t>
         </is>
       </c>
       <c r="K84" s="6" t="inlineStr"/>
       <c r="L84" s="6" t="inlineStr"/>
       <c r="M84" s="6" t="inlineStr"/>
-      <c r="N84" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="N84" s="6" t="inlineStr">
+        <is>
+          <t>아이비케이투자증권</t>
         </is>
       </c>
       <c r="O84" s="6" t="inlineStr"/>
-      <c r="P84" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="Q84" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="P84" s="7" t="inlineStr">
+        <is>
+          <t>927,000,000</t>
+        </is>
+      </c>
+      <c r="Q84" s="6" t="inlineStr">
+        <is>
+          <t>3.0%</t>
         </is>
       </c>
       <c r="R84" s="6" t="inlineStr">
@@ -14414,7 +14414,7 @@
     <row r="85" ht="30" customHeight="1">
       <c r="A85" s="6" t="inlineStr">
         <is>
-          <t>엔키화이트햇</t>
+          <t>럭스코</t>
         </is>
       </c>
       <c r="B85" s="18" t="inlineStr">
@@ -14478,7 +14478,7 @@
     <row r="86" ht="30" customHeight="1">
       <c r="A86" s="6" t="inlineStr">
         <is>
-          <t>아델</t>
+          <t>디티에스</t>
         </is>
       </c>
       <c r="B86" s="18" t="inlineStr">
@@ -14535,14 +14535,14 @@
       </c>
       <c r="R86" s="6" t="inlineStr">
         <is>
-          <t>corp_code 미확보(수동확인)</t>
+          <t>신고서 대기</t>
         </is>
       </c>
     </row>
     <row r="87" ht="30" customHeight="1">
       <c r="A87" s="6" t="inlineStr">
         <is>
-          <t>케이티이</t>
+          <t>에이엔에이치스트럭쳐</t>
         </is>
       </c>
       <c r="B87" s="18" t="inlineStr">
@@ -14599,14 +14599,14 @@
       </c>
       <c r="R87" s="6" t="inlineStr">
         <is>
-          <t>corp_code 미확보(수동확인)</t>
+          <t>신고서 대기</t>
         </is>
       </c>
     </row>
     <row r="88" ht="30" customHeight="1">
       <c r="A88" s="6" t="inlineStr">
         <is>
-          <t>씨앤엠</t>
+          <t>이에스티</t>
         </is>
       </c>
       <c r="B88" s="18" t="inlineStr">
@@ -14663,14 +14663,14 @@
       </c>
       <c r="R88" s="6" t="inlineStr">
         <is>
-          <t>corp_code 미확보(수동확인)</t>
+          <t>신고서 대기</t>
         </is>
       </c>
     </row>
     <row r="89" ht="30" customHeight="1">
       <c r="A89" s="6" t="inlineStr">
         <is>
-          <t>디티에스</t>
+          <t>우리투자제1호스팩</t>
         </is>
       </c>
       <c r="B89" s="18" t="inlineStr">
@@ -14734,7 +14734,7 @@
     <row r="90" ht="30" customHeight="1">
       <c r="A90" s="6" t="inlineStr">
         <is>
-          <t>에이엔에이치스트럭쳐</t>
+          <t>마더스제약</t>
         </is>
       </c>
       <c r="B90" s="18" t="inlineStr">
@@ -14798,7 +14798,7 @@
     <row r="91" ht="30" customHeight="1">
       <c r="A91" s="6" t="inlineStr">
         <is>
-          <t>이에스티</t>
+          <t>아델</t>
         </is>
       </c>
       <c r="B91" s="18" t="inlineStr">
@@ -14862,7 +14862,7 @@
     <row r="92" ht="30" customHeight="1">
       <c r="A92" s="6" t="inlineStr">
         <is>
-          <t>우리투자제1호스팩</t>
+          <t>케이티이</t>
         </is>
       </c>
       <c r="B92" s="18" t="inlineStr">
@@ -14926,7 +14926,7 @@
     <row r="93" ht="30" customHeight="1">
       <c r="A93" s="6" t="inlineStr">
         <is>
-          <t>마더스제약</t>
+          <t>씨앤엠</t>
         </is>
       </c>
       <c r="B93" s="18" t="inlineStr">
@@ -15019,7 +15019,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F42"/>
+  <dimension ref="A1:F43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -15389,22 +15389,22 @@
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>한국투자증권</t>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="B21" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>256,940,000,000</t>
+          <t>268,350,000,000</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>대신증권</t>
+          <t>한국투자증권</t>
         </is>
       </c>
       <c r="B22" s="6" t="n">
@@ -15412,7 +15412,7 @@
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>246,730,000,000</t>
+          <t>256,940,000,000</t>
         </is>
       </c>
     </row>
@@ -15569,97 +15569,97 @@
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>신영증권</t>
         </is>
       </c>
       <c r="B33" s="6" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>618,288</t>
+          <t>22,100,000,000</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="B34" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>154,600</t>
+          <t>618,288</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="B35" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>130,837</t>
+          <t>154,600</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>신한</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="B36" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>49,052</t>
+          <t>130,837</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>삼성</t>
+          <t>신한</t>
         </is>
       </c>
       <c r="B37" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>32,000</t>
+          <t>49,052</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>유진</t>
+          <t>삼성</t>
         </is>
       </c>
       <c r="B38" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
-          <t>25,020</t>
+          <t>32,000</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>메리츠</t>
+          <t>유진</t>
         </is>
       </c>
       <c r="B39" s="6" t="n">
@@ -15667,14 +15667,14 @@
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>14,000</t>
+          <t>25,020</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>대신</t>
+          <t>메리츠</t>
         </is>
       </c>
       <c r="B40" s="6" t="n">
@@ -15682,14 +15682,14 @@
       </c>
       <c r="C40" s="6" t="inlineStr">
         <is>
-          <t>13,000</t>
+          <t>14,000</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>키움</t>
+          <t>대신</t>
         </is>
       </c>
       <c r="B41" s="6" t="n">
@@ -15697,20 +15697,35 @@
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>12,000</t>
+          <t>13,000</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>교보</t>
+          <t>키움</t>
         </is>
       </c>
       <c r="B42" s="6" t="n">
         <v>1</v>
       </c>
       <c r="C42" s="6" t="inlineStr">
+        <is>
+          <t>12,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="6" t="inlineStr">
+        <is>
+          <t>교보</t>
+        </is>
+      </c>
+      <c r="B43" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C43" s="6" t="inlineStr">
         <is>
           <t>10,800</t>
         </is>

</xml_diff>

<commit_message>
chore: update IPO data 2026-10-12
</commit_message>
<xml_diff>
--- a/IPO_analysis.xlsx
+++ b/IPO_analysis.xlsx
@@ -618,14 +618,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>기준일 2026-10-11 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
+          <t>기준일 2026-10-12 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>■ 심사 신청(진행중)  (41건)</t>
+          <t>■ 심사 신청(진행중)  (39건)</t>
         </is>
       </c>
       <c r="B4" s="4" t="n"/>
@@ -1808,7 +1808,7 @@
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>데스틴파워</t>
+          <t>유림테크</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
@@ -1828,27 +1828,27 @@
       </c>
       <c r="F26" s="7" t="inlineStr">
         <is>
-          <t>29,851</t>
+          <t>102,586</t>
         </is>
       </c>
       <c r="G26" s="7" t="inlineStr">
         <is>
-          <t>5,852</t>
+          <t>-18,278</t>
         </is>
       </c>
       <c r="H26" s="7" t="inlineStr">
         <is>
-          <t>-30,114</t>
+          <t>-4,832</t>
         </is>
       </c>
       <c r="I26" s="6" t="inlineStr">
         <is>
-          <t>전동기, 발전기 및 전기 변환 · 공급 · 제어 장치 제조업</t>
+          <t>자동차 신품 부품 제조업</t>
         </is>
       </c>
       <c r="J26" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>대신</t>
         </is>
       </c>
       <c r="K26" s="6" t="inlineStr">
@@ -1860,12 +1860,12 @@
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>유림테크</t>
+          <t>이노보테라퓨틱스</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
@@ -1885,27 +1885,27 @@
       </c>
       <c r="F27" s="7" t="inlineStr">
         <is>
-          <t>102,586</t>
+          <t>209</t>
         </is>
       </c>
       <c r="G27" s="7" t="inlineStr">
         <is>
-          <t>-18,278</t>
+          <t>-5,429</t>
         </is>
       </c>
       <c r="H27" s="7" t="inlineStr">
         <is>
-          <t>-4,832</t>
+          <t>-53,200</t>
         </is>
       </c>
       <c r="I27" s="6" t="inlineStr">
         <is>
-          <t>자동차 신품 부품 제조업</t>
+          <t>의약품 제조업</t>
         </is>
       </c>
       <c r="J27" s="6" t="inlineStr">
         <is>
-          <t>대신</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="K27" s="6" t="inlineStr">
@@ -1917,17 +1917,17 @@
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>이노보테라퓨틱스</t>
+          <t>에스에프씨</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>코스닥</t>
+          <t>유가</t>
         </is>
       </c>
       <c r="D28" s="6" t="inlineStr">
@@ -1942,27 +1942,27 @@
       </c>
       <c r="F28" s="7" t="inlineStr">
         <is>
-          <t>209</t>
+          <t>160,792</t>
         </is>
       </c>
       <c r="G28" s="7" t="inlineStr">
         <is>
-          <t>-5,429</t>
+          <t>25,509</t>
         </is>
       </c>
       <c r="H28" s="7" t="inlineStr">
         <is>
-          <t>-53,200</t>
+          <t>243,562</t>
         </is>
       </c>
       <c r="I28" s="6" t="inlineStr">
         <is>
-          <t>의약품 제조업</t>
+          <t>기타 화학제품 제조업</t>
         </is>
       </c>
       <c r="J28" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>미래, 한국</t>
         </is>
       </c>
       <c r="K28" s="6" t="inlineStr">
@@ -1974,17 +1974,17 @@
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>에스에프씨</t>
+          <t>에버온</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>유가</t>
+          <t>코스닥</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr">
@@ -1999,27 +1999,27 @@
       </c>
       <c r="F29" s="7" t="inlineStr">
         <is>
-          <t>160,792</t>
+          <t>65,225</t>
         </is>
       </c>
       <c r="G29" s="7" t="inlineStr">
         <is>
-          <t>25,509</t>
+          <t>-3,606</t>
         </is>
       </c>
       <c r="H29" s="7" t="inlineStr">
         <is>
-          <t>243,562</t>
+          <t>54,955</t>
         </is>
       </c>
       <c r="I29" s="6" t="inlineStr">
         <is>
-          <t>기타 화학제품 제조업</t>
+          <t>전기업</t>
         </is>
       </c>
       <c r="J29" s="6" t="inlineStr">
         <is>
-          <t>미래, 한국</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K29" s="6" t="inlineStr">
@@ -2031,12 +2031,12 @@
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>에버온</t>
+          <t>씨아이에스케미칼</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
@@ -2056,27 +2056,27 @@
       </c>
       <c r="F30" s="7" t="inlineStr">
         <is>
-          <t>65,225</t>
+          <t>15,985</t>
         </is>
       </c>
       <c r="G30" s="7" t="inlineStr">
         <is>
-          <t>-3,606</t>
+          <t>-11,440</t>
         </is>
       </c>
       <c r="H30" s="7" t="inlineStr">
         <is>
-          <t>54,955</t>
+          <t>23,706</t>
         </is>
       </c>
       <c r="I30" s="6" t="inlineStr">
         <is>
-          <t>전기업</t>
+          <t>기초 화학물질 제조업</t>
         </is>
       </c>
       <c r="J30" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>KB</t>
         </is>
       </c>
       <c r="K30" s="6" t="inlineStr">
@@ -2088,12 +2088,12 @@
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>씨아이에스케미칼</t>
+          <t>엠디에스코리아</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
@@ -2113,27 +2113,27 @@
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>15,985</t>
+          <t>97,972</t>
         </is>
       </c>
       <c r="G31" s="7" t="inlineStr">
         <is>
-          <t>-11,440</t>
+          <t>6,512</t>
         </is>
       </c>
       <c r="H31" s="7" t="inlineStr">
         <is>
-          <t>23,706</t>
+          <t>53,818</t>
         </is>
       </c>
       <c r="I31" s="6" t="inlineStr">
         <is>
-          <t>기초 화학물질 제조업</t>
+          <t>기타 식품 제조업</t>
         </is>
       </c>
       <c r="J31" s="6" t="inlineStr">
         <is>
-          <t>KB</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K31" s="6" t="inlineStr">
@@ -2145,12 +2145,12 @@
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>엠디에스코리아</t>
+          <t>동승</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr">
@@ -2170,27 +2170,27 @@
       </c>
       <c r="F32" s="7" t="inlineStr">
         <is>
-          <t>97,972</t>
+          <t>78,625</t>
         </is>
       </c>
       <c r="G32" s="7" t="inlineStr">
         <is>
-          <t>6,512</t>
+          <t>14,525</t>
         </is>
       </c>
       <c r="H32" s="7" t="inlineStr">
         <is>
-          <t>53,818</t>
+          <t>5,438</t>
         </is>
       </c>
       <c r="I32" s="6" t="inlineStr">
         <is>
-          <t>기타 식품 제조업</t>
+          <t>부동산 임대 및 공급업</t>
         </is>
       </c>
       <c r="J32" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K32" s="6" t="inlineStr">
@@ -2207,7 +2207,7 @@
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>동승</t>
+          <t>에프엠더블유</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
@@ -2217,7 +2217,7 @@
       </c>
       <c r="D33" s="6" t="inlineStr">
         <is>
-          <t>신규상장</t>
+          <t>스팩 소멸합병</t>
         </is>
       </c>
       <c r="E33" s="6" t="inlineStr">
@@ -2227,27 +2227,27 @@
       </c>
       <c r="F33" s="7" t="inlineStr">
         <is>
-          <t>78,625</t>
+          <t>30,282</t>
         </is>
       </c>
       <c r="G33" s="7" t="inlineStr">
         <is>
-          <t>14,525</t>
+          <t>4,762</t>
         </is>
       </c>
       <c r="H33" s="7" t="inlineStr">
         <is>
-          <t>5,438</t>
+          <t>32</t>
         </is>
       </c>
       <c r="I33" s="6" t="inlineStr">
         <is>
-          <t>부동산 임대 및 공급업</t>
+          <t>기타 식품 제조업</t>
         </is>
       </c>
       <c r="J33" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>유진</t>
         </is>
       </c>
       <c r="K33" s="6" t="inlineStr">
@@ -2259,22 +2259,22 @@
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>에프엠더블유</t>
+          <t>소노인터내셔널</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>코스닥</t>
+          <t>유가</t>
         </is>
       </c>
       <c r="D34" s="6" t="inlineStr">
         <is>
-          <t>스팩 소멸합병</t>
+          <t>신규상장</t>
         </is>
       </c>
       <c r="E34" s="6" t="inlineStr">
@@ -2284,27 +2284,27 @@
       </c>
       <c r="F34" s="7" t="inlineStr">
         <is>
-          <t>30,282</t>
+          <t>2,093,051</t>
         </is>
       </c>
       <c r="G34" s="7" t="inlineStr">
         <is>
-          <t>4,762</t>
+          <t>-148,064</t>
         </is>
       </c>
       <c r="H34" s="7" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>852,372</t>
         </is>
       </c>
       <c r="I34" s="6" t="inlineStr">
         <is>
-          <t>기타 식품 제조업</t>
+          <t>일반 및 생활 숙박시설 운영업</t>
         </is>
       </c>
       <c r="J34" s="6" t="inlineStr">
         <is>
-          <t>유진</t>
+          <t>대신, 미래</t>
         </is>
       </c>
       <c r="K34" s="6" t="inlineStr">
@@ -2316,17 +2316,17 @@
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>소노인터내셔널</t>
+          <t>싸이몬</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>유가</t>
+          <t>코스닥</t>
         </is>
       </c>
       <c r="D35" s="6" t="inlineStr">
@@ -2341,27 +2341,27 @@
       </c>
       <c r="F35" s="7" t="inlineStr">
         <is>
-          <t>2,093,051</t>
+          <t>48,695</t>
         </is>
       </c>
       <c r="G35" s="7" t="inlineStr">
         <is>
-          <t>-148,064</t>
+          <t>15,714</t>
         </is>
       </c>
       <c r="H35" s="7" t="inlineStr">
         <is>
-          <t>852,372</t>
+          <t>61,761</t>
         </is>
       </c>
       <c r="I35" s="6" t="inlineStr">
         <is>
-          <t>일반 및 생활 숙박시설 운영업</t>
+          <t>측정, 시험, 항해, 제어 및 기타 정밀기기 제조업</t>
         </is>
       </c>
       <c r="J35" s="6" t="inlineStr">
         <is>
-          <t>대신, 미래</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K35" s="6" t="inlineStr">
@@ -2373,12 +2373,12 @@
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>싸이몬</t>
+          <t>바이다</t>
         </is>
       </c>
       <c r="C36" s="6" t="inlineStr">
@@ -2398,27 +2398,27 @@
       </c>
       <c r="F36" s="7" t="inlineStr">
         <is>
-          <t>48,695</t>
+          <t>14,432</t>
         </is>
       </c>
       <c r="G36" s="7" t="inlineStr">
         <is>
-          <t>15,714</t>
+          <t>-3,951</t>
         </is>
       </c>
       <c r="H36" s="7" t="inlineStr">
         <is>
-          <t>61,761</t>
+          <t>15,108</t>
         </is>
       </c>
       <c r="I36" s="6" t="inlineStr">
         <is>
-          <t>측정, 시험, 항해, 제어 및 기타 정밀기기 제조업</t>
+          <t>전자부품 제조업</t>
         </is>
       </c>
       <c r="J36" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K36" s="6" t="inlineStr">
@@ -2430,12 +2430,12 @@
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>바이다</t>
+          <t>아이알큐더스</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
@@ -2455,27 +2455,27 @@
       </c>
       <c r="F37" s="7" t="inlineStr">
         <is>
-          <t>14,432</t>
+          <t>10,231</t>
         </is>
       </c>
       <c r="G37" s="7" t="inlineStr">
         <is>
-          <t>-3,951</t>
+          <t>-986</t>
         </is>
       </c>
       <c r="H37" s="7" t="inlineStr">
         <is>
-          <t>15,108</t>
+          <t>1,800</t>
         </is>
       </c>
       <c r="I37" s="6" t="inlineStr">
         <is>
-          <t>전자부품 제조업</t>
+          <t>소프트웨어 개발 및 공급업</t>
         </is>
       </c>
       <c r="J37" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>DB</t>
         </is>
       </c>
       <c r="K37" s="6" t="inlineStr">
@@ -2487,12 +2487,12 @@
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>아이알큐더스</t>
+          <t>씨엔티테크</t>
         </is>
       </c>
       <c r="C38" s="6" t="inlineStr">
@@ -2512,17 +2512,17 @@
       </c>
       <c r="F38" s="7" t="inlineStr">
         <is>
-          <t>10,231</t>
+          <t>27,015</t>
         </is>
       </c>
       <c r="G38" s="7" t="inlineStr">
         <is>
-          <t>-986</t>
+          <t>3,987</t>
         </is>
       </c>
       <c r="H38" s="7" t="inlineStr">
         <is>
-          <t>1,800</t>
+          <t>2,613</t>
         </is>
       </c>
       <c r="I38" s="6" t="inlineStr">
@@ -2532,7 +2532,7 @@
       </c>
       <c r="J38" s="6" t="inlineStr">
         <is>
-          <t>DB</t>
+          <t>한화, 하나</t>
         </is>
       </c>
       <c r="K38" s="6" t="inlineStr">
@@ -2544,12 +2544,12 @@
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>씨엔티테크</t>
+          <t>인터엑스</t>
         </is>
       </c>
       <c r="C39" s="6" t="inlineStr">
@@ -2569,17 +2569,17 @@
       </c>
       <c r="F39" s="7" t="inlineStr">
         <is>
-          <t>27,015</t>
+          <t>8,645</t>
         </is>
       </c>
       <c r="G39" s="7" t="inlineStr">
         <is>
-          <t>3,987</t>
+          <t>-20,272</t>
         </is>
       </c>
       <c r="H39" s="7" t="inlineStr">
         <is>
-          <t>2,613</t>
+          <t>4,530</t>
         </is>
       </c>
       <c r="I39" s="6" t="inlineStr">
@@ -2589,7 +2589,7 @@
       </c>
       <c r="J39" s="6" t="inlineStr">
         <is>
-          <t>한화, 하나</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="K39" s="6" t="inlineStr">
@@ -2601,12 +2601,12 @@
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>제이앤티지</t>
+          <t>삼홍아크튜리온</t>
         </is>
       </c>
       <c r="C40" s="6" t="inlineStr">
@@ -2626,27 +2626,27 @@
       </c>
       <c r="F40" s="7" t="inlineStr">
         <is>
-          <t>72,378</t>
+          <t>26,162</t>
         </is>
       </c>
       <c r="G40" s="7" t="inlineStr">
         <is>
-          <t>9,904</t>
+          <t>-10,314</t>
         </is>
       </c>
       <c r="H40" s="7" t="inlineStr">
         <is>
-          <t>6,743</t>
+          <t>6,369</t>
         </is>
       </c>
       <c r="I40" s="6" t="inlineStr">
         <is>
-          <t>전자부품 제조업</t>
+          <t>구조용 금속제품, 탱크 및 증기발생기 제조업</t>
         </is>
       </c>
       <c r="J40" s="6" t="inlineStr">
         <is>
-          <t>대신, NH</t>
+          <t>삼성, 미래</t>
         </is>
       </c>
       <c r="K40" s="6" t="inlineStr">
@@ -2658,12 +2658,12 @@
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>인터엑스</t>
+          <t>비앤비코리아</t>
         </is>
       </c>
       <c r="C41" s="6" t="inlineStr">
@@ -2683,27 +2683,27 @@
       </c>
       <c r="F41" s="7" t="inlineStr">
         <is>
-          <t>8,645</t>
+          <t>141,169</t>
         </is>
       </c>
       <c r="G41" s="7" t="inlineStr">
         <is>
-          <t>-20,272</t>
+          <t>21,406</t>
         </is>
       </c>
       <c r="H41" s="7" t="inlineStr">
         <is>
-          <t>4,530</t>
+          <t>43,932</t>
         </is>
       </c>
       <c r="I41" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어 개발 및 공급업</t>
+          <t>기타 화학제품 제조업</t>
         </is>
       </c>
       <c r="J41" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K41" s="6" t="inlineStr">
@@ -2715,12 +2715,12 @@
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B42" s="6" t="inlineStr">
         <is>
-          <t>삼홍아크튜리온</t>
+          <t>오토핸즈</t>
         </is>
       </c>
       <c r="C42" s="6" t="inlineStr">
@@ -2730,7 +2730,7 @@
       </c>
       <c r="D42" s="6" t="inlineStr">
         <is>
-          <t>신규상장</t>
+          <t>스팩 소멸합병</t>
         </is>
       </c>
       <c r="E42" s="6" t="inlineStr">
@@ -2740,27 +2740,27 @@
       </c>
       <c r="F42" s="7" t="inlineStr">
         <is>
-          <t>26,162</t>
+          <t>238,564</t>
         </is>
       </c>
       <c r="G42" s="7" t="inlineStr">
         <is>
-          <t>-10,314</t>
+          <t>6,047</t>
         </is>
       </c>
       <c r="H42" s="7" t="inlineStr">
         <is>
-          <t>6,369</t>
+          <t>6,129</t>
         </is>
       </c>
       <c r="I42" s="6" t="inlineStr">
         <is>
-          <t>구조용 금속제품, 탱크 및 증기발생기 제조업</t>
+          <t>자동차 판매업</t>
         </is>
       </c>
       <c r="J42" s="6" t="inlineStr">
         <is>
-          <t>삼성, 미래</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K42" s="6" t="inlineStr">
@@ -2772,12 +2772,12 @@
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B43" s="6" t="inlineStr">
         <is>
-          <t>비앤비코리아</t>
+          <t>아이벡스메디칼시스템즈</t>
         </is>
       </c>
       <c r="C43" s="6" t="inlineStr">
@@ -2797,27 +2797,27 @@
       </c>
       <c r="F43" s="7" t="inlineStr">
         <is>
-          <t>141,169</t>
+          <t>15,282</t>
         </is>
       </c>
       <c r="G43" s="7" t="inlineStr">
         <is>
-          <t>21,406</t>
+          <t>-7,227</t>
         </is>
       </c>
       <c r="H43" s="7" t="inlineStr">
         <is>
-          <t>43,932</t>
+          <t>744</t>
         </is>
       </c>
       <c r="I43" s="6" t="inlineStr">
         <is>
-          <t>기타 화학제품 제조업</t>
+          <t>의료용 기기 제조업</t>
         </is>
       </c>
       <c r="J43" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K43" s="6" t="inlineStr">
@@ -2829,12 +2829,12 @@
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="B44" s="6" t="inlineStr">
         <is>
-          <t>오토핸즈</t>
+          <t>피지티</t>
         </is>
       </c>
       <c r="C44" s="6" t="inlineStr">
@@ -2844,7 +2844,7 @@
       </c>
       <c r="D44" s="6" t="inlineStr">
         <is>
-          <t>스팩 소멸합병</t>
+          <t>신규상장</t>
         </is>
       </c>
       <c r="E44" s="6" t="inlineStr">
@@ -2854,27 +2854,27 @@
       </c>
       <c r="F44" s="7" t="inlineStr">
         <is>
-          <t>238,564</t>
+          <t>40,141</t>
         </is>
       </c>
       <c r="G44" s="7" t="inlineStr">
         <is>
-          <t>6,047</t>
+          <t>-69,722</t>
         </is>
       </c>
       <c r="H44" s="7" t="inlineStr">
         <is>
-          <t>6,129</t>
+          <t>6,029</t>
         </is>
       </c>
       <c r="I44" s="6" t="inlineStr">
         <is>
-          <t>자동차 판매업</t>
+          <t>기타 화학제품 제조업</t>
         </is>
       </c>
       <c r="J44" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="K44" s="6" t="inlineStr">
@@ -2883,191 +2883,191 @@
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="6" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-      <c r="B45" s="6" t="inlineStr">
-        <is>
-          <t>아이벡스메디칼시스템즈</t>
-        </is>
-      </c>
-      <c r="C45" s="6" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>■ 심사 승인  (78건)</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="n"/>
+      <c r="C46" s="4" t="n"/>
+      <c r="D46" s="4" t="n"/>
+      <c r="E46" s="4" t="n"/>
+      <c r="F46" s="4" t="n"/>
+      <c r="G46" s="4" t="n"/>
+      <c r="H46" s="4" t="n"/>
+      <c r="I46" s="4" t="n"/>
+      <c r="J46" s="4" t="n"/>
+      <c r="K46" s="4" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>일자</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>회사명</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>시장</t>
+        </is>
+      </c>
+      <c r="D47" s="5" t="inlineStr">
+        <is>
+          <t>상장유형</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
+          <t>기준연도</t>
+        </is>
+      </c>
+      <c r="F47" s="5" t="inlineStr">
+        <is>
+          <t>매출액</t>
+        </is>
+      </c>
+      <c r="G47" s="5" t="inlineStr">
+        <is>
+          <t>순이익</t>
+        </is>
+      </c>
+      <c r="H47" s="5" t="inlineStr">
+        <is>
+          <t>자기자본</t>
+        </is>
+      </c>
+      <c r="I47" s="5" t="inlineStr">
+        <is>
+          <t>업종</t>
+        </is>
+      </c>
+      <c r="J47" s="5" t="inlineStr">
+        <is>
+          <t>대표주관사</t>
+        </is>
+      </c>
+      <c r="K47" s="5" t="inlineStr">
+        <is>
+          <t>현황</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B48" s="6" t="inlineStr">
+        <is>
+          <t>제이앤티지</t>
+        </is>
+      </c>
+      <c r="C48" s="6" t="inlineStr">
         <is>
           <t>코스닥</t>
         </is>
       </c>
-      <c r="D45" s="6" t="inlineStr">
+      <c r="D48" s="6" t="inlineStr">
         <is>
           <t>신규상장</t>
         </is>
       </c>
-      <c r="E45" s="6" t="inlineStr">
+      <c r="E48" s="6" t="inlineStr">
         <is>
           <t>FY25</t>
         </is>
       </c>
-      <c r="F45" s="7" t="inlineStr">
-        <is>
-          <t>15,282</t>
-        </is>
-      </c>
-      <c r="G45" s="7" t="inlineStr">
-        <is>
-          <t>-7,227</t>
-        </is>
-      </c>
-      <c r="H45" s="7" t="inlineStr">
-        <is>
-          <t>744</t>
-        </is>
-      </c>
-      <c r="I45" s="6" t="inlineStr">
-        <is>
-          <t>의료용 기기 제조업</t>
-        </is>
-      </c>
-      <c r="J45" s="6" t="inlineStr">
-        <is>
-          <t>NH</t>
-        </is>
-      </c>
-      <c r="K45" s="6" t="inlineStr">
-        <is>
-          <t>예심 진행중</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="6" t="inlineStr">
-        <is>
-          <t>2026-02-27</t>
-        </is>
-      </c>
-      <c r="B46" s="6" t="inlineStr">
-        <is>
-          <t>피지티</t>
-        </is>
-      </c>
-      <c r="C46" s="6" t="inlineStr">
+      <c r="F48" s="7" t="inlineStr">
+        <is>
+          <t>72,378</t>
+        </is>
+      </c>
+      <c r="G48" s="7" t="inlineStr">
+        <is>
+          <t>9,904</t>
+        </is>
+      </c>
+      <c r="H48" s="7" t="inlineStr">
+        <is>
+          <t>6,743</t>
+        </is>
+      </c>
+      <c r="I48" s="6" t="inlineStr">
+        <is>
+          <t>전자부품 제조업</t>
+        </is>
+      </c>
+      <c r="J48" s="6" t="inlineStr">
+        <is>
+          <t>대신, NH</t>
+        </is>
+      </c>
+      <c r="K48" s="6" t="inlineStr">
+        <is>
+          <t>상장전</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B49" s="6" t="inlineStr">
+        <is>
+          <t>데스틴파워</t>
+        </is>
+      </c>
+      <c r="C49" s="6" t="inlineStr">
         <is>
           <t>코스닥</t>
         </is>
       </c>
-      <c r="D46" s="6" t="inlineStr">
+      <c r="D49" s="6" t="inlineStr">
         <is>
           <t>신규상장</t>
         </is>
       </c>
-      <c r="E46" s="6" t="inlineStr">
+      <c r="E49" s="6" t="inlineStr">
         <is>
           <t>FY25</t>
         </is>
       </c>
-      <c r="F46" s="7" t="inlineStr">
-        <is>
-          <t>40,141</t>
-        </is>
-      </c>
-      <c r="G46" s="7" t="inlineStr">
-        <is>
-          <t>-69,722</t>
-        </is>
-      </c>
-      <c r="H46" s="7" t="inlineStr">
-        <is>
-          <t>6,029</t>
-        </is>
-      </c>
-      <c r="I46" s="6" t="inlineStr">
-        <is>
-          <t>기타 화학제품 제조업</t>
-        </is>
-      </c>
-      <c r="J46" s="6" t="inlineStr">
+      <c r="F49" s="7" t="inlineStr">
+        <is>
+          <t>29,851</t>
+        </is>
+      </c>
+      <c r="G49" s="7" t="inlineStr">
+        <is>
+          <t>5,852</t>
+        </is>
+      </c>
+      <c r="H49" s="7" t="inlineStr">
+        <is>
+          <t>-30,114</t>
+        </is>
+      </c>
+      <c r="I49" s="6" t="inlineStr">
+        <is>
+          <t>전동기, 발전기 및 전기 변환 · 공급 · 제어 장치 제조업</t>
+        </is>
+      </c>
+      <c r="J49" s="6" t="inlineStr">
         <is>
           <t>한국</t>
         </is>
       </c>
-      <c r="K46" s="6" t="inlineStr">
-        <is>
-          <t>예심 진행중</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="3" t="inlineStr">
-        <is>
-          <t>■ 심사 승인  (76건)</t>
-        </is>
-      </c>
-      <c r="B48" s="4" t="n"/>
-      <c r="C48" s="4" t="n"/>
-      <c r="D48" s="4" t="n"/>
-      <c r="E48" s="4" t="n"/>
-      <c r="F48" s="4" t="n"/>
-      <c r="G48" s="4" t="n"/>
-      <c r="H48" s="4" t="n"/>
-      <c r="I48" s="4" t="n"/>
-      <c r="J48" s="4" t="n"/>
-      <c r="K48" s="4" t="n"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="5" t="inlineStr">
-        <is>
-          <t>일자</t>
-        </is>
-      </c>
-      <c r="B49" s="5" t="inlineStr">
-        <is>
-          <t>회사명</t>
-        </is>
-      </c>
-      <c r="C49" s="5" t="inlineStr">
-        <is>
-          <t>시장</t>
-        </is>
-      </c>
-      <c r="D49" s="5" t="inlineStr">
-        <is>
-          <t>상장유형</t>
-        </is>
-      </c>
-      <c r="E49" s="5" t="inlineStr">
-        <is>
-          <t>기준연도</t>
-        </is>
-      </c>
-      <c r="F49" s="5" t="inlineStr">
-        <is>
-          <t>매출액</t>
-        </is>
-      </c>
-      <c r="G49" s="5" t="inlineStr">
-        <is>
-          <t>순이익</t>
-        </is>
-      </c>
-      <c r="H49" s="5" t="inlineStr">
-        <is>
-          <t>자기자본</t>
-        </is>
-      </c>
-      <c r="I49" s="5" t="inlineStr">
-        <is>
-          <t>업종</t>
-        </is>
-      </c>
-      <c r="J49" s="5" t="inlineStr">
-        <is>
-          <t>대표주관사</t>
-        </is>
-      </c>
-      <c r="K49" s="5" t="inlineStr">
-        <is>
-          <t>현황</t>
+      <c r="K49" s="6" t="inlineStr">
+        <is>
+          <t>상장전</t>
         </is>
       </c>
     </row>
@@ -8464,7 +8464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R97"/>
+  <dimension ref="A1:R99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -12546,7 +12546,7 @@
     <row r="56" ht="22" customHeight="1">
       <c r="A56" s="3" t="inlineStr">
         <is>
-          <t>■ 공모 진행 (예심 승인법인)  (37건)</t>
+          <t>■ 공모 진행 (예심 승인법인)  (39건)</t>
         </is>
       </c>
       <c r="B56" s="4" t="n"/>
@@ -13582,32 +13582,32 @@
     <row r="72" ht="30" customHeight="1">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>다비오</t>
+          <t>에이엘로봇</t>
         </is>
       </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>11-02~11-06</t>
+          <t>10-28~11-03</t>
         </is>
       </c>
       <c r="C72" s="6" t="inlineStr">
         <is>
-          <t>12,300~16,600</t>
+          <t>15,700~17,600</t>
         </is>
       </c>
       <c r="D72" s="7" t="inlineStr">
         <is>
-          <t>1,000,000</t>
+          <t>2,400,000</t>
         </is>
       </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
-          <t>12,300,000,000</t>
+          <t>37,680,000,000</t>
         </is>
       </c>
       <c r="F72" s="6" t="inlineStr">
         <is>
-          <t>26.70배 (PER)</t>
+          <t>37.17배 (PER)</t>
         </is>
       </c>
       <c r="G72" s="6" t="inlineStr"/>
@@ -13615,7 +13615,7 @@
       <c r="I72" s="6" t="inlineStr"/>
       <c r="J72" s="6" t="inlineStr">
         <is>
-          <t>11-10~11-11</t>
+          <t>11-06~11-09</t>
         </is>
       </c>
       <c r="K72" s="6" t="inlineStr"/>
@@ -13629,12 +13629,12 @@
       <c r="O72" s="6" t="inlineStr"/>
       <c r="P72" s="7" t="inlineStr">
         <is>
-          <t>570,105,000</t>
+          <t>1,160,399,874</t>
         </is>
       </c>
       <c r="Q72" s="6" t="inlineStr">
         <is>
-          <t>4.5%</t>
+          <t>3.0%</t>
         </is>
       </c>
       <c r="R72" s="6" t="inlineStr">
@@ -13646,59 +13646,59 @@
     <row r="73" ht="30" customHeight="1">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>바로팜</t>
-        </is>
-      </c>
-      <c r="B73" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>다비오</t>
+        </is>
+      </c>
+      <c r="B73" s="6" t="inlineStr">
+        <is>
+          <t>11-02~11-06</t>
         </is>
       </c>
       <c r="C73" s="6" t="inlineStr">
         <is>
-          <t>16,400~20,200</t>
+          <t>12,300~16,600</t>
         </is>
       </c>
       <c r="D73" s="7" t="inlineStr">
         <is>
-          <t>1,780,000</t>
+          <t>1,000,000</t>
         </is>
       </c>
       <c r="E73" s="7" t="inlineStr">
         <is>
-          <t>29,192,000,000</t>
+          <t>12,300,000,000</t>
         </is>
       </c>
       <c r="F73" s="6" t="inlineStr">
         <is>
-          <t>24.95배 (PER)</t>
+          <t>26.70배 (PER)</t>
         </is>
       </c>
       <c r="G73" s="6" t="inlineStr"/>
       <c r="H73" s="6" t="inlineStr"/>
       <c r="I73" s="6" t="inlineStr"/>
-      <c r="J73" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="J73" s="6" t="inlineStr">
+        <is>
+          <t>11-10~11-11</t>
         </is>
       </c>
       <c r="K73" s="6" t="inlineStr"/>
       <c r="L73" s="6" t="inlineStr"/>
       <c r="M73" s="6" t="inlineStr"/>
-      <c r="N73" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="N73" s="6" t="inlineStr">
+        <is>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="O73" s="6" t="inlineStr"/>
-      <c r="P73" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="Q73" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="P73" s="7" t="inlineStr">
+        <is>
+          <t>570,105,000</t>
+        </is>
+      </c>
+      <c r="Q73" s="6" t="inlineStr">
+        <is>
+          <t>4.5%</t>
         </is>
       </c>
       <c r="R73" s="6" t="inlineStr">
@@ -13710,7 +13710,7 @@
     <row r="74" ht="30" customHeight="1">
       <c r="A74" s="6" t="inlineStr">
         <is>
-          <t>셀트릭스</t>
+          <t>바로팜</t>
         </is>
       </c>
       <c r="B74" s="18" t="inlineStr">
@@ -13718,24 +13718,24 @@
           <t>수집예정</t>
         </is>
       </c>
-      <c r="C74" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="D74" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="E74" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="F74" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="C74" s="6" t="inlineStr">
+        <is>
+          <t>16,400~20,200</t>
+        </is>
+      </c>
+      <c r="D74" s="7" t="inlineStr">
+        <is>
+          <t>1,780,000</t>
+        </is>
+      </c>
+      <c r="E74" s="7" t="inlineStr">
+        <is>
+          <t>29,192,000,000</t>
+        </is>
+      </c>
+      <c r="F74" s="6" t="inlineStr">
+        <is>
+          <t>24.95배 (PER)</t>
         </is>
       </c>
       <c r="G74" s="6" t="inlineStr"/>
@@ -13774,7 +13774,7 @@
     <row r="75" ht="30" customHeight="1">
       <c r="A75" s="6" t="inlineStr">
         <is>
-          <t>솔리스</t>
+          <t>셀트릭스</t>
         </is>
       </c>
       <c r="B75" s="18" t="inlineStr">
@@ -13838,64 +13838,64 @@
     <row r="76" ht="30" customHeight="1">
       <c r="A76" s="6" t="inlineStr">
         <is>
-          <t>에이엘로봇</t>
-        </is>
-      </c>
-      <c r="B76" s="6" t="inlineStr">
-        <is>
-          <t>10-15~10-21</t>
-        </is>
-      </c>
-      <c r="C76" s="6" t="inlineStr">
-        <is>
-          <t>15,700~17,600</t>
-        </is>
-      </c>
-      <c r="D76" s="7" t="inlineStr">
-        <is>
-          <t>2,400,000</t>
-        </is>
-      </c>
-      <c r="E76" s="7" t="inlineStr">
-        <is>
-          <t>37,680,000,000</t>
-        </is>
-      </c>
-      <c r="F76" s="6" t="inlineStr">
-        <is>
-          <t>37.17배 (PER)</t>
+          <t>솔리스</t>
+        </is>
+      </c>
+      <c r="B76" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="C76" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="D76" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="E76" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="F76" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="G76" s="6" t="inlineStr"/>
       <c r="H76" s="6" t="inlineStr"/>
       <c r="I76" s="6" t="inlineStr"/>
-      <c r="J76" s="6" t="inlineStr">
-        <is>
-          <t>10-26~10-27</t>
+      <c r="J76" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="K76" s="6" t="inlineStr"/>
       <c r="L76" s="6" t="inlineStr"/>
       <c r="M76" s="6" t="inlineStr"/>
-      <c r="N76" s="6" t="inlineStr">
-        <is>
-          <t>대신증권</t>
+      <c r="N76" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="O76" s="6" t="inlineStr"/>
-      <c r="P76" s="7" t="inlineStr">
-        <is>
-          <t>1,160,399,874</t>
-        </is>
-      </c>
-      <c r="Q76" s="6" t="inlineStr">
-        <is>
-          <t>3.0%</t>
+      <c r="P76" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="Q76" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="R76" s="6" t="inlineStr">
         <is>
-          <t>최초</t>
+          <t>정정</t>
         </is>
       </c>
     </row>
@@ -14350,32 +14350,32 @@
     <row r="84" ht="30" customHeight="1">
       <c r="A84" s="6" t="inlineStr">
         <is>
-          <t>케이엠에프</t>
+          <t>아델</t>
         </is>
       </c>
       <c r="B84" s="6" t="inlineStr">
         <is>
-          <t>11-16~11-20</t>
+          <t>11-12~11-18</t>
         </is>
       </c>
       <c r="C84" s="6" t="inlineStr">
         <is>
-          <t>15,000~17,800</t>
+          <t>18,000~25,000</t>
         </is>
       </c>
       <c r="D84" s="7" t="inlineStr">
         <is>
-          <t>2,000,000</t>
+          <t>2,170,000</t>
         </is>
       </c>
       <c r="E84" s="7" t="inlineStr">
         <is>
-          <t>30,000,000,000</t>
+          <t>39,060,000,000</t>
         </is>
       </c>
       <c r="F84" s="6" t="inlineStr">
         <is>
-          <t>18.53배 (PER)</t>
+          <t>20.91배 (PER)</t>
         </is>
       </c>
       <c r="G84" s="6" t="inlineStr"/>
@@ -14383,7 +14383,7 @@
       <c r="I84" s="6" t="inlineStr"/>
       <c r="J84" s="6" t="inlineStr">
         <is>
-          <t>11-24~11-25</t>
+          <t>11-23~11-24</t>
         </is>
       </c>
       <c r="K84" s="6" t="inlineStr"/>
@@ -14391,18 +14391,18 @@
       <c r="M84" s="6" t="inlineStr"/>
       <c r="N84" s="6" t="inlineStr">
         <is>
-          <t>아이비케이투자증권</t>
+          <t>삼성증권㈜</t>
         </is>
       </c>
       <c r="O84" s="6" t="inlineStr"/>
       <c r="P84" s="7" t="inlineStr">
         <is>
-          <t>927,000,000</t>
+          <t>1,041,559,920</t>
         </is>
       </c>
       <c r="Q84" s="6" t="inlineStr">
         <is>
-          <t>3.0%</t>
+          <t>4.0%</t>
         </is>
       </c>
       <c r="R84" s="6" t="inlineStr">
@@ -14414,59 +14414,59 @@
     <row r="85" ht="30" customHeight="1">
       <c r="A85" s="6" t="inlineStr">
         <is>
-          <t>럭스코</t>
-        </is>
-      </c>
-      <c r="B85" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="C85" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="D85" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="E85" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="F85" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>케이엠에프</t>
+        </is>
+      </c>
+      <c r="B85" s="6" t="inlineStr">
+        <is>
+          <t>11-16~11-20</t>
+        </is>
+      </c>
+      <c r="C85" s="6" t="inlineStr">
+        <is>
+          <t>15,000~17,800</t>
+        </is>
+      </c>
+      <c r="D85" s="7" t="inlineStr">
+        <is>
+          <t>2,000,000</t>
+        </is>
+      </c>
+      <c r="E85" s="7" t="inlineStr">
+        <is>
+          <t>30,000,000,000</t>
+        </is>
+      </c>
+      <c r="F85" s="6" t="inlineStr">
+        <is>
+          <t>18.53배 (PER)</t>
         </is>
       </c>
       <c r="G85" s="6" t="inlineStr"/>
       <c r="H85" s="6" t="inlineStr"/>
       <c r="I85" s="6" t="inlineStr"/>
-      <c r="J85" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="J85" s="6" t="inlineStr">
+        <is>
+          <t>11-24~11-25</t>
         </is>
       </c>
       <c r="K85" s="6" t="inlineStr"/>
       <c r="L85" s="6" t="inlineStr"/>
       <c r="M85" s="6" t="inlineStr"/>
-      <c r="N85" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="N85" s="6" t="inlineStr">
+        <is>
+          <t>아이비케이투자증권</t>
         </is>
       </c>
       <c r="O85" s="6" t="inlineStr"/>
-      <c r="P85" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="Q85" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="P85" s="7" t="inlineStr">
+        <is>
+          <t>927,000,000</t>
+        </is>
+      </c>
+      <c r="Q85" s="6" t="inlineStr">
+        <is>
+          <t>3.0%</t>
         </is>
       </c>
       <c r="R85" s="6" t="inlineStr">
@@ -14478,7 +14478,7 @@
     <row r="86" ht="30" customHeight="1">
       <c r="A86" s="6" t="inlineStr">
         <is>
-          <t>디티에스</t>
+          <t>럭스코</t>
         </is>
       </c>
       <c r="B86" s="18" t="inlineStr">
@@ -14535,14 +14535,14 @@
       </c>
       <c r="R86" s="6" t="inlineStr">
         <is>
-          <t>신고서 대기</t>
+          <t>최초</t>
         </is>
       </c>
     </row>
     <row r="87" ht="30" customHeight="1">
       <c r="A87" s="6" t="inlineStr">
         <is>
-          <t>에이엔에이치스트럭쳐</t>
+          <t>디티에스</t>
         </is>
       </c>
       <c r="B87" s="18" t="inlineStr">
@@ -14606,7 +14606,7 @@
     <row r="88" ht="30" customHeight="1">
       <c r="A88" s="6" t="inlineStr">
         <is>
-          <t>이에스티</t>
+          <t>에이엔에이치스트럭쳐</t>
         </is>
       </c>
       <c r="B88" s="18" t="inlineStr">
@@ -14670,7 +14670,7 @@
     <row r="89" ht="30" customHeight="1">
       <c r="A89" s="6" t="inlineStr">
         <is>
-          <t>우리투자제1호스팩</t>
+          <t>이에스티</t>
         </is>
       </c>
       <c r="B89" s="18" t="inlineStr">
@@ -14734,7 +14734,7 @@
     <row r="90" ht="30" customHeight="1">
       <c r="A90" s="6" t="inlineStr">
         <is>
-          <t>마더스제약</t>
+          <t>우리투자제1호스팩</t>
         </is>
       </c>
       <c r="B90" s="18" t="inlineStr">
@@ -14798,7 +14798,7 @@
     <row r="91" ht="30" customHeight="1">
       <c r="A91" s="6" t="inlineStr">
         <is>
-          <t>아델</t>
+          <t>마더스제약</t>
         </is>
       </c>
       <c r="B91" s="18" t="inlineStr">
@@ -14987,22 +14987,150 @@
         </is>
       </c>
     </row>
-    <row r="95">
-      <c r="A95" s="20" t="inlineStr">
-        <is>
-          <t>※ 상장 완료 = KIND 신규상장 페이지 기준(스팩합병 포함) · 스팩 공모상장은 밴드·밸류에이션 등 해당없음(공모가 2,000원 고정).</t>
-        </is>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" s="20" t="inlineStr">
-        <is>
-          <t>※ 기재정정 신고서 내 정정 전·후 병존 → 자동수집은 "정정 후" 값만 취함.</t>
+    <row r="94" ht="30" customHeight="1">
+      <c r="A94" s="6" t="inlineStr">
+        <is>
+          <t>제이앤티지</t>
+        </is>
+      </c>
+      <c r="B94" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="C94" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="D94" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="E94" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="F94" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="G94" s="6" t="inlineStr"/>
+      <c r="H94" s="6" t="inlineStr"/>
+      <c r="I94" s="6" t="inlineStr"/>
+      <c r="J94" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="K94" s="6" t="inlineStr"/>
+      <c r="L94" s="6" t="inlineStr"/>
+      <c r="M94" s="6" t="inlineStr"/>
+      <c r="N94" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="O94" s="6" t="inlineStr"/>
+      <c r="P94" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="Q94" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="R94" s="6" t="inlineStr">
+        <is>
+          <t>신고서 대기</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="30" customHeight="1">
+      <c r="A95" s="6" t="inlineStr">
+        <is>
+          <t>데스틴파워</t>
+        </is>
+      </c>
+      <c r="B95" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="C95" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="D95" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="E95" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="F95" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="G95" s="6" t="inlineStr"/>
+      <c r="H95" s="6" t="inlineStr"/>
+      <c r="I95" s="6" t="inlineStr"/>
+      <c r="J95" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="K95" s="6" t="inlineStr"/>
+      <c r="L95" s="6" t="inlineStr"/>
+      <c r="M95" s="6" t="inlineStr"/>
+      <c r="N95" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="O95" s="6" t="inlineStr"/>
+      <c r="P95" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="Q95" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="R95" s="6" t="inlineStr">
+        <is>
+          <t>신고서 대기</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="20" t="inlineStr">
+        <is>
+          <t>※ 상장 완료 = KIND 신규상장 페이지 기준(스팩합병 포함) · 스팩 공모상장은 밴드·밸류에이션 등 해당없음(공모가 2,000원 고정).</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="20" t="inlineStr">
+        <is>
+          <t>※ 기재정정 신고서 내 정정 전·후 병존 → 자동수집은 "정정 후" 값만 취함.</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="20" t="inlineStr">
         <is>
           <t>※ 청약경쟁률=일반투자자 청약수량÷최종배정수량 · "MM-DD~"는 종료일 자동수집 예정.</t>
         </is>
@@ -15019,7 +15147,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F43"/>
+  <dimension ref="A1:F44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -15305,7 +15433,7 @@
         <v>3</v>
       </c>
       <c r="C15" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D15" s="6" t="n">
         <v>1</v>
@@ -15524,37 +15652,37 @@
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>하나증권</t>
+          <t>삼성증권㈜</t>
         </is>
       </c>
       <c r="B30" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>35,814,000,000</t>
+          <t>39,060,000,000</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>KB증권</t>
+          <t>하나증권</t>
         </is>
       </c>
       <c r="B31" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>31,200,000,000</t>
+          <t>35,814,000,000</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>신한투자증권</t>
+          <t>KB증권</t>
         </is>
       </c>
       <c r="B32" s="6" t="n">
@@ -15562,14 +15690,14 @@
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>30,240,000,000</t>
+          <t>31,200,000,000</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>신영증권</t>
+          <t>신한투자증권</t>
         </is>
       </c>
       <c r="B33" s="6" t="n">
@@ -15577,104 +15705,104 @@
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>22,100,000,000</t>
+          <t>30,240,000,000</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>신영증권</t>
         </is>
       </c>
       <c r="B34" s="6" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>618,288</t>
+          <t>22,100,000,000</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="B35" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>154,600</t>
+          <t>618,288</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="B36" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>130,837</t>
+          <t>154,600</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>신한</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="B37" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>49,052</t>
+          <t>130,837</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>삼성</t>
+          <t>신한</t>
         </is>
       </c>
       <c r="B38" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
-          <t>32,000</t>
+          <t>49,052</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>유진</t>
+          <t>삼성</t>
         </is>
       </c>
       <c r="B39" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>25,020</t>
+          <t>32,000</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>메리츠</t>
+          <t>유진</t>
         </is>
       </c>
       <c r="B40" s="6" t="n">
@@ -15682,14 +15810,14 @@
       </c>
       <c r="C40" s="6" t="inlineStr">
         <is>
-          <t>14,000</t>
+          <t>25,020</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>대신</t>
+          <t>메리츠</t>
         </is>
       </c>
       <c r="B41" s="6" t="n">
@@ -15697,14 +15825,14 @@
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>13,000</t>
+          <t>14,000</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>키움</t>
+          <t>대신</t>
         </is>
       </c>
       <c r="B42" s="6" t="n">
@@ -15712,20 +15840,35 @@
       </c>
       <c r="C42" s="6" t="inlineStr">
         <is>
-          <t>12,000</t>
+          <t>13,000</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>교보</t>
+          <t>키움</t>
         </is>
       </c>
       <c r="B43" s="6" t="n">
         <v>1</v>
       </c>
       <c r="C43" s="6" t="inlineStr">
+        <is>
+          <t>12,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="6" t="inlineStr">
+        <is>
+          <t>교보</t>
+        </is>
+      </c>
+      <c r="B44" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C44" s="6" t="inlineStr">
         <is>
           <t>10,800</t>
         </is>

</xml_diff>

<commit_message>
chore: update IPO data 2026-10-14
</commit_message>
<xml_diff>
--- a/IPO_analysis.xlsx
+++ b/IPO_analysis.xlsx
@@ -618,7 +618,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>기준일 2026-10-13 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
+          <t>기준일 2026-10-14 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
         </is>
       </c>
     </row>
@@ -13003,71 +13003,79 @@
     <row r="62" ht="30" customHeight="1">
       <c r="A62" s="6" t="inlineStr">
         <is>
-          <t>티앤이코리아</t>
+          <t>에스케이증권제14호기업인수목적</t>
         </is>
       </c>
       <c r="B62" s="6" t="inlineStr">
         <is>
-          <t>10-07~10-14</t>
-        </is>
-      </c>
-      <c r="C62" s="6" t="inlineStr">
-        <is>
-          <t>12,600~15,300</t>
+          <t>10-12~10-13</t>
+        </is>
+      </c>
+      <c r="C62" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="D62" s="7" t="inlineStr">
         <is>
-          <t>2,400,000</t>
+          <t>6,500,000</t>
         </is>
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
-          <t>30,240,000,000</t>
-        </is>
-      </c>
-      <c r="F62" s="6" t="inlineStr">
-        <is>
-          <t>19.48배 (PER)</t>
-        </is>
-      </c>
-      <c r="G62" s="6" t="inlineStr"/>
-      <c r="H62" s="6" t="inlineStr"/>
-      <c r="I62" s="6" t="inlineStr"/>
+          <t>13,000,000,000</t>
+        </is>
+      </c>
+      <c r="F62" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="G62" s="6" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
+      </c>
+      <c r="H62" s="6" t="n">
+        <v>1228.38</v>
+      </c>
+      <c r="I62" s="6" t="n">
+        <v>1945</v>
+      </c>
       <c r="J62" s="6" t="inlineStr">
         <is>
-          <t>10-20~10-21</t>
+          <t>10-15~10-16</t>
         </is>
       </c>
       <c r="K62" s="6" t="inlineStr"/>
       <c r="L62" s="6" t="inlineStr"/>
       <c r="M62" s="6" t="inlineStr"/>
-      <c r="N62" s="6" t="inlineStr">
-        <is>
-          <t>신한투자증권</t>
+      <c r="N62" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="O62" s="6" t="inlineStr"/>
-      <c r="P62" s="7" t="inlineStr">
-        <is>
-          <t>1,245,888,000</t>
+      <c r="P62" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="Q62" s="6" t="inlineStr">
         <is>
-          <t>4.0%</t>
+          <t>50%</t>
         </is>
       </c>
       <c r="R62" s="6" t="inlineStr">
         <is>
-          <t>정정</t>
+          <t>발행조건확정</t>
         </is>
       </c>
     </row>
     <row r="63" ht="30" customHeight="1">
       <c r="A63" s="6" t="inlineStr">
         <is>
-          <t>유캐스트</t>
+          <t>티앤이코리아</t>
         </is>
       </c>
       <c r="B63" s="6" t="inlineStr">
@@ -13077,22 +13085,22 @@
       </c>
       <c r="C63" s="6" t="inlineStr">
         <is>
-          <t>21,000~26,000</t>
+          <t>12,600~15,300</t>
         </is>
       </c>
       <c r="D63" s="7" t="inlineStr">
         <is>
-          <t>800,000</t>
+          <t>2,400,000</t>
         </is>
       </c>
       <c r="E63" s="7" t="inlineStr">
         <is>
-          <t>16,800,000,000</t>
+          <t>30,240,000,000</t>
         </is>
       </c>
       <c r="F63" s="6" t="inlineStr">
         <is>
-          <t>17.97배 (PER)</t>
+          <t>19.48배 (PER)</t>
         </is>
       </c>
       <c r="G63" s="6" t="inlineStr"/>
@@ -13100,7 +13108,7 @@
       <c r="I63" s="6" t="inlineStr"/>
       <c r="J63" s="6" t="inlineStr">
         <is>
-          <t>10-19~10-20</t>
+          <t>10-20~10-21</t>
         </is>
       </c>
       <c r="K63" s="6" t="inlineStr"/>
@@ -13108,18 +13116,18 @@
       <c r="M63" s="6" t="inlineStr"/>
       <c r="N63" s="6" t="inlineStr">
         <is>
-          <t>유진투자증권</t>
+          <t>신한투자증권</t>
         </is>
       </c>
       <c r="O63" s="6" t="inlineStr"/>
       <c r="P63" s="7" t="inlineStr">
         <is>
-          <t>1,181,280,000</t>
+          <t>1,245,888,000</t>
         </is>
       </c>
       <c r="Q63" s="6" t="inlineStr">
         <is>
-          <t>7.0%</t>
+          <t>4.0%</t>
         </is>
       </c>
       <c r="R63" s="6" t="inlineStr">
@@ -13131,32 +13139,32 @@
     <row r="64" ht="30" customHeight="1">
       <c r="A64" s="6" t="inlineStr">
         <is>
-          <t>에스케이증권제14호기업인수목적</t>
+          <t>유캐스트</t>
         </is>
       </c>
       <c r="B64" s="6" t="inlineStr">
         <is>
-          <t>10-12~10-13</t>
-        </is>
-      </c>
-      <c r="C64" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>10-07~10-14</t>
+        </is>
+      </c>
+      <c r="C64" s="6" t="inlineStr">
+        <is>
+          <t>21,000~26,000</t>
         </is>
       </c>
       <c r="D64" s="7" t="inlineStr">
         <is>
-          <t>6,500,000</t>
+          <t>800,000</t>
         </is>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
-          <t>13,000,000,000</t>
-        </is>
-      </c>
-      <c r="F64" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>16,800,000,000</t>
+        </is>
+      </c>
+      <c r="F64" s="6" t="inlineStr">
+        <is>
+          <t>17.97배 (PER)</t>
         </is>
       </c>
       <c r="G64" s="6" t="inlineStr"/>
@@ -13164,26 +13172,26 @@
       <c r="I64" s="6" t="inlineStr"/>
       <c r="J64" s="6" t="inlineStr">
         <is>
-          <t>10-15~10-16</t>
+          <t>10-19~10-20</t>
         </is>
       </c>
       <c r="K64" s="6" t="inlineStr"/>
       <c r="L64" s="6" t="inlineStr"/>
       <c r="M64" s="6" t="inlineStr"/>
-      <c r="N64" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="N64" s="6" t="inlineStr">
+        <is>
+          <t>유진투자증권</t>
         </is>
       </c>
       <c r="O64" s="6" t="inlineStr"/>
-      <c r="P64" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="P64" s="7" t="inlineStr">
+        <is>
+          <t>1,181,280,000</t>
         </is>
       </c>
       <c r="Q64" s="6" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>7.0%</t>
         </is>
       </c>
       <c r="R64" s="6" t="inlineStr">

</xml_diff>

<commit_message>
chore: update IPO data 2026-10-16
</commit_message>
<xml_diff>
--- a/IPO_analysis.xlsx
+++ b/IPO_analysis.xlsx
@@ -618,14 +618,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>기준일 2026-10-15 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
+          <t>기준일 2026-10-16 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>■ 심사 신청(진행중)  (34건)</t>
+          <t>■ 심사 신청(진행중)  (33건)</t>
         </is>
       </c>
       <c r="B4" s="4" t="n"/>
@@ -1746,17 +1746,17 @@
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>에스에프씨</t>
+          <t>에버온</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>유가</t>
+          <t>코스닥</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
@@ -1771,27 +1771,27 @@
       </c>
       <c r="F25" s="7" t="inlineStr">
         <is>
-          <t>160,792</t>
+          <t>65,225</t>
         </is>
       </c>
       <c r="G25" s="7" t="inlineStr">
         <is>
-          <t>25,509</t>
+          <t>-3,606</t>
         </is>
       </c>
       <c r="H25" s="7" t="inlineStr">
         <is>
-          <t>243,562</t>
+          <t>54,955</t>
         </is>
       </c>
       <c r="I25" s="6" t="inlineStr">
         <is>
-          <t>기타 화학제품 제조업</t>
+          <t>전기업</t>
         </is>
       </c>
       <c r="J25" s="6" t="inlineStr">
         <is>
-          <t>미래, 한국</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K25" s="6" t="inlineStr">
@@ -1803,12 +1803,12 @@
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>에버온</t>
+          <t>엠디에스코리아</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
@@ -1828,22 +1828,22 @@
       </c>
       <c r="F26" s="7" t="inlineStr">
         <is>
-          <t>65,225</t>
+          <t>97,972</t>
         </is>
       </c>
       <c r="G26" s="7" t="inlineStr">
         <is>
-          <t>-3,606</t>
+          <t>6,512</t>
         </is>
       </c>
       <c r="H26" s="7" t="inlineStr">
         <is>
-          <t>54,955</t>
+          <t>53,818</t>
         </is>
       </c>
       <c r="I26" s="6" t="inlineStr">
         <is>
-          <t>전기업</t>
+          <t>기타 식품 제조업</t>
         </is>
       </c>
       <c r="J26" s="6" t="inlineStr">
@@ -1860,12 +1860,12 @@
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>엠디에스코리아</t>
+          <t>동승</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
@@ -1885,27 +1885,27 @@
       </c>
       <c r="F27" s="7" t="inlineStr">
         <is>
-          <t>97,972</t>
+          <t>78,625</t>
         </is>
       </c>
       <c r="G27" s="7" t="inlineStr">
         <is>
-          <t>6,512</t>
+          <t>14,525</t>
         </is>
       </c>
       <c r="H27" s="7" t="inlineStr">
         <is>
-          <t>53,818</t>
+          <t>5,438</t>
         </is>
       </c>
       <c r="I27" s="6" t="inlineStr">
         <is>
-          <t>기타 식품 제조업</t>
+          <t>부동산 임대 및 공급업</t>
         </is>
       </c>
       <c r="J27" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K27" s="6" t="inlineStr">
@@ -1922,7 +1922,7 @@
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>동승</t>
+          <t>에프엠더블유</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
@@ -1932,7 +1932,7 @@
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
-          <t>신규상장</t>
+          <t>스팩 소멸합병</t>
         </is>
       </c>
       <c r="E28" s="6" t="inlineStr">
@@ -1942,27 +1942,27 @@
       </c>
       <c r="F28" s="7" t="inlineStr">
         <is>
-          <t>78,625</t>
+          <t>30,282</t>
         </is>
       </c>
       <c r="G28" s="7" t="inlineStr">
         <is>
-          <t>14,525</t>
+          <t>4,762</t>
         </is>
       </c>
       <c r="H28" s="7" t="inlineStr">
         <is>
-          <t>5,438</t>
+          <t>32</t>
         </is>
       </c>
       <c r="I28" s="6" t="inlineStr">
         <is>
-          <t>부동산 임대 및 공급업</t>
+          <t>기타 식품 제조업</t>
         </is>
       </c>
       <c r="J28" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>유진</t>
         </is>
       </c>
       <c r="K28" s="6" t="inlineStr">
@@ -1974,22 +1974,22 @@
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>에프엠더블유</t>
+          <t>소노인터내셔널</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>코스닥</t>
+          <t>유가</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>스팩 소멸합병</t>
+          <t>신규상장</t>
         </is>
       </c>
       <c r="E29" s="6" t="inlineStr">
@@ -1999,27 +1999,27 @@
       </c>
       <c r="F29" s="7" t="inlineStr">
         <is>
-          <t>30,282</t>
+          <t>2,093,051</t>
         </is>
       </c>
       <c r="G29" s="7" t="inlineStr">
         <is>
-          <t>4,762</t>
+          <t>-148,064</t>
         </is>
       </c>
       <c r="H29" s="7" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>852,372</t>
         </is>
       </c>
       <c r="I29" s="6" t="inlineStr">
         <is>
-          <t>기타 식품 제조업</t>
+          <t>일반 및 생활 숙박시설 운영업</t>
         </is>
       </c>
       <c r="J29" s="6" t="inlineStr">
         <is>
-          <t>유진</t>
+          <t>대신, 미래</t>
         </is>
       </c>
       <c r="K29" s="6" t="inlineStr">
@@ -2031,17 +2031,17 @@
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>소노인터내셔널</t>
+          <t>싸이몬</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>유가</t>
+          <t>코스닥</t>
         </is>
       </c>
       <c r="D30" s="6" t="inlineStr">
@@ -2056,27 +2056,27 @@
       </c>
       <c r="F30" s="7" t="inlineStr">
         <is>
-          <t>2,093,051</t>
+          <t>48,695</t>
         </is>
       </c>
       <c r="G30" s="7" t="inlineStr">
         <is>
-          <t>-148,064</t>
+          <t>15,714</t>
         </is>
       </c>
       <c r="H30" s="7" t="inlineStr">
         <is>
-          <t>852,372</t>
+          <t>61,761</t>
         </is>
       </c>
       <c r="I30" s="6" t="inlineStr">
         <is>
-          <t>일반 및 생활 숙박시설 운영업</t>
+          <t>측정, 시험, 항해, 제어 및 기타 정밀기기 제조업</t>
         </is>
       </c>
       <c r="J30" s="6" t="inlineStr">
         <is>
-          <t>대신, 미래</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K30" s="6" t="inlineStr">
@@ -2088,12 +2088,12 @@
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>싸이몬</t>
+          <t>바이다</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
@@ -2113,27 +2113,27 @@
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>48,695</t>
+          <t>14,432</t>
         </is>
       </c>
       <c r="G31" s="7" t="inlineStr">
         <is>
-          <t>15,714</t>
+          <t>-3,951</t>
         </is>
       </c>
       <c r="H31" s="7" t="inlineStr">
         <is>
-          <t>61,761</t>
+          <t>15,108</t>
         </is>
       </c>
       <c r="I31" s="6" t="inlineStr">
         <is>
-          <t>측정, 시험, 항해, 제어 및 기타 정밀기기 제조업</t>
+          <t>전자부품 제조업</t>
         </is>
       </c>
       <c r="J31" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K31" s="6" t="inlineStr">
@@ -2145,12 +2145,12 @@
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>바이다</t>
+          <t>아이알큐더스</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr">
@@ -2170,27 +2170,27 @@
       </c>
       <c r="F32" s="7" t="inlineStr">
         <is>
-          <t>14,432</t>
+          <t>10,231</t>
         </is>
       </c>
       <c r="G32" s="7" t="inlineStr">
         <is>
-          <t>-3,951</t>
+          <t>-986</t>
         </is>
       </c>
       <c r="H32" s="7" t="inlineStr">
         <is>
-          <t>15,108</t>
+          <t>1,800</t>
         </is>
       </c>
       <c r="I32" s="6" t="inlineStr">
         <is>
-          <t>전자부품 제조업</t>
+          <t>소프트웨어 개발 및 공급업</t>
         </is>
       </c>
       <c r="J32" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>DB</t>
         </is>
       </c>
       <c r="K32" s="6" t="inlineStr">
@@ -2202,12 +2202,12 @@
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>아이알큐더스</t>
+          <t>씨엔티테크</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
@@ -2227,17 +2227,17 @@
       </c>
       <c r="F33" s="7" t="inlineStr">
         <is>
-          <t>10,231</t>
+          <t>27,015</t>
         </is>
       </c>
       <c r="G33" s="7" t="inlineStr">
         <is>
-          <t>-986</t>
+          <t>3,987</t>
         </is>
       </c>
       <c r="H33" s="7" t="inlineStr">
         <is>
-          <t>1,800</t>
+          <t>2,613</t>
         </is>
       </c>
       <c r="I33" s="6" t="inlineStr">
@@ -2247,7 +2247,7 @@
       </c>
       <c r="J33" s="6" t="inlineStr">
         <is>
-          <t>DB</t>
+          <t>한화, 하나</t>
         </is>
       </c>
       <c r="K33" s="6" t="inlineStr">
@@ -2259,12 +2259,12 @@
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>씨엔티테크</t>
+          <t>삼홍아크튜리온</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
@@ -2284,27 +2284,27 @@
       </c>
       <c r="F34" s="7" t="inlineStr">
         <is>
-          <t>27,015</t>
+          <t>26,162</t>
         </is>
       </c>
       <c r="G34" s="7" t="inlineStr">
         <is>
-          <t>3,987</t>
+          <t>-10,314</t>
         </is>
       </c>
       <c r="H34" s="7" t="inlineStr">
         <is>
-          <t>2,613</t>
+          <t>6,369</t>
         </is>
       </c>
       <c r="I34" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어 개발 및 공급업</t>
+          <t>구조용 금속제품, 탱크 및 증기발생기 제조업</t>
         </is>
       </c>
       <c r="J34" s="6" t="inlineStr">
         <is>
-          <t>한화, 하나</t>
+          <t>삼성, 미래</t>
         </is>
       </c>
       <c r="K34" s="6" t="inlineStr">
@@ -2316,12 +2316,12 @@
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>삼홍아크튜리온</t>
+          <t>비앤비코리아</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
@@ -2341,27 +2341,27 @@
       </c>
       <c r="F35" s="7" t="inlineStr">
         <is>
-          <t>26,162</t>
+          <t>141,169</t>
         </is>
       </c>
       <c r="G35" s="7" t="inlineStr">
         <is>
-          <t>-10,314</t>
+          <t>21,406</t>
         </is>
       </c>
       <c r="H35" s="7" t="inlineStr">
         <is>
-          <t>6,369</t>
+          <t>43,932</t>
         </is>
       </c>
       <c r="I35" s="6" t="inlineStr">
         <is>
-          <t>구조용 금속제품, 탱크 및 증기발생기 제조업</t>
+          <t>기타 화학제품 제조업</t>
         </is>
       </c>
       <c r="J35" s="6" t="inlineStr">
         <is>
-          <t>삼성, 미래</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K35" s="6" t="inlineStr">
@@ -2373,12 +2373,12 @@
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>비앤비코리아</t>
+          <t>오토핸즈</t>
         </is>
       </c>
       <c r="C36" s="6" t="inlineStr">
@@ -2388,7 +2388,7 @@
       </c>
       <c r="D36" s="6" t="inlineStr">
         <is>
-          <t>신규상장</t>
+          <t>스팩 소멸합병</t>
         </is>
       </c>
       <c r="E36" s="6" t="inlineStr">
@@ -2398,22 +2398,22 @@
       </c>
       <c r="F36" s="7" t="inlineStr">
         <is>
-          <t>141,169</t>
+          <t>238,564</t>
         </is>
       </c>
       <c r="G36" s="7" t="inlineStr">
         <is>
-          <t>21,406</t>
+          <t>6,047</t>
         </is>
       </c>
       <c r="H36" s="7" t="inlineStr">
         <is>
-          <t>43,932</t>
+          <t>6,129</t>
         </is>
       </c>
       <c r="I36" s="6" t="inlineStr">
         <is>
-          <t>기타 화학제품 제조업</t>
+          <t>자동차 판매업</t>
         </is>
       </c>
       <c r="J36" s="6" t="inlineStr">
@@ -2430,12 +2430,12 @@
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>오토핸즈</t>
+          <t>아이벡스메디칼시스템즈</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
@@ -2445,7 +2445,7 @@
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
-          <t>스팩 소멸합병</t>
+          <t>신규상장</t>
         </is>
       </c>
       <c r="E37" s="6" t="inlineStr">
@@ -2455,27 +2455,27 @@
       </c>
       <c r="F37" s="7" t="inlineStr">
         <is>
-          <t>238,564</t>
+          <t>15,282</t>
         </is>
       </c>
       <c r="G37" s="7" t="inlineStr">
         <is>
-          <t>6,047</t>
+          <t>-7,227</t>
         </is>
       </c>
       <c r="H37" s="7" t="inlineStr">
         <is>
-          <t>6,129</t>
+          <t>744</t>
         </is>
       </c>
       <c r="I37" s="6" t="inlineStr">
         <is>
-          <t>자동차 판매업</t>
+          <t>의료용 기기 제조업</t>
         </is>
       </c>
       <c r="J37" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K37" s="6" t="inlineStr">
@@ -2487,12 +2487,12 @@
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>아이벡스메디칼시스템즈</t>
+          <t>피지티</t>
         </is>
       </c>
       <c r="C38" s="6" t="inlineStr">
@@ -2512,27 +2512,27 @@
       </c>
       <c r="F38" s="7" t="inlineStr">
         <is>
-          <t>15,282</t>
+          <t>40,141</t>
         </is>
       </c>
       <c r="G38" s="7" t="inlineStr">
         <is>
-          <t>-7,227</t>
+          <t>-69,722</t>
         </is>
       </c>
       <c r="H38" s="7" t="inlineStr">
         <is>
-          <t>744</t>
+          <t>6,029</t>
         </is>
       </c>
       <c r="I38" s="6" t="inlineStr">
         <is>
-          <t>의료용 기기 제조업</t>
+          <t>기타 화학제품 제조업</t>
         </is>
       </c>
       <c r="J38" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="K38" s="6" t="inlineStr">
@@ -2541,134 +2541,134 @@
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="6" t="inlineStr">
-        <is>
-          <t>2026-02-27</t>
-        </is>
-      </c>
-      <c r="B39" s="6" t="inlineStr">
-        <is>
-          <t>피지티</t>
-        </is>
-      </c>
-      <c r="C39" s="6" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>■ 심사 승인  (85건)</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="n"/>
+      <c r="C40" s="4" t="n"/>
+      <c r="D40" s="4" t="n"/>
+      <c r="E40" s="4" t="n"/>
+      <c r="F40" s="4" t="n"/>
+      <c r="G40" s="4" t="n"/>
+      <c r="H40" s="4" t="n"/>
+      <c r="I40" s="4" t="n"/>
+      <c r="J40" s="4" t="n"/>
+      <c r="K40" s="4" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>일자</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>회사명</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>시장</t>
+        </is>
+      </c>
+      <c r="D41" s="5" t="inlineStr">
+        <is>
+          <t>상장유형</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>기준연도</t>
+        </is>
+      </c>
+      <c r="F41" s="5" t="inlineStr">
+        <is>
+          <t>매출액</t>
+        </is>
+      </c>
+      <c r="G41" s="5" t="inlineStr">
+        <is>
+          <t>순이익</t>
+        </is>
+      </c>
+      <c r="H41" s="5" t="inlineStr">
+        <is>
+          <t>자기자본</t>
+        </is>
+      </c>
+      <c r="I41" s="5" t="inlineStr">
+        <is>
+          <t>업종</t>
+        </is>
+      </c>
+      <c r="J41" s="5" t="inlineStr">
+        <is>
+          <t>대표주관사</t>
+        </is>
+      </c>
+      <c r="K41" s="5" t="inlineStr">
+        <is>
+          <t>현황</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B42" s="6" t="inlineStr">
+        <is>
+          <t>인터엑스</t>
+        </is>
+      </c>
+      <c r="C42" s="6" t="inlineStr">
         <is>
           <t>코스닥</t>
         </is>
       </c>
-      <c r="D39" s="6" t="inlineStr">
+      <c r="D42" s="6" t="inlineStr">
         <is>
           <t>신규상장</t>
         </is>
       </c>
-      <c r="E39" s="6" t="inlineStr">
+      <c r="E42" s="6" t="inlineStr">
         <is>
           <t>FY25</t>
         </is>
       </c>
-      <c r="F39" s="7" t="inlineStr">
-        <is>
-          <t>40,141</t>
-        </is>
-      </c>
-      <c r="G39" s="7" t="inlineStr">
-        <is>
-          <t>-69,722</t>
-        </is>
-      </c>
-      <c r="H39" s="7" t="inlineStr">
-        <is>
-          <t>6,029</t>
-        </is>
-      </c>
-      <c r="I39" s="6" t="inlineStr">
-        <is>
-          <t>기타 화학제품 제조업</t>
-        </is>
-      </c>
-      <c r="J39" s="6" t="inlineStr">
+      <c r="F42" s="7" t="inlineStr">
+        <is>
+          <t>8,645</t>
+        </is>
+      </c>
+      <c r="G42" s="7" t="inlineStr">
+        <is>
+          <t>-20,272</t>
+        </is>
+      </c>
+      <c r="H42" s="7" t="inlineStr">
+        <is>
+          <t>4,530</t>
+        </is>
+      </c>
+      <c r="I42" s="6" t="inlineStr">
+        <is>
+          <t>소프트웨어 개발 및 공급업</t>
+        </is>
+      </c>
+      <c r="J42" s="6" t="inlineStr">
         <is>
           <t>한국</t>
         </is>
       </c>
-      <c r="K39" s="6" t="inlineStr">
-        <is>
-          <t>예심 진행중</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="3" t="inlineStr">
-        <is>
-          <t>■ 심사 승인  (84건)</t>
-        </is>
-      </c>
-      <c r="B41" s="4" t="n"/>
-      <c r="C41" s="4" t="n"/>
-      <c r="D41" s="4" t="n"/>
-      <c r="E41" s="4" t="n"/>
-      <c r="F41" s="4" t="n"/>
-      <c r="G41" s="4" t="n"/>
-      <c r="H41" s="4" t="n"/>
-      <c r="I41" s="4" t="n"/>
-      <c r="J41" s="4" t="n"/>
-      <c r="K41" s="4" t="n"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="5" t="inlineStr">
-        <is>
-          <t>일자</t>
-        </is>
-      </c>
-      <c r="B42" s="5" t="inlineStr">
-        <is>
-          <t>회사명</t>
-        </is>
-      </c>
-      <c r="C42" s="5" t="inlineStr">
-        <is>
-          <t>시장</t>
-        </is>
-      </c>
-      <c r="D42" s="5" t="inlineStr">
-        <is>
-          <t>상장유형</t>
-        </is>
-      </c>
-      <c r="E42" s="5" t="inlineStr">
-        <is>
-          <t>기준연도</t>
-        </is>
-      </c>
-      <c r="F42" s="5" t="inlineStr">
-        <is>
-          <t>매출액</t>
-        </is>
-      </c>
-      <c r="G42" s="5" t="inlineStr">
-        <is>
-          <t>순이익</t>
-        </is>
-      </c>
-      <c r="H42" s="5" t="inlineStr">
-        <is>
-          <t>자기자본</t>
-        </is>
-      </c>
-      <c r="I42" s="5" t="inlineStr">
-        <is>
-          <t>업종</t>
-        </is>
-      </c>
-      <c r="J42" s="5" t="inlineStr">
-        <is>
-          <t>대표주관사</t>
-        </is>
-      </c>
-      <c r="K42" s="5" t="inlineStr">
-        <is>
-          <t>현황</t>
+      <c r="K42" s="6" t="inlineStr">
+        <is>
+          <t>상장전</t>
         </is>
       </c>
     </row>
@@ -2680,7 +2680,7 @@
       </c>
       <c r="B43" s="6" t="inlineStr">
         <is>
-          <t>인터엑스</t>
+          <t>씨아이에스케미칼</t>
         </is>
       </c>
       <c r="C43" s="6" t="inlineStr">
@@ -2700,27 +2700,27 @@
       </c>
       <c r="F43" s="7" t="inlineStr">
         <is>
-          <t>8,645</t>
+          <t>15,985</t>
         </is>
       </c>
       <c r="G43" s="7" t="inlineStr">
         <is>
-          <t>-20,272</t>
+          <t>-11,440</t>
         </is>
       </c>
       <c r="H43" s="7" t="inlineStr">
         <is>
-          <t>4,530</t>
+          <t>23,706</t>
         </is>
       </c>
       <c r="I43" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어 개발 및 공급업</t>
+          <t>기초 화학물질 제조업</t>
         </is>
       </c>
       <c r="J43" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>KB</t>
         </is>
       </c>
       <c r="K43" s="6" t="inlineStr">
@@ -2737,12 +2737,12 @@
       </c>
       <c r="B44" s="6" t="inlineStr">
         <is>
-          <t>씨아이에스케미칼</t>
+          <t>에스에프씨</t>
         </is>
       </c>
       <c r="C44" s="6" t="inlineStr">
         <is>
-          <t>코스닥</t>
+          <t>유가</t>
         </is>
       </c>
       <c r="D44" s="6" t="inlineStr">
@@ -2757,27 +2757,27 @@
       </c>
       <c r="F44" s="7" t="inlineStr">
         <is>
-          <t>15,985</t>
+          <t>160,792</t>
         </is>
       </c>
       <c r="G44" s="7" t="inlineStr">
         <is>
-          <t>-11,440</t>
+          <t>25,509</t>
         </is>
       </c>
       <c r="H44" s="7" t="inlineStr">
         <is>
-          <t>23,706</t>
+          <t>243,562</t>
         </is>
       </c>
       <c r="I44" s="6" t="inlineStr">
         <is>
-          <t>기초 화학물질 제조업</t>
+          <t>기타 화학제품 제조업</t>
         </is>
       </c>
       <c r="J44" s="6" t="inlineStr">
         <is>
-          <t>KB</t>
+          <t>미래, 한국</t>
         </is>
       </c>
       <c r="K44" s="6" t="inlineStr">
@@ -4570,7 +4570,7 @@
       </c>
       <c r="K76" s="6" t="inlineStr">
         <is>
-          <t>상장전</t>
+          <t>상장승인(상장예정)</t>
         </is>
       </c>
     </row>
@@ -8521,7 +8521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R105"/>
+  <dimension ref="A1:R106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -12767,7 +12767,7 @@
     <row r="58" ht="22" customHeight="1">
       <c r="A58" s="3" t="inlineStr">
         <is>
-          <t>■ 공모 진행 (예심 승인법인)  (43건)</t>
+          <t>■ 공모 진행 (예심 승인법인)  (44건)</t>
         </is>
       </c>
       <c r="B58" s="4" t="n"/>
@@ -13023,67 +13023,67 @@
     <row r="62" ht="30" customHeight="1">
       <c r="A62" s="6" t="inlineStr">
         <is>
-          <t>에스케이증권제14호기업인수목적</t>
+          <t>티앤이코리아</t>
         </is>
       </c>
       <c r="B62" s="6" t="inlineStr">
         <is>
-          <t>10-12~10-13</t>
-        </is>
-      </c>
-      <c r="C62" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>10-07~10-14</t>
+        </is>
+      </c>
+      <c r="C62" s="6" t="inlineStr">
+        <is>
+          <t>12,600~15,300</t>
         </is>
       </c>
       <c r="D62" s="7" t="inlineStr">
         <is>
-          <t>6,500,000</t>
+          <t>2,400,000</t>
         </is>
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
-          <t>13,000,000,000</t>
-        </is>
-      </c>
-      <c r="F62" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>36,720,000,000</t>
+        </is>
+      </c>
+      <c r="F62" s="6" t="inlineStr">
+        <is>
+          <t>19.48배 (PER)</t>
         </is>
       </c>
       <c r="G62" s="6" t="inlineStr">
         <is>
-          <t>2,000</t>
+          <t>15,300</t>
         </is>
       </c>
       <c r="H62" s="6" t="n">
-        <v>1228.38</v>
+        <v>1041.02</v>
       </c>
       <c r="I62" s="6" t="n">
-        <v>1945</v>
+        <v>2274</v>
       </c>
       <c r="J62" s="6" t="inlineStr">
         <is>
-          <t>10-15~10-16</t>
+          <t>10-20~10-21</t>
         </is>
       </c>
       <c r="K62" s="6" t="inlineStr"/>
       <c r="L62" s="6" t="inlineStr"/>
       <c r="M62" s="6" t="inlineStr"/>
-      <c r="N62" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="N62" s="6" t="inlineStr">
+        <is>
+          <t>신한투자증권</t>
         </is>
       </c>
       <c r="O62" s="6" t="inlineStr"/>
-      <c r="P62" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="P62" s="7" t="inlineStr">
+        <is>
+          <t>1,245,888,000</t>
         </is>
       </c>
       <c r="Q62" s="6" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>4.0%</t>
         </is>
       </c>
       <c r="R62" s="6" t="inlineStr">
@@ -13095,64 +13095,72 @@
     <row r="63" ht="30" customHeight="1">
       <c r="A63" s="6" t="inlineStr">
         <is>
-          <t>티앤이코리아</t>
+          <t>에스케이증권제14호기업인수목적</t>
         </is>
       </c>
       <c r="B63" s="6" t="inlineStr">
         <is>
-          <t>10-07~10-14</t>
-        </is>
-      </c>
-      <c r="C63" s="6" t="inlineStr">
-        <is>
-          <t>12,600~15,300</t>
+          <t>10-12~10-13</t>
+        </is>
+      </c>
+      <c r="C63" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="D63" s="7" t="inlineStr">
         <is>
-          <t>2,400,000</t>
+          <t>6,500,000</t>
         </is>
       </c>
       <c r="E63" s="7" t="inlineStr">
         <is>
-          <t>30,240,000,000</t>
-        </is>
-      </c>
-      <c r="F63" s="6" t="inlineStr">
-        <is>
-          <t>19.48배 (PER)</t>
-        </is>
-      </c>
-      <c r="G63" s="6" t="inlineStr"/>
-      <c r="H63" s="6" t="inlineStr"/>
-      <c r="I63" s="6" t="inlineStr"/>
+          <t>13,000,000,000</t>
+        </is>
+      </c>
+      <c r="F63" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="G63" s="6" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
+      </c>
+      <c r="H63" s="6" t="n">
+        <v>1228.38</v>
+      </c>
+      <c r="I63" s="6" t="n">
+        <v>1945</v>
+      </c>
       <c r="J63" s="6" t="inlineStr">
         <is>
-          <t>10-20~10-21</t>
+          <t>10-15~10-16</t>
         </is>
       </c>
       <c r="K63" s="6" t="inlineStr"/>
       <c r="L63" s="6" t="inlineStr"/>
       <c r="M63" s="6" t="inlineStr"/>
-      <c r="N63" s="6" t="inlineStr">
-        <is>
-          <t>신한투자증권</t>
+      <c r="N63" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="O63" s="6" t="inlineStr"/>
-      <c r="P63" s="7" t="inlineStr">
-        <is>
-          <t>1,245,888,000</t>
+      <c r="P63" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="Q63" s="6" t="inlineStr">
         <is>
-          <t>4.0%</t>
+          <t>50%</t>
         </is>
       </c>
       <c r="R63" s="6" t="inlineStr">
         <is>
-          <t>정정</t>
+          <t>발행조건확정</t>
         </is>
       </c>
     </row>
@@ -13607,32 +13615,32 @@
     <row r="71" ht="30" customHeight="1">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>에이엘로봇</t>
+          <t>넥스아이</t>
         </is>
       </c>
       <c r="B71" s="6" t="inlineStr">
         <is>
-          <t>10-28~11-03</t>
+          <t>10-22~10-28</t>
         </is>
       </c>
       <c r="C71" s="6" t="inlineStr">
         <is>
-          <t>15,700~17,600</t>
+          <t>10,500~13,000</t>
         </is>
       </c>
       <c r="D71" s="7" t="inlineStr">
         <is>
-          <t>2,400,000</t>
+          <t>5,000,000</t>
         </is>
       </c>
       <c r="E71" s="7" t="inlineStr">
         <is>
-          <t>37,680,000,000</t>
+          <t>52,500,000,000</t>
         </is>
       </c>
       <c r="F71" s="6" t="inlineStr">
         <is>
-          <t>37.17배 (PER)</t>
+          <t>19.15배 (PER)</t>
         </is>
       </c>
       <c r="G71" s="6" t="inlineStr"/>
@@ -13640,7 +13648,7 @@
       <c r="I71" s="6" t="inlineStr"/>
       <c r="J71" s="6" t="inlineStr">
         <is>
-          <t>11-06~11-09</t>
+          <t>11-03~11-04</t>
         </is>
       </c>
       <c r="K71" s="6" t="inlineStr"/>
@@ -13648,18 +13656,18 @@
       <c r="M71" s="6" t="inlineStr"/>
       <c r="N71" s="6" t="inlineStr">
         <is>
-          <t>대신증권</t>
+          <t>한국투자증권</t>
         </is>
       </c>
       <c r="O71" s="6" t="inlineStr"/>
       <c r="P71" s="7" t="inlineStr">
         <is>
-          <t>1,160,399,874</t>
+          <t>2,407,500,000</t>
         </is>
       </c>
       <c r="Q71" s="6" t="inlineStr">
         <is>
-          <t>3.0%</t>
+          <t>4.5%</t>
         </is>
       </c>
       <c r="R71" s="6" t="inlineStr">
@@ -13671,32 +13679,32 @@
     <row r="72" ht="30" customHeight="1">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>엠비디</t>
+          <t>에이엘로봇</t>
         </is>
       </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>11-02~11-06</t>
+          <t>10-28~11-03</t>
         </is>
       </c>
       <c r="C72" s="6" t="inlineStr">
         <is>
-          <t>9,600~11,700</t>
+          <t>15,700~17,600</t>
         </is>
       </c>
       <c r="D72" s="7" t="inlineStr">
         <is>
-          <t>2,000,000</t>
+          <t>2,400,000</t>
         </is>
       </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
-          <t>19,200,000,000</t>
+          <t>37,680,000,000</t>
         </is>
       </c>
       <c r="F72" s="6" t="inlineStr">
         <is>
-          <t>27.36배 (PER)</t>
+          <t>37.17배 (PER)</t>
         </is>
       </c>
       <c r="G72" s="6" t="inlineStr"/>
@@ -13704,7 +13712,7 @@
       <c r="I72" s="6" t="inlineStr"/>
       <c r="J72" s="6" t="inlineStr">
         <is>
-          <t>11-12~11-13</t>
+          <t>11-06~11-09</t>
         </is>
       </c>
       <c r="K72" s="6" t="inlineStr"/>
@@ -13712,18 +13720,18 @@
       <c r="M72" s="6" t="inlineStr"/>
       <c r="N72" s="6" t="inlineStr">
         <is>
-          <t>하나증권</t>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="O72" s="6" t="inlineStr"/>
       <c r="P72" s="7" t="inlineStr">
         <is>
-          <t>988,800,000</t>
+          <t>1,160,399,874</t>
         </is>
       </c>
       <c r="Q72" s="6" t="inlineStr">
         <is>
-          <t>5.0%</t>
+          <t>3.0%</t>
         </is>
       </c>
       <c r="R72" s="6" t="inlineStr">
@@ -13735,7 +13743,7 @@
     <row r="73" ht="30" customHeight="1">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>다비오</t>
+          <t>엠비디</t>
         </is>
       </c>
       <c r="B73" s="6" t="inlineStr">
@@ -13745,22 +13753,22 @@
       </c>
       <c r="C73" s="6" t="inlineStr">
         <is>
-          <t>12,300~16,600</t>
+          <t>9,600~11,700</t>
         </is>
       </c>
       <c r="D73" s="7" t="inlineStr">
         <is>
-          <t>1,000,000</t>
+          <t>2,000,000</t>
         </is>
       </c>
       <c r="E73" s="7" t="inlineStr">
         <is>
-          <t>12,300,000,000</t>
+          <t>19,200,000,000</t>
         </is>
       </c>
       <c r="F73" s="6" t="inlineStr">
         <is>
-          <t>26.70배 (PER)</t>
+          <t>27.36배 (PER)</t>
         </is>
       </c>
       <c r="G73" s="6" t="inlineStr"/>
@@ -13768,7 +13776,7 @@
       <c r="I73" s="6" t="inlineStr"/>
       <c r="J73" s="6" t="inlineStr">
         <is>
-          <t>11-10~11-11</t>
+          <t>11-12~11-13</t>
         </is>
       </c>
       <c r="K73" s="6" t="inlineStr"/>
@@ -13776,18 +13784,18 @@
       <c r="M73" s="6" t="inlineStr"/>
       <c r="N73" s="6" t="inlineStr">
         <is>
-          <t>대신증권</t>
+          <t>하나증권</t>
         </is>
       </c>
       <c r="O73" s="6" t="inlineStr"/>
       <c r="P73" s="7" t="inlineStr">
         <is>
-          <t>570,105,000</t>
+          <t>988,800,000</t>
         </is>
       </c>
       <c r="Q73" s="6" t="inlineStr">
         <is>
-          <t>4.5%</t>
+          <t>5.0%</t>
         </is>
       </c>
       <c r="R73" s="6" t="inlineStr">
@@ -13799,59 +13807,59 @@
     <row r="74" ht="30" customHeight="1">
       <c r="A74" s="6" t="inlineStr">
         <is>
-          <t>바로팜</t>
-        </is>
-      </c>
-      <c r="B74" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>다비오</t>
+        </is>
+      </c>
+      <c r="B74" s="6" t="inlineStr">
+        <is>
+          <t>11-02~11-06</t>
         </is>
       </c>
       <c r="C74" s="6" t="inlineStr">
         <is>
-          <t>16,400~20,200</t>
+          <t>12,300~16,600</t>
         </is>
       </c>
       <c r="D74" s="7" t="inlineStr">
         <is>
-          <t>1,780,000</t>
+          <t>1,000,000</t>
         </is>
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
-          <t>29,192,000,000</t>
+          <t>12,300,000,000</t>
         </is>
       </c>
       <c r="F74" s="6" t="inlineStr">
         <is>
-          <t>25.27배 (PER)</t>
+          <t>26.70배 (PER)</t>
         </is>
       </c>
       <c r="G74" s="6" t="inlineStr"/>
       <c r="H74" s="6" t="inlineStr"/>
       <c r="I74" s="6" t="inlineStr"/>
-      <c r="J74" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="J74" s="6" t="inlineStr">
+        <is>
+          <t>11-10~11-11</t>
         </is>
       </c>
       <c r="K74" s="6" t="inlineStr"/>
       <c r="L74" s="6" t="inlineStr"/>
       <c r="M74" s="6" t="inlineStr"/>
-      <c r="N74" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="N74" s="6" t="inlineStr">
+        <is>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="O74" s="6" t="inlineStr"/>
-      <c r="P74" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="Q74" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="P74" s="7" t="inlineStr">
+        <is>
+          <t>570,105,000</t>
+        </is>
+      </c>
+      <c r="Q74" s="6" t="inlineStr">
+        <is>
+          <t>4.5%</t>
         </is>
       </c>
       <c r="R74" s="6" t="inlineStr">
@@ -13863,54 +13871,54 @@
     <row r="75" ht="30" customHeight="1">
       <c r="A75" s="6" t="inlineStr">
         <is>
-          <t>셀트릭스</t>
-        </is>
-      </c>
-      <c r="B75" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="C75" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="D75" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="E75" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="F75" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>하나에어로다이내믹스</t>
+        </is>
+      </c>
+      <c r="B75" s="6" t="inlineStr">
+        <is>
+          <t>11-02~11-06</t>
+        </is>
+      </c>
+      <c r="C75" s="6" t="inlineStr">
+        <is>
+          <t>4,700~5,700</t>
+        </is>
+      </c>
+      <c r="D75" s="7" t="inlineStr">
+        <is>
+          <t>4,400,000</t>
+        </is>
+      </c>
+      <c r="E75" s="7" t="inlineStr">
+        <is>
+          <t>20,680,000,000</t>
+        </is>
+      </c>
+      <c r="F75" s="6" t="inlineStr">
+        <is>
+          <t>17.89배 (EV/EBITDA)</t>
         </is>
       </c>
       <c r="G75" s="6" t="inlineStr"/>
       <c r="H75" s="6" t="inlineStr"/>
       <c r="I75" s="6" t="inlineStr"/>
-      <c r="J75" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="J75" s="6" t="inlineStr">
+        <is>
+          <t>11-10~11-11</t>
         </is>
       </c>
       <c r="K75" s="6" t="inlineStr"/>
       <c r="L75" s="6" t="inlineStr"/>
       <c r="M75" s="6" t="inlineStr"/>
-      <c r="N75" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="N75" s="6" t="inlineStr">
+        <is>
+          <t>아이비케이투자증권</t>
         </is>
       </c>
       <c r="O75" s="6" t="inlineStr"/>
-      <c r="P75" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="P75" s="7" t="inlineStr">
+        <is>
+          <t>850,000,000</t>
         </is>
       </c>
       <c r="Q75" s="18" t="inlineStr">
@@ -13927,7 +13935,7 @@
     <row r="76" ht="30" customHeight="1">
       <c r="A76" s="6" t="inlineStr">
         <is>
-          <t>솔리스</t>
+          <t>바로팜</t>
         </is>
       </c>
       <c r="B76" s="18" t="inlineStr">
@@ -13935,24 +13943,24 @@
           <t>수집예정</t>
         </is>
       </c>
-      <c r="C76" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="D76" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="E76" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="F76" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="C76" s="6" t="inlineStr">
+        <is>
+          <t>16,400~20,200</t>
+        </is>
+      </c>
+      <c r="D76" s="7" t="inlineStr">
+        <is>
+          <t>1,780,000</t>
+        </is>
+      </c>
+      <c r="E76" s="7" t="inlineStr">
+        <is>
+          <t>29,192,000,000</t>
+        </is>
+      </c>
+      <c r="F76" s="6" t="inlineStr">
+        <is>
+          <t>25.27배 (PER)</t>
         </is>
       </c>
       <c r="G76" s="6" t="inlineStr"/>
@@ -13991,209 +13999,209 @@
     <row r="77" ht="30" customHeight="1">
       <c r="A77" s="6" t="inlineStr">
         <is>
-          <t>옵토닉스</t>
-        </is>
-      </c>
-      <c r="B77" s="6" t="inlineStr">
-        <is>
-          <t>10-21~10-27</t>
-        </is>
-      </c>
-      <c r="C77" s="6" t="inlineStr">
-        <is>
-          <t>10,000~12,000</t>
-        </is>
-      </c>
-      <c r="D77" s="7" t="inlineStr">
-        <is>
-          <t>2,200,000</t>
-        </is>
-      </c>
-      <c r="E77" s="7" t="inlineStr">
-        <is>
-          <t>22,000,000,000</t>
-        </is>
-      </c>
-      <c r="F77" s="6" t="inlineStr">
-        <is>
-          <t>25.27배 (EV/EBITDA)</t>
+          <t>셀트릭스</t>
+        </is>
+      </c>
+      <c r="B77" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="C77" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="D77" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="E77" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="F77" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="G77" s="6" t="inlineStr"/>
       <c r="H77" s="6" t="inlineStr"/>
       <c r="I77" s="6" t="inlineStr"/>
-      <c r="J77" s="6" t="inlineStr">
-        <is>
-          <t>11-05~11-06</t>
+      <c r="J77" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="K77" s="6" t="inlineStr"/>
       <c r="L77" s="6" t="inlineStr"/>
       <c r="M77" s="6" t="inlineStr"/>
-      <c r="N77" s="6" t="inlineStr">
-        <is>
-          <t>한국투자증권</t>
+      <c r="N77" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="O77" s="6" t="inlineStr"/>
-      <c r="P77" s="7" t="inlineStr">
-        <is>
-          <t>1,133,000,000</t>
-        </is>
-      </c>
-      <c r="Q77" s="6" t="inlineStr">
-        <is>
-          <t>5.0%</t>
+      <c r="P77" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="Q77" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="R77" s="6" t="inlineStr">
         <is>
-          <t>최초</t>
+          <t>정정</t>
         </is>
       </c>
     </row>
     <row r="78" ht="30" customHeight="1">
       <c r="A78" s="6" t="inlineStr">
         <is>
-          <t>동원파츠</t>
-        </is>
-      </c>
-      <c r="B78" s="6" t="inlineStr">
-        <is>
-          <t>10-22~10-28</t>
-        </is>
-      </c>
-      <c r="C78" s="6" t="inlineStr">
-        <is>
-          <t>23,000~26,500</t>
-        </is>
-      </c>
-      <c r="D78" s="7" t="inlineStr">
-        <is>
-          <t>2,030,000</t>
-        </is>
-      </c>
-      <c r="E78" s="7" t="inlineStr">
-        <is>
-          <t>46,690,000,000</t>
-        </is>
-      </c>
-      <c r="F78" s="6" t="inlineStr">
-        <is>
-          <t>22.91배 (PER)</t>
+          <t>럭스코</t>
+        </is>
+      </c>
+      <c r="B78" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="C78" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="D78" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="E78" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="F78" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="G78" s="6" t="inlineStr"/>
       <c r="H78" s="6" t="inlineStr"/>
       <c r="I78" s="6" t="inlineStr"/>
-      <c r="J78" s="6" t="inlineStr">
-        <is>
-          <t>11-02~11-03</t>
+      <c r="J78" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="K78" s="6" t="inlineStr"/>
       <c r="L78" s="6" t="inlineStr"/>
       <c r="M78" s="6" t="inlineStr"/>
-      <c r="N78" s="6" t="inlineStr">
-        <is>
-          <t>삼성증권</t>
+      <c r="N78" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="O78" s="6" t="inlineStr"/>
-      <c r="P78" s="7" t="inlineStr">
-        <is>
-          <t>1,430,699,820</t>
-        </is>
-      </c>
-      <c r="Q78" s="6" t="inlineStr">
-        <is>
-          <t>3.0%</t>
+      <c r="P78" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="Q78" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="R78" s="6" t="inlineStr">
         <is>
-          <t>최초</t>
+          <t>정정</t>
         </is>
       </c>
     </row>
     <row r="79" ht="30" customHeight="1">
       <c r="A79" s="6" t="inlineStr">
         <is>
-          <t>넥스아이</t>
-        </is>
-      </c>
-      <c r="B79" s="6" t="inlineStr">
-        <is>
-          <t>10-22~10-28</t>
-        </is>
-      </c>
-      <c r="C79" s="6" t="inlineStr">
-        <is>
-          <t>10,500~13,000</t>
-        </is>
-      </c>
-      <c r="D79" s="7" t="inlineStr">
-        <is>
-          <t>5,000,000</t>
-        </is>
-      </c>
-      <c r="E79" s="7" t="inlineStr">
-        <is>
-          <t>52,500,000,000</t>
-        </is>
-      </c>
-      <c r="F79" s="6" t="inlineStr">
-        <is>
-          <t>19.15배 (PER)</t>
+          <t>솔리스</t>
+        </is>
+      </c>
+      <c r="B79" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="C79" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="D79" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="E79" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="F79" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="G79" s="6" t="inlineStr"/>
       <c r="H79" s="6" t="inlineStr"/>
       <c r="I79" s="6" t="inlineStr"/>
-      <c r="J79" s="6" t="inlineStr">
-        <is>
-          <t>11-03~11-04</t>
+      <c r="J79" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="K79" s="6" t="inlineStr"/>
       <c r="L79" s="6" t="inlineStr"/>
       <c r="M79" s="6" t="inlineStr"/>
-      <c r="N79" s="6" t="inlineStr">
-        <is>
-          <t>한국투자증권</t>
+      <c r="N79" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="O79" s="6" t="inlineStr"/>
-      <c r="P79" s="7" t="inlineStr">
-        <is>
-          <t>2,407,500,000</t>
-        </is>
-      </c>
-      <c r="Q79" s="6" t="inlineStr">
-        <is>
-          <t>4.5%</t>
+      <c r="P79" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="Q79" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="R79" s="6" t="inlineStr">
         <is>
-          <t>최초</t>
+          <t>정정</t>
         </is>
       </c>
     </row>
     <row r="80" ht="30" customHeight="1">
       <c r="A80" s="6" t="inlineStr">
         <is>
-          <t>제논</t>
+          <t>옵토닉스</t>
         </is>
       </c>
       <c r="B80" s="6" t="inlineStr">
         <is>
-          <t>10-26~10-30</t>
+          <t>10-21~10-27</t>
         </is>
       </c>
       <c r="C80" s="6" t="inlineStr">
         <is>
-          <t>9,700~12,200</t>
+          <t>10,000~12,000</t>
         </is>
       </c>
       <c r="D80" s="7" t="inlineStr">
@@ -14203,12 +14211,12 @@
       </c>
       <c r="E80" s="7" t="inlineStr">
         <is>
-          <t>21,340,000,000</t>
+          <t>22,000,000,000</t>
         </is>
       </c>
       <c r="F80" s="6" t="inlineStr">
         <is>
-          <t>36.49배 (PER)</t>
+          <t>25.27배 (EV/EBITDA)</t>
         </is>
       </c>
       <c r="G80" s="6" t="inlineStr"/>
@@ -14216,7 +14224,7 @@
       <c r="I80" s="6" t="inlineStr"/>
       <c r="J80" s="6" t="inlineStr">
         <is>
-          <t>11-04~11-05</t>
+          <t>11-05~11-06</t>
         </is>
       </c>
       <c r="K80" s="6" t="inlineStr"/>
@@ -14224,18 +14232,18 @@
       <c r="M80" s="6" t="inlineStr"/>
       <c r="N80" s="6" t="inlineStr">
         <is>
-          <t>삼성증권</t>
+          <t>한국투자증권</t>
         </is>
       </c>
       <c r="O80" s="6" t="inlineStr"/>
       <c r="P80" s="7" t="inlineStr">
         <is>
-          <t>835,247,600</t>
+          <t>1,133,000,000</t>
         </is>
       </c>
       <c r="Q80" s="6" t="inlineStr">
         <is>
-          <t>3.80%</t>
+          <t>5.0%</t>
         </is>
       </c>
       <c r="R80" s="6" t="inlineStr">
@@ -14247,27 +14255,27 @@
     <row r="81" ht="30" customHeight="1">
       <c r="A81" s="6" t="inlineStr">
         <is>
-          <t>영광와이케이엠씨</t>
+          <t>동원파츠</t>
         </is>
       </c>
       <c r="B81" s="6" t="inlineStr">
         <is>
-          <t>10-27~11-02</t>
+          <t>10-22~10-28</t>
         </is>
       </c>
       <c r="C81" s="6" t="inlineStr">
         <is>
-          <t>9,400~11,000</t>
+          <t>23,000~26,500</t>
         </is>
       </c>
       <c r="D81" s="7" t="inlineStr">
         <is>
-          <t>2,300,000</t>
+          <t>2,030,000</t>
         </is>
       </c>
       <c r="E81" s="7" t="inlineStr">
         <is>
-          <t>21,620,000,000</t>
+          <t>46,690,000,000</t>
         </is>
       </c>
       <c r="F81" s="6" t="inlineStr">
@@ -14280,7 +14288,7 @@
       <c r="I81" s="6" t="inlineStr"/>
       <c r="J81" s="6" t="inlineStr">
         <is>
-          <t>11-04~11-05</t>
+          <t>11-02~11-03</t>
         </is>
       </c>
       <c r="K81" s="6" t="inlineStr"/>
@@ -14288,18 +14296,18 @@
       <c r="M81" s="6" t="inlineStr"/>
       <c r="N81" s="6" t="inlineStr">
         <is>
-          <t>대신증권</t>
+          <t>삼성증권</t>
         </is>
       </c>
       <c r="O81" s="6" t="inlineStr"/>
       <c r="P81" s="7" t="inlineStr">
         <is>
-          <t>1,002,087,000</t>
+          <t>1,430,699,820</t>
         </is>
       </c>
       <c r="Q81" s="6" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>3.0%</t>
         </is>
       </c>
       <c r="R81" s="6" t="inlineStr">
@@ -14311,32 +14319,32 @@
     <row r="82" ht="30" customHeight="1">
       <c r="A82" s="6" t="inlineStr">
         <is>
-          <t>하나에어로다이내믹스</t>
+          <t>제논</t>
         </is>
       </c>
       <c r="B82" s="6" t="inlineStr">
         <is>
-          <t>11-02~11-06</t>
+          <t>10-26~10-30</t>
         </is>
       </c>
       <c r="C82" s="6" t="inlineStr">
         <is>
-          <t>4,700~5,700</t>
+          <t>9,700~12,200</t>
         </is>
       </c>
       <c r="D82" s="7" t="inlineStr">
         <is>
-          <t>4,400,000</t>
+          <t>2,200,000</t>
         </is>
       </c>
       <c r="E82" s="7" t="inlineStr">
         <is>
-          <t>20,680,000,000</t>
+          <t>21,340,000,000</t>
         </is>
       </c>
       <c r="F82" s="6" t="inlineStr">
         <is>
-          <t>17.89배 (EV/EBITDA)</t>
+          <t>36.49배 (PER)</t>
         </is>
       </c>
       <c r="G82" s="6" t="inlineStr"/>
@@ -14344,7 +14352,7 @@
       <c r="I82" s="6" t="inlineStr"/>
       <c r="J82" s="6" t="inlineStr">
         <is>
-          <t>11-10~11-11</t>
+          <t>11-04~11-05</t>
         </is>
       </c>
       <c r="K82" s="6" t="inlineStr"/>
@@ -14352,18 +14360,18 @@
       <c r="M82" s="6" t="inlineStr"/>
       <c r="N82" s="6" t="inlineStr">
         <is>
-          <t>아이비케이투자증권</t>
+          <t>삼성증권</t>
         </is>
       </c>
       <c r="O82" s="6" t="inlineStr"/>
       <c r="P82" s="7" t="inlineStr">
         <is>
-          <t>850,000,000</t>
-        </is>
-      </c>
-      <c r="Q82" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>835,247,600</t>
+        </is>
+      </c>
+      <c r="Q82" s="6" t="inlineStr">
+        <is>
+          <t>3.80%</t>
         </is>
       </c>
       <c r="R82" s="6" t="inlineStr">
@@ -14375,32 +14383,32 @@
     <row r="83" ht="30" customHeight="1">
       <c r="A83" s="6" t="inlineStr">
         <is>
-          <t>엔키화이트햇</t>
+          <t>영광와이케이엠씨</t>
         </is>
       </c>
       <c r="B83" s="6" t="inlineStr">
         <is>
-          <t>11-03~11-09</t>
+          <t>10-27~11-02</t>
         </is>
       </c>
       <c r="C83" s="6" t="inlineStr">
         <is>
-          <t>13,000~16,500</t>
+          <t>9,400~11,000</t>
         </is>
       </c>
       <c r="D83" s="7" t="inlineStr">
         <is>
-          <t>1,700,000</t>
+          <t>2,300,000</t>
         </is>
       </c>
       <c r="E83" s="7" t="inlineStr">
         <is>
-          <t>22,100,000,000</t>
+          <t>21,620,000,000</t>
         </is>
       </c>
       <c r="F83" s="6" t="inlineStr">
         <is>
-          <t>24.86배 (PER)</t>
+          <t>22.91배 (PER)</t>
         </is>
       </c>
       <c r="G83" s="6" t="inlineStr"/>
@@ -14408,7 +14416,7 @@
       <c r="I83" s="6" t="inlineStr"/>
       <c r="J83" s="6" t="inlineStr">
         <is>
-          <t>11-12~11-13</t>
+          <t>11-04~11-05</t>
         </is>
       </c>
       <c r="K83" s="6" t="inlineStr"/>
@@ -14416,18 +14424,18 @@
       <c r="M83" s="6" t="inlineStr"/>
       <c r="N83" s="6" t="inlineStr">
         <is>
-          <t>신영증권</t>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="O83" s="6" t="inlineStr"/>
       <c r="P83" s="7" t="inlineStr">
         <is>
-          <t>1,138,150,000</t>
+          <t>1,002,087,000</t>
         </is>
       </c>
       <c r="Q83" s="6" t="inlineStr">
         <is>
-          <t>5.0%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="R83" s="6" t="inlineStr">
@@ -14439,32 +14447,32 @@
     <row r="84" ht="30" customHeight="1">
       <c r="A84" s="6" t="inlineStr">
         <is>
-          <t>아델</t>
+          <t>엔키화이트햇</t>
         </is>
       </c>
       <c r="B84" s="6" t="inlineStr">
         <is>
-          <t>11-12~11-18</t>
+          <t>11-03~11-09</t>
         </is>
       </c>
       <c r="C84" s="6" t="inlineStr">
         <is>
-          <t>18,000~25,000</t>
+          <t>13,000~16,500</t>
         </is>
       </c>
       <c r="D84" s="7" t="inlineStr">
         <is>
-          <t>2,170,000</t>
+          <t>1,700,000</t>
         </is>
       </c>
       <c r="E84" s="7" t="inlineStr">
         <is>
-          <t>39,060,000,000</t>
+          <t>22,100,000,000</t>
         </is>
       </c>
       <c r="F84" s="6" t="inlineStr">
         <is>
-          <t>20.91배 (PER)</t>
+          <t>24.86배 (PER)</t>
         </is>
       </c>
       <c r="G84" s="6" t="inlineStr"/>
@@ -14472,7 +14480,7 @@
       <c r="I84" s="6" t="inlineStr"/>
       <c r="J84" s="6" t="inlineStr">
         <is>
-          <t>11-23~11-24</t>
+          <t>11-12~11-13</t>
         </is>
       </c>
       <c r="K84" s="6" t="inlineStr"/>
@@ -14480,18 +14488,18 @@
       <c r="M84" s="6" t="inlineStr"/>
       <c r="N84" s="6" t="inlineStr">
         <is>
-          <t>삼성증권㈜</t>
+          <t>신영증권</t>
         </is>
       </c>
       <c r="O84" s="6" t="inlineStr"/>
       <c r="P84" s="7" t="inlineStr">
         <is>
-          <t>1,041,559,920</t>
+          <t>1,138,150,000</t>
         </is>
       </c>
       <c r="Q84" s="6" t="inlineStr">
         <is>
-          <t>4.0%</t>
+          <t>5.0%</t>
         </is>
       </c>
       <c r="R84" s="6" t="inlineStr">
@@ -14503,32 +14511,32 @@
     <row r="85" ht="30" customHeight="1">
       <c r="A85" s="6" t="inlineStr">
         <is>
-          <t>케이엠에프</t>
+          <t>제이앤티지</t>
         </is>
       </c>
       <c r="B85" s="6" t="inlineStr">
         <is>
-          <t>11-16~11-20</t>
+          <t>11-03~11-09</t>
         </is>
       </c>
       <c r="C85" s="6" t="inlineStr">
         <is>
-          <t>15,000~17,800</t>
+          <t>26,400~31,900</t>
         </is>
       </c>
       <c r="D85" s="7" t="inlineStr">
         <is>
-          <t>2,000,000</t>
+          <t>4,300,000</t>
         </is>
       </c>
       <c r="E85" s="7" t="inlineStr">
         <is>
-          <t>30,000,000,000</t>
+          <t>113,520,000,000</t>
         </is>
       </c>
       <c r="F85" s="6" t="inlineStr">
         <is>
-          <t>18.53배 (PER)</t>
+          <t>21.25배 (EV/EBITDA)</t>
         </is>
       </c>
       <c r="G85" s="6" t="inlineStr"/>
@@ -14536,7 +14544,7 @@
       <c r="I85" s="6" t="inlineStr"/>
       <c r="J85" s="6" t="inlineStr">
         <is>
-          <t>11-24~11-25</t>
+          <t>11-12~11-13</t>
         </is>
       </c>
       <c r="K85" s="6" t="inlineStr"/>
@@ -14544,18 +14552,22 @@
       <c r="M85" s="6" t="inlineStr"/>
       <c r="N85" s="6" t="inlineStr">
         <is>
-          <t>아이비케이투자증권</t>
-        </is>
-      </c>
-      <c r="O85" s="6" t="inlineStr"/>
+          <t>대신증권</t>
+        </is>
+      </c>
+      <c r="O85" s="6" t="inlineStr">
+        <is>
+          <t>NH</t>
+        </is>
+      </c>
       <c r="P85" s="7" t="inlineStr">
         <is>
-          <t>927,000,000</t>
+          <t>2,147,249,940</t>
         </is>
       </c>
       <c r="Q85" s="6" t="inlineStr">
         <is>
-          <t>3.0%</t>
+          <t>2.5%</t>
         </is>
       </c>
       <c r="R85" s="6" t="inlineStr">
@@ -14567,59 +14579,59 @@
     <row r="86" ht="30" customHeight="1">
       <c r="A86" s="6" t="inlineStr">
         <is>
-          <t>럭스코</t>
-        </is>
-      </c>
-      <c r="B86" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="C86" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="D86" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="E86" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="F86" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>아델</t>
+        </is>
+      </c>
+      <c r="B86" s="6" t="inlineStr">
+        <is>
+          <t>11-12~11-18</t>
+        </is>
+      </c>
+      <c r="C86" s="6" t="inlineStr">
+        <is>
+          <t>18,000~25,000</t>
+        </is>
+      </c>
+      <c r="D86" s="7" t="inlineStr">
+        <is>
+          <t>2,170,000</t>
+        </is>
+      </c>
+      <c r="E86" s="7" t="inlineStr">
+        <is>
+          <t>39,060,000,000</t>
+        </is>
+      </c>
+      <c r="F86" s="6" t="inlineStr">
+        <is>
+          <t>20.91배 (PER)</t>
         </is>
       </c>
       <c r="G86" s="6" t="inlineStr"/>
       <c r="H86" s="6" t="inlineStr"/>
       <c r="I86" s="6" t="inlineStr"/>
-      <c r="J86" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="J86" s="6" t="inlineStr">
+        <is>
+          <t>11-23~11-24</t>
         </is>
       </c>
       <c r="K86" s="6" t="inlineStr"/>
       <c r="L86" s="6" t="inlineStr"/>
       <c r="M86" s="6" t="inlineStr"/>
-      <c r="N86" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="N86" s="6" t="inlineStr">
+        <is>
+          <t>삼성증권㈜</t>
         </is>
       </c>
       <c r="O86" s="6" t="inlineStr"/>
-      <c r="P86" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="Q86" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="P86" s="7" t="inlineStr">
+        <is>
+          <t>1,041,559,920</t>
+        </is>
+      </c>
+      <c r="Q86" s="6" t="inlineStr">
+        <is>
+          <t>4.0%</t>
         </is>
       </c>
       <c r="R86" s="6" t="inlineStr">
@@ -14631,71 +14643,71 @@
     <row r="87" ht="30" customHeight="1">
       <c r="A87" s="6" t="inlineStr">
         <is>
-          <t>(주)태석광학</t>
-        </is>
-      </c>
-      <c r="B87" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="C87" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="D87" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="E87" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="F87" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>케이엠에프</t>
+        </is>
+      </c>
+      <c r="B87" s="6" t="inlineStr">
+        <is>
+          <t>11-16~11-20</t>
+        </is>
+      </c>
+      <c r="C87" s="6" t="inlineStr">
+        <is>
+          <t>15,000~17,800</t>
+        </is>
+      </c>
+      <c r="D87" s="7" t="inlineStr">
+        <is>
+          <t>2,000,000</t>
+        </is>
+      </c>
+      <c r="E87" s="7" t="inlineStr">
+        <is>
+          <t>30,000,000,000</t>
+        </is>
+      </c>
+      <c r="F87" s="6" t="inlineStr">
+        <is>
+          <t>18.53배 (PER)</t>
         </is>
       </c>
       <c r="G87" s="6" t="inlineStr"/>
       <c r="H87" s="6" t="inlineStr"/>
       <c r="I87" s="6" t="inlineStr"/>
-      <c r="J87" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="J87" s="6" t="inlineStr">
+        <is>
+          <t>11-24~11-25</t>
         </is>
       </c>
       <c r="K87" s="6" t="inlineStr"/>
       <c r="L87" s="6" t="inlineStr"/>
       <c r="M87" s="6" t="inlineStr"/>
-      <c r="N87" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="N87" s="6" t="inlineStr">
+        <is>
+          <t>아이비케이투자증권</t>
         </is>
       </c>
       <c r="O87" s="6" t="inlineStr"/>
-      <c r="P87" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="Q87" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="P87" s="7" t="inlineStr">
+        <is>
+          <t>927,000,000</t>
+        </is>
+      </c>
+      <c r="Q87" s="6" t="inlineStr">
+        <is>
+          <t>3.0%</t>
         </is>
       </c>
       <c r="R87" s="6" t="inlineStr">
         <is>
-          <t>corp_code 미확보(수동확인)</t>
+          <t>최초</t>
         </is>
       </c>
     </row>
     <row r="88" ht="30" customHeight="1">
       <c r="A88" s="6" t="inlineStr">
         <is>
-          <t>디티에스</t>
+          <t>씨앤엠</t>
         </is>
       </c>
       <c r="B88" s="18" t="inlineStr">
@@ -14703,24 +14715,24 @@
           <t>수집예정</t>
         </is>
       </c>
-      <c r="C88" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="D88" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="E88" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="F88" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="C88" s="6" t="inlineStr">
+        <is>
+          <t>10,000~13,000</t>
+        </is>
+      </c>
+      <c r="D88" s="7" t="inlineStr">
+        <is>
+          <t>2,950,000</t>
+        </is>
+      </c>
+      <c r="E88" s="7" t="inlineStr">
+        <is>
+          <t>29,500,000,000</t>
+        </is>
+      </c>
+      <c r="F88" s="6" t="inlineStr">
+        <is>
+          <t>24.96배 (PER)</t>
         </is>
       </c>
       <c r="G88" s="6" t="inlineStr"/>
@@ -14752,14 +14764,14 @@
       </c>
       <c r="R88" s="6" t="inlineStr">
         <is>
-          <t>신고서 대기</t>
+          <t>최초</t>
         </is>
       </c>
     </row>
     <row r="89" ht="30" customHeight="1">
       <c r="A89" s="6" t="inlineStr">
         <is>
-          <t>에이엔에이치스트럭쳐</t>
+          <t>(주)태석광학</t>
         </is>
       </c>
       <c r="B89" s="18" t="inlineStr">
@@ -14816,14 +14828,14 @@
       </c>
       <c r="R89" s="6" t="inlineStr">
         <is>
-          <t>신고서 대기</t>
+          <t>corp_code 미확보(수동확인)</t>
         </is>
       </c>
     </row>
     <row r="90" ht="30" customHeight="1">
       <c r="A90" s="6" t="inlineStr">
         <is>
-          <t>이에스티</t>
+          <t>디티에스</t>
         </is>
       </c>
       <c r="B90" s="18" t="inlineStr">
@@ -14887,7 +14899,7 @@
     <row r="91" ht="30" customHeight="1">
       <c r="A91" s="6" t="inlineStr">
         <is>
-          <t>우리투자제1호스팩</t>
+          <t>에이엔에이치스트럭쳐</t>
         </is>
       </c>
       <c r="B91" s="18" t="inlineStr">
@@ -14951,7 +14963,7 @@
     <row r="92" ht="30" customHeight="1">
       <c r="A92" s="6" t="inlineStr">
         <is>
-          <t>마더스제약</t>
+          <t>이에스티</t>
         </is>
       </c>
       <c r="B92" s="18" t="inlineStr">
@@ -15015,7 +15027,7 @@
     <row r="93" ht="30" customHeight="1">
       <c r="A93" s="6" t="inlineStr">
         <is>
-          <t>케이티이</t>
+          <t>우리투자제1호스팩</t>
         </is>
       </c>
       <c r="B93" s="18" t="inlineStr">
@@ -15079,7 +15091,7 @@
     <row r="94" ht="30" customHeight="1">
       <c r="A94" s="6" t="inlineStr">
         <is>
-          <t>씨앤엠</t>
+          <t>마더스제약</t>
         </is>
       </c>
       <c r="B94" s="18" t="inlineStr">
@@ -15143,7 +15155,7 @@
     <row r="95" ht="30" customHeight="1">
       <c r="A95" s="6" t="inlineStr">
         <is>
-          <t>제이앤티지</t>
+          <t>케이티이</t>
         </is>
       </c>
       <c r="B95" s="18" t="inlineStr">
@@ -15588,22 +15600,86 @@
         </is>
       </c>
     </row>
-    <row r="103">
-      <c r="A103" s="20" t="inlineStr">
-        <is>
-          <t>※ 상장 완료 = KIND 신규상장 페이지 기준(스팩합병 포함) · 스팩 공모상장은 밴드·밸류에이션 등 해당없음(공모가 2,000원 고정).</t>
+    <row r="102" ht="30" customHeight="1">
+      <c r="A102" s="6" t="inlineStr">
+        <is>
+          <t>에스에프씨</t>
+        </is>
+      </c>
+      <c r="B102" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="C102" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="D102" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="E102" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="F102" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="G102" s="6" t="inlineStr"/>
+      <c r="H102" s="6" t="inlineStr"/>
+      <c r="I102" s="6" t="inlineStr"/>
+      <c r="J102" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="K102" s="6" t="inlineStr"/>
+      <c r="L102" s="6" t="inlineStr"/>
+      <c r="M102" s="6" t="inlineStr"/>
+      <c r="N102" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="O102" s="6" t="inlineStr"/>
+      <c r="P102" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="Q102" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="R102" s="6" t="inlineStr">
+        <is>
+          <t>신고서 대기</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="20" t="inlineStr">
         <is>
-          <t>※ 기재정정 신고서 내 정정 전·후 병존 → 자동수집은 "정정 후" 값만 취함.</t>
+          <t>※ 상장 완료 = KIND 신규상장 페이지 기준(스팩합병 포함) · 스팩 공모상장은 밴드·밸류에이션 등 해당없음(공모가 2,000원 고정).</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="20" t="inlineStr">
+        <is>
+          <t>※ 기재정정 신고서 내 정정 전·후 병존 → 자동수집은 "정정 후" 값만 취함.</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="20" t="inlineStr">
         <is>
           <t>※ 청약경쟁률=일반투자자 청약수량÷최종배정수량 · "MM-DD~"는 종료일 자동수집 예정.</t>
         </is>
@@ -15906,7 +15982,7 @@
         <v>3</v>
       </c>
       <c r="C15" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D15" s="6" t="n">
         <v>1</v>
@@ -15979,11 +16055,11 @@
         </is>
       </c>
       <c r="B20" s="6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>299,100,000,000</t>
+          <t>412,620,000,000</t>
         </is>
       </c>
     </row>
@@ -16155,7 +16231,7 @@
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>KB증권</t>
+          <t>신한투자증권</t>
         </is>
       </c>
       <c r="B32" s="6" t="n">
@@ -16163,14 +16239,14 @@
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>31,200,000,000</t>
+          <t>36,720,000,000</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>신한투자증권</t>
+          <t>KB증권</t>
         </is>
       </c>
       <c r="B33" s="6" t="n">
@@ -16178,7 +16254,7 @@
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>30,240,000,000</t>
+          <t>31,200,000,000</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update IPO data 2026-10-19
</commit_message>
<xml_diff>
--- a/IPO_analysis.xlsx
+++ b/IPO_analysis.xlsx
@@ -618,14 +618,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>기준일 2026-10-18 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
+          <t>기준일 2026-10-19 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>■ 심사 신청(진행중)  (33건)</t>
+          <t>■ 심사 신청(진행중)  (32건)</t>
         </is>
       </c>
       <c r="B4" s="4" t="n"/>
@@ -1587,12 +1587,12 @@
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>신영스팩12호</t>
+          <t>범한메카텍</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
@@ -1610,17 +1610,29 @@
           <t>FY25</t>
         </is>
       </c>
-      <c r="F22" s="7" t="inlineStr"/>
-      <c r="G22" s="7" t="inlineStr"/>
-      <c r="H22" s="7" t="inlineStr"/>
+      <c r="F22" s="7" t="inlineStr">
+        <is>
+          <t>339,209</t>
+        </is>
+      </c>
+      <c r="G22" s="7" t="inlineStr">
+        <is>
+          <t>-18,141</t>
+        </is>
+      </c>
+      <c r="H22" s="7" t="inlineStr">
+        <is>
+          <t>265,955</t>
+        </is>
+      </c>
       <c r="I22" s="6" t="inlineStr">
         <is>
-          <t>금융 지원 서비스업</t>
+          <t>구조용 금속제품, 탱크 및 증기발생기 제조업</t>
         </is>
       </c>
       <c r="J22" s="6" t="inlineStr">
         <is>
-          <t>신영</t>
+          <t>유진, NH</t>
         </is>
       </c>
       <c r="K22" s="6" t="inlineStr">
@@ -1632,12 +1644,12 @@
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>범한메카텍</t>
+          <t>유림테크</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
@@ -1657,27 +1669,27 @@
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
-          <t>339,209</t>
+          <t>102,586</t>
         </is>
       </c>
       <c r="G23" s="7" t="inlineStr">
         <is>
-          <t>-18,141</t>
+          <t>-18,278</t>
         </is>
       </c>
       <c r="H23" s="7" t="inlineStr">
         <is>
-          <t>265,955</t>
+          <t>-4,832</t>
         </is>
       </c>
       <c r="I23" s="6" t="inlineStr">
         <is>
-          <t>구조용 금속제품, 탱크 및 증기발생기 제조업</t>
+          <t>자동차 신품 부품 제조업</t>
         </is>
       </c>
       <c r="J23" s="6" t="inlineStr">
         <is>
-          <t>유진, NH</t>
+          <t>대신</t>
         </is>
       </c>
       <c r="K23" s="6" t="inlineStr">
@@ -1689,12 +1701,12 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>유림테크</t>
+          <t>에버온</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
@@ -1714,27 +1726,27 @@
       </c>
       <c r="F24" s="7" t="inlineStr">
         <is>
-          <t>102,586</t>
+          <t>65,225</t>
         </is>
       </c>
       <c r="G24" s="7" t="inlineStr">
         <is>
-          <t>-18,278</t>
+          <t>-3,606</t>
         </is>
       </c>
       <c r="H24" s="7" t="inlineStr">
         <is>
-          <t>-4,832</t>
+          <t>54,955</t>
         </is>
       </c>
       <c r="I24" s="6" t="inlineStr">
         <is>
-          <t>자동차 신품 부품 제조업</t>
+          <t>전기업</t>
         </is>
       </c>
       <c r="J24" s="6" t="inlineStr">
         <is>
-          <t>대신</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K24" s="6" t="inlineStr">
@@ -1746,12 +1758,12 @@
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>에버온</t>
+          <t>엠디에스코리아</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
@@ -1771,22 +1783,22 @@
       </c>
       <c r="F25" s="7" t="inlineStr">
         <is>
-          <t>65,225</t>
+          <t>97,972</t>
         </is>
       </c>
       <c r="G25" s="7" t="inlineStr">
         <is>
-          <t>-3,606</t>
+          <t>6,512</t>
         </is>
       </c>
       <c r="H25" s="7" t="inlineStr">
         <is>
-          <t>54,955</t>
+          <t>53,818</t>
         </is>
       </c>
       <c r="I25" s="6" t="inlineStr">
         <is>
-          <t>전기업</t>
+          <t>기타 식품 제조업</t>
         </is>
       </c>
       <c r="J25" s="6" t="inlineStr">
@@ -1803,12 +1815,12 @@
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>엠디에스코리아</t>
+          <t>동승</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
@@ -1828,27 +1840,27 @@
       </c>
       <c r="F26" s="7" t="inlineStr">
         <is>
-          <t>97,972</t>
+          <t>78,625</t>
         </is>
       </c>
       <c r="G26" s="7" t="inlineStr">
         <is>
-          <t>6,512</t>
+          <t>14,525</t>
         </is>
       </c>
       <c r="H26" s="7" t="inlineStr">
         <is>
-          <t>53,818</t>
+          <t>5,438</t>
         </is>
       </c>
       <c r="I26" s="6" t="inlineStr">
         <is>
-          <t>기타 식품 제조업</t>
+          <t>부동산 임대 및 공급업</t>
         </is>
       </c>
       <c r="J26" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K26" s="6" t="inlineStr">
@@ -1865,7 +1877,7 @@
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>동승</t>
+          <t>에프엠더블유</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
@@ -1875,7 +1887,7 @@
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>신규상장</t>
+          <t>스팩 소멸합병</t>
         </is>
       </c>
       <c r="E27" s="6" t="inlineStr">
@@ -1885,27 +1897,27 @@
       </c>
       <c r="F27" s="7" t="inlineStr">
         <is>
-          <t>78,625</t>
+          <t>30,282</t>
         </is>
       </c>
       <c r="G27" s="7" t="inlineStr">
         <is>
-          <t>14,525</t>
+          <t>4,762</t>
         </is>
       </c>
       <c r="H27" s="7" t="inlineStr">
         <is>
-          <t>5,438</t>
+          <t>32</t>
         </is>
       </c>
       <c r="I27" s="6" t="inlineStr">
         <is>
-          <t>부동산 임대 및 공급업</t>
+          <t>기타 식품 제조업</t>
         </is>
       </c>
       <c r="J27" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>유진</t>
         </is>
       </c>
       <c r="K27" s="6" t="inlineStr">
@@ -1917,22 +1929,22 @@
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>에프엠더블유</t>
+          <t>소노인터내셔널</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>코스닥</t>
+          <t>유가</t>
         </is>
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
-          <t>스팩 소멸합병</t>
+          <t>신규상장</t>
         </is>
       </c>
       <c r="E28" s="6" t="inlineStr">
@@ -1942,27 +1954,27 @@
       </c>
       <c r="F28" s="7" t="inlineStr">
         <is>
-          <t>30,282</t>
+          <t>2,093,051</t>
         </is>
       </c>
       <c r="G28" s="7" t="inlineStr">
         <is>
-          <t>4,762</t>
+          <t>-148,064</t>
         </is>
       </c>
       <c r="H28" s="7" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>852,372</t>
         </is>
       </c>
       <c r="I28" s="6" t="inlineStr">
         <is>
-          <t>기타 식품 제조업</t>
+          <t>일반 및 생활 숙박시설 운영업</t>
         </is>
       </c>
       <c r="J28" s="6" t="inlineStr">
         <is>
-          <t>유진</t>
+          <t>대신, 미래</t>
         </is>
       </c>
       <c r="K28" s="6" t="inlineStr">
@@ -1974,17 +1986,17 @@
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>소노인터내셔널</t>
+          <t>싸이몬</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>유가</t>
+          <t>코스닥</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr">
@@ -1999,27 +2011,27 @@
       </c>
       <c r="F29" s="7" t="inlineStr">
         <is>
-          <t>2,093,051</t>
+          <t>48,695</t>
         </is>
       </c>
       <c r="G29" s="7" t="inlineStr">
         <is>
-          <t>-148,064</t>
+          <t>15,714</t>
         </is>
       </c>
       <c r="H29" s="7" t="inlineStr">
         <is>
-          <t>852,372</t>
+          <t>61,761</t>
         </is>
       </c>
       <c r="I29" s="6" t="inlineStr">
         <is>
-          <t>일반 및 생활 숙박시설 운영업</t>
+          <t>측정, 시험, 항해, 제어 및 기타 정밀기기 제조업</t>
         </is>
       </c>
       <c r="J29" s="6" t="inlineStr">
         <is>
-          <t>대신, 미래</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K29" s="6" t="inlineStr">
@@ -2031,12 +2043,12 @@
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>싸이몬</t>
+          <t>바이다</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
@@ -2056,27 +2068,27 @@
       </c>
       <c r="F30" s="7" t="inlineStr">
         <is>
-          <t>48,695</t>
+          <t>14,432</t>
         </is>
       </c>
       <c r="G30" s="7" t="inlineStr">
         <is>
-          <t>15,714</t>
+          <t>-3,951</t>
         </is>
       </c>
       <c r="H30" s="7" t="inlineStr">
         <is>
-          <t>61,761</t>
+          <t>15,108</t>
         </is>
       </c>
       <c r="I30" s="6" t="inlineStr">
         <is>
-          <t>측정, 시험, 항해, 제어 및 기타 정밀기기 제조업</t>
+          <t>전자부품 제조업</t>
         </is>
       </c>
       <c r="J30" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K30" s="6" t="inlineStr">
@@ -2088,12 +2100,12 @@
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>바이다</t>
+          <t>아이알큐더스</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
@@ -2113,27 +2125,27 @@
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>14,432</t>
+          <t>10,231</t>
         </is>
       </c>
       <c r="G31" s="7" t="inlineStr">
         <is>
-          <t>-3,951</t>
+          <t>-986</t>
         </is>
       </c>
       <c r="H31" s="7" t="inlineStr">
         <is>
-          <t>15,108</t>
+          <t>1,800</t>
         </is>
       </c>
       <c r="I31" s="6" t="inlineStr">
         <is>
-          <t>전자부품 제조업</t>
+          <t>소프트웨어 개발 및 공급업</t>
         </is>
       </c>
       <c r="J31" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>DB</t>
         </is>
       </c>
       <c r="K31" s="6" t="inlineStr">
@@ -2145,12 +2157,12 @@
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>아이알큐더스</t>
+          <t>씨엔티테크</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr">
@@ -2170,17 +2182,17 @@
       </c>
       <c r="F32" s="7" t="inlineStr">
         <is>
-          <t>10,231</t>
+          <t>27,015</t>
         </is>
       </c>
       <c r="G32" s="7" t="inlineStr">
         <is>
-          <t>-986</t>
+          <t>3,987</t>
         </is>
       </c>
       <c r="H32" s="7" t="inlineStr">
         <is>
-          <t>1,800</t>
+          <t>2,613</t>
         </is>
       </c>
       <c r="I32" s="6" t="inlineStr">
@@ -2190,7 +2202,7 @@
       </c>
       <c r="J32" s="6" t="inlineStr">
         <is>
-          <t>DB</t>
+          <t>한화, 하나</t>
         </is>
       </c>
       <c r="K32" s="6" t="inlineStr">
@@ -2202,12 +2214,12 @@
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>씨엔티테크</t>
+          <t>삼홍아크튜리온</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
@@ -2227,27 +2239,27 @@
       </c>
       <c r="F33" s="7" t="inlineStr">
         <is>
-          <t>27,015</t>
+          <t>26,162</t>
         </is>
       </c>
       <c r="G33" s="7" t="inlineStr">
         <is>
-          <t>3,987</t>
+          <t>-10,314</t>
         </is>
       </c>
       <c r="H33" s="7" t="inlineStr">
         <is>
-          <t>2,613</t>
+          <t>6,369</t>
         </is>
       </c>
       <c r="I33" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어 개발 및 공급업</t>
+          <t>구조용 금속제품, 탱크 및 증기발생기 제조업</t>
         </is>
       </c>
       <c r="J33" s="6" t="inlineStr">
         <is>
-          <t>한화, 하나</t>
+          <t>삼성, 미래</t>
         </is>
       </c>
       <c r="K33" s="6" t="inlineStr">
@@ -2259,12 +2271,12 @@
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>삼홍아크튜리온</t>
+          <t>비앤비코리아</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
@@ -2284,27 +2296,27 @@
       </c>
       <c r="F34" s="7" t="inlineStr">
         <is>
-          <t>26,162</t>
+          <t>141,169</t>
         </is>
       </c>
       <c r="G34" s="7" t="inlineStr">
         <is>
-          <t>-10,314</t>
+          <t>21,406</t>
         </is>
       </c>
       <c r="H34" s="7" t="inlineStr">
         <is>
-          <t>6,369</t>
+          <t>43,932</t>
         </is>
       </c>
       <c r="I34" s="6" t="inlineStr">
         <is>
-          <t>구조용 금속제품, 탱크 및 증기발생기 제조업</t>
+          <t>기타 화학제품 제조업</t>
         </is>
       </c>
       <c r="J34" s="6" t="inlineStr">
         <is>
-          <t>삼성, 미래</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K34" s="6" t="inlineStr">
@@ -2316,12 +2328,12 @@
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>비앤비코리아</t>
+          <t>오토핸즈</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
@@ -2331,7 +2343,7 @@
       </c>
       <c r="D35" s="6" t="inlineStr">
         <is>
-          <t>신규상장</t>
+          <t>스팩 소멸합병</t>
         </is>
       </c>
       <c r="E35" s="6" t="inlineStr">
@@ -2341,22 +2353,22 @@
       </c>
       <c r="F35" s="7" t="inlineStr">
         <is>
-          <t>141,169</t>
+          <t>238,564</t>
         </is>
       </c>
       <c r="G35" s="7" t="inlineStr">
         <is>
-          <t>21,406</t>
+          <t>6,047</t>
         </is>
       </c>
       <c r="H35" s="7" t="inlineStr">
         <is>
-          <t>43,932</t>
+          <t>6,129</t>
         </is>
       </c>
       <c r="I35" s="6" t="inlineStr">
         <is>
-          <t>기타 화학제품 제조업</t>
+          <t>자동차 판매업</t>
         </is>
       </c>
       <c r="J35" s="6" t="inlineStr">
@@ -2373,12 +2385,12 @@
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>오토핸즈</t>
+          <t>아이벡스메디칼시스템즈</t>
         </is>
       </c>
       <c r="C36" s="6" t="inlineStr">
@@ -2388,7 +2400,7 @@
       </c>
       <c r="D36" s="6" t="inlineStr">
         <is>
-          <t>스팩 소멸합병</t>
+          <t>신규상장</t>
         </is>
       </c>
       <c r="E36" s="6" t="inlineStr">
@@ -2398,27 +2410,27 @@
       </c>
       <c r="F36" s="7" t="inlineStr">
         <is>
-          <t>238,564</t>
+          <t>15,282</t>
         </is>
       </c>
       <c r="G36" s="7" t="inlineStr">
         <is>
-          <t>6,047</t>
+          <t>-7,227</t>
         </is>
       </c>
       <c r="H36" s="7" t="inlineStr">
         <is>
-          <t>6,129</t>
+          <t>744</t>
         </is>
       </c>
       <c r="I36" s="6" t="inlineStr">
         <is>
-          <t>자동차 판매업</t>
+          <t>의료용 기기 제조업</t>
         </is>
       </c>
       <c r="J36" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K36" s="6" t="inlineStr">
@@ -2430,12 +2442,12 @@
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>아이벡스메디칼시스템즈</t>
+          <t>피지티</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
@@ -2455,27 +2467,27 @@
       </c>
       <c r="F37" s="7" t="inlineStr">
         <is>
-          <t>15,282</t>
+          <t>40,141</t>
         </is>
       </c>
       <c r="G37" s="7" t="inlineStr">
         <is>
-          <t>-7,227</t>
+          <t>-69,722</t>
         </is>
       </c>
       <c r="H37" s="7" t="inlineStr">
         <is>
-          <t>744</t>
+          <t>6,029</t>
         </is>
       </c>
       <c r="I37" s="6" t="inlineStr">
         <is>
-          <t>의료용 기기 제조업</t>
+          <t>기타 화학제품 제조업</t>
         </is>
       </c>
       <c r="J37" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="K37" s="6" t="inlineStr">
@@ -2484,134 +2496,122 @@
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="6" t="inlineStr">
-        <is>
-          <t>2026-02-27</t>
-        </is>
-      </c>
-      <c r="B38" s="6" t="inlineStr">
-        <is>
-          <t>피지티</t>
-        </is>
-      </c>
-      <c r="C38" s="6" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>■ 심사 승인  (86건)</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="n"/>
+      <c r="C39" s="4" t="n"/>
+      <c r="D39" s="4" t="n"/>
+      <c r="E39" s="4" t="n"/>
+      <c r="F39" s="4" t="n"/>
+      <c r="G39" s="4" t="n"/>
+      <c r="H39" s="4" t="n"/>
+      <c r="I39" s="4" t="n"/>
+      <c r="J39" s="4" t="n"/>
+      <c r="K39" s="4" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>일자</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>회사명</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>시장</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>상장유형</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>기준연도</t>
+        </is>
+      </c>
+      <c r="F40" s="5" t="inlineStr">
+        <is>
+          <t>매출액</t>
+        </is>
+      </c>
+      <c r="G40" s="5" t="inlineStr">
+        <is>
+          <t>순이익</t>
+        </is>
+      </c>
+      <c r="H40" s="5" t="inlineStr">
+        <is>
+          <t>자기자본</t>
+        </is>
+      </c>
+      <c r="I40" s="5" t="inlineStr">
+        <is>
+          <t>업종</t>
+        </is>
+      </c>
+      <c r="J40" s="5" t="inlineStr">
+        <is>
+          <t>대표주관사</t>
+        </is>
+      </c>
+      <c r="K40" s="5" t="inlineStr">
+        <is>
+          <t>현황</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B41" s="6" t="inlineStr">
+        <is>
+          <t>신영스팩12호</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="inlineStr">
         <is>
           <t>코스닥</t>
         </is>
       </c>
-      <c r="D38" s="6" t="inlineStr">
+      <c r="D41" s="6" t="inlineStr">
         <is>
           <t>신규상장</t>
         </is>
       </c>
-      <c r="E38" s="6" t="inlineStr">
+      <c r="E41" s="6" t="inlineStr">
         <is>
           <t>FY25</t>
         </is>
       </c>
-      <c r="F38" s="7" t="inlineStr">
-        <is>
-          <t>40,141</t>
-        </is>
-      </c>
-      <c r="G38" s="7" t="inlineStr">
-        <is>
-          <t>-69,722</t>
-        </is>
-      </c>
-      <c r="H38" s="7" t="inlineStr">
-        <is>
-          <t>6,029</t>
-        </is>
-      </c>
-      <c r="I38" s="6" t="inlineStr">
-        <is>
-          <t>기타 화학제품 제조업</t>
-        </is>
-      </c>
-      <c r="J38" s="6" t="inlineStr">
-        <is>
-          <t>한국</t>
-        </is>
-      </c>
-      <c r="K38" s="6" t="inlineStr">
-        <is>
-          <t>예심 진행중</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="3" t="inlineStr">
-        <is>
-          <t>■ 심사 승인  (85건)</t>
-        </is>
-      </c>
-      <c r="B40" s="4" t="n"/>
-      <c r="C40" s="4" t="n"/>
-      <c r="D40" s="4" t="n"/>
-      <c r="E40" s="4" t="n"/>
-      <c r="F40" s="4" t="n"/>
-      <c r="G40" s="4" t="n"/>
-      <c r="H40" s="4" t="n"/>
-      <c r="I40" s="4" t="n"/>
-      <c r="J40" s="4" t="n"/>
-      <c r="K40" s="4" t="n"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="5" t="inlineStr">
-        <is>
-          <t>일자</t>
-        </is>
-      </c>
-      <c r="B41" s="5" t="inlineStr">
-        <is>
-          <t>회사명</t>
-        </is>
-      </c>
-      <c r="C41" s="5" t="inlineStr">
-        <is>
-          <t>시장</t>
-        </is>
-      </c>
-      <c r="D41" s="5" t="inlineStr">
-        <is>
-          <t>상장유형</t>
-        </is>
-      </c>
-      <c r="E41" s="5" t="inlineStr">
-        <is>
-          <t>기준연도</t>
-        </is>
-      </c>
-      <c r="F41" s="5" t="inlineStr">
-        <is>
-          <t>매출액</t>
-        </is>
-      </c>
-      <c r="G41" s="5" t="inlineStr">
-        <is>
-          <t>순이익</t>
-        </is>
-      </c>
-      <c r="H41" s="5" t="inlineStr">
-        <is>
-          <t>자기자본</t>
-        </is>
-      </c>
-      <c r="I41" s="5" t="inlineStr">
-        <is>
-          <t>업종</t>
-        </is>
-      </c>
-      <c r="J41" s="5" t="inlineStr">
-        <is>
-          <t>대표주관사</t>
-        </is>
-      </c>
-      <c r="K41" s="5" t="inlineStr">
-        <is>
-          <t>현황</t>
+      <c r="F41" s="7" t="inlineStr"/>
+      <c r="G41" s="7" t="inlineStr"/>
+      <c r="H41" s="7" t="inlineStr"/>
+      <c r="I41" s="6" t="inlineStr">
+        <is>
+          <t>금융 지원 서비스업</t>
+        </is>
+      </c>
+      <c r="J41" s="6" t="inlineStr">
+        <is>
+          <t>신영</t>
+        </is>
+      </c>
+      <c r="K41" s="6" t="inlineStr">
+        <is>
+          <t>상장전</t>
         </is>
       </c>
     </row>
@@ -8521,7 +8521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R106"/>
+  <dimension ref="A1:R107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -12767,7 +12767,7 @@
     <row r="58" ht="22" customHeight="1">
       <c r="A58" s="3" t="inlineStr">
         <is>
-          <t>■ 공모 진행 (예심 승인법인)  (44건)</t>
+          <t>■ 공모 진행 (예심 승인법인)  (45건)</t>
         </is>
       </c>
       <c r="B58" s="4" t="n"/>
@@ -13167,40 +13167,48 @@
     <row r="64" ht="30" customHeight="1">
       <c r="A64" s="6" t="inlineStr">
         <is>
-          <t>유캐스트</t>
+          <t>크리에이츠</t>
         </is>
       </c>
       <c r="B64" s="6" t="inlineStr">
         <is>
-          <t>10-07~10-14</t>
+          <t>10-12~10-16</t>
         </is>
       </c>
       <c r="C64" s="6" t="inlineStr">
         <is>
-          <t>21,000~26,000</t>
+          <t>15,000~18,000</t>
         </is>
       </c>
       <c r="D64" s="7" t="inlineStr">
         <is>
-          <t>800,000</t>
+          <t>1,400,000</t>
         </is>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
-          <t>16,800,000,000</t>
+          <t>21,000,000,000</t>
         </is>
       </c>
       <c r="F64" s="6" t="inlineStr">
         <is>
-          <t>17.97배 (PER)</t>
-        </is>
-      </c>
-      <c r="G64" s="6" t="inlineStr"/>
-      <c r="H64" s="6" t="inlineStr"/>
-      <c r="I64" s="6" t="inlineStr"/>
+          <t>19.15배 (PER)</t>
+        </is>
+      </c>
+      <c r="G64" s="6" t="inlineStr">
+        <is>
+          <t>15,000</t>
+        </is>
+      </c>
+      <c r="H64" s="6" t="n">
+        <v>240.46</v>
+      </c>
+      <c r="I64" s="6" t="n">
+        <v>831</v>
+      </c>
       <c r="J64" s="6" t="inlineStr">
         <is>
-          <t>10-19~10-20</t>
+          <t>10-20~10-21</t>
         </is>
       </c>
       <c r="K64" s="6" t="inlineStr"/>
@@ -13208,60 +13216,68 @@
       <c r="M64" s="6" t="inlineStr"/>
       <c r="N64" s="6" t="inlineStr">
         <is>
-          <t>유진투자증권</t>
+          <t>삼성증권</t>
         </is>
       </c>
       <c r="O64" s="6" t="inlineStr"/>
       <c r="P64" s="7" t="inlineStr">
         <is>
-          <t>1,181,280,000</t>
+          <t>865,200,000</t>
         </is>
       </c>
       <c r="Q64" s="6" t="inlineStr">
         <is>
-          <t>7.0%</t>
+          <t>4.0%</t>
         </is>
       </c>
       <c r="R64" s="6" t="inlineStr">
         <is>
-          <t>정정</t>
+          <t>발행조건확정</t>
         </is>
       </c>
     </row>
     <row r="65" ht="30" customHeight="1">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>크리에이츠</t>
+          <t>한화플러스제6호스팩</t>
         </is>
       </c>
       <c r="B65" s="6" t="inlineStr">
         <is>
-          <t>10-12~10-16</t>
-        </is>
-      </c>
-      <c r="C65" s="6" t="inlineStr">
-        <is>
-          <t>15,000~18,000</t>
+          <t>10-14~10-15</t>
+        </is>
+      </c>
+      <c r="C65" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="D65" s="7" t="inlineStr">
         <is>
-          <t>1,400,000</t>
+          <t>6,000,000</t>
         </is>
       </c>
       <c r="E65" s="7" t="inlineStr">
         <is>
-          <t>21,000,000,000</t>
-        </is>
-      </c>
-      <c r="F65" s="6" t="inlineStr">
-        <is>
-          <t>19.15배 (PER)</t>
-        </is>
-      </c>
-      <c r="G65" s="6" t="inlineStr"/>
-      <c r="H65" s="6" t="inlineStr"/>
-      <c r="I65" s="6" t="inlineStr"/>
+          <t>12,000,000,000</t>
+        </is>
+      </c>
+      <c r="F65" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="G65" s="6" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
+      </c>
+      <c r="H65" s="6" t="n">
+        <v>1256.48</v>
+      </c>
+      <c r="I65" s="6" t="n">
+        <v>1927</v>
+      </c>
       <c r="J65" s="6" t="inlineStr">
         <is>
           <t>10-20~10-21</t>
@@ -13270,57 +13286,57 @@
       <c r="K65" s="6" t="inlineStr"/>
       <c r="L65" s="6" t="inlineStr"/>
       <c r="M65" s="6" t="inlineStr"/>
-      <c r="N65" s="6" t="inlineStr">
-        <is>
-          <t>삼성증권</t>
+      <c r="N65" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="O65" s="6" t="inlineStr"/>
-      <c r="P65" s="7" t="inlineStr">
-        <is>
-          <t>865,200,000</t>
+      <c r="P65" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="Q65" s="6" t="inlineStr">
         <is>
-          <t>4.0%</t>
+          <t>50%</t>
         </is>
       </c>
       <c r="R65" s="6" t="inlineStr">
         <is>
-          <t>정정</t>
+          <t>발행조건확정</t>
         </is>
       </c>
     </row>
     <row r="66" ht="30" customHeight="1">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>인텔리빅스</t>
+          <t>유캐스트</t>
         </is>
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
-          <t>10-12~10-16</t>
+          <t>10-07~10-14</t>
         </is>
       </c>
       <c r="C66" s="6" t="inlineStr">
         <is>
-          <t>7,600~9,000</t>
+          <t>21,000~26,000</t>
         </is>
       </c>
       <c r="D66" s="7" t="inlineStr">
         <is>
-          <t>2,500,000</t>
+          <t>800,000</t>
         </is>
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
-          <t>19,000,000,000</t>
+          <t>16,800,000,000</t>
         </is>
       </c>
       <c r="F66" s="6" t="inlineStr">
         <is>
-          <t>22.02배 (PER)</t>
+          <t>17.97배 (PER)</t>
         </is>
       </c>
       <c r="G66" s="6" t="inlineStr"/>
@@ -13328,7 +13344,7 @@
       <c r="I66" s="6" t="inlineStr"/>
       <c r="J66" s="6" t="inlineStr">
         <is>
-          <t>10-21~10-22</t>
+          <t>10-19~10-20</t>
         </is>
       </c>
       <c r="K66" s="6" t="inlineStr"/>
@@ -13336,18 +13352,18 @@
       <c r="M66" s="6" t="inlineStr"/>
       <c r="N66" s="6" t="inlineStr">
         <is>
-          <t>미래에셋증권</t>
+          <t>유진투자증권</t>
         </is>
       </c>
       <c r="O66" s="6" t="inlineStr"/>
       <c r="P66" s="7" t="inlineStr">
         <is>
-          <t>782,800,000</t>
+          <t>1,181,280,000</t>
         </is>
       </c>
       <c r="Q66" s="6" t="inlineStr">
         <is>
-          <t>4.0%</t>
+          <t>7.0%</t>
         </is>
       </c>
       <c r="R66" s="6" t="inlineStr">
@@ -13359,32 +13375,32 @@
     <row r="67" ht="30" customHeight="1">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>래블업</t>
+          <t>인텔리빅스</t>
         </is>
       </c>
       <c r="B67" s="6" t="inlineStr">
         <is>
-          <t>10-13~10-19</t>
+          <t>10-12~10-16</t>
         </is>
       </c>
       <c r="C67" s="6" t="inlineStr">
         <is>
-          <t>19,000~22,000</t>
+          <t>7,600~9,000</t>
         </is>
       </c>
       <c r="D67" s="7" t="inlineStr">
         <is>
-          <t>2,180,000</t>
+          <t>2,500,000</t>
         </is>
       </c>
       <c r="E67" s="7" t="inlineStr">
         <is>
-          <t>41,420,000,000</t>
+          <t>19,000,000,000</t>
         </is>
       </c>
       <c r="F67" s="6" t="inlineStr">
         <is>
-          <t>33.6배 (PER)</t>
+          <t>22.02배 (PER)</t>
         </is>
       </c>
       <c r="G67" s="6" t="inlineStr"/>
@@ -13392,7 +13408,7 @@
       <c r="I67" s="6" t="inlineStr"/>
       <c r="J67" s="6" t="inlineStr">
         <is>
-          <t>10-22~10-23</t>
+          <t>10-21~10-22</t>
         </is>
       </c>
       <c r="K67" s="6" t="inlineStr"/>
@@ -13400,18 +13416,18 @@
       <c r="M67" s="6" t="inlineStr"/>
       <c r="N67" s="6" t="inlineStr">
         <is>
-          <t>NH투자증권</t>
+          <t>미래에셋증권</t>
         </is>
       </c>
       <c r="O67" s="6" t="inlineStr"/>
       <c r="P67" s="7" t="inlineStr">
         <is>
-          <t>1,908,899,000</t>
+          <t>782,800,000</t>
         </is>
       </c>
       <c r="Q67" s="6" t="inlineStr">
         <is>
-          <t>4.5%</t>
+          <t>4.0%</t>
         </is>
       </c>
       <c r="R67" s="6" t="inlineStr">
@@ -13423,7 +13439,7 @@
     <row r="68" ht="30" customHeight="1">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>영광</t>
+          <t>래블업</t>
         </is>
       </c>
       <c r="B68" s="6" t="inlineStr">
@@ -13433,22 +13449,22 @@
       </c>
       <c r="C68" s="6" t="inlineStr">
         <is>
-          <t>14,000~17,000</t>
+          <t>19,000~22,000</t>
         </is>
       </c>
       <c r="D68" s="7" t="inlineStr">
         <is>
-          <t>2,260,000</t>
+          <t>2,180,000</t>
         </is>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
-          <t>31,640,000,000</t>
+          <t>41,420,000,000</t>
         </is>
       </c>
       <c r="F68" s="6" t="inlineStr">
         <is>
-          <t>11.98배 (EV/EBITDA)</t>
+          <t>33.6배 (PER)</t>
         </is>
       </c>
       <c r="G68" s="6" t="inlineStr"/>
@@ -13464,18 +13480,18 @@
       <c r="M68" s="6" t="inlineStr"/>
       <c r="N68" s="6" t="inlineStr">
         <is>
-          <t>한국투자증권</t>
+          <t>NH투자증권</t>
         </is>
       </c>
       <c r="O68" s="6" t="inlineStr"/>
       <c r="P68" s="7" t="inlineStr">
         <is>
-          <t>977,676,000</t>
-        </is>
-      </c>
-      <c r="Q68" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>1,908,899,000</t>
+        </is>
+      </c>
+      <c r="Q68" s="6" t="inlineStr">
+        <is>
+          <t>4.5%</t>
         </is>
       </c>
       <c r="R68" s="6" t="inlineStr">
@@ -13487,32 +13503,32 @@
     <row r="69" ht="30" customHeight="1">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>한화플러스제6호스팩</t>
+          <t>영광</t>
         </is>
       </c>
       <c r="B69" s="6" t="inlineStr">
         <is>
-          <t>10-14~10-15</t>
-        </is>
-      </c>
-      <c r="C69" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>10-13~10-19</t>
+        </is>
+      </c>
+      <c r="C69" s="6" t="inlineStr">
+        <is>
+          <t>14,000~17,000</t>
         </is>
       </c>
       <c r="D69" s="7" t="inlineStr">
         <is>
-          <t>6,000,000</t>
+          <t>2,260,000</t>
         </is>
       </c>
       <c r="E69" s="7" t="inlineStr">
         <is>
-          <t>12,000,000,000</t>
-        </is>
-      </c>
-      <c r="F69" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>31,640,000,000</t>
+        </is>
+      </c>
+      <c r="F69" s="6" t="inlineStr">
+        <is>
+          <t>11.98배 (EV/EBITDA)</t>
         </is>
       </c>
       <c r="G69" s="6" t="inlineStr"/>
@@ -13520,26 +13536,26 @@
       <c r="I69" s="6" t="inlineStr"/>
       <c r="J69" s="6" t="inlineStr">
         <is>
-          <t>10-20~10-21</t>
+          <t>10-22~10-23</t>
         </is>
       </c>
       <c r="K69" s="6" t="inlineStr"/>
       <c r="L69" s="6" t="inlineStr"/>
       <c r="M69" s="6" t="inlineStr"/>
-      <c r="N69" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="N69" s="6" t="inlineStr">
+        <is>
+          <t>한국투자증권</t>
         </is>
       </c>
       <c r="O69" s="6" t="inlineStr"/>
-      <c r="P69" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="Q69" s="6" t="inlineStr">
-        <is>
-          <t>3.50%</t>
+      <c r="P69" s="7" t="inlineStr">
+        <is>
+          <t>977,676,000</t>
+        </is>
+      </c>
+      <c r="Q69" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="R69" s="6" t="inlineStr">
@@ -14771,7 +14787,7 @@
     <row r="89" ht="30" customHeight="1">
       <c r="A89" s="6" t="inlineStr">
         <is>
-          <t>(주)태석광학</t>
+          <t>씨아이에스케미칼</t>
         </is>
       </c>
       <c r="B89" s="18" t="inlineStr">
@@ -14779,24 +14795,24 @@
           <t>수집예정</t>
         </is>
       </c>
-      <c r="C89" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="D89" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="E89" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="F89" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="C89" s="6" t="inlineStr">
+        <is>
+          <t>5,400~6,800</t>
+        </is>
+      </c>
+      <c r="D89" s="7" t="inlineStr">
+        <is>
+          <t>4,000,000</t>
+        </is>
+      </c>
+      <c r="E89" s="7" t="inlineStr">
+        <is>
+          <t>21,600,000,000</t>
+        </is>
+      </c>
+      <c r="F89" s="6" t="inlineStr">
+        <is>
+          <t>21.24배 (PER)</t>
         </is>
       </c>
       <c r="G89" s="6" t="inlineStr"/>
@@ -14828,14 +14844,14 @@
       </c>
       <c r="R89" s="6" t="inlineStr">
         <is>
-          <t>corp_code 미확보(수동확인)</t>
+          <t>최초</t>
         </is>
       </c>
     </row>
     <row r="90" ht="30" customHeight="1">
       <c r="A90" s="6" t="inlineStr">
         <is>
-          <t>디티에스</t>
+          <t>(주)태석광학</t>
         </is>
       </c>
       <c r="B90" s="18" t="inlineStr">
@@ -14892,14 +14908,14 @@
       </c>
       <c r="R90" s="6" t="inlineStr">
         <is>
-          <t>신고서 대기</t>
+          <t>corp_code 미확보(수동확인)</t>
         </is>
       </c>
     </row>
     <row r="91" ht="30" customHeight="1">
       <c r="A91" s="6" t="inlineStr">
         <is>
-          <t>에이엔에이치스트럭쳐</t>
+          <t>신영스팩12호</t>
         </is>
       </c>
       <c r="B91" s="18" t="inlineStr">
@@ -14956,14 +14972,14 @@
       </c>
       <c r="R91" s="6" t="inlineStr">
         <is>
-          <t>신고서 대기</t>
+          <t>corp_code 미확보(수동확인)</t>
         </is>
       </c>
     </row>
     <row r="92" ht="30" customHeight="1">
       <c r="A92" s="6" t="inlineStr">
         <is>
-          <t>이에스티</t>
+          <t>디티에스</t>
         </is>
       </c>
       <c r="B92" s="18" t="inlineStr">
@@ -15027,7 +15043,7 @@
     <row r="93" ht="30" customHeight="1">
       <c r="A93" s="6" t="inlineStr">
         <is>
-          <t>우리투자제1호스팩</t>
+          <t>에이엔에이치스트럭쳐</t>
         </is>
       </c>
       <c r="B93" s="18" t="inlineStr">
@@ -15091,7 +15107,7 @@
     <row r="94" ht="30" customHeight="1">
       <c r="A94" s="6" t="inlineStr">
         <is>
-          <t>마더스제약</t>
+          <t>이에스티</t>
         </is>
       </c>
       <c r="B94" s="18" t="inlineStr">
@@ -15155,7 +15171,7 @@
     <row r="95" ht="30" customHeight="1">
       <c r="A95" s="6" t="inlineStr">
         <is>
-          <t>케이티이</t>
+          <t>우리투자제1호스팩</t>
         </is>
       </c>
       <c r="B95" s="18" t="inlineStr">
@@ -15219,7 +15235,7 @@
     <row r="96" ht="30" customHeight="1">
       <c r="A96" s="6" t="inlineStr">
         <is>
-          <t>데스틴파워</t>
+          <t>마더스제약</t>
         </is>
       </c>
       <c r="B96" s="18" t="inlineStr">
@@ -15283,7 +15299,7 @@
     <row r="97" ht="30" customHeight="1">
       <c r="A97" s="6" t="inlineStr">
         <is>
-          <t>엘리스</t>
+          <t>케이티이</t>
         </is>
       </c>
       <c r="B97" s="18" t="inlineStr">
@@ -15347,7 +15363,7 @@
     <row r="98" ht="30" customHeight="1">
       <c r="A98" s="6" t="inlineStr">
         <is>
-          <t>인터엑스</t>
+          <t>데스틴파워</t>
         </is>
       </c>
       <c r="B98" s="18" t="inlineStr">
@@ -15411,7 +15427,7 @@
     <row r="99" ht="30" customHeight="1">
       <c r="A99" s="6" t="inlineStr">
         <is>
-          <t>씨아이에스케미칼</t>
+          <t>엘리스</t>
         </is>
       </c>
       <c r="B99" s="18" t="inlineStr">
@@ -15475,7 +15491,7 @@
     <row r="100" ht="30" customHeight="1">
       <c r="A100" s="6" t="inlineStr">
         <is>
-          <t>이노보테라퓨틱스</t>
+          <t>인터엑스</t>
         </is>
       </c>
       <c r="B100" s="18" t="inlineStr">
@@ -15539,7 +15555,7 @@
     <row r="101" ht="30" customHeight="1">
       <c r="A101" s="6" t="inlineStr">
         <is>
-          <t>이나인페이</t>
+          <t>이노보테라퓨틱스</t>
         </is>
       </c>
       <c r="B101" s="18" t="inlineStr">
@@ -15603,7 +15619,7 @@
     <row r="102" ht="30" customHeight="1">
       <c r="A102" s="6" t="inlineStr">
         <is>
-          <t>에스에프씨</t>
+          <t>이나인페이</t>
         </is>
       </c>
       <c r="B102" s="18" t="inlineStr">
@@ -15664,22 +15680,86 @@
         </is>
       </c>
     </row>
-    <row r="104">
-      <c r="A104" s="20" t="inlineStr">
-        <is>
-          <t>※ 상장 완료 = KIND 신규상장 페이지 기준(스팩합병 포함) · 스팩 공모상장은 밴드·밸류에이션 등 해당없음(공모가 2,000원 고정).</t>
+    <row r="103" ht="30" customHeight="1">
+      <c r="A103" s="6" t="inlineStr">
+        <is>
+          <t>에스에프씨</t>
+        </is>
+      </c>
+      <c r="B103" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="C103" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="D103" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="E103" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="F103" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="G103" s="6" t="inlineStr"/>
+      <c r="H103" s="6" t="inlineStr"/>
+      <c r="I103" s="6" t="inlineStr"/>
+      <c r="J103" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="K103" s="6" t="inlineStr"/>
+      <c r="L103" s="6" t="inlineStr"/>
+      <c r="M103" s="6" t="inlineStr"/>
+      <c r="N103" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="O103" s="6" t="inlineStr"/>
+      <c r="P103" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="Q103" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="R103" s="6" t="inlineStr">
+        <is>
+          <t>신고서 대기</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="20" t="inlineStr">
         <is>
-          <t>※ 기재정정 신고서 내 정정 전·후 병존 → 자동수집은 "정정 후" 값만 취함.</t>
+          <t>※ 상장 완료 = KIND 신규상장 페이지 기준(스팩합병 포함) · 스팩 공모상장은 밴드·밸류에이션 등 해당없음(공모가 2,000원 고정).</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="20" t="inlineStr">
+        <is>
+          <t>※ 기재정정 신고서 내 정정 전·후 병존 → 자동수집은 "정정 후" 값만 취함.</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="20" t="inlineStr">
         <is>
           <t>※ 청약경쟁률=일반투자자 청약수량÷최종배정수량 · "MM-DD~"는 종료일 자동수집 예정.</t>
         </is>
@@ -15982,7 +16062,7 @@
         <v>3</v>
       </c>
       <c r="C15" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D15" s="6" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
chore: update IPO data 2026-10-21
</commit_message>
<xml_diff>
--- a/IPO_analysis.xlsx
+++ b/IPO_analysis.xlsx
@@ -618,7 +618,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>기준일 2026-10-20 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
+          <t>기준일 2026-10-21 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
         </is>
       </c>
     </row>
@@ -5368,7 +5368,7 @@
       </c>
       <c r="K90" s="6" t="inlineStr">
         <is>
-          <t>상장전</t>
+          <t>상장승인(상장예정)</t>
         </is>
       </c>
     </row>
@@ -13399,67 +13399,67 @@
     <row r="67" ht="30" customHeight="1">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>한화플러스제6호스팩</t>
+          <t>래블업</t>
         </is>
       </c>
       <c r="B67" s="6" t="inlineStr">
         <is>
-          <t>10-14~10-15</t>
-        </is>
-      </c>
-      <c r="C67" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>10-13~10-19</t>
+        </is>
+      </c>
+      <c r="C67" s="6" t="inlineStr">
+        <is>
+          <t>19,000~22,000</t>
         </is>
       </c>
       <c r="D67" s="7" t="inlineStr">
         <is>
-          <t>6,000,000</t>
+          <t>2,180,000</t>
         </is>
       </c>
       <c r="E67" s="7" t="inlineStr">
         <is>
-          <t>12,000,000,000</t>
-        </is>
-      </c>
-      <c r="F67" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>41,420,000,000</t>
+        </is>
+      </c>
+      <c r="F67" s="6" t="inlineStr">
+        <is>
+          <t>33.6배 (PER)</t>
         </is>
       </c>
       <c r="G67" s="6" t="inlineStr">
         <is>
-          <t>2,000</t>
+          <t>19,000</t>
         </is>
       </c>
       <c r="H67" s="6" t="n">
-        <v>1256.48</v>
+        <v>284.53</v>
       </c>
       <c r="I67" s="6" t="n">
-        <v>1927</v>
+        <v>1129</v>
       </c>
       <c r="J67" s="6" t="inlineStr">
         <is>
-          <t>10-20~10-21</t>
+          <t>10-22~10-23</t>
         </is>
       </c>
       <c r="K67" s="6" t="inlineStr"/>
       <c r="L67" s="6" t="inlineStr"/>
       <c r="M67" s="6" t="inlineStr"/>
-      <c r="N67" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="N67" s="6" t="inlineStr">
+        <is>
+          <t>NH투자증권</t>
         </is>
       </c>
       <c r="O67" s="6" t="inlineStr"/>
-      <c r="P67" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="P67" s="7" t="inlineStr">
+        <is>
+          <t>1,908,899,000</t>
         </is>
       </c>
       <c r="Q67" s="6" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>4.5%</t>
         </is>
       </c>
       <c r="R67" s="6" t="inlineStr">
@@ -13471,40 +13471,48 @@
     <row r="68" ht="30" customHeight="1">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>유캐스트</t>
+          <t>영광</t>
         </is>
       </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t>10-07~10-14</t>
+          <t>10-13~10-19</t>
         </is>
       </c>
       <c r="C68" s="6" t="inlineStr">
         <is>
-          <t>21,000~26,000</t>
+          <t>14,000~17,000</t>
         </is>
       </c>
       <c r="D68" s="7" t="inlineStr">
         <is>
-          <t>800,000</t>
+          <t>2,260,000</t>
         </is>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
-          <t>16,800,000,000</t>
+          <t>38,420,000,000</t>
         </is>
       </c>
       <c r="F68" s="6" t="inlineStr">
         <is>
-          <t>17.97배 (PER)</t>
-        </is>
-      </c>
-      <c r="G68" s="6" t="inlineStr"/>
-      <c r="H68" s="6" t="inlineStr"/>
-      <c r="I68" s="6" t="inlineStr"/>
+          <t>11.98배 (EV/EBITDA)</t>
+        </is>
+      </c>
+      <c r="G68" s="6" t="inlineStr">
+        <is>
+          <t>17,000</t>
+        </is>
+      </c>
+      <c r="H68" s="6" t="n">
+        <v>1000.07</v>
+      </c>
+      <c r="I68" s="6" t="n">
+        <v>2276</v>
+      </c>
       <c r="J68" s="6" t="inlineStr">
         <is>
-          <t>10-19~10-20</t>
+          <t>10-22~10-23</t>
         </is>
       </c>
       <c r="K68" s="6" t="inlineStr"/>
@@ -13512,119 +13520,127 @@
       <c r="M68" s="6" t="inlineStr"/>
       <c r="N68" s="6" t="inlineStr">
         <is>
-          <t>유진투자증권</t>
+          <t>한국투자증권</t>
         </is>
       </c>
       <c r="O68" s="6" t="inlineStr"/>
       <c r="P68" s="7" t="inlineStr">
         <is>
-          <t>1,181,280,000</t>
-        </is>
-      </c>
-      <c r="Q68" s="6" t="inlineStr">
-        <is>
-          <t>7.0%</t>
+          <t>977,676,000</t>
+        </is>
+      </c>
+      <c r="Q68" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="R68" s="6" t="inlineStr">
         <is>
-          <t>정정</t>
+          <t>발행조건확정</t>
         </is>
       </c>
     </row>
     <row r="69" ht="30" customHeight="1">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>래블업</t>
+          <t>한화플러스제6호스팩</t>
         </is>
       </c>
       <c r="B69" s="6" t="inlineStr">
         <is>
-          <t>10-13~10-19</t>
-        </is>
-      </c>
-      <c r="C69" s="6" t="inlineStr">
-        <is>
-          <t>19,000~22,000</t>
+          <t>10-14~10-15</t>
+        </is>
+      </c>
+      <c r="C69" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="D69" s="7" t="inlineStr">
         <is>
-          <t>2,180,000</t>
+          <t>6,000,000</t>
         </is>
       </c>
       <c r="E69" s="7" t="inlineStr">
         <is>
-          <t>41,420,000,000</t>
-        </is>
-      </c>
-      <c r="F69" s="6" t="inlineStr">
-        <is>
-          <t>33.6배 (PER)</t>
-        </is>
-      </c>
-      <c r="G69" s="6" t="inlineStr"/>
-      <c r="H69" s="6" t="inlineStr"/>
-      <c r="I69" s="6" t="inlineStr"/>
+          <t>12,000,000,000</t>
+        </is>
+      </c>
+      <c r="F69" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="G69" s="6" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
+      </c>
+      <c r="H69" s="6" t="n">
+        <v>1256.48</v>
+      </c>
+      <c r="I69" s="6" t="n">
+        <v>1927</v>
+      </c>
       <c r="J69" s="6" t="inlineStr">
         <is>
-          <t>10-22~10-23</t>
+          <t>10-20~10-21</t>
         </is>
       </c>
       <c r="K69" s="6" t="inlineStr"/>
       <c r="L69" s="6" t="inlineStr"/>
       <c r="M69" s="6" t="inlineStr"/>
-      <c r="N69" s="6" t="inlineStr">
-        <is>
-          <t>NH투자증권</t>
+      <c r="N69" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="O69" s="6" t="inlineStr"/>
-      <c r="P69" s="7" t="inlineStr">
-        <is>
-          <t>1,908,899,000</t>
+      <c r="P69" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="Q69" s="6" t="inlineStr">
         <is>
-          <t>4.5%</t>
+          <t>50%</t>
         </is>
       </c>
       <c r="R69" s="6" t="inlineStr">
         <is>
-          <t>정정</t>
+          <t>발행조건확정</t>
         </is>
       </c>
     </row>
     <row r="70" ht="30" customHeight="1">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>영광</t>
+          <t>아이엠스팩1호</t>
         </is>
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>10-13~10-19</t>
-        </is>
-      </c>
-      <c r="C70" s="6" t="inlineStr">
-        <is>
-          <t>14,000~17,000</t>
+          <t>10-19~10-20</t>
+        </is>
+      </c>
+      <c r="C70" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="D70" s="7" t="inlineStr">
         <is>
-          <t>2,260,000</t>
+          <t>5,000,000</t>
         </is>
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
-          <t>31,640,000,000</t>
-        </is>
-      </c>
-      <c r="F70" s="6" t="inlineStr">
-        <is>
-          <t>11.98배 (EV/EBITDA)</t>
+          <t>10,000,000,000</t>
+        </is>
+      </c>
+      <c r="F70" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="G70" s="6" t="inlineStr"/>
@@ -13632,26 +13648,26 @@
       <c r="I70" s="6" t="inlineStr"/>
       <c r="J70" s="6" t="inlineStr">
         <is>
-          <t>10-22~10-23</t>
+          <t>10-26~10-27</t>
         </is>
       </c>
       <c r="K70" s="6" t="inlineStr"/>
       <c r="L70" s="6" t="inlineStr"/>
       <c r="M70" s="6" t="inlineStr"/>
-      <c r="N70" s="6" t="inlineStr">
-        <is>
-          <t>한국투자증권</t>
+      <c r="N70" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="O70" s="6" t="inlineStr"/>
-      <c r="P70" s="7" t="inlineStr">
-        <is>
-          <t>977,676,000</t>
-        </is>
-      </c>
-      <c r="Q70" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="P70" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="Q70" s="6" t="inlineStr">
+        <is>
+          <t>3.00%</t>
         </is>
       </c>
       <c r="R70" s="6" t="inlineStr">
@@ -13663,32 +13679,32 @@
     <row r="71" ht="30" customHeight="1">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>아이엠스팩1호</t>
+          <t>옵토닉스</t>
         </is>
       </c>
       <c r="B71" s="6" t="inlineStr">
         <is>
-          <t>10-19~10-20</t>
-        </is>
-      </c>
-      <c r="C71" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>10-21~10-27</t>
+        </is>
+      </c>
+      <c r="C71" s="6" t="inlineStr">
+        <is>
+          <t>10,000~12,000</t>
         </is>
       </c>
       <c r="D71" s="7" t="inlineStr">
         <is>
-          <t>5,000,000</t>
+          <t>2,200,000</t>
         </is>
       </c>
       <c r="E71" s="7" t="inlineStr">
         <is>
-          <t>10,000,000,000</t>
-        </is>
-      </c>
-      <c r="F71" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>22,000,000,000</t>
+        </is>
+      </c>
+      <c r="F71" s="6" t="inlineStr">
+        <is>
+          <t>25.27배 (EV/EBITDA)</t>
         </is>
       </c>
       <c r="G71" s="6" t="inlineStr"/>
@@ -13696,26 +13712,26 @@
       <c r="I71" s="6" t="inlineStr"/>
       <c r="J71" s="6" t="inlineStr">
         <is>
-          <t>10-26~10-27</t>
+          <t>11-05~11-06</t>
         </is>
       </c>
       <c r="K71" s="6" t="inlineStr"/>
       <c r="L71" s="6" t="inlineStr"/>
       <c r="M71" s="6" t="inlineStr"/>
-      <c r="N71" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="N71" s="6" t="inlineStr">
+        <is>
+          <t>한국투자증권</t>
         </is>
       </c>
       <c r="O71" s="6" t="inlineStr"/>
-      <c r="P71" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="P71" s="7" t="inlineStr">
+        <is>
+          <t>1,133,000,000</t>
         </is>
       </c>
       <c r="Q71" s="6" t="inlineStr">
         <is>
-          <t>3.00%</t>
+          <t>5.0%</t>
         </is>
       </c>
       <c r="R71" s="6" t="inlineStr">
@@ -14047,59 +14063,59 @@
     <row r="77" ht="30" customHeight="1">
       <c r="A77" s="6" t="inlineStr">
         <is>
-          <t>바로팜</t>
-        </is>
-      </c>
-      <c r="B77" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>유캐스트</t>
+        </is>
+      </c>
+      <c r="B77" s="6" t="inlineStr">
+        <is>
+          <t>11-09~11-13</t>
         </is>
       </c>
       <c r="C77" s="6" t="inlineStr">
         <is>
-          <t>16,400~20,200</t>
+          <t>19,000~23,000</t>
         </is>
       </c>
       <c r="D77" s="7" t="inlineStr">
         <is>
-          <t>1,780,000</t>
+          <t>800,000</t>
         </is>
       </c>
       <c r="E77" s="7" t="inlineStr">
         <is>
-          <t>29,192,000,000</t>
+          <t>15,200,000,000</t>
         </is>
       </c>
       <c r="F77" s="6" t="inlineStr">
         <is>
-          <t>25.27배 (PER)</t>
+          <t>17.97배 (PER)</t>
         </is>
       </c>
       <c r="G77" s="6" t="inlineStr"/>
       <c r="H77" s="6" t="inlineStr"/>
       <c r="I77" s="6" t="inlineStr"/>
-      <c r="J77" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="J77" s="6" t="inlineStr">
+        <is>
+          <t>11-18~11-19</t>
         </is>
       </c>
       <c r="K77" s="6" t="inlineStr"/>
       <c r="L77" s="6" t="inlineStr"/>
       <c r="M77" s="6" t="inlineStr"/>
-      <c r="N77" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="N77" s="6" t="inlineStr">
+        <is>
+          <t>유진투자증권</t>
         </is>
       </c>
       <c r="O77" s="6" t="inlineStr"/>
-      <c r="P77" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="Q77" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="P77" s="7" t="inlineStr">
+        <is>
+          <t>1,065,920,000</t>
+        </is>
+      </c>
+      <c r="Q77" s="6" t="inlineStr">
+        <is>
+          <t>7.0%</t>
         </is>
       </c>
       <c r="R77" s="6" t="inlineStr">
@@ -14111,7 +14127,7 @@
     <row r="78" ht="30" customHeight="1">
       <c r="A78" s="6" t="inlineStr">
         <is>
-          <t>셀트릭스</t>
+          <t>바로팜</t>
         </is>
       </c>
       <c r="B78" s="18" t="inlineStr">
@@ -14119,24 +14135,24 @@
           <t>수집예정</t>
         </is>
       </c>
-      <c r="C78" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="D78" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="E78" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="F78" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="C78" s="6" t="inlineStr">
+        <is>
+          <t>16,400~20,200</t>
+        </is>
+      </c>
+      <c r="D78" s="7" t="inlineStr">
+        <is>
+          <t>1,780,000</t>
+        </is>
+      </c>
+      <c r="E78" s="7" t="inlineStr">
+        <is>
+          <t>29,192,000,000</t>
+        </is>
+      </c>
+      <c r="F78" s="6" t="inlineStr">
+        <is>
+          <t>25.27배 (PER)</t>
         </is>
       </c>
       <c r="G78" s="6" t="inlineStr"/>
@@ -14175,7 +14191,7 @@
     <row r="79" ht="30" customHeight="1">
       <c r="A79" s="6" t="inlineStr">
         <is>
-          <t>럭스코</t>
+          <t>셀트릭스</t>
         </is>
       </c>
       <c r="B79" s="18" t="inlineStr">
@@ -14239,7 +14255,7 @@
     <row r="80" ht="30" customHeight="1">
       <c r="A80" s="6" t="inlineStr">
         <is>
-          <t>솔리스</t>
+          <t>럭스코</t>
         </is>
       </c>
       <c r="B80" s="18" t="inlineStr">
@@ -14303,64 +14319,64 @@
     <row r="81" ht="30" customHeight="1">
       <c r="A81" s="6" t="inlineStr">
         <is>
-          <t>옵토닉스</t>
-        </is>
-      </c>
-      <c r="B81" s="6" t="inlineStr">
-        <is>
-          <t>10-21~10-27</t>
-        </is>
-      </c>
-      <c r="C81" s="6" t="inlineStr">
-        <is>
-          <t>10,000~12,000</t>
-        </is>
-      </c>
-      <c r="D81" s="7" t="inlineStr">
-        <is>
-          <t>2,200,000</t>
-        </is>
-      </c>
-      <c r="E81" s="7" t="inlineStr">
-        <is>
-          <t>22,000,000,000</t>
-        </is>
-      </c>
-      <c r="F81" s="6" t="inlineStr">
-        <is>
-          <t>25.27배 (EV/EBITDA)</t>
+          <t>솔리스</t>
+        </is>
+      </c>
+      <c r="B81" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="C81" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="D81" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="E81" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="F81" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="G81" s="6" t="inlineStr"/>
       <c r="H81" s="6" t="inlineStr"/>
       <c r="I81" s="6" t="inlineStr"/>
-      <c r="J81" s="6" t="inlineStr">
-        <is>
-          <t>11-05~11-06</t>
+      <c r="J81" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="K81" s="6" t="inlineStr"/>
       <c r="L81" s="6" t="inlineStr"/>
       <c r="M81" s="6" t="inlineStr"/>
-      <c r="N81" s="6" t="inlineStr">
-        <is>
-          <t>한국투자증권</t>
+      <c r="N81" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="O81" s="6" t="inlineStr"/>
-      <c r="P81" s="7" t="inlineStr">
-        <is>
-          <t>1,133,000,000</t>
-        </is>
-      </c>
-      <c r="Q81" s="6" t="inlineStr">
-        <is>
-          <t>5.0%</t>
+      <c r="P81" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="Q81" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="R81" s="6" t="inlineStr">
         <is>
-          <t>최초</t>
+          <t>정정</t>
         </is>
       </c>
     </row>
@@ -14883,59 +14899,59 @@
     <row r="90" ht="30" customHeight="1">
       <c r="A90" s="6" t="inlineStr">
         <is>
-          <t>씨앤엠</t>
-        </is>
-      </c>
-      <c r="B90" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>이노보테라퓨틱스</t>
+        </is>
+      </c>
+      <c r="B90" s="6" t="inlineStr">
+        <is>
+          <t>11-26~12-02</t>
         </is>
       </c>
       <c r="C90" s="6" t="inlineStr">
         <is>
-          <t>10,000~13,000</t>
+          <t>20,000~24,000</t>
         </is>
       </c>
       <c r="D90" s="7" t="inlineStr">
         <is>
-          <t>2,950,000</t>
+          <t>2,200,000</t>
         </is>
       </c>
       <c r="E90" s="7" t="inlineStr">
         <is>
-          <t>29,500,000,000</t>
+          <t>44,000,000,000</t>
         </is>
       </c>
       <c r="F90" s="6" t="inlineStr">
         <is>
-          <t>24.96배 (PER)</t>
+          <t>25.53배 (PER)</t>
         </is>
       </c>
       <c r="G90" s="6" t="inlineStr"/>
       <c r="H90" s="6" t="inlineStr"/>
       <c r="I90" s="6" t="inlineStr"/>
-      <c r="J90" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="J90" s="6" t="inlineStr">
+        <is>
+          <t>12-07~12-08</t>
         </is>
       </c>
       <c r="K90" s="6" t="inlineStr"/>
       <c r="L90" s="6" t="inlineStr"/>
       <c r="M90" s="6" t="inlineStr"/>
-      <c r="N90" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="N90" s="6" t="inlineStr">
+        <is>
+          <t>한국투자증권</t>
         </is>
       </c>
       <c r="O90" s="6" t="inlineStr"/>
-      <c r="P90" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="Q90" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="P90" s="7" t="inlineStr">
+        <is>
+          <t>2,025,000,000</t>
+        </is>
+      </c>
+      <c r="Q90" s="6" t="inlineStr">
+        <is>
+          <t>4.5%</t>
         </is>
       </c>
       <c r="R90" s="6" t="inlineStr">
@@ -14947,7 +14963,7 @@
     <row r="91" ht="30" customHeight="1">
       <c r="A91" s="6" t="inlineStr">
         <is>
-          <t>씨아이에스케미칼</t>
+          <t>씨앤엠</t>
         </is>
       </c>
       <c r="B91" s="18" t="inlineStr">
@@ -14957,22 +14973,22 @@
       </c>
       <c r="C91" s="6" t="inlineStr">
         <is>
-          <t>5,400~6,800</t>
+          <t>10,000~13,000</t>
         </is>
       </c>
       <c r="D91" s="7" t="inlineStr">
         <is>
-          <t>4,000,000</t>
+          <t>2,950,000</t>
         </is>
       </c>
       <c r="E91" s="7" t="inlineStr">
         <is>
-          <t>21,600,000,000</t>
+          <t>29,500,000,000</t>
         </is>
       </c>
       <c r="F91" s="6" t="inlineStr">
         <is>
-          <t>21.24배 (PER)</t>
+          <t>24.96배 (PER)</t>
         </is>
       </c>
       <c r="G91" s="6" t="inlineStr"/>
@@ -15011,7 +15027,7 @@
     <row r="92" ht="30" customHeight="1">
       <c r="A92" s="6" t="inlineStr">
         <is>
-          <t>(주)태석광학</t>
+          <t>씨아이에스케미칼</t>
         </is>
       </c>
       <c r="B92" s="18" t="inlineStr">
@@ -15019,24 +15035,24 @@
           <t>수집예정</t>
         </is>
       </c>
-      <c r="C92" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="D92" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="E92" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="F92" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="C92" s="6" t="inlineStr">
+        <is>
+          <t>5,400~6,800</t>
+        </is>
+      </c>
+      <c r="D92" s="7" t="inlineStr">
+        <is>
+          <t>4,000,000</t>
+        </is>
+      </c>
+      <c r="E92" s="7" t="inlineStr">
+        <is>
+          <t>21,600,000,000</t>
+        </is>
+      </c>
+      <c r="F92" s="6" t="inlineStr">
+        <is>
+          <t>21.24배 (PER)</t>
         </is>
       </c>
       <c r="G92" s="6" t="inlineStr"/>
@@ -15068,14 +15084,14 @@
       </c>
       <c r="R92" s="6" t="inlineStr">
         <is>
-          <t>corp_code 미확보(수동확인)</t>
+          <t>최초</t>
         </is>
       </c>
     </row>
     <row r="93" ht="30" customHeight="1">
       <c r="A93" s="6" t="inlineStr">
         <is>
-          <t>신영스팩12호</t>
+          <t>(주)태석광학</t>
         </is>
       </c>
       <c r="B93" s="18" t="inlineStr">
@@ -15139,7 +15155,7 @@
     <row r="94" ht="30" customHeight="1">
       <c r="A94" s="6" t="inlineStr">
         <is>
-          <t>디티에스</t>
+          <t>신영스팩12호</t>
         </is>
       </c>
       <c r="B94" s="18" t="inlineStr">
@@ -15196,14 +15212,14 @@
       </c>
       <c r="R94" s="6" t="inlineStr">
         <is>
-          <t>신고서 대기</t>
+          <t>corp_code 미확보(수동확인)</t>
         </is>
       </c>
     </row>
     <row r="95" ht="30" customHeight="1">
       <c r="A95" s="6" t="inlineStr">
         <is>
-          <t>이에스티</t>
+          <t>디티에스</t>
         </is>
       </c>
       <c r="B95" s="18" t="inlineStr">
@@ -15267,7 +15283,7 @@
     <row r="96" ht="30" customHeight="1">
       <c r="A96" s="6" t="inlineStr">
         <is>
-          <t>우리투자제1호스팩</t>
+          <t>이에스티</t>
         </is>
       </c>
       <c r="B96" s="18" t="inlineStr">
@@ -15331,7 +15347,7 @@
     <row r="97" ht="30" customHeight="1">
       <c r="A97" s="6" t="inlineStr">
         <is>
-          <t>마더스제약</t>
+          <t>우리투자제1호스팩</t>
         </is>
       </c>
       <c r="B97" s="18" t="inlineStr">
@@ -15395,7 +15411,7 @@
     <row r="98" ht="30" customHeight="1">
       <c r="A98" s="6" t="inlineStr">
         <is>
-          <t>케이티이</t>
+          <t>마더스제약</t>
         </is>
       </c>
       <c r="B98" s="18" t="inlineStr">
@@ -15459,7 +15475,7 @@
     <row r="99" ht="30" customHeight="1">
       <c r="A99" s="6" t="inlineStr">
         <is>
-          <t>데스틴파워</t>
+          <t>케이티이</t>
         </is>
       </c>
       <c r="B99" s="18" t="inlineStr">
@@ -15523,7 +15539,7 @@
     <row r="100" ht="30" customHeight="1">
       <c r="A100" s="6" t="inlineStr">
         <is>
-          <t>인터엑스</t>
+          <t>데스틴파워</t>
         </is>
       </c>
       <c r="B100" s="18" t="inlineStr">
@@ -15587,7 +15603,7 @@
     <row r="101" ht="30" customHeight="1">
       <c r="A101" s="6" t="inlineStr">
         <is>
-          <t>이노보테라퓨틱스</t>
+          <t>인터엑스</t>
         </is>
       </c>
       <c r="B101" s="18" t="inlineStr">
@@ -16178,30 +16194,30 @@
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>삼성증권</t>
+          <t>한국투자증권</t>
         </is>
       </c>
       <c r="B21" s="6" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>284,014,000,000</t>
+          <t>307,720,000,000</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>한국투자증권</t>
+          <t>삼성증권</t>
         </is>
       </c>
       <c r="B22" s="6" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>256,940,000,000</t>
+          <t>284,014,000,000</t>
         </is>
       </c>
     </row>
@@ -16276,7 +16292,7 @@
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>74,400,000,000</t>
+          <t>72,800,000,000</t>
         </is>
       </c>
     </row>

</xml_diff>